<commit_message>
Adiciona Procfile e runtime.txt para deploy
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1284" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E71837B-B8AE-4205-AAB6-E409BB9F6695}"/>
+  <xr:revisionPtr revIDLastSave="1297" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{059BBA56-177A-4633-A0D8-C9B286ACB5B3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$288</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$294</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1425" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="245">
   <si>
     <t>DATA</t>
   </si>
@@ -8620,7 +8620,9 @@
       </c>
       <c r="K288" s="9"/>
       <c r="L288" s="4"/>
-      <c r="M288" s="4"/>
+      <c r="M288" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N288" s="6">
         <v>3</v>
       </c>
@@ -8635,10 +8637,18 @@
       <c r="I289" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="J289" s="4"/>
-      <c r="K289" s="9"/>
-      <c r="L289" s="4"/>
-      <c r="M289" s="4"/>
+      <c r="J289" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K289" s="9">
+        <v>200</v>
+      </c>
+      <c r="L289" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="M289" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N289" s="6">
         <v>2</v>
       </c>
@@ -8698,7 +8708,9 @@
       <c r="J292" s="4"/>
       <c r="K292" s="9"/>
       <c r="L292" s="4"/>
-      <c r="M292" s="4"/>
+      <c r="M292" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N292" s="6">
         <v>2</v>
       </c>
@@ -8713,10 +8725,18 @@
       <c r="I293" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="J293" s="4"/>
-      <c r="K293" s="9"/>
-      <c r="L293" s="4"/>
-      <c r="M293" s="4"/>
+      <c r="J293" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="K293" s="9">
+        <v>160</v>
+      </c>
+      <c r="L293" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M293" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N293" s="6">
         <v>4</v>
       </c>
@@ -8736,7 +8756,9 @@
       </c>
       <c r="K294" s="9"/>
       <c r="L294" s="4"/>
-      <c r="M294" s="4"/>
+      <c r="M294" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N294" s="6">
         <v>1</v>
       </c>
@@ -8765,7 +8787,7 @@
       <c r="M302" s="20"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N288" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:N294" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2025" month="10" day="6" dateTimeGrouping="day"/>

</xml_diff>

<commit_message>
Dependências testadas localmente — compatíveis com Render
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1297" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{059BBA56-177A-4633-A0D8-C9B286ACB5B3}"/>
+  <xr:revisionPtr revIDLastSave="1298" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF32D39D-A310-4AAB-A93C-E7BB425A1FBD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="245">
   <si>
     <t>DATA</t>
   </si>
@@ -8705,7 +8705,9 @@
       <c r="I292" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="J292" s="4"/>
+      <c r="J292" s="4" t="s">
+        <v>71</v>
+      </c>
       <c r="K292" s="9"/>
       <c r="L292" s="4"/>
       <c r="M292" s="4" t="s">

</xml_diff>

<commit_message>
Adiciona setuptools e wheel para compatibilidade no Render
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1298" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF32D39D-A310-4AAB-A93C-E7BB425A1FBD}"/>
+  <xr:revisionPtr revIDLastSave="1310" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06537F08-80EA-4E1B-9BE3-481AFAFE9EE7}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1435" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="246">
   <si>
     <t>DATA</t>
   </si>
@@ -773,6 +773,9 @@
   </si>
   <si>
     <t>HOTEL FELICIDADE</t>
+  </si>
+  <si>
+    <t>LEGALOP</t>
   </si>
 </sst>
 </file>
@@ -8423,7 +8426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="281" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G281" s="3">
         <v>45936</v>
       </c>
@@ -8449,7 +8452,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="282" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="282" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G282" s="3">
         <v>45936</v>
       </c>
@@ -8475,7 +8478,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="283" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="283" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G283" s="3">
         <v>45936</v>
       </c>
@@ -8501,7 +8504,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="284" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="284" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G284" s="3">
         <v>45936</v>
       </c>
@@ -8527,7 +8530,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="285" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="285" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G285" s="3">
         <v>45936</v>
       </c>
@@ -8553,7 +8556,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="286" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="286" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G286" s="3">
         <v>45936</v>
       </c>
@@ -8579,7 +8582,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="287" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="287" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G287" s="3">
         <v>45936</v>
       </c>
@@ -8618,8 +8621,12 @@
       <c r="J288" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K288" s="9"/>
-      <c r="L288" s="4"/>
+      <c r="K288" s="9">
+        <v>140</v>
+      </c>
+      <c r="L288" s="4" t="s">
+        <v>245</v>
+      </c>
       <c r="M288" s="4" t="s">
         <v>8</v>
       </c>
@@ -8664,7 +8671,7 @@
         <v>147</v>
       </c>
       <c r="J290" s="4" t="s">
-        <v>105</v>
+        <v>186</v>
       </c>
       <c r="K290" s="9"/>
       <c r="L290" s="4"/>
@@ -8708,8 +8715,12 @@
       <c r="J292" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="K292" s="9"/>
-      <c r="L292" s="4"/>
+      <c r="K292" s="9">
+        <v>280</v>
+      </c>
+      <c r="L292" s="4" t="s">
+        <v>62</v>
+      </c>
       <c r="M292" s="4" t="s">
         <v>8</v>
       </c>
@@ -8792,7 +8803,6 @@
   <autoFilter ref="G5:N294" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="10" day="6" dateTimeGrouping="day"/>
         <dateGroupItem year="2025" month="10" day="7" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Corrige versão do Python para 3.12.4 no runtime.txt
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1310" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06537F08-80EA-4E1B-9BE3-481AFAFE9EE7}"/>
+  <xr:revisionPtr revIDLastSave="1315" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DA88DB1-F3F7-4DEE-981A-0E19305D221E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1437" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="247">
   <si>
     <t>DATA</t>
   </si>
@@ -776,6 +776,9 @@
   </si>
   <si>
     <t>LEGALOP</t>
+  </si>
+  <si>
+    <t>HOTEL MARIO ARMANDO</t>
   </si>
 </sst>
 </file>
@@ -8673,8 +8676,12 @@
       <c r="J290" s="4" t="s">
         <v>186</v>
       </c>
-      <c r="K290" s="9"/>
-      <c r="L290" s="4"/>
+      <c r="K290" s="9">
+        <v>179.9</v>
+      </c>
+      <c r="L290" s="4" t="s">
+        <v>246</v>
+      </c>
       <c r="M290" s="4" t="s">
         <v>8</v>
       </c>
@@ -8692,9 +8699,15 @@
       <c r="I291" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="J291" s="4"/>
-      <c r="K291" s="9"/>
-      <c r="L291" s="4"/>
+      <c r="J291" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="K291" s="9">
+        <v>200</v>
+      </c>
+      <c r="L291" s="4" t="s">
+        <v>184</v>
+      </c>
       <c r="M291" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Atualiza planilha de dados e ajustes no dashboard
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1315" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9DA88DB1-F3F7-4DEE-981A-0E19305D221E}"/>
+  <xr:revisionPtr revIDLastSave="1318" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D072A378-B193-4403-8283-AEFB3FD951A8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1440" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="247">
   <si>
     <t>DATA</t>
   </si>
@@ -8778,10 +8778,14 @@
         <v>197</v>
       </c>
       <c r="J294" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K294" s="9"/>
-      <c r="L294" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="K294" s="9">
+        <v>220</v>
+      </c>
+      <c r="L294" s="4" t="s">
+        <v>205</v>
+      </c>
       <c r="M294" s="4" t="s">
         <v>8</v>
       </c>

</xml_diff>

<commit_message>
Atualiza app.py, planilha e páginas HTML
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1318" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D072A378-B193-4403-8283-AEFB3FD951A8}"/>
+  <xr:revisionPtr revIDLastSave="1353" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29599A41-A61D-48FB-B93E-D0AC35753B0F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$302</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1457" uniqueCount="247">
   <si>
     <t>DATA</t>
   </si>
@@ -932,7 +932,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1273,7 +1273,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:O302"/>
+  <dimension ref="G5:O315"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -8611,7 +8611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="288" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G288" s="3">
         <v>45937</v>
       </c>
@@ -8637,7 +8637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="289" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G289" s="3">
         <v>45937</v>
       </c>
@@ -8663,7 +8663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="290" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="290" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G290" s="3">
         <v>45937</v>
       </c>
@@ -8689,7 +8689,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="291" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="291" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G291" s="3">
         <v>45937</v>
       </c>
@@ -8715,7 +8715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="292" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="292" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G292" s="3">
         <v>45937</v>
       </c>
@@ -8741,7 +8741,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="293" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="293" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G293" s="3">
         <v>45937</v>
       </c>
@@ -8767,7 +8767,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="294" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="294" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G294" s="3">
         <v>45937</v>
       </c>
@@ -8794,33 +8794,284 @@
       </c>
     </row>
     <row r="295" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G295" s="3"/>
-      <c r="H295" s="4"/>
-      <c r="I295" s="6"/>
+      <c r="G295" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H295" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I295" s="6" t="s">
+        <v>155</v>
+      </c>
       <c r="J295" s="4"/>
       <c r="K295" s="9"/>
       <c r="L295" s="4"/>
       <c r="M295" s="4"/>
-      <c r="N295" s="6"/>
+      <c r="N295" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="296" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G296" s="3"/>
-      <c r="H296" s="4"/>
-      <c r="I296" s="6"/>
+      <c r="G296" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H296" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I296" s="6" t="s">
+        <v>147</v>
+      </c>
       <c r="J296" s="4"/>
-      <c r="K296" s="9"/>
+      <c r="K296" s="4"/>
       <c r="L296" s="4"/>
       <c r="M296" s="4"/>
-      <c r="N296" s="6"/>
+      <c r="N296" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="297" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G297" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H297" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="I297" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="J297" s="4"/>
+      <c r="K297" s="4"/>
+      <c r="L297" s="4"/>
+      <c r="M297" s="4"/>
+      <c r="N297" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="298" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G298" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H298" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I298" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="J298" s="4"/>
+      <c r="K298" s="9"/>
+      <c r="L298" s="4"/>
+      <c r="M298" s="4"/>
+      <c r="N298" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="299" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G299" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H299" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="I299" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="J299" s="4"/>
+      <c r="K299" s="9"/>
+      <c r="L299" s="4"/>
+      <c r="M299" s="4"/>
+      <c r="N299" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="300" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G300" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H300" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I300" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="J300" s="4"/>
+      <c r="K300" s="9"/>
+      <c r="L300" s="4"/>
+      <c r="M300" s="4"/>
+      <c r="N300" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="301" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G301" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H301" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="I301" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="J301" s="4"/>
+      <c r="K301" s="9"/>
+      <c r="L301" s="4"/>
+      <c r="M301" s="4"/>
+      <c r="N301" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="302" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G302" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H302" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="I302" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="J302" s="4"/>
+      <c r="K302" s="9"/>
+      <c r="L302" s="4"/>
       <c r="M302" s="20"/>
+      <c r="N302" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="303" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G303" s="4"/>
+      <c r="H303" s="4"/>
+      <c r="I303" s="6"/>
+      <c r="J303" s="4"/>
+      <c r="K303" s="9"/>
+      <c r="L303" s="4"/>
+      <c r="M303" s="4"/>
+      <c r="N303" s="6"/>
+    </row>
+    <row r="304" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G304" s="4"/>
+      <c r="H304" s="4"/>
+      <c r="I304" s="6"/>
+      <c r="J304" s="4"/>
+      <c r="K304" s="9"/>
+      <c r="L304" s="4"/>
+      <c r="M304" s="4"/>
+      <c r="N304" s="6"/>
+    </row>
+    <row r="305" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G305" s="4"/>
+      <c r="H305" s="4"/>
+      <c r="I305" s="6"/>
+      <c r="J305" s="4"/>
+      <c r="K305" s="9"/>
+      <c r="L305" s="4"/>
+      <c r="M305" s="4"/>
+      <c r="N305" s="6"/>
+    </row>
+    <row r="306" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G306" s="4"/>
+      <c r="H306" s="4"/>
+      <c r="I306" s="6"/>
+      <c r="J306" s="4"/>
+      <c r="K306" s="9"/>
+      <c r="L306" s="4"/>
+      <c r="M306" s="4"/>
+      <c r="N306" s="6"/>
+    </row>
+    <row r="307" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G307" s="4"/>
+      <c r="H307" s="4"/>
+      <c r="I307" s="6"/>
+      <c r="J307" s="4"/>
+      <c r="K307" s="9"/>
+      <c r="L307" s="4"/>
+      <c r="M307" s="4"/>
+      <c r="N307" s="6"/>
+    </row>
+    <row r="308" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G308" s="4"/>
+      <c r="H308" s="4"/>
+      <c r="I308" s="6"/>
+      <c r="J308" s="4"/>
+      <c r="K308" s="9"/>
+      <c r="L308" s="4"/>
+      <c r="M308" s="4"/>
+      <c r="N308" s="6"/>
+    </row>
+    <row r="309" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G309" s="4"/>
+      <c r="H309" s="4"/>
+      <c r="I309" s="6"/>
+      <c r="J309" s="4"/>
+      <c r="K309" s="9"/>
+      <c r="L309" s="4"/>
+      <c r="M309" s="4"/>
+      <c r="N309" s="6"/>
+    </row>
+    <row r="310" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G310" s="4"/>
+      <c r="H310" s="4"/>
+      <c r="I310" s="6"/>
+      <c r="J310" s="4"/>
+      <c r="K310" s="9"/>
+      <c r="L310" s="4"/>
+      <c r="M310" s="4"/>
+      <c r="N310" s="6"/>
+    </row>
+    <row r="311" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G311" s="4"/>
+      <c r="H311" s="4"/>
+      <c r="I311" s="6"/>
+      <c r="J311" s="4"/>
+      <c r="K311" s="9"/>
+      <c r="L311" s="4"/>
+      <c r="M311" s="4"/>
+      <c r="N311" s="6"/>
+    </row>
+    <row r="312" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G312" s="4"/>
+      <c r="H312" s="4"/>
+      <c r="I312" s="6"/>
+      <c r="J312" s="4"/>
+      <c r="K312" s="9"/>
+      <c r="L312" s="4"/>
+      <c r="M312" s="4"/>
+      <c r="N312" s="6"/>
+    </row>
+    <row r="313" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G313" s="4"/>
+      <c r="H313" s="4"/>
+      <c r="I313" s="6"/>
+      <c r="J313" s="4"/>
+      <c r="K313" s="9"/>
+      <c r="L313" s="4"/>
+      <c r="M313" s="4"/>
+      <c r="N313" s="6"/>
+    </row>
+    <row r="314" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G314" s="4"/>
+      <c r="H314" s="4"/>
+      <c r="I314" s="6"/>
+      <c r="J314" s="4"/>
+      <c r="K314" s="9"/>
+      <c r="L314" s="4"/>
+      <c r="M314" s="4"/>
+      <c r="N314" s="6"/>
+    </row>
+    <row r="315" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G315" s="4"/>
+      <c r="H315" s="4"/>
+      <c r="I315" s="6"/>
+      <c r="J315" s="4"/>
+      <c r="K315" s="9"/>
+      <c r="L315" s="4"/>
+      <c r="M315" s="4"/>
+      <c r="N315" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N294" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:N302" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="10" day="7" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="10" day="8" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-08 12:32
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1357" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{63CC10C0-96A9-4905-9476-14CAA7463DD2}"/>
+  <xr:revisionPtr revIDLastSave="1364" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5F85806-09B3-4E24-9BDF-4AB0900C819A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="248">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="246">
   <si>
     <t>DATA</t>
   </si>
@@ -751,9 +751,6 @@
     <t>HOTEL PLAZARO</t>
   </si>
   <si>
-    <t>pix</t>
-  </si>
-  <si>
     <t>IBIA</t>
   </si>
   <si>
@@ -779,9 +776,6 @@
   </si>
   <si>
     <t>HOTEL MARIO ARMANDO</t>
-  </si>
-  <si>
-    <t>HOTEL COSTA E FILHO</t>
   </si>
 </sst>
 </file>
@@ -1273,7 +1267,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-  <sheetPr codeName="Planilha1" filterMode="1">
+  <sheetPr codeName="Planilha1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="G5:O315"/>
@@ -1316,7 +1310,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>45873</v>
       </c>
@@ -1342,7 +1336,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>45873</v>
       </c>
@@ -1368,7 +1362,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>45873</v>
       </c>
@@ -1394,7 +1388,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>45873</v>
       </c>
@@ -1420,7 +1414,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>45875</v>
       </c>
@@ -1446,7 +1440,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>45875</v>
       </c>
@@ -1472,7 +1466,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>45875</v>
       </c>
@@ -1498,7 +1492,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>45875</v>
       </c>
@@ -1524,7 +1518,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>45875</v>
       </c>
@@ -1550,7 +1544,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>45875</v>
       </c>
@@ -1576,7 +1570,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>45875</v>
       </c>
@@ -1602,7 +1596,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>45875</v>
       </c>
@@ -1628,7 +1622,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>45876</v>
       </c>
@@ -1654,7 +1648,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>45876</v>
       </c>
@@ -1680,7 +1674,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>45876</v>
       </c>
@@ -1706,7 +1700,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>45876</v>
       </c>
@@ -1732,7 +1726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
         <v>45876</v>
       </c>
@@ -1758,7 +1752,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
         <v>45876</v>
       </c>
@@ -1784,7 +1778,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
         <v>45876</v>
       </c>
@@ -1810,7 +1804,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
         <v>45876</v>
       </c>
@@ -1836,7 +1830,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
         <v>45876</v>
       </c>
@@ -1862,7 +1856,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
         <v>45876</v>
       </c>
@@ -1888,7 +1882,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>45876</v>
       </c>
@@ -1914,7 +1908,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
         <v>45880</v>
       </c>
@@ -1940,7 +1934,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
         <v>45880</v>
       </c>
@@ -1966,7 +1960,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
         <v>45880</v>
       </c>
@@ -1992,7 +1986,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
         <v>45880</v>
       </c>
@@ -2018,7 +2012,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
         <v>45880</v>
       </c>
@@ -2044,7 +2038,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G34" s="3">
         <v>45881</v>
       </c>
@@ -2070,7 +2064,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G35" s="3">
         <v>45881</v>
       </c>
@@ -2096,7 +2090,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>45881</v>
       </c>
@@ -2122,7 +2116,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G37" s="3">
         <v>45881</v>
       </c>
@@ -2148,7 +2142,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G38" s="3">
         <v>45881</v>
       </c>
@@ -2174,7 +2168,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G39" s="3">
         <v>45881</v>
       </c>
@@ -2200,7 +2194,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G40" s="3">
         <v>45881</v>
       </c>
@@ -2226,7 +2220,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G41" s="3">
         <v>45882</v>
       </c>
@@ -2252,7 +2246,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G42" s="3">
         <v>45882</v>
       </c>
@@ -2278,7 +2272,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G43" s="3">
         <v>45882</v>
       </c>
@@ -2304,7 +2298,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G44" s="3">
         <v>45882</v>
       </c>
@@ -2330,7 +2324,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G45" s="3">
         <v>45882</v>
       </c>
@@ -2356,7 +2350,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G46" s="3">
         <v>45882</v>
       </c>
@@ -2380,7 +2374,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G47" s="3">
         <v>45883</v>
       </c>
@@ -2406,7 +2400,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G48" s="3">
         <v>45883</v>
       </c>
@@ -2432,7 +2426,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G49" s="3">
         <v>45883</v>
       </c>
@@ -2456,7 +2450,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G50" s="3">
         <v>45883</v>
       </c>
@@ -2482,7 +2476,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G51" s="3">
         <v>45883</v>
       </c>
@@ -2508,7 +2502,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G52" s="3">
         <v>45883</v>
       </c>
@@ -2534,7 +2528,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G53" s="3">
         <v>45883</v>
       </c>
@@ -2560,7 +2554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G54" s="3">
         <v>45883</v>
       </c>
@@ -2586,7 +2580,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G55" s="3">
         <v>45883</v>
       </c>
@@ -2612,7 +2606,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G56" s="3">
         <v>45883</v>
       </c>
@@ -2638,7 +2632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G57" s="3">
         <v>45883</v>
       </c>
@@ -2664,7 +2658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G58" s="3">
         <v>45883</v>
       </c>
@@ -2690,7 +2684,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G59" s="3">
         <v>45883</v>
       </c>
@@ -2716,7 +2710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G60" s="3">
         <v>45883</v>
       </c>
@@ -2742,7 +2736,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G61" s="3">
         <v>45883</v>
       </c>
@@ -2768,7 +2762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G62" s="3">
         <v>45883</v>
       </c>
@@ -2794,7 +2788,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>45887</v>
       </c>
@@ -2820,7 +2814,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G64" s="3">
         <v>45887</v>
       </c>
@@ -2846,7 +2840,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G65" s="3">
         <v>45887</v>
       </c>
@@ -2872,7 +2866,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G66" s="3">
         <v>45887</v>
       </c>
@@ -2898,7 +2892,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G67" s="3">
         <v>45887</v>
       </c>
@@ -2924,7 +2918,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G68" s="3">
         <v>45887</v>
       </c>
@@ -2950,7 +2944,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G69" s="3">
         <v>45887</v>
       </c>
@@ -2976,7 +2970,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G70" s="3">
         <v>45888</v>
       </c>
@@ -3002,7 +2996,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G71" s="3">
         <v>45888</v>
       </c>
@@ -3028,7 +3022,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>45888</v>
       </c>
@@ -3054,7 +3048,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G73" s="3">
         <v>45888</v>
       </c>
@@ -3080,7 +3074,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G74" s="3">
         <v>45888</v>
       </c>
@@ -3106,7 +3100,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G75" s="3">
         <v>45889</v>
       </c>
@@ -3132,7 +3126,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G76" s="3">
         <v>45889</v>
       </c>
@@ -3158,7 +3152,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G77" s="3">
         <v>45889</v>
       </c>
@@ -3184,7 +3178,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G78" s="3">
         <v>45889</v>
       </c>
@@ -3210,7 +3204,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G79" s="3">
         <v>45889</v>
       </c>
@@ -3236,7 +3230,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G80" s="3">
         <v>45889</v>
       </c>
@@ -3262,7 +3256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G81" s="3">
         <v>45889</v>
       </c>
@@ -3288,7 +3282,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G82" s="3">
         <v>45890</v>
       </c>
@@ -3314,7 +3308,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G83" s="3">
         <v>45890</v>
       </c>
@@ -3340,7 +3334,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G84" s="3">
         <v>45890</v>
       </c>
@@ -3366,7 +3360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G85" s="3">
         <v>45890</v>
       </c>
@@ -3392,7 +3386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G86" s="3">
         <v>45890</v>
       </c>
@@ -3418,7 +3412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G87" s="3">
         <v>45890</v>
       </c>
@@ -3444,7 +3438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G88" s="3">
         <v>45890</v>
       </c>
@@ -3470,7 +3464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G89" s="3">
         <v>45890</v>
       </c>
@@ -3496,7 +3490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G90" s="3">
         <v>45890</v>
       </c>
@@ -3522,7 +3516,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G91" s="3">
         <v>45890</v>
       </c>
@@ -3546,7 +3540,7 @@
       </c>
       <c r="N91" s="6"/>
     </row>
-    <row r="92" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G92" s="3">
         <v>45890</v>
       </c>
@@ -3572,7 +3566,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G93" s="3">
         <v>45894</v>
       </c>
@@ -3598,7 +3592,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G94" s="3">
         <v>45894</v>
       </c>
@@ -3624,7 +3618,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G95" s="3">
         <v>45894</v>
       </c>
@@ -3650,7 +3644,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G96" s="3">
         <v>45894</v>
       </c>
@@ -3676,7 +3670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G97" s="3">
         <v>45895</v>
       </c>
@@ -3702,7 +3696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G98" s="3">
         <v>45895</v>
       </c>
@@ -3728,7 +3722,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G99" s="3">
         <v>45895</v>
       </c>
@@ -3754,7 +3748,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G100" s="3">
         <v>45895</v>
       </c>
@@ -3780,7 +3774,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G101" s="3">
         <v>45895</v>
       </c>
@@ -3806,7 +3800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G102" s="3">
         <v>45895</v>
       </c>
@@ -3832,7 +3826,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G103" s="3">
         <v>45895</v>
       </c>
@@ -3858,7 +3852,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G104" s="3">
         <v>45896</v>
       </c>
@@ -3884,7 +3878,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G105" s="3">
         <v>45896</v>
       </c>
@@ -3910,7 +3904,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G106" s="3">
         <v>45896</v>
       </c>
@@ -3936,7 +3930,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G107" s="3">
         <v>45896</v>
       </c>
@@ -3962,7 +3956,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G108" s="3">
         <v>45896</v>
       </c>
@@ -3988,7 +3982,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G109" s="3">
         <v>45896</v>
       </c>
@@ -4014,7 +4008,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G110" s="3">
         <v>45896</v>
       </c>
@@ -4040,7 +4034,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G111" s="3">
         <v>45896</v>
       </c>
@@ -4066,7 +4060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G112" s="3">
         <v>45897</v>
       </c>
@@ -4092,7 +4086,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G113" s="3">
         <v>45897</v>
       </c>
@@ -4118,7 +4112,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G114" s="3">
         <v>45897</v>
       </c>
@@ -4144,7 +4138,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G115" s="3">
         <v>45897</v>
       </c>
@@ -4170,7 +4164,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G116" s="3">
         <v>45897</v>
       </c>
@@ -4196,7 +4190,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G117" s="3">
         <v>45897</v>
       </c>
@@ -4222,7 +4216,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G118" s="3">
         <v>45897</v>
       </c>
@@ -4241,12 +4235,14 @@
       <c r="L118" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="M118" s="4"/>
+      <c r="M118" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N118" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G119" s="3">
         <v>45897</v>
       </c>
@@ -4272,7 +4268,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="120" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G120" s="3">
         <v>45897</v>
       </c>
@@ -4298,7 +4294,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G121" s="3">
         <v>45897</v>
       </c>
@@ -4324,7 +4320,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G122" s="3">
         <v>45897</v>
       </c>
@@ -4350,7 +4346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G123" s="3">
         <v>45901</v>
       </c>
@@ -4376,7 +4372,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G124" s="3">
         <v>45901</v>
       </c>
@@ -4402,7 +4398,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G125" s="3">
         <v>45901</v>
       </c>
@@ -4428,7 +4424,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G126" s="3">
         <v>45901</v>
       </c>
@@ -4454,7 +4450,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G127" s="3">
         <v>45902</v>
       </c>
@@ -4480,7 +4476,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G128" s="3">
         <v>45902</v>
       </c>
@@ -4506,7 +4502,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G129" s="3">
         <v>45902</v>
       </c>
@@ -4532,7 +4528,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G130" s="3">
         <v>45902</v>
       </c>
@@ -4558,7 +4554,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G131" s="3">
         <v>45902</v>
       </c>
@@ -4584,7 +4580,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G132" s="3">
         <v>45902</v>
       </c>
@@ -4610,7 +4606,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G133" s="3">
         <v>45902</v>
       </c>
@@ -4636,7 +4632,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G134" s="3">
         <v>45903</v>
       </c>
@@ -4662,7 +4658,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G135" s="3">
         <v>45903</v>
       </c>
@@ -4688,7 +4684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G136" s="3">
         <v>45903</v>
       </c>
@@ -4714,7 +4710,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G137" s="3">
         <v>45903</v>
       </c>
@@ -4740,7 +4736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G138" s="3">
         <v>45903</v>
       </c>
@@ -4766,7 +4762,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G139" s="3">
         <v>45903</v>
       </c>
@@ -4792,7 +4788,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G140" s="3">
         <v>45903</v>
       </c>
@@ -4816,7 +4812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G141" s="3">
         <v>45903</v>
       </c>
@@ -4842,7 +4838,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="142" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G142" s="3">
         <v>45903</v>
       </c>
@@ -4866,7 +4862,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G143" s="3">
         <v>45904</v>
       </c>
@@ -4892,7 +4888,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="144" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G144" s="3">
         <v>45904</v>
       </c>
@@ -4918,7 +4914,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="145" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G145" s="3">
         <v>45904</v>
       </c>
@@ -4944,7 +4940,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G146" s="3">
         <v>45904</v>
       </c>
@@ -4970,7 +4966,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G147" s="3">
         <v>45904</v>
       </c>
@@ -4996,7 +4992,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G148" s="3">
         <v>45904</v>
       </c>
@@ -5022,7 +5018,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
         <v>45904</v>
       </c>
@@ -5048,7 +5044,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G150" s="3">
         <v>45904</v>
       </c>
@@ -5074,7 +5070,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G151" s="3">
         <v>45904</v>
       </c>
@@ -5100,7 +5096,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G152" s="3">
         <v>45908</v>
       </c>
@@ -5126,7 +5122,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>45908</v>
       </c>
@@ -5152,7 +5148,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G154" s="3">
         <v>45908</v>
       </c>
@@ -5178,7 +5174,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="155" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G155" s="3">
         <v>45908</v>
       </c>
@@ -5204,7 +5200,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="156" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>45909</v>
       </c>
@@ -5230,7 +5226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="157" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G157" s="3">
         <v>45909</v>
       </c>
@@ -5256,7 +5252,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="158" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G158" s="3">
         <v>45909</v>
       </c>
@@ -5282,7 +5278,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="159" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G159" s="3">
         <v>45909</v>
       </c>
@@ -5308,7 +5304,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="160" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>45909</v>
       </c>
@@ -5334,7 +5330,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G161" s="3">
         <v>45909</v>
       </c>
@@ -5360,7 +5356,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G162" s="3">
         <v>45910</v>
       </c>
@@ -5386,7 +5382,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="163" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G163" s="3">
         <v>45910</v>
       </c>
@@ -5406,7 +5402,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="164" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G164" s="3">
         <v>45910</v>
       </c>
@@ -5432,7 +5428,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="165" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G165" s="3">
         <v>45910</v>
       </c>
@@ -5458,7 +5454,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G166" s="3">
         <v>45910</v>
       </c>
@@ -5484,7 +5480,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G167" s="3">
         <v>45910</v>
       </c>
@@ -5510,7 +5506,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G168" s="3">
         <v>45910</v>
       </c>
@@ -5536,7 +5532,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="169" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G169" s="3">
         <v>45911</v>
       </c>
@@ -5556,7 +5552,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G170" s="3">
         <v>45911</v>
       </c>
@@ -5582,7 +5578,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="171" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G171" s="3">
         <v>45911</v>
       </c>
@@ -5608,7 +5604,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G172" s="3">
         <v>45911</v>
       </c>
@@ -5634,7 +5630,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="173" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G173" s="3">
         <v>45911</v>
       </c>
@@ -5649,12 +5645,14 @@
       </c>
       <c r="K173" s="9"/>
       <c r="L173" s="4"/>
-      <c r="M173" s="4"/>
+      <c r="M173" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N173" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="174" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G174" s="3">
         <v>45911</v>
       </c>
@@ -5680,7 +5678,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G175" s="3">
         <v>45911</v>
       </c>
@@ -5706,7 +5704,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G176" s="3">
         <v>45911</v>
       </c>
@@ -5732,7 +5730,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="177" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
         <v>45911</v>
       </c>
@@ -5758,7 +5756,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
         <v>45911</v>
       </c>
@@ -5784,7 +5782,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="179" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
         <v>45911</v>
       </c>
@@ -5810,7 +5808,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="180" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
         <v>45911</v>
       </c>
@@ -5836,7 +5834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="181" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>45911</v>
       </c>
@@ -5862,7 +5860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>45915</v>
       </c>
@@ -5888,7 +5886,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="183" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>45915</v>
       </c>
@@ -5914,7 +5912,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="184" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>45915</v>
       </c>
@@ -5940,7 +5938,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G185" s="3">
         <v>45915</v>
       </c>
@@ -5966,7 +5964,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G186" s="3">
         <v>45915</v>
       </c>
@@ -5992,7 +5990,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G187" s="3">
         <v>45915</v>
       </c>
@@ -6018,7 +6016,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G188" s="3">
         <v>45915</v>
       </c>
@@ -6044,7 +6042,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G189" s="3">
         <v>45916</v>
       </c>
@@ -6070,7 +6068,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="190" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G190" s="3">
         <v>45916</v>
       </c>
@@ -6096,7 +6094,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G191" s="3">
         <v>45916</v>
       </c>
@@ -6122,7 +6120,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G192" s="3">
         <v>45916</v>
       </c>
@@ -6148,7 +6146,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="193" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G193" s="3">
         <v>45916</v>
       </c>
@@ -6174,7 +6172,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="194" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G194" s="3">
         <v>45917</v>
       </c>
@@ -6200,7 +6198,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="195" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G195" s="3">
         <v>45917</v>
       </c>
@@ -6226,7 +6224,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="196" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G196" s="3">
         <v>45917</v>
       </c>
@@ -6252,7 +6250,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G197" s="3">
         <v>45917</v>
       </c>
@@ -6278,7 +6276,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="198" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G198" s="3">
         <v>45917</v>
       </c>
@@ -6304,7 +6302,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="199" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G199" s="3">
         <v>45917</v>
       </c>
@@ -6330,7 +6328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G200" s="3">
         <v>45917</v>
       </c>
@@ -6356,7 +6354,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="201" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G201" s="3">
         <v>45918</v>
       </c>
@@ -6382,7 +6380,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="202" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G202" s="3">
         <v>45918</v>
       </c>
@@ -6408,7 +6406,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G203" s="3">
         <v>45918</v>
       </c>
@@ -6434,7 +6432,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G204" s="3">
         <v>45918</v>
       </c>
@@ -6460,7 +6458,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G205" s="3">
         <v>45918</v>
       </c>
@@ -6486,7 +6484,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G206" s="3">
         <v>45918</v>
       </c>
@@ -6512,7 +6510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G207" s="3">
         <v>45918</v>
       </c>
@@ -6538,7 +6536,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G208" s="3">
         <v>45918</v>
       </c>
@@ -6555,7 +6553,7 @@
         <v>230</v>
       </c>
       <c r="L208" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M208" s="4" t="s">
         <v>8</v>
@@ -6564,7 +6562,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G209" s="3">
         <v>45918</v>
       </c>
@@ -6590,7 +6588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G210" s="3">
         <v>45918</v>
       </c>
@@ -6616,7 +6614,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G211" s="3">
         <v>45918</v>
       </c>
@@ -6629,12 +6627,14 @@
       <c r="J211" s="4"/>
       <c r="K211" s="9"/>
       <c r="L211" s="4"/>
-      <c r="M211" s="4"/>
+      <c r="M211" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N211" s="6">
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G212" s="3">
         <v>45918</v>
       </c>
@@ -6660,7 +6660,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G213" s="3">
         <v>45918</v>
       </c>
@@ -6684,7 +6684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G214" s="3">
         <v>45922</v>
       </c>
@@ -6710,7 +6710,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="215" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G215" s="3">
         <v>45922</v>
       </c>
@@ -6736,7 +6736,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G216" s="3">
         <v>45922</v>
       </c>
@@ -6762,7 +6762,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G217" s="3">
         <v>45922</v>
       </c>
@@ -6788,7 +6788,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G218" s="3">
         <v>45922</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G219" s="3">
         <v>45922</v>
       </c>
@@ -6840,7 +6840,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="220" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G220" s="3">
         <v>45922</v>
       </c>
@@ -6866,7 +6866,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G221" s="3">
         <v>45923</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="222" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G222" s="3">
         <v>45923</v>
       </c>
@@ -6918,7 +6918,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G223" s="3">
         <v>45923</v>
       </c>
@@ -6944,7 +6944,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G224" s="3">
         <v>45923</v>
       </c>
@@ -6970,7 +6970,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="225" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G225" s="3">
         <v>45923</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="226" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G226" s="3">
         <v>45923</v>
       </c>
@@ -7022,7 +7022,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="227" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G227" s="3">
         <v>45924</v>
       </c>
@@ -7048,7 +7048,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="228" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G228" s="3">
         <v>45924</v>
       </c>
@@ -7074,7 +7074,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="229" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G229" s="3">
         <v>45924</v>
       </c>
@@ -7100,7 +7100,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="230" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G230" s="3">
         <v>45924</v>
       </c>
@@ -7126,7 +7126,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="231" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G231" s="3">
         <v>45924</v>
       </c>
@@ -7152,7 +7152,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="232" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G232" s="3">
         <v>45924</v>
       </c>
@@ -7178,7 +7178,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="233" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G233" s="3">
         <v>45924</v>
       </c>
@@ -7204,7 +7204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G234" s="3">
         <v>45924</v>
       </c>
@@ -7230,7 +7230,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G235" s="3">
         <v>45925</v>
       </c>
@@ -7256,7 +7256,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="236" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G236" s="3">
         <v>45925</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="237" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G237" s="3">
         <v>45925</v>
       </c>
@@ -7308,7 +7308,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G238" s="3">
         <v>45925</v>
       </c>
@@ -7334,7 +7334,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="239" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G239" s="3">
         <v>45925</v>
       </c>
@@ -7360,7 +7360,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="240" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G240" s="3">
         <v>45925</v>
       </c>
@@ -7386,7 +7386,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G241" s="3">
         <v>45925</v>
       </c>
@@ -7412,7 +7412,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G242" s="3">
         <v>45925</v>
       </c>
@@ -7438,7 +7438,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="243" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G243" s="3">
         <v>45925</v>
       </c>
@@ -7464,7 +7464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G244" s="3">
         <v>45925</v>
       </c>
@@ -7490,7 +7490,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="245" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G245" s="3">
         <v>45929</v>
       </c>
@@ -7516,7 +7516,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G246" s="3">
         <v>45925</v>
       </c>
@@ -7542,7 +7542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G247" s="3">
         <v>45929</v>
       </c>
@@ -7568,7 +7568,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="248" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G248" s="3">
         <v>45929</v>
       </c>
@@ -7594,7 +7594,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="249" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G249" s="3">
         <v>45929</v>
       </c>
@@ -7620,7 +7620,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="250" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G250" s="3">
         <v>45929</v>
       </c>
@@ -7646,7 +7646,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="251" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G251" s="3">
         <v>45929</v>
       </c>
@@ -7672,7 +7672,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="252" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G252" s="3">
         <v>45929</v>
       </c>
@@ -7698,7 +7698,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G253" s="3">
         <v>45930</v>
       </c>
@@ -7724,7 +7724,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="254" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G254" s="3">
         <v>45930</v>
       </c>
@@ -7750,7 +7750,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="255" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G255" s="3">
         <v>45930</v>
       </c>
@@ -7776,7 +7776,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="256" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G256" s="3">
         <v>45930</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="257" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G257" s="3">
         <v>45930</v>
       </c>
@@ -7828,7 +7828,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="258" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G258" s="3">
         <v>45930</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="259" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G259" s="3">
         <v>45931</v>
       </c>
@@ -7880,7 +7880,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="260" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G260" s="3">
         <v>45931</v>
       </c>
@@ -7906,7 +7906,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G261" s="3">
         <v>45931</v>
       </c>
@@ -7923,7 +7923,7 @@
         <v>210</v>
       </c>
       <c r="L261" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="M261" s="4" t="s">
         <v>8</v>
@@ -7932,7 +7932,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G262" s="3">
         <v>45931</v>
       </c>
@@ -7958,7 +7958,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="263" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G263" s="3">
         <v>45931</v>
       </c>
@@ -7984,7 +7984,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="264" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G264" s="3">
         <v>45931</v>
       </c>
@@ -8010,7 +8010,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="265" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G265" s="3">
         <v>45931</v>
       </c>
@@ -8036,7 +8036,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="266" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G266" s="3">
         <v>45931</v>
       </c>
@@ -8062,7 +8062,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="267" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G267" s="3">
         <v>45932</v>
       </c>
@@ -8088,7 +8088,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="268" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G268" s="3">
         <v>45932</v>
       </c>
@@ -8114,7 +8114,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="269" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G269" s="3">
         <v>45932</v>
       </c>
@@ -8140,7 +8140,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="270" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G270" s="3">
         <v>45932</v>
       </c>
@@ -8151,7 +8151,7 @@
         <v>151</v>
       </c>
       <c r="J270" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K270" s="9">
         <v>235</v>
@@ -8166,7 +8166,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="271" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G271" s="3">
         <v>45932</v>
       </c>
@@ -8191,11 +8191,8 @@
       <c r="N271" s="6">
         <v>2</v>
       </c>
-      <c r="O271" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="272" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="272" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G272" s="3">
         <v>45932</v>
       </c>
@@ -8212,7 +8209,7 @@
         <v>240</v>
       </c>
       <c r="L272" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="M272" s="4" t="s">
         <v>8</v>
@@ -8221,7 +8218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="273" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G273" s="3">
         <v>45932</v>
       </c>
@@ -8246,11 +8243,9 @@
       <c r="N273" s="6">
         <v>2</v>
       </c>
-      <c r="O273" s="19" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="274" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O273" s="19"/>
+    </row>
+    <row r="274" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G274" s="3">
         <v>45932</v>
       </c>
@@ -8276,7 +8271,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="275" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G275" s="3">
         <v>45932</v>
       </c>
@@ -8302,7 +8297,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="276" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G276" s="3">
         <v>45932</v>
       </c>
@@ -8328,7 +8323,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="277" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G277" s="3">
         <v>45932</v>
       </c>
@@ -8354,7 +8349,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="278" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G278" s="3">
         <v>45903</v>
       </c>
@@ -8380,7 +8375,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G279" s="3">
         <v>45933</v>
       </c>
@@ -8406,7 +8401,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="280" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="280" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G280" s="3">
         <v>45933</v>
       </c>
@@ -8432,7 +8427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="281" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G281" s="3">
         <v>45936</v>
       </c>
@@ -8458,12 +8453,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="282" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G282" s="3">
         <v>45936</v>
       </c>
       <c r="H282" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I282" s="6" t="s">
         <v>215</v>
@@ -8484,7 +8479,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="283" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G283" s="3">
         <v>45936</v>
       </c>
@@ -8510,7 +8505,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="284" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G284" s="3">
         <v>45936</v>
       </c>
@@ -8536,7 +8531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="285" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G285" s="3">
         <v>45936</v>
       </c>
@@ -8562,7 +8557,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="286" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G286" s="3">
         <v>45936</v>
       </c>
@@ -8588,15 +8583,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="287" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G287" s="3">
         <v>45936</v>
       </c>
       <c r="H287" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="I287" s="6" t="s">
         <v>241</v>
-      </c>
-      <c r="I287" s="6" t="s">
-        <v>242</v>
       </c>
       <c r="J287" s="4" t="s">
         <v>27</v>
@@ -8614,7 +8609,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="288" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G288" s="3">
         <v>45937</v>
       </c>
@@ -8631,7 +8626,7 @@
         <v>140</v>
       </c>
       <c r="L288" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M288" s="4" t="s">
         <v>8</v>
@@ -8640,7 +8635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="289" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G289" s="3">
         <v>45937</v>
       </c>
@@ -8666,7 +8661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="290" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G290" s="3">
         <v>45937</v>
       </c>
@@ -8683,7 +8678,7 @@
         <v>179.9</v>
       </c>
       <c r="L290" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="M290" s="4" t="s">
         <v>8</v>
@@ -8692,7 +8687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="291" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G291" s="3">
         <v>45937</v>
       </c>
@@ -8718,7 +8713,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="292" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G292" s="3">
         <v>45937</v>
       </c>
@@ -8744,7 +8739,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="293" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G293" s="3">
         <v>45937</v>
       </c>
@@ -8770,7 +8765,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="294" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G294" s="3">
         <v>45937</v>
       </c>
@@ -8797,156 +8792,84 @@
       </c>
     </row>
     <row r="295" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G295" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H295" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="I295" s="6" t="s">
-        <v>155</v>
-      </c>
+      <c r="G295" s="3"/>
+      <c r="H295" s="4"/>
+      <c r="I295" s="6"/>
       <c r="J295" s="4"/>
       <c r="K295" s="9"/>
       <c r="L295" s="4"/>
       <c r="M295" s="4"/>
-      <c r="N295" s="6">
-        <v>2</v>
-      </c>
+      <c r="N295" s="6"/>
     </row>
     <row r="296" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G296" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H296" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="I296" s="6" t="s">
-        <v>147</v>
-      </c>
+      <c r="G296" s="3"/>
+      <c r="H296" s="4"/>
+      <c r="I296" s="6"/>
       <c r="J296" s="4"/>
       <c r="K296" s="4"/>
       <c r="L296" s="4"/>
       <c r="M296" s="4"/>
-      <c r="N296" s="6">
-        <v>3</v>
-      </c>
+      <c r="N296" s="6"/>
     </row>
     <row r="297" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G297" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H297" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="I297" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="J297" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="K297" s="4">
-        <v>160</v>
-      </c>
-      <c r="L297" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="M297" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N297" s="4">
-        <v>3</v>
-      </c>
+      <c r="G297" s="3"/>
+      <c r="H297" s="4"/>
+      <c r="I297" s="6"/>
+      <c r="J297" s="4"/>
+      <c r="K297" s="4"/>
+      <c r="L297" s="4"/>
+      <c r="M297" s="4"/>
+      <c r="N297" s="4"/>
     </row>
     <row r="298" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G298" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H298" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I298" s="6" t="s">
-        <v>154</v>
-      </c>
+      <c r="G298" s="3"/>
+      <c r="H298" s="4"/>
+      <c r="I298" s="6"/>
       <c r="J298" s="4"/>
       <c r="K298" s="9"/>
       <c r="L298" s="4"/>
       <c r="M298" s="4"/>
-      <c r="N298" s="6">
-        <v>3</v>
-      </c>
+      <c r="N298" s="6"/>
     </row>
     <row r="299" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G299" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H299" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="I299" s="6" t="s">
-        <v>144</v>
-      </c>
+      <c r="G299" s="3"/>
+      <c r="H299" s="4"/>
+      <c r="I299" s="6"/>
       <c r="J299" s="4"/>
       <c r="K299" s="9"/>
       <c r="L299" s="4"/>
       <c r="M299" s="4"/>
-      <c r="N299" s="6">
-        <v>3</v>
-      </c>
+      <c r="N299" s="6"/>
     </row>
     <row r="300" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G300" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H300" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="I300" s="6" t="s">
-        <v>145</v>
-      </c>
+      <c r="G300" s="3"/>
+      <c r="H300" s="4"/>
+      <c r="I300" s="6"/>
       <c r="J300" s="4"/>
       <c r="K300" s="9"/>
       <c r="L300" s="4"/>
       <c r="M300" s="4"/>
-      <c r="N300" s="6">
-        <v>3</v>
-      </c>
+      <c r="N300" s="6"/>
     </row>
     <row r="301" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G301" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H301" s="4" t="s">
-        <v>160</v>
-      </c>
-      <c r="I301" s="6" t="s">
-        <v>151</v>
-      </c>
+      <c r="G301" s="3"/>
+      <c r="H301" s="4"/>
+      <c r="I301" s="6"/>
       <c r="J301" s="4"/>
       <c r="K301" s="9"/>
       <c r="L301" s="4"/>
       <c r="M301" s="4"/>
-      <c r="N301" s="6">
-        <v>3</v>
-      </c>
+      <c r="N301" s="6"/>
     </row>
     <row r="302" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G302" s="3">
-        <v>45938</v>
-      </c>
-      <c r="H302" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="I302" s="6" t="s">
-        <v>149</v>
-      </c>
+      <c r="G302" s="3"/>
+      <c r="H302" s="4"/>
+      <c r="I302" s="6"/>
       <c r="J302" s="4"/>
       <c r="K302" s="9"/>
       <c r="L302" s="4"/>
       <c r="M302" s="20"/>
-      <c r="N302" s="6">
-        <v>2</v>
-      </c>
+      <c r="N302" s="6"/>
     </row>
     <row r="303" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G303" s="4"/>
@@ -9079,13 +9002,7 @@
       <c r="N315" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N302" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-    <filterColumn colId="0">
-      <filters>
-        <dateGroupItem year="2025" month="10" day="8" dateTimeGrouping="day"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="G5:N302" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-08 17:16
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1364" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5F85806-09B3-4E24-9BDF-4AB0900C819A}"/>
+  <xr:revisionPtr revIDLastSave="1428" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCBFF874-08D1-4740-B44F-BB1ACAAFA21F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$302</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$309</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="248">
   <si>
     <t>DATA</t>
   </si>
@@ -637,9 +637,6 @@
     <t>HOTEL LAGO DOS ENCANTOS</t>
   </si>
   <si>
-    <t>HOTEL CAMPEAO</t>
-  </si>
-  <si>
     <t>LUIS EDUARDO</t>
   </si>
   <si>
@@ -776,6 +773,15 @@
   </si>
   <si>
     <t>HOTEL MARIO ARMANDO</t>
+  </si>
+  <si>
+    <t>HOTEL CAMPEÃO</t>
+  </si>
+  <si>
+    <t>HOTEL COSTA E FILHO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POUSADA AMERICA </t>
   </si>
 </sst>
 </file>
@@ -4331,7 +4337,7 @@
         <v>148</v>
       </c>
       <c r="J122" s="17" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K122" s="9">
         <v>110</v>
@@ -5445,7 +5451,7 @@
         <v>170</v>
       </c>
       <c r="L165" s="4" t="s">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="M165" s="4" t="s">
         <v>8</v>
@@ -5471,7 +5477,7 @@
         <v>170</v>
       </c>
       <c r="L166" s="4" t="s">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="M166" s="4" t="s">
         <v>8</v>
@@ -5663,13 +5669,13 @@
         <v>152</v>
       </c>
       <c r="J174" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K174" s="9">
         <v>250</v>
       </c>
       <c r="L174" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M174" s="4" t="s">
         <v>8</v>
@@ -5686,7 +5692,7 @@
         <v>171</v>
       </c>
       <c r="I175" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J175" s="4" t="s">
         <v>73</v>
@@ -5695,7 +5701,7 @@
         <v>220</v>
       </c>
       <c r="L175" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="M175" s="4" t="s">
         <v>8</v>
@@ -5877,7 +5883,7 @@
         <v>140</v>
       </c>
       <c r="L182" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="M182" s="4" t="s">
         <v>7</v>
@@ -5894,7 +5900,7 @@
         <v>167</v>
       </c>
       <c r="I183" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J183" s="4" t="s">
         <v>59</v>
@@ -5981,7 +5987,7 @@
         <v>220</v>
       </c>
       <c r="L186" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M186" s="4" t="s">
         <v>8</v>
@@ -6183,7 +6189,7 @@
         <v>148</v>
       </c>
       <c r="J194" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K194" s="9">
         <v>150</v>
@@ -6215,7 +6221,7 @@
         <v>240</v>
       </c>
       <c r="L195" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="M195" s="4" t="s">
         <v>8</v>
@@ -6293,7 +6299,7 @@
         <v>230</v>
       </c>
       <c r="L198" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M198" s="4" t="s">
         <v>8</v>
@@ -6365,7 +6371,7 @@
         <v>148</v>
       </c>
       <c r="J201" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K201" s="9">
         <v>180</v>
@@ -6501,7 +6507,7 @@
         <v>200</v>
       </c>
       <c r="L206" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M206" s="4" t="s">
         <v>8</v>
@@ -6547,13 +6553,13 @@
         <v>152</v>
       </c>
       <c r="J208" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K208" s="9">
         <v>230</v>
       </c>
       <c r="L208" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="M208" s="4" t="s">
         <v>8</v>
@@ -6692,16 +6698,16 @@
         <v>176</v>
       </c>
       <c r="I214" s="6" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="J214" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K214" s="9">
         <v>170</v>
       </c>
       <c r="L214" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M214" s="4" t="s">
         <v>8</v>
@@ -6805,7 +6811,7 @@
         <v>250</v>
       </c>
       <c r="L218" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M218" s="4" t="s">
         <v>8</v>
@@ -6857,7 +6863,7 @@
         <v>275</v>
       </c>
       <c r="L220" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M220" s="4" t="s">
         <v>8</v>
@@ -6935,7 +6941,7 @@
         <v>220</v>
       </c>
       <c r="L223" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M223" s="4" t="s">
         <v>8</v>
@@ -7033,13 +7039,13 @@
         <v>148</v>
       </c>
       <c r="J227" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K227" s="9">
         <v>110</v>
       </c>
       <c r="L227" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="M227" s="4" t="s">
         <v>8</v>
@@ -7082,7 +7088,7 @@
         <v>160</v>
       </c>
       <c r="I229" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J229" s="4" t="s">
         <v>51</v>
@@ -7134,7 +7140,7 @@
         <v>164</v>
       </c>
       <c r="I231" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J231" s="4" t="s">
         <v>22</v>
@@ -7221,7 +7227,7 @@
         <v>170</v>
       </c>
       <c r="L234" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="M234" s="4" t="s">
         <v>8</v>
@@ -7247,7 +7253,7 @@
         <v>250</v>
       </c>
       <c r="L235" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M235" s="4" t="s">
         <v>8</v>
@@ -7290,16 +7296,16 @@
         <v>160</v>
       </c>
       <c r="I237" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J237" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K237" s="9">
         <v>180</v>
       </c>
       <c r="L237" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="M237" s="4" t="s">
         <v>8</v>
@@ -7342,7 +7348,7 @@
         <v>164</v>
       </c>
       <c r="I239" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J239" s="4" t="s">
         <v>37</v>
@@ -7368,10 +7374,10 @@
         <v>175</v>
       </c>
       <c r="I240" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="J240" s="4" t="s">
         <v>219</v>
-      </c>
-      <c r="J240" s="4" t="s">
-        <v>220</v>
       </c>
       <c r="K240" s="9">
         <v>209</v>
@@ -7423,13 +7429,13 @@
         <v>152</v>
       </c>
       <c r="J242" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K242" s="9">
         <v>200</v>
       </c>
       <c r="L242" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="M242" s="4" t="s">
         <v>8</v>
@@ -7495,7 +7501,7 @@
         <v>45929</v>
       </c>
       <c r="H245" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I245" s="6" t="s">
         <v>197</v>
@@ -7507,7 +7513,7 @@
         <v>220</v>
       </c>
       <c r="L245" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M245" s="4" t="s">
         <v>8</v>
@@ -7527,13 +7533,13 @@
         <v>147</v>
       </c>
       <c r="J246" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K246" s="9">
         <v>240</v>
       </c>
       <c r="L246" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="M246" s="4" t="s">
         <v>8</v>
@@ -7550,10 +7556,10 @@
         <v>175</v>
       </c>
       <c r="I247" s="6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="J247" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="K247" s="9">
         <v>209</v>
@@ -7637,7 +7643,7 @@
         <v>250</v>
       </c>
       <c r="L250" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M250" s="4" t="s">
         <v>8</v>
@@ -7651,10 +7657,10 @@
         <v>45929</v>
       </c>
       <c r="H251" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="I251" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J251" s="4" t="s">
         <v>27</v>
@@ -7663,7 +7669,7 @@
         <v>265</v>
       </c>
       <c r="L251" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M251" s="4" t="s">
         <v>8</v>
@@ -7859,7 +7865,7 @@
         <v>45931</v>
       </c>
       <c r="H259" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I259" s="6" t="s">
         <v>149</v>
@@ -7923,7 +7929,7 @@
         <v>210</v>
       </c>
       <c r="L261" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="M261" s="4" t="s">
         <v>8</v>
@@ -7943,7 +7949,7 @@
         <v>148</v>
       </c>
       <c r="J262" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K262" s="9">
         <v>110</v>
@@ -8015,7 +8021,7 @@
         <v>45931</v>
       </c>
       <c r="H265" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I265" s="6" t="s">
         <v>145</v>
@@ -8041,7 +8047,7 @@
         <v>45931</v>
       </c>
       <c r="H266" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I266" s="6" t="s">
         <v>151</v>
@@ -8119,7 +8125,7 @@
         <v>45932</v>
       </c>
       <c r="H269" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="I269" s="6" t="s">
         <v>145</v>
@@ -8145,13 +8151,13 @@
         <v>45932</v>
       </c>
       <c r="H270" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="I270" s="6" t="s">
         <v>151</v>
       </c>
       <c r="J270" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="K270" s="9">
         <v>235</v>
@@ -8174,10 +8180,10 @@
         <v>175</v>
       </c>
       <c r="I271" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J271" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="K271" s="9">
         <v>259</v>
@@ -8203,13 +8209,13 @@
         <v>141</v>
       </c>
       <c r="J272" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K272" s="9">
         <v>240</v>
       </c>
       <c r="L272" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="M272" s="4" t="s">
         <v>8</v>
@@ -8226,16 +8232,16 @@
         <v>170</v>
       </c>
       <c r="I273" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J273" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="K273" s="9">
         <v>200</v>
       </c>
       <c r="L273" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M273" s="4" t="s">
         <v>8</v>
@@ -8256,13 +8262,13 @@
         <v>152</v>
       </c>
       <c r="J274" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K274" s="9">
         <v>250</v>
       </c>
       <c r="L274" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="M274" s="4" t="s">
         <v>8</v>
@@ -8340,7 +8346,7 @@
         <v>250</v>
       </c>
       <c r="L277" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M277" s="4" t="s">
         <v>8</v>
@@ -8366,7 +8372,7 @@
         <v>240</v>
       </c>
       <c r="L278" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="M278" s="4" t="s">
         <v>8</v>
@@ -8432,7 +8438,7 @@
         <v>45936</v>
       </c>
       <c r="H281" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I281" s="6" t="s">
         <v>197</v>
@@ -8444,7 +8450,7 @@
         <v>220</v>
       </c>
       <c r="L281" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M281" s="4" t="s">
         <v>8</v>
@@ -8458,13 +8464,13 @@
         <v>45936</v>
       </c>
       <c r="H282" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I282" s="6" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J282" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="K282" s="9">
         <v>259</v>
@@ -8574,7 +8580,7 @@
         <v>250</v>
       </c>
       <c r="L286" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M286" s="4" t="s">
         <v>8</v>
@@ -8588,10 +8594,10 @@
         <v>45936</v>
       </c>
       <c r="H287" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="I287" s="6" t="s">
         <v>240</v>
-      </c>
-      <c r="I287" s="6" t="s">
-        <v>241</v>
       </c>
       <c r="J287" s="4" t="s">
         <v>27</v>
@@ -8600,7 +8606,7 @@
         <v>265</v>
       </c>
       <c r="L287" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="M287" s="4" t="s">
         <v>8</v>
@@ -8626,7 +8632,7 @@
         <v>140</v>
       </c>
       <c r="L288" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="M288" s="4" t="s">
         <v>8</v>
@@ -8678,7 +8684,7 @@
         <v>179.9</v>
       </c>
       <c r="L290" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="M290" s="4" t="s">
         <v>8</v>
@@ -8770,7 +8776,7 @@
         <v>45937</v>
       </c>
       <c r="H294" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="I294" s="6" t="s">
         <v>197</v>
@@ -8782,7 +8788,7 @@
         <v>220</v>
       </c>
       <c r="L294" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="M294" s="4" t="s">
         <v>8</v>
@@ -8872,74 +8878,186 @@
       <c r="N302" s="6"/>
     </row>
     <row r="303" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G303" s="4"/>
-      <c r="H303" s="4"/>
-      <c r="I303" s="6"/>
-      <c r="J303" s="4"/>
-      <c r="K303" s="9"/>
-      <c r="L303" s="4"/>
-      <c r="M303" s="4"/>
-      <c r="N303" s="6"/>
+      <c r="G303" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H303" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="I303" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="J303" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="K303" s="9">
+        <v>200</v>
+      </c>
+      <c r="L303" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="M303" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N303" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="304" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G304" s="4"/>
-      <c r="H304" s="4"/>
-      <c r="I304" s="6"/>
-      <c r="J304" s="4"/>
-      <c r="K304" s="9"/>
-      <c r="L304" s="4"/>
-      <c r="M304" s="4"/>
-      <c r="N304" s="6"/>
+      <c r="G304" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H304" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I304" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="J304" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="K304" s="9">
+        <v>280</v>
+      </c>
+      <c r="L304" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M304" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N304" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="305" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G305" s="4"/>
-      <c r="H305" s="4"/>
-      <c r="I305" s="6"/>
-      <c r="J305" s="4"/>
-      <c r="K305" s="9"/>
-      <c r="L305" s="4"/>
-      <c r="M305" s="4"/>
-      <c r="N305" s="6"/>
+      <c r="G305" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H305" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="I305" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="J305" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="K305" s="9">
+        <v>160</v>
+      </c>
+      <c r="L305" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="M305" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N305" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="306" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G306" s="4"/>
-      <c r="H306" s="4"/>
-      <c r="I306" s="6"/>
-      <c r="J306" s="4"/>
-      <c r="K306" s="9"/>
-      <c r="L306" s="4"/>
-      <c r="M306" s="4"/>
-      <c r="N306" s="6"/>
+      <c r="G306" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H306" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I306" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="J306" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K306" s="9">
+        <v>170</v>
+      </c>
+      <c r="L306" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="M306" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N306" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="307" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G307" s="4"/>
-      <c r="H307" s="4"/>
-      <c r="I307" s="6"/>
-      <c r="J307" s="4"/>
-      <c r="K307" s="9"/>
-      <c r="L307" s="4"/>
-      <c r="M307" s="4"/>
-      <c r="N307" s="6"/>
+      <c r="G307" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H307" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="I307" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="J307" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="K307" s="9">
+        <v>200</v>
+      </c>
+      <c r="L307" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="M307" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N307" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="308" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G308" s="4"/>
-      <c r="H308" s="4"/>
-      <c r="I308" s="6"/>
-      <c r="J308" s="4"/>
-      <c r="K308" s="9"/>
-      <c r="L308" s="4"/>
-      <c r="M308" s="4"/>
-      <c r="N308" s="6"/>
+      <c r="G308" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H308" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="I308" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="J308" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="K308" s="9">
+        <v>170</v>
+      </c>
+      <c r="L308" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="M308" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N308" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="309" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G309" s="4"/>
-      <c r="H309" s="4"/>
-      <c r="I309" s="6"/>
-      <c r="J309" s="4"/>
-      <c r="K309" s="9"/>
-      <c r="L309" s="4"/>
-      <c r="M309" s="4"/>
-      <c r="N309" s="6"/>
+      <c r="G309" s="3">
+        <v>45938</v>
+      </c>
+      <c r="H309" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="I309" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="J309" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K309" s="9">
+        <v>230</v>
+      </c>
+      <c r="L309" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="M309" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N309" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="310" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G310" s="4"/>
@@ -9002,7 +9120,7 @@
       <c r="N315" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N302" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:N309" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-13 17:38
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD COMBUSTIVEL/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1579" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7C01DA02-E3E2-463E-A5AC-4FB97D537685}"/>
+  <xr:revisionPtr revIDLastSave="1640" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C544A0D2-D567-4BF9-B006-FE026D3C524F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$323</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$324</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1550" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1585" uniqueCount="264">
   <si>
     <t>DATA</t>
   </si>
@@ -824,6 +824,12 @@
   </si>
   <si>
     <t xml:space="preserve">HOTEL PARAISO </t>
+  </si>
+  <si>
+    <t>BARBACENA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SERRA DAS VERTENTES </t>
   </si>
 </sst>
 </file>
@@ -834,7 +840,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -843,14 +849,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -977,7 +975,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -9032,64 +9030,160 @@
       </c>
     </row>
     <row r="302" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G302" s="3"/>
-      <c r="H302" s="4"/>
-      <c r="I302" s="6"/>
-      <c r="J302" s="4"/>
-      <c r="K302" s="9"/>
-      <c r="L302" s="4"/>
-      <c r="M302" s="20"/>
-      <c r="N302" s="6"/>
+      <c r="G302" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H302" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="I302" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J302" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K302" s="9">
+        <v>220</v>
+      </c>
+      <c r="L302" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="M302" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="N302" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="303" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G303" s="4"/>
-      <c r="H303" s="4"/>
-      <c r="I303" s="6"/>
-      <c r="J303" s="4"/>
-      <c r="K303" s="9"/>
-      <c r="L303" s="4"/>
-      <c r="M303" s="4"/>
-      <c r="N303" s="6"/>
+      <c r="G303" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H303" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I303" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="J303" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K303" s="9">
+        <v>140</v>
+      </c>
+      <c r="L303" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="M303" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N303" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="304" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G304" s="4"/>
-      <c r="H304" s="4"/>
-      <c r="I304" s="6"/>
-      <c r="J304" s="4"/>
-      <c r="K304" s="9"/>
-      <c r="L304" s="4"/>
-      <c r="M304" s="4"/>
-      <c r="N304" s="6"/>
+      <c r="G304" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H304" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="I304" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="J304" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="K304" s="9">
+        <v>200</v>
+      </c>
+      <c r="L304" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="M304" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N304" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="305" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G305" s="4"/>
-      <c r="H305" s="4"/>
-      <c r="I305" s="6"/>
-      <c r="J305" s="4"/>
-      <c r="K305" s="9"/>
-      <c r="L305" s="4"/>
-      <c r="M305" s="4"/>
-      <c r="N305" s="6"/>
+      <c r="G305" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H305" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I305" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="J305" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K305" s="9">
+        <v>220</v>
+      </c>
+      <c r="L305" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="M305" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N305" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="306" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G306" s="4"/>
-      <c r="H306" s="4"/>
-      <c r="I306" s="6"/>
-      <c r="J306" s="4"/>
-      <c r="K306" s="9"/>
-      <c r="L306" s="4"/>
-      <c r="M306" s="4"/>
-      <c r="N306" s="6"/>
+      <c r="G306" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H306" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I306" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="J306" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="K306" s="9">
+        <v>180</v>
+      </c>
+      <c r="L306" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="M306" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N306" s="6">
+        <v>3</v>
+      </c>
     </row>
     <row r="307" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G307" s="4"/>
-      <c r="H307" s="4"/>
-      <c r="I307" s="6"/>
-      <c r="J307" s="4"/>
-      <c r="K307" s="9"/>
-      <c r="L307" s="4"/>
-      <c r="M307" s="4"/>
-      <c r="N307" s="6"/>
+      <c r="G307" s="3">
+        <v>45943</v>
+      </c>
+      <c r="H307" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I307" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="J307" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="K307" s="9">
+        <v>220</v>
+      </c>
+      <c r="L307" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="M307" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N307" s="6">
+        <v>2</v>
+      </c>
     </row>
     <row r="308" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G308" s="4"/>
@@ -9476,14 +9570,30 @@
       </c>
     </row>
     <row r="324" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G324" s="4"/>
-      <c r="H324" s="4"/>
-      <c r="I324" s="6"/>
-      <c r="J324" s="4"/>
-      <c r="K324" s="9"/>
-      <c r="L324" s="4"/>
-      <c r="M324" s="4"/>
-      <c r="N324" s="6"/>
+      <c r="G324" s="3">
+        <v>45940</v>
+      </c>
+      <c r="H324" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="I324" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="J324" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="K324" s="9">
+        <v>220</v>
+      </c>
+      <c r="L324" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="M324" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N324" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="325" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G325" s="4"/>
@@ -9506,7 +9616,7 @@
       <c r="N326" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N323" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:N324" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-16 11:01
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1916" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1881563-2C13-41C2-929F-4DF6F0932D55}"/>
+  <xr:revisionPtr revIDLastSave="1921" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A04E4BE9-DF24-4B82-95D4-AC891A319130}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$342</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$347</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -10226,7 +10226,7 @@
       <c r="N356" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N342" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:N347" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2025" month="10" day="16" dateTimeGrouping="day"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-21 14:16
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2158" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C511DE0-C4CA-4B4D-9DF8-A873E18EE2FB}"/>
+  <xr:revisionPtr revIDLastSave="2166" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECB91BB1-8156-4A16-82D1-4CD0A7B86BAD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1778" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1781" uniqueCount="256">
   <si>
     <t>DATA</t>
   </si>
@@ -803,6 +803,9 @@
   </si>
   <si>
     <t>JOSE ARILDO</t>
+  </si>
+  <si>
+    <t>TRES PONTAS</t>
   </si>
 </sst>
 </file>
@@ -1306,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-  <sheetPr codeName="Planilha1">
+  <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="G5:O369"/>
@@ -1349,7 +1352,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>45873</v>
       </c>
@@ -1376,7 +1379,7 @@
       </c>
       <c r="O6"/>
     </row>
-    <row r="7" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>45873</v>
       </c>
@@ -1403,7 +1406,7 @@
       </c>
       <c r="O7"/>
     </row>
-    <row r="8" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>45873</v>
       </c>
@@ -1430,7 +1433,7 @@
       </c>
       <c r="O8"/>
     </row>
-    <row r="9" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>45873</v>
       </c>
@@ -1457,7 +1460,7 @@
       </c>
       <c r="O9"/>
     </row>
-    <row r="10" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>45875</v>
       </c>
@@ -1484,7 +1487,7 @@
       </c>
       <c r="O10"/>
     </row>
-    <row r="11" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>45875</v>
       </c>
@@ -1511,7 +1514,7 @@
       </c>
       <c r="O11"/>
     </row>
-    <row r="12" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>45875</v>
       </c>
@@ -1538,7 +1541,7 @@
       </c>
       <c r="O12"/>
     </row>
-    <row r="13" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>45875</v>
       </c>
@@ -1565,7 +1568,7 @@
       </c>
       <c r="O13"/>
     </row>
-    <row r="14" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>45875</v>
       </c>
@@ -1592,7 +1595,7 @@
       </c>
       <c r="O14"/>
     </row>
-    <row r="15" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>45875</v>
       </c>
@@ -1619,7 +1622,7 @@
       </c>
       <c r="O15"/>
     </row>
-    <row r="16" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>45875</v>
       </c>
@@ -1646,7 +1649,7 @@
       </c>
       <c r="O16"/>
     </row>
-    <row r="17" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>45875</v>
       </c>
@@ -1672,7 +1675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>45876</v>
       </c>
@@ -1698,7 +1701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>45876</v>
       </c>
@@ -1724,7 +1727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>45876</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>45876</v>
       </c>
@@ -1776,7 +1779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
         <v>45876</v>
       </c>
@@ -1802,7 +1805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
         <v>45876</v>
       </c>
@@ -1828,7 +1831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
         <v>45876</v>
       </c>
@@ -1854,7 +1857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
         <v>45876</v>
       </c>
@@ -1880,7 +1883,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
         <v>45876</v>
       </c>
@@ -1906,7 +1909,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
         <v>45876</v>
       </c>
@@ -1932,7 +1935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>45876</v>
       </c>
@@ -1958,7 +1961,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
         <v>45880</v>
       </c>
@@ -1984,7 +1987,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
         <v>45880</v>
       </c>
@@ -2010,7 +2013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
         <v>45880</v>
       </c>
@@ -2036,7 +2039,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
         <v>45880</v>
       </c>
@@ -2062,7 +2065,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
         <v>45880</v>
       </c>
@@ -2088,7 +2091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G34" s="3">
         <v>45881</v>
       </c>
@@ -2114,7 +2117,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G35" s="3">
         <v>45881</v>
       </c>
@@ -2140,7 +2143,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>45881</v>
       </c>
@@ -2166,7 +2169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G37" s="3">
         <v>45881</v>
       </c>
@@ -2192,7 +2195,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G38" s="3">
         <v>45881</v>
       </c>
@@ -2218,7 +2221,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G39" s="3">
         <v>45881</v>
       </c>
@@ -2244,7 +2247,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G40" s="3">
         <v>45881</v>
       </c>
@@ -2270,7 +2273,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G41" s="3">
         <v>45882</v>
       </c>
@@ -2296,7 +2299,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G42" s="3">
         <v>45882</v>
       </c>
@@ -2322,7 +2325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G43" s="3">
         <v>45882</v>
       </c>
@@ -2348,7 +2351,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G44" s="3">
         <v>45882</v>
       </c>
@@ -2374,7 +2377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G45" s="3">
         <v>45882</v>
       </c>
@@ -2400,7 +2403,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G46" s="3">
         <v>45882</v>
       </c>
@@ -2426,7 +2429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G47" s="3">
         <v>45883</v>
       </c>
@@ -2452,7 +2455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G48" s="3">
         <v>45883</v>
       </c>
@@ -2478,7 +2481,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G49" s="3">
         <v>45883</v>
       </c>
@@ -2504,7 +2507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G50" s="3">
         <v>45883</v>
       </c>
@@ -2530,7 +2533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G51" s="3">
         <v>45883</v>
       </c>
@@ -2556,7 +2559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G52" s="3">
         <v>45883</v>
       </c>
@@ -2582,7 +2585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G53" s="3">
         <v>45883</v>
       </c>
@@ -2608,7 +2611,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G54" s="3">
         <v>45883</v>
       </c>
@@ -2634,7 +2637,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G55" s="3">
         <v>45883</v>
       </c>
@@ -2660,7 +2663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G56" s="3">
         <v>45883</v>
       </c>
@@ -2686,7 +2689,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G57" s="3">
         <v>45883</v>
       </c>
@@ -2712,7 +2715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G58" s="3">
         <v>45883</v>
       </c>
@@ -2738,7 +2741,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G59" s="3">
         <v>45883</v>
       </c>
@@ -2764,7 +2767,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G60" s="3">
         <v>45883</v>
       </c>
@@ -2790,7 +2793,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G61" s="3">
         <v>45883</v>
       </c>
@@ -2816,7 +2819,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G62" s="3">
         <v>45883</v>
       </c>
@@ -2842,7 +2845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>45887</v>
       </c>
@@ -2868,7 +2871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G64" s="3">
         <v>45887</v>
       </c>
@@ -2894,7 +2897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G65" s="3">
         <v>45887</v>
       </c>
@@ -2920,7 +2923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G66" s="3">
         <v>45887</v>
       </c>
@@ -2946,7 +2949,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G67" s="3">
         <v>45887</v>
       </c>
@@ -2972,7 +2975,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G68" s="3">
         <v>45887</v>
       </c>
@@ -2998,7 +3001,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G69" s="3">
         <v>45887</v>
       </c>
@@ -3024,7 +3027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G70" s="3">
         <v>45888</v>
       </c>
@@ -3050,7 +3053,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G71" s="3">
         <v>45888</v>
       </c>
@@ -3076,7 +3079,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>45888</v>
       </c>
@@ -3102,7 +3105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G73" s="3">
         <v>45888</v>
       </c>
@@ -3128,7 +3131,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G74" s="3">
         <v>45888</v>
       </c>
@@ -3154,7 +3157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G75" s="3">
         <v>45889</v>
       </c>
@@ -3180,7 +3183,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G76" s="3">
         <v>45889</v>
       </c>
@@ -3206,7 +3209,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G77" s="3">
         <v>45889</v>
       </c>
@@ -3232,7 +3235,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G78" s="3">
         <v>45889</v>
       </c>
@@ -3258,7 +3261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G79" s="3">
         <v>45889</v>
       </c>
@@ -3284,7 +3287,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G80" s="3">
         <v>45889</v>
       </c>
@@ -3310,7 +3313,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G81" s="3">
         <v>45889</v>
       </c>
@@ -3336,7 +3339,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G82" s="3">
         <v>45890</v>
       </c>
@@ -3362,7 +3365,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G83" s="3">
         <v>45890</v>
       </c>
@@ -3388,7 +3391,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G84" s="3">
         <v>45890</v>
       </c>
@@ -3414,7 +3417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G85" s="3">
         <v>45890</v>
       </c>
@@ -3440,7 +3443,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G86" s="3">
         <v>45890</v>
       </c>
@@ -3466,7 +3469,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G87" s="3">
         <v>45890</v>
       </c>
@@ -3492,7 +3495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G88" s="3">
         <v>45890</v>
       </c>
@@ -3518,7 +3521,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G89" s="3">
         <v>45890</v>
       </c>
@@ -3544,7 +3547,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G90" s="3">
         <v>45890</v>
       </c>
@@ -3570,7 +3573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G91" s="3">
         <v>45890</v>
       </c>
@@ -3594,7 +3597,7 @@
       </c>
       <c r="N91" s="6"/>
     </row>
-    <row r="92" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G92" s="3">
         <v>45890</v>
       </c>
@@ -3620,7 +3623,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G93" s="3">
         <v>45894</v>
       </c>
@@ -3646,7 +3649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G94" s="3">
         <v>45894</v>
       </c>
@@ -3672,7 +3675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G95" s="3">
         <v>45894</v>
       </c>
@@ -3698,7 +3701,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G96" s="3">
         <v>45894</v>
       </c>
@@ -3724,7 +3727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G97" s="3">
         <v>45895</v>
       </c>
@@ -3750,7 +3753,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G98" s="3">
         <v>45895</v>
       </c>
@@ -3776,7 +3779,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G99" s="3">
         <v>45895</v>
       </c>
@@ -3802,7 +3805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G100" s="3">
         <v>45895</v>
       </c>
@@ -3828,7 +3831,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G101" s="3">
         <v>45895</v>
       </c>
@@ -3854,7 +3857,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G102" s="3">
         <v>45895</v>
       </c>
@@ -3880,7 +3883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G103" s="3">
         <v>45895</v>
       </c>
@@ -3906,7 +3909,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G104" s="3">
         <v>45896</v>
       </c>
@@ -3932,7 +3935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G105" s="3">
         <v>45896</v>
       </c>
@@ -3958,7 +3961,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G106" s="3">
         <v>45896</v>
       </c>
@@ -3984,7 +3987,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G107" s="3">
         <v>45896</v>
       </c>
@@ -4010,7 +4013,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G108" s="3">
         <v>45896</v>
       </c>
@@ -4036,7 +4039,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G109" s="3">
         <v>45896</v>
       </c>
@@ -4062,7 +4065,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G110" s="3">
         <v>45896</v>
       </c>
@@ -4088,7 +4091,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G111" s="3">
         <v>45896</v>
       </c>
@@ -4114,7 +4117,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G112" s="3">
         <v>45897</v>
       </c>
@@ -4140,7 +4143,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G113" s="3">
         <v>45897</v>
       </c>
@@ -4166,7 +4169,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G114" s="3">
         <v>45897</v>
       </c>
@@ -4192,7 +4195,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G115" s="3">
         <v>45897</v>
       </c>
@@ -4218,7 +4221,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G116" s="3">
         <v>45897</v>
       </c>
@@ -4244,7 +4247,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G117" s="3">
         <v>45897</v>
       </c>
@@ -4270,7 +4273,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G118" s="3">
         <v>45897</v>
       </c>
@@ -4296,7 +4299,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G119" s="3">
         <v>45897</v>
       </c>
@@ -4322,7 +4325,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="120" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G120" s="3">
         <v>45897</v>
       </c>
@@ -4348,7 +4351,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G121" s="3">
         <v>45897</v>
       </c>
@@ -4374,7 +4377,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G122" s="3">
         <v>45897</v>
       </c>
@@ -4400,7 +4403,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G123" s="3">
         <v>45901</v>
       </c>
@@ -4426,7 +4429,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G124" s="3">
         <v>45901</v>
       </c>
@@ -4452,7 +4455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G125" s="3">
         <v>45901</v>
       </c>
@@ -4478,7 +4481,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G126" s="3">
         <v>45901</v>
       </c>
@@ -4504,7 +4507,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G127" s="3">
         <v>45902</v>
       </c>
@@ -4530,7 +4533,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G128" s="3">
         <v>45902</v>
       </c>
@@ -4556,7 +4559,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G129" s="3">
         <v>45902</v>
       </c>
@@ -4582,7 +4585,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G130" s="3">
         <v>45902</v>
       </c>
@@ -4608,7 +4611,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G131" s="3">
         <v>45902</v>
       </c>
@@ -4634,7 +4637,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G132" s="3">
         <v>45902</v>
       </c>
@@ -4660,7 +4663,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G133" s="3">
         <v>45902</v>
       </c>
@@ -4686,7 +4689,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G134" s="3">
         <v>45903</v>
       </c>
@@ -4712,7 +4715,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G135" s="3">
         <v>45903</v>
       </c>
@@ -4738,7 +4741,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G136" s="3">
         <v>45903</v>
       </c>
@@ -4764,7 +4767,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G137" s="3">
         <v>45903</v>
       </c>
@@ -4790,7 +4793,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G138" s="3">
         <v>45903</v>
       </c>
@@ -4816,7 +4819,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G139" s="3">
         <v>45903</v>
       </c>
@@ -4842,7 +4845,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G140" s="3">
         <v>45903</v>
       </c>
@@ -4866,7 +4869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G141" s="3">
         <v>45903</v>
       </c>
@@ -4892,7 +4895,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="142" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G142" s="3">
         <v>45903</v>
       </c>
@@ -4916,7 +4919,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G143" s="3">
         <v>45903</v>
       </c>
@@ -4942,7 +4945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G144" s="3">
         <v>45904</v>
       </c>
@@ -4968,7 +4971,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="145" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G145" s="3">
         <v>45904</v>
       </c>
@@ -4994,7 +4997,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G146" s="3">
         <v>45904</v>
       </c>
@@ -5020,7 +5023,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G147" s="3">
         <v>45904</v>
       </c>
@@ -5046,7 +5049,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G148" s="3">
         <v>45904</v>
       </c>
@@ -5072,7 +5075,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
         <v>45904</v>
       </c>
@@ -5098,7 +5101,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G150" s="3">
         <v>45904</v>
       </c>
@@ -5124,7 +5127,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G151" s="3">
         <v>45904</v>
       </c>
@@ -5150,7 +5153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G152" s="3">
         <v>45904</v>
       </c>
@@ -5176,7 +5179,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>45908</v>
       </c>
@@ -5202,7 +5205,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G154" s="3">
         <v>45908</v>
       </c>
@@ -5228,7 +5231,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="155" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G155" s="3">
         <v>45908</v>
       </c>
@@ -5254,7 +5257,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>45908</v>
       </c>
@@ -5280,7 +5283,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="157" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G157" s="3">
         <v>45909</v>
       </c>
@@ -5306,7 +5309,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="158" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G158" s="3">
         <v>45909</v>
       </c>
@@ -5332,7 +5335,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G159" s="3">
         <v>45909</v>
       </c>
@@ -5358,7 +5361,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="160" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>45909</v>
       </c>
@@ -5384,7 +5387,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G161" s="3">
         <v>45909</v>
       </c>
@@ -5410,7 +5413,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G162" s="3">
         <v>45909</v>
       </c>
@@ -5436,7 +5439,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="163" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G163" s="3">
         <v>45910</v>
       </c>
@@ -5462,7 +5465,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="164" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G164" s="3">
         <v>45910</v>
       </c>
@@ -5482,7 +5485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="165" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G165" s="3">
         <v>45910</v>
       </c>
@@ -5508,7 +5511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G166" s="3">
         <v>45910</v>
       </c>
@@ -5534,7 +5537,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G167" s="3">
         <v>45910</v>
       </c>
@@ -5560,7 +5563,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G168" s="3">
         <v>45910</v>
       </c>
@@ -5586,7 +5589,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="169" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G169" s="3">
         <v>45910</v>
       </c>
@@ -5612,7 +5615,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G170" s="3">
         <v>45911</v>
       </c>
@@ -5632,7 +5635,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="171" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G171" s="3">
         <v>45911</v>
       </c>
@@ -5658,7 +5661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G172" s="3">
         <v>45911</v>
       </c>
@@ -5684,7 +5687,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="173" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G173" s="3">
         <v>45911</v>
       </c>
@@ -5710,7 +5713,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="174" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G174" s="3">
         <v>45911</v>
       </c>
@@ -5736,7 +5739,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G175" s="3">
         <v>45911</v>
       </c>
@@ -5762,7 +5765,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G176" s="3">
         <v>45911</v>
       </c>
@@ -5788,7 +5791,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="177" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
         <v>45911</v>
       </c>
@@ -5814,7 +5817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
         <v>45911</v>
       </c>
@@ -5840,7 +5843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="179" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
         <v>45911</v>
       </c>
@@ -5866,7 +5869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="180" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
         <v>45911</v>
       </c>
@@ -5892,7 +5895,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>45911</v>
       </c>
@@ -5918,7 +5921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>45911</v>
       </c>
@@ -5944,7 +5947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>45915</v>
       </c>
@@ -5970,7 +5973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>45915</v>
       </c>
@@ -5996,7 +5999,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G185" s="3">
         <v>45915</v>
       </c>
@@ -6022,7 +6025,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G186" s="3">
         <v>45915</v>
       </c>
@@ -6048,7 +6051,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G187" s="3">
         <v>45915</v>
       </c>
@@ -6074,7 +6077,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G188" s="3">
         <v>45915</v>
       </c>
@@ -6100,7 +6103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G189" s="3">
         <v>45915</v>
       </c>
@@ -6126,7 +6129,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G190" s="3">
         <v>45916</v>
       </c>
@@ -6152,7 +6155,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G191" s="3">
         <v>45916</v>
       </c>
@@ -6178,7 +6181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G192" s="3">
         <v>45916</v>
       </c>
@@ -6204,7 +6207,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G193" s="3">
         <v>45916</v>
       </c>
@@ -6230,7 +6233,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="194" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G194" s="3">
         <v>45916</v>
       </c>
@@ -6256,7 +6259,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="195" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G195" s="3">
         <v>45917</v>
       </c>
@@ -6282,7 +6285,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="196" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G196" s="3">
         <v>45917</v>
       </c>
@@ -6308,7 +6311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G197" s="3">
         <v>45917</v>
       </c>
@@ -6334,7 +6337,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G198" s="3">
         <v>45917</v>
       </c>
@@ -6360,7 +6363,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="199" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G199" s="3">
         <v>45917</v>
       </c>
@@ -6386,7 +6389,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G200" s="3">
         <v>45917</v>
       </c>
@@ -6412,7 +6415,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="201" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G201" s="3">
         <v>45917</v>
       </c>
@@ -6438,7 +6441,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="202" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G202" s="3">
         <v>45918</v>
       </c>
@@ -6464,7 +6467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G203" s="3">
         <v>45918</v>
       </c>
@@ -6490,7 +6493,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G204" s="3">
         <v>45918</v>
       </c>
@@ -6516,7 +6519,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G205" s="3">
         <v>45918</v>
       </c>
@@ -6542,7 +6545,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G206" s="3">
         <v>45918</v>
       </c>
@@ -6568,7 +6571,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G207" s="3">
         <v>45918</v>
       </c>
@@ -6594,7 +6597,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G208" s="3">
         <v>45918</v>
       </c>
@@ -6620,7 +6623,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G209" s="3">
         <v>45918</v>
       </c>
@@ -6646,7 +6649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G210" s="3">
         <v>45918</v>
       </c>
@@ -6672,7 +6675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G211" s="3">
         <v>45918</v>
       </c>
@@ -6698,7 +6701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G212" s="3">
         <v>45918</v>
       </c>
@@ -6718,7 +6721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G213" s="3">
         <v>45918</v>
       </c>
@@ -6744,7 +6747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G214" s="3">
         <v>45918</v>
       </c>
@@ -6770,7 +6773,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G215" s="3">
         <v>45922</v>
       </c>
@@ -6796,7 +6799,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G216" s="3">
         <v>45922</v>
       </c>
@@ -6822,7 +6825,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G217" s="3">
         <v>45922</v>
       </c>
@@ -6848,7 +6851,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G218" s="3">
         <v>45922</v>
       </c>
@@ -6874,7 +6877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G219" s="3">
         <v>45922</v>
       </c>
@@ -6900,7 +6903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="220" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G220" s="3">
         <v>45922</v>
       </c>
@@ -6926,7 +6929,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="221" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G221" s="3">
         <v>45922</v>
       </c>
@@ -6952,7 +6955,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G222" s="3">
         <v>45923</v>
       </c>
@@ -6978,7 +6981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G223" s="3">
         <v>45923</v>
       </c>
@@ -7004,7 +7007,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G224" s="3">
         <v>45923</v>
       </c>
@@ -7030,7 +7033,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="225" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G225" s="3">
         <v>45923</v>
       </c>
@@ -7056,7 +7059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G226" s="3">
         <v>45923</v>
       </c>
@@ -7082,7 +7085,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G227" s="3">
         <v>45923</v>
       </c>
@@ -7108,7 +7111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G228" s="3">
         <v>45924</v>
       </c>
@@ -7134,7 +7137,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="229" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G229" s="3">
         <v>45924</v>
       </c>
@@ -7160,7 +7163,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="230" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G230" s="3">
         <v>45924</v>
       </c>
@@ -7186,7 +7189,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="231" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G231" s="3">
         <v>45924</v>
       </c>
@@ -7212,7 +7215,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="232" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G232" s="3">
         <v>45924</v>
       </c>
@@ -7238,7 +7241,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G233" s="3">
         <v>45924</v>
       </c>
@@ -7264,7 +7267,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G234" s="3">
         <v>45924</v>
       </c>
@@ -7290,7 +7293,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G235" s="3">
         <v>45924</v>
       </c>
@@ -7316,7 +7319,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G236" s="3">
         <v>45925</v>
       </c>
@@ -7342,7 +7345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="237" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G237" s="3">
         <v>45925</v>
       </c>
@@ -7368,7 +7371,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G238" s="3">
         <v>45925</v>
       </c>
@@ -7394,7 +7397,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="239" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G239" s="3">
         <v>45925</v>
       </c>
@@ -7420,7 +7423,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="240" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G240" s="3">
         <v>45925</v>
       </c>
@@ -7446,7 +7449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G241" s="3">
         <v>45925</v>
       </c>
@@ -7472,7 +7475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G242" s="3">
         <v>45925</v>
       </c>
@@ -7498,7 +7501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="243" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G243" s="3">
         <v>45925</v>
       </c>
@@ -7524,7 +7527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G244" s="3">
         <v>45925</v>
       </c>
@@ -7550,7 +7553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="245" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G245" s="3">
         <v>45925</v>
       </c>
@@ -7576,7 +7579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G246" s="3">
         <v>45925</v>
       </c>
@@ -7602,7 +7605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G247" s="3">
         <v>45929</v>
       </c>
@@ -7628,7 +7631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="248" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G248" s="3">
         <v>45929</v>
       </c>
@@ -7654,7 +7657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="249" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G249" s="3">
         <v>45929</v>
       </c>
@@ -7680,7 +7683,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="250" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G250" s="3">
         <v>45929</v>
       </c>
@@ -7706,7 +7709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="251" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G251" s="3">
         <v>45929</v>
       </c>
@@ -7732,7 +7735,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="252" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G252" s="3">
         <v>45929</v>
       </c>
@@ -7758,7 +7761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G253" s="3">
         <v>45929</v>
       </c>
@@ -7784,7 +7787,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="254" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G254" s="3">
         <v>45930</v>
       </c>
@@ -7810,7 +7813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G255" s="3">
         <v>45930</v>
       </c>
@@ -7836,7 +7839,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G256" s="3">
         <v>45930</v>
       </c>
@@ -7862,7 +7865,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="257" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G257" s="3">
         <v>45930</v>
       </c>
@@ -7888,7 +7891,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="258" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G258" s="3">
         <v>45930</v>
       </c>
@@ -7914,7 +7917,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="259" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G259" s="3">
         <v>45930</v>
       </c>
@@ -7940,7 +7943,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="260" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G260" s="3">
         <v>45931</v>
       </c>
@@ -7966,7 +7969,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="261" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G261" s="3">
         <v>45931</v>
       </c>
@@ -7992,7 +7995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="262" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G262" s="3">
         <v>45931</v>
       </c>
@@ -8018,7 +8021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="263" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G263" s="3">
         <v>45931</v>
       </c>
@@ -8044,7 +8047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="264" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G264" s="3">
         <v>45931</v>
       </c>
@@ -8070,7 +8073,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="265" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G265" s="3">
         <v>45931</v>
       </c>
@@ -8096,7 +8099,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="266" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G266" s="3">
         <v>45931</v>
       </c>
@@ -8122,7 +8125,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="267" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G267" s="3">
         <v>45931</v>
       </c>
@@ -8148,7 +8151,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="268" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G268" s="3">
         <v>45932</v>
       </c>
@@ -8174,7 +8177,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="269" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G269" s="3">
         <v>45932</v>
       </c>
@@ -8200,7 +8203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="270" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G270" s="3">
         <v>45932</v>
       </c>
@@ -8226,7 +8229,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="271" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G271" s="3">
         <v>45932</v>
       </c>
@@ -8252,7 +8255,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="272" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G272" s="3">
         <v>45932</v>
       </c>
@@ -8278,7 +8281,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="273" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="273" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G273" s="3">
         <v>45932</v>
       </c>
@@ -8305,7 +8308,7 @@
       </c>
       <c r="O273" s="19"/>
     </row>
-    <row r="274" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="274" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G274" s="3">
         <v>45932</v>
       </c>
@@ -8332,7 +8335,7 @@
       </c>
       <c r="O274"/>
     </row>
-    <row r="275" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="275" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G275" s="3">
         <v>45932</v>
       </c>
@@ -8359,7 +8362,7 @@
       </c>
       <c r="O275"/>
     </row>
-    <row r="276" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="276" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G276" s="3">
         <v>45932</v>
       </c>
@@ -8386,7 +8389,7 @@
       </c>
       <c r="O276"/>
     </row>
-    <row r="277" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="277" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G277" s="3">
         <v>45932</v>
       </c>
@@ -8413,7 +8416,7 @@
       </c>
       <c r="O277"/>
     </row>
-    <row r="278" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="278" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G278" s="3">
         <v>45932</v>
       </c>
@@ -8440,7 +8443,7 @@
       </c>
       <c r="O278"/>
     </row>
-    <row r="279" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="279" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G279" s="3">
         <v>45933</v>
       </c>
@@ -8467,7 +8470,7 @@
       </c>
       <c r="O279"/>
     </row>
-    <row r="280" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="280" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G280" s="3">
         <v>45933</v>
       </c>
@@ -8494,7 +8497,7 @@
       </c>
       <c r="O280"/>
     </row>
-    <row r="281" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="281" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G281" s="3">
         <v>45936</v>
       </c>
@@ -8521,7 +8524,7 @@
       </c>
       <c r="O281"/>
     </row>
-    <row r="282" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="282" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G282" s="3">
         <v>45936</v>
       </c>
@@ -8548,7 +8551,7 @@
       </c>
       <c r="O282"/>
     </row>
-    <row r="283" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="283" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G283" s="3">
         <v>45936</v>
       </c>
@@ -8575,7 +8578,7 @@
       </c>
       <c r="O283"/>
     </row>
-    <row r="284" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="284" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G284" s="3">
         <v>45936</v>
       </c>
@@ -8602,7 +8605,7 @@
       </c>
       <c r="O284"/>
     </row>
-    <row r="285" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="285" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G285" s="3">
         <v>45936</v>
       </c>
@@ -8629,7 +8632,7 @@
       </c>
       <c r="O285"/>
     </row>
-    <row r="286" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="286" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G286" s="3">
         <v>45936</v>
       </c>
@@ -8656,7 +8659,7 @@
       </c>
       <c r="O286"/>
     </row>
-    <row r="287" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="287" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G287" s="3">
         <v>45936</v>
       </c>
@@ -8683,7 +8686,7 @@
       </c>
       <c r="O287"/>
     </row>
-    <row r="288" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="288" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G288" s="3">
         <v>45937</v>
       </c>
@@ -8710,7 +8713,7 @@
       </c>
       <c r="O288"/>
     </row>
-    <row r="289" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G289" s="3">
         <v>45937</v>
       </c>
@@ -8736,7 +8739,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="290" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G290" s="3">
         <v>45937</v>
       </c>
@@ -8762,7 +8765,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="291" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G291" s="3">
         <v>45937</v>
       </c>
@@ -8788,7 +8791,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="292" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G292" s="3">
         <v>45937</v>
       </c>
@@ -8814,7 +8817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="293" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G293" s="3">
         <v>45937</v>
       </c>
@@ -8840,7 +8843,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="294" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G294" s="3">
         <v>45937</v>
       </c>
@@ -8866,7 +8869,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="295" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G295" s="3">
         <v>45938</v>
       </c>
@@ -8892,7 +8895,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="296" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G296" s="3">
         <v>45938</v>
       </c>
@@ -8918,7 +8921,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="297" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G297" s="3">
         <v>45938</v>
       </c>
@@ -8944,7 +8947,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="298" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G298" s="3">
         <v>45938</v>
       </c>
@@ -8970,7 +8973,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="299" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G299" s="3">
         <v>45938</v>
       </c>
@@ -8996,7 +8999,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="300" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G300" s="3">
         <v>45938</v>
       </c>
@@ -9022,7 +9025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="301" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G301" s="3">
         <v>45938</v>
       </c>
@@ -9048,7 +9051,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="302" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G302" s="3">
         <v>45939</v>
       </c>
@@ -9074,7 +9077,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="303" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G303" s="3">
         <v>45939</v>
       </c>
@@ -9100,7 +9103,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="304" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G304" s="3">
         <v>45939</v>
       </c>
@@ -9126,7 +9129,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="305" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G305" s="3">
         <v>45939</v>
       </c>
@@ -9152,7 +9155,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="306" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G306" s="3">
         <v>45939</v>
       </c>
@@ -9178,7 +9181,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="307" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G307" s="3">
         <v>45939</v>
       </c>
@@ -9204,7 +9207,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="308" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G308" s="3">
         <v>45939</v>
       </c>
@@ -9230,7 +9233,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="309" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G309" s="3">
         <v>45939</v>
       </c>
@@ -9256,7 +9259,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="310" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G310" s="3">
         <v>45939</v>
       </c>
@@ -9282,7 +9285,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="311" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G311" s="3">
         <v>45939</v>
       </c>
@@ -9308,7 +9311,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="312" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G312" s="3">
         <v>45939</v>
       </c>
@@ -9334,7 +9337,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="313" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G313" s="3">
         <v>45939</v>
       </c>
@@ -9360,7 +9363,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="314" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G314" s="3">
         <v>45939</v>
       </c>
@@ -9386,7 +9389,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="315" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G315" s="3">
         <v>45939</v>
       </c>
@@ -9412,7 +9415,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="316" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G316" s="3">
         <v>45940</v>
       </c>
@@ -9438,7 +9441,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G317" s="3">
         <v>45943</v>
       </c>
@@ -9464,7 +9467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="318" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G318" s="3">
         <v>45943</v>
       </c>
@@ -9490,7 +9493,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="319" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G319" s="3">
         <v>45943</v>
       </c>
@@ -9516,7 +9519,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="320" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G320" s="3">
         <v>45943</v>
       </c>
@@ -9542,7 +9545,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="321" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G321" s="3">
         <v>45943</v>
       </c>
@@ -9568,7 +9571,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="322" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="322" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G322" s="3">
         <v>45943</v>
       </c>
@@ -9594,7 +9597,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="323" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G323" s="3">
         <v>45944</v>
       </c>
@@ -9620,7 +9623,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="324" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G324" s="3">
         <v>45944</v>
       </c>
@@ -9646,7 +9649,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="325" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G325" s="3">
         <v>45944</v>
       </c>
@@ -9672,7 +9675,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="326" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G326" s="3">
         <v>45944</v>
       </c>
@@ -9698,7 +9701,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="327" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G327" s="3">
         <v>45944</v>
       </c>
@@ -9724,7 +9727,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="328" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G328" s="3">
         <v>45944</v>
       </c>
@@ -9750,7 +9753,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="329" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G329" s="20">
         <v>45944</v>
       </c>
@@ -9776,7 +9779,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G330" s="3">
         <v>45945</v>
       </c>
@@ -9802,7 +9805,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="331" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G331" s="3">
         <v>45945</v>
       </c>
@@ -9828,7 +9831,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="332" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G332" s="3">
         <v>45945</v>
       </c>
@@ -9854,7 +9857,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="333" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G333" s="3">
         <v>45945</v>
       </c>
@@ -9880,7 +9883,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="334" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G334" s="3">
         <v>45945</v>
       </c>
@@ -9906,7 +9909,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="335" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G335" s="3">
         <v>45945</v>
       </c>
@@ -9932,7 +9935,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="336" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="G336" s="3">
         <v>45945</v>
       </c>
@@ -9958,7 +9961,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="337" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="337" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G337" s="3">
         <v>45946</v>
       </c>
@@ -9985,7 +9988,7 @@
       </c>
       <c r="O337"/>
     </row>
-    <row r="338" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="338" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G338" s="3">
         <v>45946</v>
       </c>
@@ -10012,7 +10015,7 @@
       </c>
       <c r="O338"/>
     </row>
-    <row r="339" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="339" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G339" s="3">
         <v>45946</v>
       </c>
@@ -10039,7 +10042,7 @@
       </c>
       <c r="O339"/>
     </row>
-    <row r="340" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="340" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G340" s="3">
         <v>45946</v>
       </c>
@@ -10066,7 +10069,7 @@
       </c>
       <c r="O340"/>
     </row>
-    <row r="341" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="341" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G341" s="3">
         <v>45946</v>
       </c>
@@ -10093,7 +10096,7 @@
       </c>
       <c r="O341"/>
     </row>
-    <row r="342" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="342" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G342" s="3">
         <v>45946</v>
       </c>
@@ -10120,7 +10123,7 @@
       </c>
       <c r="O342"/>
     </row>
-    <row r="343" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="343" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G343" s="3">
         <v>45946</v>
       </c>
@@ -10147,7 +10150,7 @@
       </c>
       <c r="O343"/>
     </row>
-    <row r="344" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="344" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G344" s="3">
         <v>45946</v>
       </c>
@@ -10174,7 +10177,7 @@
       </c>
       <c r="O344"/>
     </row>
-    <row r="345" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="345" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G345" s="3">
         <v>45946</v>
       </c>
@@ -10201,7 +10204,7 @@
       </c>
       <c r="O345"/>
     </row>
-    <row r="346" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="346" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G346" s="3">
         <v>45946</v>
       </c>
@@ -10228,7 +10231,7 @@
       </c>
       <c r="O346"/>
     </row>
-    <row r="347" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="347" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G347" s="3">
         <v>45946</v>
       </c>
@@ -10255,7 +10258,7 @@
       </c>
       <c r="O347"/>
     </row>
-    <row r="348" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="348" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G348" s="3">
         <v>45946</v>
       </c>
@@ -10282,7 +10285,7 @@
       </c>
       <c r="O348"/>
     </row>
-    <row r="349" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="349" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G349" s="3">
         <v>45946</v>
       </c>
@@ -10309,7 +10312,7 @@
       </c>
       <c r="O349"/>
     </row>
-    <row r="350" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="350" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G350" s="3">
         <v>45947</v>
       </c>
@@ -10334,7 +10337,7 @@
       </c>
       <c r="O350"/>
     </row>
-    <row r="351" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="351" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G351" s="3">
         <v>45950</v>
       </c>
@@ -10360,7 +10363,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="352" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="352" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G352" s="3">
         <v>45950</v>
       </c>
@@ -10386,7 +10389,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="353" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="353" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G353" s="3">
         <v>45950</v>
       </c>
@@ -10412,7 +10415,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="354" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="354" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G354" s="3">
         <v>45950</v>
       </c>
@@ -10438,7 +10441,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="355" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="355" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G355" s="3">
         <v>45950</v>
       </c>
@@ -10464,7 +10467,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="356" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="356" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G356" s="3">
         <v>45950</v>
       </c>
@@ -10490,7 +10493,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="357" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="357" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G357" s="3">
         <v>45950</v>
       </c>
@@ -10516,7 +10519,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="358" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="358" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G358" s="3"/>
       <c r="H358" s="4"/>
       <c r="I358" s="6"/>
@@ -10556,10 +10559,18 @@
       <c r="I360" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="J360" s="4"/>
-      <c r="K360" s="9"/>
-      <c r="L360" s="4"/>
-      <c r="M360" s="4"/>
+      <c r="J360" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="K360" s="9">
+        <v>270</v>
+      </c>
+      <c r="L360" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M360" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N360" s="6">
         <v>3</v>
       </c>
@@ -10653,11 +10664,15 @@
       </c>
     </row>
     <row r="365" spans="7:14" x14ac:dyDescent="0.25">
-      <c r="G365" s="4"/>
+      <c r="G365" s="3">
+        <v>45948</v>
+      </c>
       <c r="H365" s="4"/>
       <c r="I365" s="6"/>
       <c r="J365" s="4"/>
-      <c r="K365" s="9"/>
+      <c r="K365" s="9">
+        <v>1000</v>
+      </c>
       <c r="L365" s="4"/>
       <c r="M365" s="4"/>
       <c r="N365" s="6"/>
@@ -10703,7 +10718,13 @@
       <c r="N369" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:N364" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:N364" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+    <filterColumn colId="0">
+      <filters>
+        <dateGroupItem year="2025" month="10" day="21" dateTimeGrouping="day"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G6:N339">
     <sortCondition ref="G6:G339"/>
   </sortState>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-23 16:32
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2295" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5A02DA4-45F1-47F9-9B61-F6E7269EF944}"/>
+  <xr:revisionPtr revIDLastSave="2391" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57400DA2-A8F2-4783-BE94-621E43F72E5B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$372</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$N$384</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1832" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1887" uniqueCount="265">
   <si>
     <t>DATA</t>
   </si>
@@ -824,6 +824,15 @@
   </si>
   <si>
     <t>1</t>
+  </si>
+  <si>
+    <t>HOTEL PAULISTA</t>
+  </si>
+  <si>
+    <t>HOTEL VITORIA</t>
+  </si>
+  <si>
+    <t>HOTEL BARBACENA</t>
   </si>
 </sst>
 </file>
@@ -870,7 +879,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -919,12 +928,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -994,6 +1016,7 @@
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -1329,10 +1352,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-  <sheetPr codeName="Planilha1" filterMode="1">
+  <sheetPr codeName="Planilha1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:O374"/>
+  <dimension ref="G5:O386"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -1375,7 +1398,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="6" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>45873</v>
       </c>
@@ -1402,7 +1425,7 @@
       </c>
       <c r="O6"/>
     </row>
-    <row r="7" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>45873</v>
       </c>
@@ -1429,7 +1452,7 @@
       </c>
       <c r="O7"/>
     </row>
-    <row r="8" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>45873</v>
       </c>
@@ -1456,7 +1479,7 @@
       </c>
       <c r="O8"/>
     </row>
-    <row r="9" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>45873</v>
       </c>
@@ -1483,7 +1506,7 @@
       </c>
       <c r="O9"/>
     </row>
-    <row r="10" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>45875</v>
       </c>
@@ -1510,7 +1533,7 @@
       </c>
       <c r="O10"/>
     </row>
-    <row r="11" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>45875</v>
       </c>
@@ -1537,7 +1560,7 @@
       </c>
       <c r="O11"/>
     </row>
-    <row r="12" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>45875</v>
       </c>
@@ -1564,7 +1587,7 @@
       </c>
       <c r="O12"/>
     </row>
-    <row r="13" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>45875</v>
       </c>
@@ -1591,7 +1614,7 @@
       </c>
       <c r="O13"/>
     </row>
-    <row r="14" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>45875</v>
       </c>
@@ -1618,7 +1641,7 @@
       </c>
       <c r="O14"/>
     </row>
-    <row r="15" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>45875</v>
       </c>
@@ -1645,7 +1668,7 @@
       </c>
       <c r="O15"/>
     </row>
-    <row r="16" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>45875</v>
       </c>
@@ -1672,7 +1695,7 @@
       </c>
       <c r="O16"/>
     </row>
-    <row r="17" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>45875</v>
       </c>
@@ -1698,7 +1721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>45876</v>
       </c>
@@ -1724,7 +1747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>45876</v>
       </c>
@@ -1750,7 +1773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>45876</v>
       </c>
@@ -1776,7 +1799,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>45876</v>
       </c>
@@ -1802,7 +1825,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
         <v>45876</v>
       </c>
@@ -1828,7 +1851,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
         <v>45876</v>
       </c>
@@ -1854,7 +1877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
         <v>45876</v>
       </c>
@@ -1880,7 +1903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
         <v>45876</v>
       </c>
@@ -1906,7 +1929,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
         <v>45876</v>
       </c>
@@ -1932,7 +1955,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
         <v>45876</v>
       </c>
@@ -1958,7 +1981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>45876</v>
       </c>
@@ -1984,7 +2007,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
         <v>45880</v>
       </c>
@@ -2010,7 +2033,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
         <v>45880</v>
       </c>
@@ -2036,7 +2059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
         <v>45880</v>
       </c>
@@ -2062,7 +2085,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
         <v>45880</v>
       </c>
@@ -2088,7 +2111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
         <v>45880</v>
       </c>
@@ -2114,7 +2137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G34" s="3">
         <v>45881</v>
       </c>
@@ -2140,7 +2163,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G35" s="3">
         <v>45881</v>
       </c>
@@ -2166,7 +2189,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>45881</v>
       </c>
@@ -2192,7 +2215,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G37" s="3">
         <v>45881</v>
       </c>
@@ -2218,7 +2241,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G38" s="3">
         <v>45881</v>
       </c>
@@ -2244,7 +2267,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G39" s="3">
         <v>45881</v>
       </c>
@@ -2270,7 +2293,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="40" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G40" s="3">
         <v>45881</v>
       </c>
@@ -2296,7 +2319,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G41" s="3">
         <v>45882</v>
       </c>
@@ -2322,7 +2345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G42" s="3">
         <v>45882</v>
       </c>
@@ -2348,7 +2371,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G43" s="3">
         <v>45882</v>
       </c>
@@ -2374,7 +2397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G44" s="3">
         <v>45882</v>
       </c>
@@ -2400,7 +2423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G45" s="3">
         <v>45882</v>
       </c>
@@ -2426,7 +2449,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G46" s="3">
         <v>45882</v>
       </c>
@@ -2452,7 +2475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="47" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G47" s="3">
         <v>45883</v>
       </c>
@@ -2478,7 +2501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G48" s="3">
         <v>45883</v>
       </c>
@@ -2504,7 +2527,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G49" s="3">
         <v>45883</v>
       </c>
@@ -2530,7 +2553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="50" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G50" s="3">
         <v>45883</v>
       </c>
@@ -2556,7 +2579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G51" s="3">
         <v>45883</v>
       </c>
@@ -2582,7 +2605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G52" s="3">
         <v>45883</v>
       </c>
@@ -2608,7 +2631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="53" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G53" s="3">
         <v>45883</v>
       </c>
@@ -2634,7 +2657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G54" s="3">
         <v>45883</v>
       </c>
@@ -2660,7 +2683,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G55" s="3">
         <v>45883</v>
       </c>
@@ -2686,7 +2709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G56" s="3">
         <v>45883</v>
       </c>
@@ -2712,7 +2735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G57" s="3">
         <v>45883</v>
       </c>
@@ -2738,7 +2761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G58" s="3">
         <v>45883</v>
       </c>
@@ -2764,7 +2787,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G59" s="3">
         <v>45883</v>
       </c>
@@ -2790,7 +2813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G60" s="3">
         <v>45883</v>
       </c>
@@ -2816,7 +2839,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G61" s="3">
         <v>45883</v>
       </c>
@@ -2842,7 +2865,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G62" s="3">
         <v>45883</v>
       </c>
@@ -2868,7 +2891,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="63" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>45887</v>
       </c>
@@ -2894,7 +2917,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G64" s="3">
         <v>45887</v>
       </c>
@@ -2920,7 +2943,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G65" s="3">
         <v>45887</v>
       </c>
@@ -2946,7 +2969,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G66" s="3">
         <v>45887</v>
       </c>
@@ -2972,7 +2995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G67" s="3">
         <v>45887</v>
       </c>
@@ -2998,7 +3021,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G68" s="3">
         <v>45887</v>
       </c>
@@ -3024,7 +3047,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G69" s="3">
         <v>45887</v>
       </c>
@@ -3050,7 +3073,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="70" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G70" s="3">
         <v>45888</v>
       </c>
@@ -3076,7 +3099,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G71" s="3">
         <v>45888</v>
       </c>
@@ -3102,7 +3125,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>45888</v>
       </c>
@@ -3128,7 +3151,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G73" s="3">
         <v>45888</v>
       </c>
@@ -3154,7 +3177,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="74" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G74" s="3">
         <v>45888</v>
       </c>
@@ -3180,7 +3203,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="75" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G75" s="3">
         <v>45889</v>
       </c>
@@ -3206,7 +3229,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G76" s="3">
         <v>45889</v>
       </c>
@@ -3232,7 +3255,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="77" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G77" s="3">
         <v>45889</v>
       </c>
@@ -3258,7 +3281,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="78" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G78" s="3">
         <v>45889</v>
       </c>
@@ -3284,7 +3307,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="79" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G79" s="3">
         <v>45889</v>
       </c>
@@ -3310,7 +3333,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="80" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G80" s="3">
         <v>45889</v>
       </c>
@@ -3336,7 +3359,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="81" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G81" s="3">
         <v>45889</v>
       </c>
@@ -3362,7 +3385,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="82" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G82" s="3">
         <v>45890</v>
       </c>
@@ -3388,7 +3411,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="83" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G83" s="3">
         <v>45890</v>
       </c>
@@ -3414,7 +3437,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="84" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G84" s="3">
         <v>45890</v>
       </c>
@@ -3440,7 +3463,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="85" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G85" s="3">
         <v>45890</v>
       </c>
@@ -3466,7 +3489,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="86" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G86" s="3">
         <v>45890</v>
       </c>
@@ -3492,7 +3515,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="87" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G87" s="3">
         <v>45890</v>
       </c>
@@ -3518,7 +3541,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="88" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G88" s="3">
         <v>45890</v>
       </c>
@@ -3544,7 +3567,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="89" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G89" s="3">
         <v>45890</v>
       </c>
@@ -3570,7 +3593,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="90" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G90" s="3">
         <v>45890</v>
       </c>
@@ -3596,7 +3619,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="91" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G91" s="3">
         <v>45890</v>
       </c>
@@ -3620,7 +3643,7 @@
       </c>
       <c r="N91" s="6"/>
     </row>
-    <row r="92" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G92" s="3">
         <v>45890</v>
       </c>
@@ -3646,7 +3669,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G93" s="3">
         <v>45894</v>
       </c>
@@ -3672,7 +3695,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="94" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G94" s="3">
         <v>45894</v>
       </c>
@@ -3698,7 +3721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="95" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G95" s="3">
         <v>45894</v>
       </c>
@@ -3724,7 +3747,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G96" s="3">
         <v>45894</v>
       </c>
@@ -3750,7 +3773,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="97" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G97" s="3">
         <v>45895</v>
       </c>
@@ -3776,7 +3799,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="98" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G98" s="3">
         <v>45895</v>
       </c>
@@ -3802,7 +3825,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="99" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G99" s="3">
         <v>45895</v>
       </c>
@@ -3828,7 +3851,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="100" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G100" s="3">
         <v>45895</v>
       </c>
@@ -3854,7 +3877,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="101" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G101" s="3">
         <v>45895</v>
       </c>
@@ -3880,7 +3903,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="102" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G102" s="3">
         <v>45895</v>
       </c>
@@ -3906,7 +3929,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G103" s="3">
         <v>45895</v>
       </c>
@@ -3932,7 +3955,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="104" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G104" s="3">
         <v>45896</v>
       </c>
@@ -3958,7 +3981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G105" s="3">
         <v>45896</v>
       </c>
@@ -3984,7 +4007,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G106" s="3">
         <v>45896</v>
       </c>
@@ -4010,7 +4033,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G107" s="3">
         <v>45896</v>
       </c>
@@ -4036,7 +4059,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G108" s="3">
         <v>45896</v>
       </c>
@@ -4062,7 +4085,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G109" s="3">
         <v>45896</v>
       </c>
@@ -4088,7 +4111,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="110" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G110" s="3">
         <v>45896</v>
       </c>
@@ -4114,7 +4137,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G111" s="3">
         <v>45896</v>
       </c>
@@ -4140,7 +4163,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G112" s="3">
         <v>45897</v>
       </c>
@@ -4166,7 +4189,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="113" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="113" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G113" s="3">
         <v>45897</v>
       </c>
@@ -4192,7 +4215,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="114" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="114" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G114" s="3">
         <v>45897</v>
       </c>
@@ -4218,7 +4241,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="115" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="115" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G115" s="3">
         <v>45897</v>
       </c>
@@ -4244,7 +4267,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="116" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="116" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G116" s="3">
         <v>45897</v>
       </c>
@@ -4270,7 +4293,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="117" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="117" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G117" s="3">
         <v>45897</v>
       </c>
@@ -4296,7 +4319,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="118" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G118" s="3">
         <v>45897</v>
       </c>
@@ -4322,7 +4345,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="119" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G119" s="3">
         <v>45897</v>
       </c>
@@ -4348,7 +4371,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="120" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G120" s="3">
         <v>45897</v>
       </c>
@@ -4374,7 +4397,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="121" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G121" s="3">
         <v>45897</v>
       </c>
@@ -4400,7 +4423,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="122" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G122" s="3">
         <v>45897</v>
       </c>
@@ -4426,7 +4449,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G123" s="3">
         <v>45901</v>
       </c>
@@ -4452,7 +4475,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="124" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G124" s="3">
         <v>45901</v>
       </c>
@@ -4478,7 +4501,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="125" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G125" s="3">
         <v>45901</v>
       </c>
@@ -4504,7 +4527,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G126" s="3">
         <v>45901</v>
       </c>
@@ -4530,7 +4553,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="127" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G127" s="3">
         <v>45902</v>
       </c>
@@ -4556,7 +4579,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="128" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G128" s="3">
         <v>45902</v>
       </c>
@@ -4582,7 +4605,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="129" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G129" s="3">
         <v>45902</v>
       </c>
@@ -4608,7 +4631,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G130" s="3">
         <v>45902</v>
       </c>
@@ -4634,7 +4657,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="131" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G131" s="3">
         <v>45902</v>
       </c>
@@ -4660,7 +4683,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="132" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G132" s="3">
         <v>45902</v>
       </c>
@@ -4686,7 +4709,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="133" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G133" s="3">
         <v>45902</v>
       </c>
@@ -4712,7 +4735,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="134" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G134" s="3">
         <v>45903</v>
       </c>
@@ -4738,7 +4761,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="135" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G135" s="3">
         <v>45903</v>
       </c>
@@ -4764,7 +4787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G136" s="3">
         <v>45903</v>
       </c>
@@ -4790,7 +4813,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="137" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G137" s="3">
         <v>45903</v>
       </c>
@@ -4816,7 +4839,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="138" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="138" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G138" s="3">
         <v>45903</v>
       </c>
@@ -4842,7 +4865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="139" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="139" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G139" s="3">
         <v>45903</v>
       </c>
@@ -4868,7 +4891,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="140" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G140" s="3">
         <v>45903</v>
       </c>
@@ -4892,7 +4915,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="141" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="141" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G141" s="3">
         <v>45903</v>
       </c>
@@ -4918,7 +4941,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="142" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="142" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G142" s="3">
         <v>45903</v>
       </c>
@@ -4942,7 +4965,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="143" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G143" s="3">
         <v>45903</v>
       </c>
@@ -4968,7 +4991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="144" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G144" s="3">
         <v>45904</v>
       </c>
@@ -4994,7 +5017,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="145" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="145" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G145" s="3">
         <v>45904</v>
       </c>
@@ -5020,7 +5043,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="146" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="146" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G146" s="3">
         <v>45904</v>
       </c>
@@ -5046,7 +5069,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="147" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="147" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G147" s="3">
         <v>45904</v>
       </c>
@@ -5072,7 +5095,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="148" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G148" s="3">
         <v>45904</v>
       </c>
@@ -5098,7 +5121,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="149" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
         <v>45904</v>
       </c>
@@ -5124,7 +5147,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="150" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="150" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G150" s="3">
         <v>45904</v>
       </c>
@@ -5150,7 +5173,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="151" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="151" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G151" s="3">
         <v>45904</v>
       </c>
@@ -5176,7 +5199,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="152" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="152" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G152" s="3">
         <v>45904</v>
       </c>
@@ -5202,7 +5225,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="153" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>45908</v>
       </c>
@@ -5228,7 +5251,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="154" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="154" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G154" s="3">
         <v>45908</v>
       </c>
@@ -5254,7 +5277,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="155" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="155" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G155" s="3">
         <v>45908</v>
       </c>
@@ -5280,7 +5303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>45908</v>
       </c>
@@ -5306,7 +5329,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="157" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="157" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G157" s="3">
         <v>45909</v>
       </c>
@@ -5332,7 +5355,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="158" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="158" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G158" s="3">
         <v>45909</v>
       </c>
@@ -5358,7 +5381,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="159" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="159" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G159" s="3">
         <v>45909</v>
       </c>
@@ -5384,7 +5407,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="160" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>45909</v>
       </c>
@@ -5410,7 +5433,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="161" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="161" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G161" s="3">
         <v>45909</v>
       </c>
@@ -5436,7 +5459,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="162" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="162" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G162" s="3">
         <v>45909</v>
       </c>
@@ -5462,7 +5485,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="163" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="163" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G163" s="3">
         <v>45910</v>
       </c>
@@ -5488,7 +5511,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="164" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="164" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G164" s="3">
         <v>45910</v>
       </c>
@@ -5508,7 +5531,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="165" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="165" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G165" s="3">
         <v>45910</v>
       </c>
@@ -5534,7 +5557,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="166" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="166" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G166" s="3">
         <v>45910</v>
       </c>
@@ -5560,7 +5583,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="167" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="167" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G167" s="3">
         <v>45910</v>
       </c>
@@ -5586,7 +5609,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="168" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="168" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G168" s="3">
         <v>45910</v>
       </c>
@@ -5612,7 +5635,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="169" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="169" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G169" s="3">
         <v>45910</v>
       </c>
@@ -5638,7 +5661,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="170" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G170" s="3">
         <v>45911</v>
       </c>
@@ -5658,7 +5681,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="171" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G171" s="3">
         <v>45911</v>
       </c>
@@ -5684,7 +5707,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="172" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="172" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G172" s="3">
         <v>45911</v>
       </c>
@@ -5710,7 +5733,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="173" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G173" s="3">
         <v>45911</v>
       </c>
@@ -5736,7 +5759,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="174" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G174" s="3">
         <v>45911</v>
       </c>
@@ -5762,7 +5785,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="175" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G175" s="3">
         <v>45911</v>
       </c>
@@ -5788,7 +5811,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="176" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G176" s="3">
         <v>45911</v>
       </c>
@@ -5814,7 +5837,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="177" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
         <v>45911</v>
       </c>
@@ -5840,7 +5863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="178" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
         <v>45911</v>
       </c>
@@ -5866,7 +5889,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="179" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
         <v>45911</v>
       </c>
@@ -5892,7 +5915,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="180" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
         <v>45911</v>
       </c>
@@ -5918,7 +5941,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="181" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>45911</v>
       </c>
@@ -5944,7 +5967,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>45911</v>
       </c>
@@ -5970,7 +5993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>45915</v>
       </c>
@@ -5996,7 +6019,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>45915</v>
       </c>
@@ -6022,7 +6045,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="185" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G185" s="3">
         <v>45915</v>
       </c>
@@ -6048,7 +6071,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="186" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G186" s="3">
         <v>45915</v>
       </c>
@@ -6074,7 +6097,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="187" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G187" s="3">
         <v>45915</v>
       </c>
@@ -6100,7 +6123,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="188" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G188" s="3">
         <v>45915</v>
       </c>
@@ -6126,7 +6149,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="189" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G189" s="3">
         <v>45915</v>
       </c>
@@ -6152,7 +6175,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="190" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="190" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G190" s="3">
         <v>45916</v>
       </c>
@@ -6178,7 +6201,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="191" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="191" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G191" s="3">
         <v>45916</v>
       </c>
@@ -6204,7 +6227,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="192" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="192" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G192" s="3">
         <v>45916</v>
       </c>
@@ -6230,7 +6253,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="193" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="193" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G193" s="3">
         <v>45916</v>
       </c>
@@ -6256,7 +6279,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="194" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="194" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G194" s="3">
         <v>45916</v>
       </c>
@@ -6282,7 +6305,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="195" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="195" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G195" s="3">
         <v>45917</v>
       </c>
@@ -6308,7 +6331,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="196" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="196" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G196" s="3">
         <v>45917</v>
       </c>
@@ -6334,7 +6357,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="197" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="197" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G197" s="3">
         <v>45917</v>
       </c>
@@ -6360,7 +6383,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="198" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="198" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G198" s="3">
         <v>45917</v>
       </c>
@@ -6386,7 +6409,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="199" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="199" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G199" s="3">
         <v>45917</v>
       </c>
@@ -6412,7 +6435,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="200" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G200" s="3">
         <v>45917</v>
       </c>
@@ -6438,7 +6461,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="201" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="201" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G201" s="3">
         <v>45917</v>
       </c>
@@ -6464,7 +6487,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="202" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="202" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G202" s="3">
         <v>45918</v>
       </c>
@@ -6490,7 +6513,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="203" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="203" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G203" s="3">
         <v>45918</v>
       </c>
@@ -6516,7 +6539,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="204" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="204" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G204" s="3">
         <v>45918</v>
       </c>
@@ -6542,7 +6565,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="205" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G205" s="3">
         <v>45918</v>
       </c>
@@ -6568,7 +6591,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="206" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="206" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G206" s="3">
         <v>45918</v>
       </c>
@@ -6594,7 +6617,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="207" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="207" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G207" s="3">
         <v>45918</v>
       </c>
@@ -6620,7 +6643,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="208" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="208" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G208" s="3">
         <v>45918</v>
       </c>
@@ -6646,7 +6669,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="209" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="209" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G209" s="3">
         <v>45918</v>
       </c>
@@ -6672,7 +6695,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="210" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="210" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G210" s="3">
         <v>45918</v>
       </c>
@@ -6698,7 +6721,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="211" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="211" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G211" s="3">
         <v>45918</v>
       </c>
@@ -6724,7 +6747,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="212" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="212" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G212" s="3">
         <v>45918</v>
       </c>
@@ -6744,7 +6767,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="213" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="213" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G213" s="3">
         <v>45918</v>
       </c>
@@ -6770,7 +6793,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="214" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="214" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G214" s="3">
         <v>45918</v>
       </c>
@@ -6796,7 +6819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="215" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="215" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G215" s="3">
         <v>45922</v>
       </c>
@@ -6822,7 +6845,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="216" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="216" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G216" s="3">
         <v>45922</v>
       </c>
@@ -6848,7 +6871,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="217" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="217" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G217" s="3">
         <v>45922</v>
       </c>
@@ -6874,7 +6897,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="218" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="218" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G218" s="3">
         <v>45922</v>
       </c>
@@ -6900,7 +6923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="219" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="219" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G219" s="3">
         <v>45922</v>
       </c>
@@ -6926,7 +6949,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="220" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="220" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G220" s="3">
         <v>45922</v>
       </c>
@@ -6952,7 +6975,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="221" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="221" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G221" s="3">
         <v>45922</v>
       </c>
@@ -6978,7 +7001,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="222" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G222" s="3">
         <v>45923</v>
       </c>
@@ -7004,7 +7027,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="223" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="223" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G223" s="3">
         <v>45923</v>
       </c>
@@ -7030,7 +7053,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="224" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="224" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G224" s="3">
         <v>45923</v>
       </c>
@@ -7056,7 +7079,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="225" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="225" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G225" s="3">
         <v>45923</v>
       </c>
@@ -7082,7 +7105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="226" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G226" s="3">
         <v>45923</v>
       </c>
@@ -7108,7 +7131,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="227" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="227" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G227" s="3">
         <v>45923</v>
       </c>
@@ -7134,7 +7157,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="228" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G228" s="3">
         <v>45924</v>
       </c>
@@ -7160,7 +7183,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="229" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="229" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G229" s="3">
         <v>45924</v>
       </c>
@@ -7186,7 +7209,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="230" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="230" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G230" s="3">
         <v>45924</v>
       </c>
@@ -7212,7 +7235,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="231" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="231" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G231" s="3">
         <v>45924</v>
       </c>
@@ -7238,7 +7261,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="232" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G232" s="3">
         <v>45924</v>
       </c>
@@ -7264,7 +7287,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="233" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G233" s="3">
         <v>45924</v>
       </c>
@@ -7290,7 +7313,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="234" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G234" s="3">
         <v>45924</v>
       </c>
@@ -7316,7 +7339,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="235" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="235" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G235" s="3">
         <v>45924</v>
       </c>
@@ -7342,7 +7365,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="236" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="236" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G236" s="3">
         <v>45925</v>
       </c>
@@ -7368,7 +7391,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="237" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="237" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G237" s="3">
         <v>45925</v>
       </c>
@@ -7394,7 +7417,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="238" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="238" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G238" s="3">
         <v>45925</v>
       </c>
@@ -7420,7 +7443,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="239" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="239" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G239" s="3">
         <v>45925</v>
       </c>
@@ -7446,7 +7469,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="240" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="240" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G240" s="3">
         <v>45925</v>
       </c>
@@ -7472,7 +7495,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="241" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="241" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G241" s="3">
         <v>45925</v>
       </c>
@@ -7498,7 +7521,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="242" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="242" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G242" s="3">
         <v>45925</v>
       </c>
@@ -7524,7 +7547,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="243" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="243" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G243" s="3">
         <v>45925</v>
       </c>
@@ -7550,7 +7573,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="244" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="244" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G244" s="3">
         <v>45925</v>
       </c>
@@ -7576,7 +7599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="245" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="245" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G245" s="3">
         <v>45925</v>
       </c>
@@ -7602,7 +7625,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="246" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="246" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G246" s="3">
         <v>45925</v>
       </c>
@@ -7628,7 +7651,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="247" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="247" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G247" s="3">
         <v>45929</v>
       </c>
@@ -7654,7 +7677,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="248" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="248" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G248" s="3">
         <v>45929</v>
       </c>
@@ -7680,7 +7703,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="249" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="249" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G249" s="3">
         <v>45929</v>
       </c>
@@ -7706,7 +7729,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="250" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="250" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G250" s="3">
         <v>45929</v>
       </c>
@@ -7732,7 +7755,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="251" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="251" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G251" s="3">
         <v>45929</v>
       </c>
@@ -7758,7 +7781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="252" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G252" s="3">
         <v>45929</v>
       </c>
@@ -7784,7 +7807,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="253" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="253" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G253" s="3">
         <v>45929</v>
       </c>
@@ -7810,7 +7833,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="254" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="254" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G254" s="3">
         <v>45930</v>
       </c>
@@ -7836,7 +7859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="255" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G255" s="3">
         <v>45930</v>
       </c>
@@ -7862,7 +7885,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" spans="7:14" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="256" spans="7:14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="G256" s="3">
         <v>45930</v>
       </c>
@@ -7888,7 +7911,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="257" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="257" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G257" s="3">
         <v>45930</v>
       </c>
@@ -7915,7 +7938,7 @@
       </c>
       <c r="O257"/>
     </row>
-    <row r="258" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="258" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G258" s="3">
         <v>45930</v>
       </c>
@@ -7942,7 +7965,7 @@
       </c>
       <c r="O258"/>
     </row>
-    <row r="259" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="259" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G259" s="3">
         <v>45930</v>
       </c>
@@ -10619,7 +10642,7 @@
       </c>
       <c r="O357" s="27"/>
     </row>
-    <row r="358" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="358" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G358" s="3"/>
       <c r="H358" s="4"/>
       <c r="I358" s="6"/>
@@ -11010,35 +11033,329 @@
       </c>
     </row>
     <row r="373" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G373" s="4"/>
-      <c r="H373" s="4"/>
-      <c r="I373" s="6"/>
-      <c r="J373" s="4"/>
-      <c r="K373" s="9"/>
-      <c r="L373" s="4"/>
-      <c r="M373" s="4"/>
-      <c r="N373" s="6"/>
+      <c r="G373" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H373" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I373" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="J373" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="K373" s="9">
+        <v>198</v>
+      </c>
+      <c r="L373" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M373" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N373" s="6">
+        <v>2</v>
+      </c>
       <c r="O373" s="27"/>
     </row>
     <row r="374" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G374" s="4"/>
-      <c r="H374" s="4"/>
-      <c r="I374" s="6"/>
-      <c r="J374" s="4"/>
-      <c r="K374" s="9"/>
-      <c r="L374" s="4"/>
-      <c r="M374" s="4"/>
-      <c r="N374" s="6"/>
+      <c r="G374" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H374" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I374" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="J374" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K374" s="9">
+        <v>170</v>
+      </c>
+      <c r="L374" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M374" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N374" s="6">
+        <v>2</v>
+      </c>
       <c r="O374" s="27"/>
     </row>
+    <row r="375" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G375" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H375" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I375" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J375" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K375" s="9">
+        <v>150</v>
+      </c>
+      <c r="L375" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="M375" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N375" s="6">
+        <v>2</v>
+      </c>
+      <c r="O375" s="27"/>
+    </row>
+    <row r="376" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G376" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H376" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I376" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J376" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="K376" s="9">
+        <v>200</v>
+      </c>
+      <c r="L376" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="M376" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N376" s="6">
+        <v>2</v>
+      </c>
+      <c r="O376" s="27"/>
+    </row>
+    <row r="377" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G377" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H377" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="I377" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="J377" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="K377" s="9">
+        <v>190</v>
+      </c>
+      <c r="L377" s="4" t="s">
+        <v>264</v>
+      </c>
+      <c r="M377" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N377" s="6">
+        <v>2</v>
+      </c>
+      <c r="O377" s="27"/>
+    </row>
+    <row r="378" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G378" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H378" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="I378" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J378" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K378" s="9">
+        <v>240</v>
+      </c>
+      <c r="L378" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="M378" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N378" s="6">
+        <v>2</v>
+      </c>
+      <c r="O378" s="27"/>
+    </row>
+    <row r="379" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G379" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H379" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I379" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J379" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="K379" s="9">
+        <v>150</v>
+      </c>
+      <c r="L379" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="M379" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N379" s="6">
+        <v>2</v>
+      </c>
+      <c r="O379" s="27"/>
+    </row>
+    <row r="380" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G380" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H380" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="I380" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="J380" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K380" s="9">
+        <v>280</v>
+      </c>
+      <c r="L380" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M380" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N380" s="6">
+        <v>2</v>
+      </c>
+      <c r="O380" s="27"/>
+    </row>
+    <row r="381" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G381" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H381" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I381" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="J381" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="K381" s="9">
+        <v>200</v>
+      </c>
+      <c r="L381" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="M381" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N381" s="6">
+        <v>2</v>
+      </c>
+      <c r="O381" s="27"/>
+    </row>
+    <row r="382" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G382" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H382" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I382" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J382" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K382" s="9">
+        <v>180</v>
+      </c>
+      <c r="L382" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="M382" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N382" s="6">
+        <v>1</v>
+      </c>
+      <c r="O382" s="27"/>
+    </row>
+    <row r="383" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="O383" s="29"/>
+    </row>
+    <row r="384" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G384" s="3">
+        <v>45953</v>
+      </c>
+      <c r="H384" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="I384" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J384" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="K384" s="9">
+        <v>170</v>
+      </c>
+      <c r="L384" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="M384" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N384" s="6">
+        <v>1</v>
+      </c>
+      <c r="O384" s="27"/>
+    </row>
+    <row r="385" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G385" s="4"/>
+      <c r="H385" s="4"/>
+      <c r="I385" s="6"/>
+      <c r="J385" s="4"/>
+      <c r="K385" s="9"/>
+      <c r="L385" s="4"/>
+      <c r="M385" s="4"/>
+      <c r="N385" s="6"/>
+      <c r="O385" s="27"/>
+    </row>
+    <row r="386" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G386" s="4"/>
+      <c r="H386" s="4"/>
+      <c r="I386" s="6"/>
+      <c r="J386" s="4"/>
+      <c r="K386" s="9"/>
+      <c r="L386" s="4"/>
+      <c r="M386" s="4"/>
+      <c r="N386" s="6"/>
+      <c r="O386" s="27"/>
+    </row>
   </sheetData>
-  <autoFilter ref="G5:N372" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-    <filterColumn colId="0">
-      <filters>
-        <dateGroupItem year="2025" month="10" dateTimeGrouping="month"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="G5:N384" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G6:N339">
     <sortCondition ref="G6:G339"/>
   </sortState>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-24 16:57
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2399" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACEBB2A5-DBDC-490F-BCB3-316D4B0A50DA}"/>
+  <xr:revisionPtr revIDLastSave="2401" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FCCFA95-2D75-4E70-8CD0-F8A1FAFF7A61}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -8451,7 +8451,7 @@
       </c>
       <c r="O276" s="6"/>
     </row>
-    <row r="277" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G277" s="3">
         <v>45932</v>
       </c>
@@ -8667,7 +8667,7 @@
       </c>
       <c r="O284" s="6"/>
     </row>
-    <row r="285" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G285" s="3">
         <v>45936</v>
       </c>
@@ -9450,7 +9450,7 @@
       </c>
       <c r="O313" s="6"/>
     </row>
-    <row r="314" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="314" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G314" s="3">
         <v>45939</v>
       </c>
@@ -9533,7 +9533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="317" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G317" s="3">
         <v>45943</v>
       </c>
@@ -9560,7 +9560,7 @@
       </c>
       <c r="O317" s="6"/>
     </row>
-    <row r="318" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="318" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G318" s="3">
         <v>45943</v>
       </c>
@@ -9587,7 +9587,7 @@
       </c>
       <c r="O318" s="6"/>
     </row>
-    <row r="319" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="319" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G319" s="3">
         <v>45943</v>
       </c>
@@ -9614,7 +9614,7 @@
       </c>
       <c r="O319" s="6"/>
     </row>
-    <row r="320" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="320" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G320" s="3">
         <v>45943</v>
       </c>
@@ -9641,7 +9641,7 @@
       </c>
       <c r="O320" s="6"/>
     </row>
-    <row r="321" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="321" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G321" s="3">
         <v>45943</v>
       </c>
@@ -9695,7 +9695,7 @@
       </c>
       <c r="O322" s="6"/>
     </row>
-    <row r="323" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="323" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G323" s="3">
         <v>45944</v>
       </c>
@@ -9722,7 +9722,7 @@
       </c>
       <c r="O323" s="6"/>
     </row>
-    <row r="324" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="324" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G324" s="3">
         <v>45944</v>
       </c>
@@ -9749,7 +9749,7 @@
       </c>
       <c r="O324" s="6"/>
     </row>
-    <row r="325" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="325" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G325" s="3">
         <v>45944</v>
       </c>
@@ -9776,7 +9776,7 @@
       </c>
       <c r="O325" s="6"/>
     </row>
-    <row r="326" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="326" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G326" s="3">
         <v>45944</v>
       </c>
@@ -9803,7 +9803,7 @@
       </c>
       <c r="O326" s="6"/>
     </row>
-    <row r="327" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="327" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G327" s="3">
         <v>45944</v>
       </c>
@@ -9830,7 +9830,7 @@
       </c>
       <c r="O327" s="6"/>
     </row>
-    <row r="328" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="328" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G328" s="3">
         <v>45944</v>
       </c>
@@ -9857,7 +9857,7 @@
       </c>
       <c r="O328" s="6"/>
     </row>
-    <row r="329" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="329" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G329" s="19">
         <v>45944</v>
       </c>
@@ -9886,7 +9886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="330" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G330" s="3">
         <v>45945</v>
       </c>
@@ -9913,7 +9913,7 @@
       </c>
       <c r="O330" s="6"/>
     </row>
-    <row r="331" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="331" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G331" s="3">
         <v>45945</v>
       </c>
@@ -9940,7 +9940,7 @@
       </c>
       <c r="O331" s="6"/>
     </row>
-    <row r="332" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="332" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G332" s="3">
         <v>45945</v>
       </c>
@@ -9967,7 +9967,7 @@
       </c>
       <c r="O332" s="6"/>
     </row>
-    <row r="333" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="333" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G333" s="3">
         <v>45945</v>
       </c>
@@ -9994,7 +9994,7 @@
       </c>
       <c r="O333" s="6"/>
     </row>
-    <row r="334" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="334" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G334" s="3">
         <v>45945</v>
       </c>
@@ -10021,7 +10021,7 @@
       </c>
       <c r="O334" s="6"/>
     </row>
-    <row r="335" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="335" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G335" s="3">
         <v>45945</v>
       </c>
@@ -10048,7 +10048,7 @@
       </c>
       <c r="O335" s="6"/>
     </row>
-    <row r="336" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="336" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G336" s="3">
         <v>45945</v>
       </c>
@@ -10075,7 +10075,7 @@
       </c>
       <c r="O336" s="6"/>
     </row>
-    <row r="337" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="337" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G337" s="3">
         <v>45946</v>
       </c>
@@ -10102,7 +10102,7 @@
       </c>
       <c r="O337" s="6"/>
     </row>
-    <row r="338" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="338" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G338" s="3">
         <v>45946</v>
       </c>
@@ -10129,7 +10129,7 @@
       </c>
       <c r="O338" s="6"/>
     </row>
-    <row r="339" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="339" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G339" s="3">
         <v>45946</v>
       </c>
@@ -10156,7 +10156,7 @@
       </c>
       <c r="O339" s="6"/>
     </row>
-    <row r="340" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="340" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G340" s="3">
         <v>45946</v>
       </c>
@@ -10183,7 +10183,7 @@
       </c>
       <c r="O340" s="6"/>
     </row>
-    <row r="341" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="341" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G341" s="3">
         <v>45946</v>
       </c>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="O341" s="6"/>
     </row>
-    <row r="342" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="342" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G342" s="3">
         <v>45946</v>
       </c>
@@ -10237,7 +10237,7 @@
       </c>
       <c r="O342" s="6"/>
     </row>
-    <row r="343" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="343" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G343" s="3">
         <v>45946</v>
       </c>
@@ -10264,7 +10264,7 @@
       </c>
       <c r="O343" s="6"/>
     </row>
-    <row r="344" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="344" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G344" s="3">
         <v>45946</v>
       </c>
@@ -10291,7 +10291,7 @@
       </c>
       <c r="O344" s="6"/>
     </row>
-    <row r="345" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="345" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G345" s="3">
         <v>45946</v>
       </c>
@@ -10345,7 +10345,7 @@
       </c>
       <c r="O346" s="6"/>
     </row>
-    <row r="347" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="347" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G347" s="3">
         <v>45946</v>
       </c>
@@ -10372,7 +10372,7 @@
       </c>
       <c r="O347" s="6"/>
     </row>
-    <row r="348" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="348" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G348" s="3">
         <v>45946</v>
       </c>
@@ -10399,7 +10399,7 @@
       </c>
       <c r="O348" s="6"/>
     </row>
-    <row r="349" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="349" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G349" s="3">
         <v>45946</v>
       </c>
@@ -10426,7 +10426,7 @@
       </c>
       <c r="O349" s="6"/>
     </row>
-    <row r="350" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="350" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G350" s="19">
         <v>45947</v>
       </c>
@@ -10617,7 +10617,7 @@
       </c>
       <c r="O356" s="27"/>
     </row>
-    <row r="357" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="357" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G357" s="3">
         <v>45950</v>
       </c>
@@ -11250,7 +11250,7 @@
       </c>
       <c r="O380" s="27"/>
     </row>
-    <row r="381" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="381" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G381" s="3">
         <v>45953</v>
       </c>
@@ -11360,11 +11360,12 @@
   <autoFilter ref="G5:N384" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="10" day="13" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="10" day="14" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="10" day="15" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="10" day="16" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="10" day="17" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="10" dateTimeGrouping="month"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="1">
+      <filters>
+        <filter val="CRISTIANO"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-24 17:13
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2401" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FCCFA95-2D75-4E70-8CD0-F8A1FAFF7A61}"/>
+  <xr:revisionPtr revIDLastSave="2406" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9350F7B-74DC-4F83-807A-DA83B4C03AB8}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -7992,7 +7992,7 @@
       </c>
       <c r="O259"/>
     </row>
-    <row r="260" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="260" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G260" s="3">
         <v>45931</v>
       </c>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="O260" s="6"/>
     </row>
-    <row r="261" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="261" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G261" s="3">
         <v>45931</v>
       </c>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="O261" s="6"/>
     </row>
-    <row r="262" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="262" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G262" s="3">
         <v>45931</v>
       </c>
@@ -8073,7 +8073,7 @@
       </c>
       <c r="O262" s="6"/>
     </row>
-    <row r="263" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="263" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G263" s="3">
         <v>45931</v>
       </c>
@@ -8100,7 +8100,7 @@
       </c>
       <c r="O263" s="6"/>
     </row>
-    <row r="264" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="264" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G264" s="3">
         <v>45931</v>
       </c>
@@ -8127,7 +8127,7 @@
       </c>
       <c r="O264" s="6"/>
     </row>
-    <row r="265" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="265" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G265" s="3">
         <v>45931</v>
       </c>
@@ -8154,7 +8154,7 @@
       </c>
       <c r="O265" s="6"/>
     </row>
-    <row r="266" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="266" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G266" s="3">
         <v>45931</v>
       </c>
@@ -8181,7 +8181,7 @@
       </c>
       <c r="O266" s="6"/>
     </row>
-    <row r="267" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="267" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G267" s="3">
         <v>45931</v>
       </c>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="O267" s="6"/>
     </row>
-    <row r="268" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="268" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G268" s="3">
         <v>45932</v>
       </c>
@@ -8235,7 +8235,7 @@
       </c>
       <c r="O268" s="6"/>
     </row>
-    <row r="269" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="269" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G269" s="3">
         <v>45932</v>
       </c>
@@ -8262,7 +8262,7 @@
       </c>
       <c r="O269" s="6"/>
     </row>
-    <row r="270" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="270" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G270" s="3">
         <v>45932</v>
       </c>
@@ -8289,7 +8289,7 @@
       </c>
       <c r="O270" s="6"/>
     </row>
-    <row r="271" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="271" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G271" s="3">
         <v>45932</v>
       </c>
@@ -8316,7 +8316,7 @@
       </c>
       <c r="O271" s="6"/>
     </row>
-    <row r="272" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G272" s="3">
         <v>45932</v>
       </c>
@@ -8343,7 +8343,7 @@
       </c>
       <c r="O272" s="6"/>
     </row>
-    <row r="273" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G273" s="3">
         <v>45932</v>
       </c>
@@ -8370,7 +8370,7 @@
       </c>
       <c r="O273" s="4"/>
     </row>
-    <row r="274" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G274" s="3">
         <v>45932</v>
       </c>
@@ -8397,7 +8397,7 @@
       </c>
       <c r="O274" s="6"/>
     </row>
-    <row r="275" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G275" s="3">
         <v>45932</v>
       </c>
@@ -8424,7 +8424,7 @@
       </c>
       <c r="O275" s="6"/>
     </row>
-    <row r="276" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G276" s="3">
         <v>45932</v>
       </c>
@@ -8478,7 +8478,7 @@
       </c>
       <c r="O277" s="6"/>
     </row>
-    <row r="278" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G278" s="3">
         <v>45932</v>
       </c>
@@ -8505,61 +8505,65 @@
       </c>
       <c r="O278" s="6"/>
     </row>
-    <row r="279" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G279" s="3">
+    <row r="279" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G279" s="19">
         <v>45933</v>
       </c>
-      <c r="H279" s="4" t="s">
+      <c r="H279" s="20" t="s">
         <v>143</v>
       </c>
-      <c r="I279" s="6" t="s">
+      <c r="I279" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="J279" s="4" t="s">
+      <c r="J279" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="K279" s="9">
+      <c r="K279" s="22">
         <v>230</v>
       </c>
-      <c r="L279" s="4" t="s">
+      <c r="L279" s="20" t="s">
         <v>176</v>
       </c>
-      <c r="M279" s="4" t="s">
+      <c r="M279" s="20" t="s">
         <v>8</v>
       </c>
       <c r="N279" s="6">
         <v>1</v>
       </c>
-      <c r="O279" s="6"/>
-    </row>
-    <row r="280" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G280" s="3">
+      <c r="O279" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="280" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G280" s="19">
         <v>45933</v>
       </c>
-      <c r="H280" s="4" t="s">
+      <c r="H280" s="20" t="s">
         <v>140</v>
       </c>
-      <c r="I280" s="6" t="s">
+      <c r="I280" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="J280" s="4" t="s">
+      <c r="J280" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="K280" s="9">
+      <c r="K280" s="22">
         <v>200</v>
       </c>
-      <c r="L280" s="4" t="s">
+      <c r="L280" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="M280" s="4" t="s">
+      <c r="M280" s="20" t="s">
         <v>8</v>
       </c>
       <c r="N280" s="6">
         <v>1</v>
       </c>
-      <c r="O280" s="6"/>
-    </row>
-    <row r="281" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O280" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="281" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G281" s="3">
         <v>45936</v>
       </c>
@@ -8586,7 +8590,7 @@
       </c>
       <c r="O281" s="6"/>
     </row>
-    <row r="282" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G282" s="3">
         <v>45936</v>
       </c>
@@ -8613,7 +8617,7 @@
       </c>
       <c r="O282" s="6"/>
     </row>
-    <row r="283" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G283" s="3">
         <v>45936</v>
       </c>
@@ -8640,7 +8644,7 @@
       </c>
       <c r="O283" s="6"/>
     </row>
-    <row r="284" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G284" s="3">
         <v>45936</v>
       </c>
@@ -8694,7 +8698,7 @@
       </c>
       <c r="O285" s="6"/>
     </row>
-    <row r="286" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G286" s="3">
         <v>45936</v>
       </c>
@@ -8721,7 +8725,7 @@
       </c>
       <c r="O286" s="6"/>
     </row>
-    <row r="287" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G287" s="3">
         <v>45936</v>
       </c>
@@ -8748,7 +8752,7 @@
       </c>
       <c r="O287" s="6"/>
     </row>
-    <row r="288" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G288" s="3">
         <v>45937</v>
       </c>
@@ -8775,7 +8779,7 @@
       </c>
       <c r="O288" s="6"/>
     </row>
-    <row r="289" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G289" s="3">
         <v>45937</v>
       </c>
@@ -8802,7 +8806,7 @@
       </c>
       <c r="O289" s="6"/>
     </row>
-    <row r="290" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="290" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G290" s="3">
         <v>45937</v>
       </c>
@@ -8829,7 +8833,7 @@
       </c>
       <c r="O290" s="6"/>
     </row>
-    <row r="291" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="291" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G291" s="3">
         <v>45937</v>
       </c>
@@ -8856,7 +8860,7 @@
       </c>
       <c r="O291" s="6"/>
     </row>
-    <row r="292" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="292" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G292" s="3">
         <v>45937</v>
       </c>
@@ -8883,7 +8887,7 @@
       </c>
       <c r="O292" s="6"/>
     </row>
-    <row r="293" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="293" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G293" s="3">
         <v>45937</v>
       </c>
@@ -8910,7 +8914,7 @@
       </c>
       <c r="O293" s="6"/>
     </row>
-    <row r="294" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="294" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G294" s="3">
         <v>45937</v>
       </c>
@@ -8937,7 +8941,7 @@
       </c>
       <c r="O294" s="6"/>
     </row>
-    <row r="295" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="295" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G295" s="3">
         <v>45938</v>
       </c>
@@ -8964,7 +8968,7 @@
       </c>
       <c r="O295" s="6"/>
     </row>
-    <row r="296" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="296" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G296" s="3">
         <v>45938</v>
       </c>
@@ -8991,7 +8995,7 @@
       </c>
       <c r="O296" s="6"/>
     </row>
-    <row r="297" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="297" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G297" s="3">
         <v>45938</v>
       </c>
@@ -9018,7 +9022,7 @@
       </c>
       <c r="O297" s="6"/>
     </row>
-    <row r="298" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="298" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G298" s="3">
         <v>45938</v>
       </c>
@@ -9045,7 +9049,7 @@
       </c>
       <c r="O298" s="6"/>
     </row>
-    <row r="299" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="299" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G299" s="3">
         <v>45938</v>
       </c>
@@ -9072,7 +9076,7 @@
       </c>
       <c r="O299" s="6"/>
     </row>
-    <row r="300" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="300" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G300" s="3">
         <v>45938</v>
       </c>
@@ -9099,7 +9103,7 @@
       </c>
       <c r="O300" s="6"/>
     </row>
-    <row r="301" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="301" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G301" s="3">
         <v>45938</v>
       </c>
@@ -9126,7 +9130,7 @@
       </c>
       <c r="O301" s="6"/>
     </row>
-    <row r="302" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="302" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G302" s="3">
         <v>45939</v>
       </c>
@@ -9153,7 +9157,7 @@
       </c>
       <c r="O302" s="6"/>
     </row>
-    <row r="303" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="303" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G303" s="3">
         <v>45939</v>
       </c>
@@ -9180,7 +9184,7 @@
       </c>
       <c r="O303" s="6"/>
     </row>
-    <row r="304" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G304" s="3">
         <v>45939</v>
       </c>
@@ -9207,7 +9211,7 @@
       </c>
       <c r="O304" s="6"/>
     </row>
-    <row r="305" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="305" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G305" s="3">
         <v>45939</v>
       </c>
@@ -9234,7 +9238,7 @@
       </c>
       <c r="O305" s="6"/>
     </row>
-    <row r="306" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="306" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G306" s="3">
         <v>45939</v>
       </c>
@@ -9261,7 +9265,7 @@
       </c>
       <c r="O306" s="6"/>
     </row>
-    <row r="307" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="307" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G307" s="3">
         <v>45939</v>
       </c>
@@ -9288,7 +9292,7 @@
       </c>
       <c r="O307" s="6"/>
     </row>
-    <row r="308" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="308" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G308" s="3">
         <v>45939</v>
       </c>
@@ -9315,7 +9319,7 @@
       </c>
       <c r="O308" s="6"/>
     </row>
-    <row r="309" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="309" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G309" s="3">
         <v>45939</v>
       </c>
@@ -9342,7 +9346,7 @@
       </c>
       <c r="O309" s="6"/>
     </row>
-    <row r="310" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="310" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G310" s="3">
         <v>45939</v>
       </c>
@@ -9369,7 +9373,7 @@
       </c>
       <c r="O310" s="6"/>
     </row>
-    <row r="311" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="311" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G311" s="3">
         <v>45939</v>
       </c>
@@ -9396,7 +9400,7 @@
       </c>
       <c r="O311" s="6"/>
     </row>
-    <row r="312" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="312" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G312" s="3">
         <v>45939</v>
       </c>
@@ -9423,7 +9427,7 @@
       </c>
       <c r="O312" s="6"/>
     </row>
-    <row r="313" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="313" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G313" s="3">
         <v>45939</v>
       </c>
@@ -9477,7 +9481,7 @@
       </c>
       <c r="O314" s="6"/>
     </row>
-    <row r="315" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="315" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G315" s="3">
         <v>45939</v>
       </c>
@@ -9504,7 +9508,7 @@
       </c>
       <c r="O315" s="6"/>
     </row>
-    <row r="316" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="316" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G316" s="19">
         <v>45940</v>
       </c>
@@ -9533,7 +9537,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="317" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="317" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G317" s="3">
         <v>45943</v>
       </c>
@@ -9560,7 +9564,7 @@
       </c>
       <c r="O317" s="6"/>
     </row>
-    <row r="318" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="318" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G318" s="3">
         <v>45943</v>
       </c>
@@ -9587,7 +9591,7 @@
       </c>
       <c r="O318" s="6"/>
     </row>
-    <row r="319" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="319" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G319" s="3">
         <v>45943</v>
       </c>
@@ -9614,7 +9618,7 @@
       </c>
       <c r="O319" s="6"/>
     </row>
-    <row r="320" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="320" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G320" s="3">
         <v>45943</v>
       </c>
@@ -9641,7 +9645,7 @@
       </c>
       <c r="O320" s="6"/>
     </row>
-    <row r="321" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="321" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G321" s="3">
         <v>45943</v>
       </c>
@@ -9695,7 +9699,7 @@
       </c>
       <c r="O322" s="6"/>
     </row>
-    <row r="323" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="323" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G323" s="3">
         <v>45944</v>
       </c>
@@ -9722,7 +9726,7 @@
       </c>
       <c r="O323" s="6"/>
     </row>
-    <row r="324" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="324" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G324" s="3">
         <v>45944</v>
       </c>
@@ -9749,7 +9753,7 @@
       </c>
       <c r="O324" s="6"/>
     </row>
-    <row r="325" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="325" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G325" s="3">
         <v>45944</v>
       </c>
@@ -9776,7 +9780,7 @@
       </c>
       <c r="O325" s="6"/>
     </row>
-    <row r="326" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="326" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G326" s="3">
         <v>45944</v>
       </c>
@@ -9803,7 +9807,7 @@
       </c>
       <c r="O326" s="6"/>
     </row>
-    <row r="327" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="327" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G327" s="3">
         <v>45944</v>
       </c>
@@ -9830,7 +9834,7 @@
       </c>
       <c r="O327" s="6"/>
     </row>
-    <row r="328" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="328" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G328" s="3">
         <v>45944</v>
       </c>
@@ -9857,7 +9861,7 @@
       </c>
       <c r="O328" s="6"/>
     </row>
-    <row r="329" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="329" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G329" s="19">
         <v>45944</v>
       </c>
@@ -9886,7 +9890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="330" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="330" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G330" s="3">
         <v>45945</v>
       </c>
@@ -9913,7 +9917,7 @@
       </c>
       <c r="O330" s="6"/>
     </row>
-    <row r="331" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="331" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G331" s="3">
         <v>45945</v>
       </c>
@@ -9940,7 +9944,7 @@
       </c>
       <c r="O331" s="6"/>
     </row>
-    <row r="332" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="332" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G332" s="3">
         <v>45945</v>
       </c>
@@ -9967,7 +9971,7 @@
       </c>
       <c r="O332" s="6"/>
     </row>
-    <row r="333" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="333" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G333" s="3">
         <v>45945</v>
       </c>
@@ -9994,7 +9998,7 @@
       </c>
       <c r="O333" s="6"/>
     </row>
-    <row r="334" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="334" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G334" s="3">
         <v>45945</v>
       </c>
@@ -10021,7 +10025,7 @@
       </c>
       <c r="O334" s="6"/>
     </row>
-    <row r="335" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="335" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G335" s="3">
         <v>45945</v>
       </c>
@@ -10048,7 +10052,7 @@
       </c>
       <c r="O335" s="6"/>
     </row>
-    <row r="336" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="336" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G336" s="3">
         <v>45945</v>
       </c>
@@ -10075,7 +10079,7 @@
       </c>
       <c r="O336" s="6"/>
     </row>
-    <row r="337" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G337" s="3">
         <v>45946</v>
       </c>
@@ -10102,7 +10106,7 @@
       </c>
       <c r="O337" s="6"/>
     </row>
-    <row r="338" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G338" s="3">
         <v>45946</v>
       </c>
@@ -10129,7 +10133,7 @@
       </c>
       <c r="O338" s="6"/>
     </row>
-    <row r="339" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G339" s="3">
         <v>45946</v>
       </c>
@@ -10156,7 +10160,7 @@
       </c>
       <c r="O339" s="6"/>
     </row>
-    <row r="340" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G340" s="3">
         <v>45946</v>
       </c>
@@ -10183,7 +10187,7 @@
       </c>
       <c r="O340" s="6"/>
     </row>
-    <row r="341" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="341" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G341" s="3">
         <v>45946</v>
       </c>
@@ -10210,7 +10214,7 @@
       </c>
       <c r="O341" s="6"/>
     </row>
-    <row r="342" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="342" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G342" s="3">
         <v>45946</v>
       </c>
@@ -10237,7 +10241,7 @@
       </c>
       <c r="O342" s="6"/>
     </row>
-    <row r="343" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="343" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G343" s="3">
         <v>45946</v>
       </c>
@@ -10264,7 +10268,7 @@
       </c>
       <c r="O343" s="6"/>
     </row>
-    <row r="344" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="344" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G344" s="3">
         <v>45946</v>
       </c>
@@ -10291,7 +10295,7 @@
       </c>
       <c r="O344" s="6"/>
     </row>
-    <row r="345" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="345" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G345" s="3">
         <v>45946</v>
       </c>
@@ -10345,7 +10349,7 @@
       </c>
       <c r="O346" s="6"/>
     </row>
-    <row r="347" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="347" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G347" s="3">
         <v>45946</v>
       </c>
@@ -10372,7 +10376,7 @@
       </c>
       <c r="O347" s="6"/>
     </row>
-    <row r="348" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="348" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G348" s="3">
         <v>45946</v>
       </c>
@@ -10399,7 +10403,7 @@
       </c>
       <c r="O348" s="6"/>
     </row>
-    <row r="349" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="349" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G349" s="3">
         <v>45946</v>
       </c>
@@ -10426,7 +10430,7 @@
       </c>
       <c r="O349" s="6"/>
     </row>
-    <row r="350" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="350" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G350" s="19">
         <v>45947</v>
       </c>
@@ -10455,7 +10459,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="351" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="351" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G351" s="3">
         <v>45950</v>
       </c>
@@ -10482,7 +10486,7 @@
       </c>
       <c r="O351" s="27"/>
     </row>
-    <row r="352" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="352" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G352" s="3">
         <v>45950</v>
       </c>
@@ -10509,7 +10513,7 @@
       </c>
       <c r="O352" s="27"/>
     </row>
-    <row r="353" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="353" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G353" s="3">
         <v>45950</v>
       </c>
@@ -10536,7 +10540,7 @@
       </c>
       <c r="O353" s="27"/>
     </row>
-    <row r="354" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="354" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G354" s="3">
         <v>45950</v>
       </c>
@@ -10563,7 +10567,7 @@
       </c>
       <c r="O354" s="27"/>
     </row>
-    <row r="355" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="355" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G355" s="3">
         <v>45950</v>
       </c>
@@ -10590,7 +10594,7 @@
       </c>
       <c r="O355" s="27"/>
     </row>
-    <row r="356" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="356" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G356" s="3">
         <v>45950</v>
       </c>
@@ -10654,7 +10658,7 @@
       <c r="M358" s="4"/>
       <c r="N358" s="6"/>
     </row>
-    <row r="359" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="359" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G359" s="3">
         <v>45951</v>
       </c>
@@ -10681,7 +10685,7 @@
       </c>
       <c r="O359" s="27"/>
     </row>
-    <row r="360" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="360" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G360" s="3">
         <v>45951</v>
       </c>
@@ -10708,7 +10712,7 @@
       </c>
       <c r="O360" s="27"/>
     </row>
-    <row r="361" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="361" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G361" s="3">
         <v>45951</v>
       </c>
@@ -10735,7 +10739,7 @@
       </c>
       <c r="O361" s="27"/>
     </row>
-    <row r="362" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="362" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G362" s="3">
         <v>45951</v>
       </c>
@@ -10762,7 +10766,7 @@
       </c>
       <c r="O362" s="27"/>
     </row>
-    <row r="363" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="363" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G363" s="3">
         <v>45951</v>
       </c>
@@ -10789,7 +10793,7 @@
       </c>
       <c r="O363" s="27"/>
     </row>
-    <row r="364" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="364" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G364" s="3">
         <v>45951</v>
       </c>
@@ -10816,7 +10820,7 @@
       </c>
       <c r="O364" s="27"/>
     </row>
-    <row r="365" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="365" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G365" s="3">
         <v>45952</v>
       </c>
@@ -10843,7 +10847,7 @@
       </c>
       <c r="O365" s="28"/>
     </row>
-    <row r="366" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="366" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G366" s="3">
         <v>45952</v>
       </c>
@@ -10870,7 +10874,7 @@
       </c>
       <c r="O366" s="27"/>
     </row>
-    <row r="367" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="367" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G367" s="3">
         <v>45952</v>
       </c>
@@ -10897,7 +10901,7 @@
       </c>
       <c r="O367" s="27"/>
     </row>
-    <row r="368" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="368" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G368" s="3">
         <v>45952</v>
       </c>
@@ -10924,7 +10928,7 @@
       </c>
       <c r="O368" s="27"/>
     </row>
-    <row r="369" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="369" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G369" s="3">
         <v>45952</v>
       </c>
@@ -10951,7 +10955,7 @@
       </c>
       <c r="O369" s="27"/>
     </row>
-    <row r="370" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="370" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G370" s="3">
         <v>45952</v>
       </c>
@@ -10978,7 +10982,7 @@
       </c>
       <c r="O370" s="27"/>
     </row>
-    <row r="371" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="371" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G371" s="3">
         <v>45952</v>
       </c>
@@ -11005,7 +11009,7 @@
       </c>
       <c r="O371" s="27"/>
     </row>
-    <row r="372" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="372" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G372" s="19">
         <v>45952</v>
       </c>
@@ -11034,7 +11038,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="373" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="373" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G373" s="3">
         <v>45953</v>
       </c>
@@ -11061,7 +11065,7 @@
       </c>
       <c r="O373" s="27"/>
     </row>
-    <row r="374" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="374" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G374" s="3">
         <v>45953</v>
       </c>
@@ -11088,7 +11092,7 @@
       </c>
       <c r="O374" s="27"/>
     </row>
-    <row r="375" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="375" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G375" s="3">
         <v>45953</v>
       </c>
@@ -11115,7 +11119,7 @@
       </c>
       <c r="O375" s="27"/>
     </row>
-    <row r="376" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="376" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G376" s="3">
         <v>45953</v>
       </c>
@@ -11142,7 +11146,7 @@
       </c>
       <c r="O376" s="27"/>
     </row>
-    <row r="377" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="377" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G377" s="3">
         <v>45953</v>
       </c>
@@ -11169,7 +11173,7 @@
       </c>
       <c r="O377" s="27"/>
     </row>
-    <row r="378" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="378" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G378" s="3">
         <v>45953</v>
       </c>
@@ -11196,7 +11200,7 @@
       </c>
       <c r="O378" s="27"/>
     </row>
-    <row r="379" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="379" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G379" s="3">
         <v>45953</v>
       </c>
@@ -11223,7 +11227,7 @@
       </c>
       <c r="O379" s="27"/>
     </row>
-    <row r="380" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="380" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G380" s="3">
         <v>45953</v>
       </c>
@@ -11277,7 +11281,7 @@
       </c>
       <c r="O381" s="27"/>
     </row>
-    <row r="382" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="382" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G382" s="3">
         <v>45953</v>
       </c>
@@ -11307,7 +11311,7 @@
     <row r="383" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="O383" s="29"/>
     </row>
-    <row r="384" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+    <row r="384" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G384" s="3">
         <v>45953</v>
       </c>
@@ -11363,11 +11367,6 @@
         <dateGroupItem year="2025" month="10" dateTimeGrouping="month"/>
       </filters>
     </filterColumn>
-    <filterColumn colId="1">
-      <filters>
-        <filter val="CRISTIANO"/>
-      </filters>
-    </filterColumn>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G6:N339">
     <sortCondition ref="G6:G339"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-28  8:30
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2488" documentId="13_ncr:1_{E95D9CB3-09C0-4BE2-98CB-FDF0DD0373BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7BBEAD03-6A20-4489-96FB-82D42DCD26A7}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F75F6097-1719-484D-B058-F6814CEA406A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$O$389</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$G$5:$O$398</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1940" uniqueCount="270">
   <si>
     <t>DATA</t>
   </si>
@@ -1370,7 +1370,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:O392"/>
+  <dimension ref="G5:O399"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -11515,7 +11515,7 @@
         <v>27</v>
       </c>
       <c r="K389" s="9">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="L389" s="4" t="s">
         <v>56</v>
@@ -11529,43 +11529,193 @@
       <c r="O389" s="27"/>
     </row>
     <row r="390" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G390" s="4"/>
-      <c r="H390" s="4"/>
-      <c r="I390" s="6"/>
+      <c r="G390" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H390" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="I390" s="6" t="s">
+        <v>128</v>
+      </c>
       <c r="J390" s="4"/>
       <c r="K390" s="9"/>
       <c r="L390" s="4"/>
       <c r="M390" s="4"/>
-      <c r="N390" s="6"/>
+      <c r="N390" s="6">
+        <v>1</v>
+      </c>
       <c r="O390" s="27"/>
     </row>
     <row r="391" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G391" s="4"/>
-      <c r="H391" s="4"/>
-      <c r="I391" s="6"/>
+      <c r="G391" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H391" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="I391" s="6" t="s">
+        <v>139</v>
+      </c>
       <c r="J391" s="4"/>
       <c r="K391" s="9"/>
       <c r="L391" s="4"/>
       <c r="M391" s="4"/>
-      <c r="N391" s="6"/>
+      <c r="N391" s="6">
+        <v>3</v>
+      </c>
       <c r="O391" s="27"/>
     </row>
     <row r="392" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G392" s="4"/>
-      <c r="H392" s="4"/>
-      <c r="I392" s="6"/>
+      <c r="G392" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H392" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="I392" s="6" t="s">
+        <v>178</v>
+      </c>
       <c r="J392" s="4"/>
       <c r="K392" s="9"/>
       <c r="L392" s="4"/>
       <c r="M392" s="4"/>
-      <c r="N392" s="6"/>
+      <c r="N392" s="6">
+        <v>1</v>
+      </c>
       <c r="O392" s="27"/>
     </row>
+    <row r="393" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G393" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H393" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="I393" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J393" s="4"/>
+      <c r="K393" s="9"/>
+      <c r="L393" s="4"/>
+      <c r="M393" s="4"/>
+      <c r="N393" s="6">
+        <v>1</v>
+      </c>
+      <c r="O393" s="27"/>
+    </row>
+    <row r="394" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G394" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H394" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="I394" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J394" s="4"/>
+      <c r="K394" s="9"/>
+      <c r="L394" s="4"/>
+      <c r="M394" s="4"/>
+      <c r="N394" s="6">
+        <v>2</v>
+      </c>
+      <c r="O394" s="27"/>
+    </row>
+    <row r="395" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G395" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H395" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="I395" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J395" s="4"/>
+      <c r="K395" s="9"/>
+      <c r="L395" s="4"/>
+      <c r="M395" s="4"/>
+      <c r="N395" s="6">
+        <v>3</v>
+      </c>
+      <c r="O395" s="27"/>
+    </row>
+    <row r="396" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G396" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H396" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="I396" s="6" t="s">
+        <v>223</v>
+      </c>
+      <c r="J396" s="4"/>
+      <c r="K396" s="9"/>
+      <c r="L396" s="4"/>
+      <c r="M396" s="4"/>
+      <c r="N396" s="6">
+        <v>2</v>
+      </c>
+      <c r="O396" s="27"/>
+    </row>
+    <row r="397" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G397" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H397" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="I397" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="J397" s="4"/>
+      <c r="K397" s="9"/>
+      <c r="L397" s="4"/>
+      <c r="M397" s="4"/>
+      <c r="N397" s="6">
+        <v>2</v>
+      </c>
+      <c r="O397" s="27"/>
+    </row>
+    <row r="398" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G398" s="3">
+        <v>45958</v>
+      </c>
+      <c r="H398" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="I398" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J398" s="4"/>
+      <c r="K398" s="9"/>
+      <c r="L398" s="4"/>
+      <c r="M398" s="4"/>
+      <c r="N398" s="6">
+        <v>3</v>
+      </c>
+      <c r="O398" s="27"/>
+    </row>
+    <row r="399" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G399" s="4"/>
+      <c r="H399" s="4"/>
+      <c r="I399" s="6"/>
+      <c r="J399" s="4"/>
+      <c r="K399" s="9"/>
+      <c r="L399" s="4"/>
+      <c r="M399" s="4"/>
+      <c r="N399" s="6"/>
+      <c r="O399" s="27"/>
+    </row>
   </sheetData>
-  <autoFilter ref="G5:O389" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O398" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2025" month="10" day="27" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="10" day="28" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-04 16:42
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="628" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29527798-37B8-424B-84ED-6A189F904098}"/>
+  <xr:revisionPtr revIDLastSave="650" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66725069-CD65-4A44-B7B3-AE978AD05254}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2262" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2274" uniqueCount="345">
   <si>
     <t>DATA</t>
   </si>
@@ -1062,6 +1062,18 @@
   </si>
   <si>
     <t>HOTEL JOAOZINHO</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CAFÉ PALACE</t>
+  </si>
+  <si>
+    <t>carmo do rio claro</t>
+  </si>
+  <si>
+    <t>pousada oasis</t>
+  </si>
+  <si>
+    <t>JOAO MONLEVADE</t>
   </si>
 </sst>
 </file>
@@ -12951,22 +12963,14 @@
       <c r="O429" s="25"/>
     </row>
     <row r="430" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G430" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H430" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="I430" s="6" t="s">
-        <v>125</v>
-      </c>
+      <c r="G430" s="3"/>
+      <c r="H430" s="4"/>
+      <c r="I430" s="6"/>
       <c r="J430" s="4"/>
       <c r="K430" s="8"/>
       <c r="L430" s="4"/>
       <c r="M430" s="4"/>
-      <c r="N430" s="6">
-        <v>1</v>
-      </c>
+      <c r="N430" s="6"/>
       <c r="O430" s="25"/>
     </row>
     <row r="431" spans="7:15" x14ac:dyDescent="0.25">
@@ -12979,10 +12983,18 @@
       <c r="I431" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="J431" s="4"/>
-      <c r="K431" s="8"/>
-      <c r="L431" s="4"/>
-      <c r="M431" s="4"/>
+      <c r="J431" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K431" s="8">
+        <v>180</v>
+      </c>
+      <c r="L431" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M431" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N431" s="6">
         <v>3</v>
       </c>
@@ -12998,10 +13010,18 @@
       <c r="I432" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="J432" s="4"/>
-      <c r="K432" s="8"/>
-      <c r="L432" s="4"/>
-      <c r="M432" s="4"/>
+      <c r="J432" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K432" s="8">
+        <v>240</v>
+      </c>
+      <c r="L432" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="M432" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N432" s="6">
         <v>2</v>
       </c>
@@ -13015,12 +13035,20 @@
         <v>146</v>
       </c>
       <c r="I433" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="J433" s="4"/>
-      <c r="K433" s="8"/>
-      <c r="L433" s="4"/>
-      <c r="M433" s="4"/>
+        <v>124</v>
+      </c>
+      <c r="J433" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="K433" s="8">
+        <v>280</v>
+      </c>
+      <c r="L433" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="M433" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N433" s="6">
         <v>3</v>
       </c>
@@ -13036,10 +13064,18 @@
       <c r="I434" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="J434" s="4"/>
-      <c r="K434" s="8"/>
-      <c r="L434" s="4"/>
-      <c r="M434" s="4"/>
+      <c r="J434" s="4" t="s">
+        <v>342</v>
+      </c>
+      <c r="K434" s="8">
+        <v>200</v>
+      </c>
+      <c r="L434" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="M434" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N434" s="6">
         <v>2</v>
       </c>
@@ -13055,9 +13091,15 @@
       <c r="I435" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="J435" s="4"/>
-      <c r="K435" s="8"/>
-      <c r="L435" s="4"/>
+      <c r="J435" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="K435" s="8">
+        <v>280</v>
+      </c>
+      <c r="L435" s="4" t="s">
+        <v>261</v>
+      </c>
       <c r="M435" s="4"/>
       <c r="N435" s="6">
         <v>2</v>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-06 12:13
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="650" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66725069-CD65-4A44-B7B3-AE978AD05254}"/>
+  <xr:revisionPtr revIDLastSave="764" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D318BD8C-6BB6-4C96-B513-A9C3A49B0E5F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$437</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$455</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2274" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2335" uniqueCount="356">
   <si>
     <t>DATA</t>
   </si>
@@ -1074,6 +1074,39 @@
   </si>
   <si>
     <t>JOAO MONLEVADE</t>
+  </si>
+  <si>
+    <t>WESLEY ANTONIO</t>
+  </si>
+  <si>
+    <t>HOTEL CAMPEAO</t>
+  </si>
+  <si>
+    <t>SAO JOAO EVANGELISTA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">HOTEL MIRIAN </t>
+  </si>
+  <si>
+    <t>HOTEL SANTOS DUMMOND</t>
+  </si>
+  <si>
+    <t>ELÓI MENDES</t>
+  </si>
+  <si>
+    <t>HOTEL FRATELLI</t>
+  </si>
+  <si>
+    <t>ÁGUAS CLARAS</t>
+  </si>
+  <si>
+    <t>douglas rodrigues</t>
+  </si>
+  <si>
+    <t>lucas gabriel</t>
+  </si>
+  <si>
+    <t>SÃO JOAO DEL REY</t>
   </si>
 </sst>
 </file>
@@ -1128,7 +1161,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -1187,6 +1220,30 @@
       <top style="thin">
         <color indexed="64"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -1276,18 +1333,16 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -1627,7 +1682,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:O440"/>
+  <dimension ref="G5:O455"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -9367,56 +9422,80 @@
       <c r="O291" s="6"/>
     </row>
     <row r="292" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="O292" s="25"/>
+      <c r="G292" s="3">
+        <v>45873</v>
+      </c>
+      <c r="H292" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I292" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="J292" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="K292" s="8">
+        <v>110</v>
+      </c>
+      <c r="L292" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M292" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="N292" s="4">
+        <v>2</v>
+      </c>
+      <c r="O292" s="6"/>
     </row>
     <row r="293" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G293" s="3">
-        <v>45873</v>
+        <v>45932</v>
       </c>
       <c r="H293" s="4" t="s">
-        <v>141</v>
+        <v>155</v>
       </c>
       <c r="I293" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="J293" s="13" t="s">
-        <v>100</v>
+        <v>133</v>
+      </c>
+      <c r="J293" s="4" t="s">
+        <v>178</v>
       </c>
       <c r="K293" s="8">
-        <v>110</v>
+        <v>250</v>
       </c>
       <c r="L293" s="4" t="s">
-        <v>55</v>
+        <v>179</v>
       </c>
       <c r="M293" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="N293" s="4">
+        <v>8</v>
+      </c>
+      <c r="N293" s="6">
         <v>2</v>
       </c>
       <c r="O293" s="6"/>
     </row>
     <row r="294" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G294" s="3">
-        <v>45932</v>
+        <v>45876</v>
       </c>
       <c r="H294" s="4" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I294" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="J294" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="K294" s="8">
-        <v>250</v>
-      </c>
-      <c r="L294" s="4" t="s">
-        <v>179</v>
+        <v>124</v>
+      </c>
+      <c r="J294" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="K294" s="9">
+        <v>100</v>
+      </c>
+      <c r="L294" s="7" t="s">
+        <v>59</v>
       </c>
       <c r="M294" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N294" s="6">
         <v>2</v>
@@ -9425,21 +9504,21 @@
     </row>
     <row r="295" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G295" s="3">
-        <v>45876</v>
+        <v>45883</v>
       </c>
       <c r="H295" s="4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="I295" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J295" s="21" t="s">
+      <c r="J295" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="K295" s="9">
+      <c r="K295" s="5">
         <v>100</v>
       </c>
-      <c r="L295" s="7" t="s">
+      <c r="L295" s="4" t="s">
         <v>59</v>
       </c>
       <c r="M295" s="4" t="s">
@@ -9452,34 +9531,34 @@
     </row>
     <row r="296" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G296" s="3">
-        <v>45883</v>
+        <v>45889</v>
       </c>
       <c r="H296" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="I296" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J296" s="4" t="s">
+      <c r="J296" s="15" t="s">
         <v>64</v>
       </c>
       <c r="K296" s="5">
-        <v>100</v>
+        <v>155</v>
       </c>
       <c r="L296" s="4" t="s">
-        <v>59</v>
+        <v>103</v>
       </c>
       <c r="M296" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N296" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O296" s="6"/>
     </row>
     <row r="297" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G297" s="3">
-        <v>45889</v>
+        <v>45896</v>
       </c>
       <c r="H297" s="4" t="s">
         <v>142</v>
@@ -9487,7 +9566,7 @@
       <c r="I297" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J297" s="15" t="s">
+      <c r="J297" s="4" t="s">
         <v>64</v>
       </c>
       <c r="K297" s="5">
@@ -9506,7 +9585,7 @@
     </row>
     <row r="298" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G298" s="3">
-        <v>45896</v>
+        <v>45917</v>
       </c>
       <c r="H298" s="4" t="s">
         <v>142</v>
@@ -9517,8 +9596,8 @@
       <c r="J298" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="K298" s="5">
-        <v>155</v>
+      <c r="K298" s="8">
+        <v>280</v>
       </c>
       <c r="L298" s="4" t="s">
         <v>103</v>
@@ -9533,7 +9612,7 @@
     </row>
     <row r="299" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G299" s="3">
-        <v>45917</v>
+        <v>45924</v>
       </c>
       <c r="H299" s="4" t="s">
         <v>142</v>
@@ -9545,7 +9624,7 @@
         <v>64</v>
       </c>
       <c r="K299" s="8">
-        <v>280</v>
+        <v>205</v>
       </c>
       <c r="L299" s="4" t="s">
         <v>103</v>
@@ -9560,19 +9639,19 @@
     </row>
     <row r="300" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G300" s="3">
-        <v>45924</v>
+        <v>45939</v>
       </c>
       <c r="H300" s="4" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="I300" s="6" t="s">
-        <v>124</v>
+        <v>209</v>
       </c>
       <c r="J300" s="4" t="s">
         <v>64</v>
       </c>
       <c r="K300" s="8">
-        <v>205</v>
+        <v>180</v>
       </c>
       <c r="L300" s="4" t="s">
         <v>103</v>
@@ -9581,28 +9660,28 @@
         <v>8</v>
       </c>
       <c r="N300" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O300" s="6"/>
     </row>
     <row r="301" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G301" s="3">
-        <v>45939</v>
+        <v>45903</v>
       </c>
       <c r="H301" s="4" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="I301" s="6" t="s">
-        <v>209</v>
+        <v>134</v>
       </c>
       <c r="J301" s="4" t="s">
-        <v>64</v>
+        <v>166</v>
       </c>
       <c r="K301" s="8">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="L301" s="4" t="s">
-        <v>103</v>
+        <v>167</v>
       </c>
       <c r="M301" s="4" t="s">
         <v>8</v>
@@ -9614,72 +9693,72 @@
     </row>
     <row r="302" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G302" s="3">
-        <v>45903</v>
-      </c>
-      <c r="H302" s="4" t="s">
-        <v>137</v>
+        <v>45875</v>
+      </c>
+      <c r="H302" s="7" t="s">
+        <v>144</v>
       </c>
       <c r="I302" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J302" s="4" t="s">
-        <v>166</v>
+        <v>126</v>
+      </c>
+      <c r="J302" s="21" t="s">
+        <v>46</v>
       </c>
       <c r="K302" s="8">
-        <v>120</v>
+        <v>85</v>
       </c>
       <c r="L302" s="4" t="s">
-        <v>167</v>
+        <v>48</v>
       </c>
       <c r="M302" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N302" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O302" s="6"/>
     </row>
     <row r="303" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G303" s="3">
-        <v>45875</v>
-      </c>
-      <c r="H303" s="7" t="s">
-        <v>144</v>
+        <v>45889</v>
+      </c>
+      <c r="H303" s="4" t="s">
+        <v>143</v>
       </c>
       <c r="I303" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J303" s="21" t="s">
+      <c r="J303" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="K303" s="8">
-        <v>85</v>
+      <c r="K303" s="5">
+        <v>170</v>
       </c>
       <c r="L303" s="4" t="s">
         <v>48</v>
       </c>
       <c r="M303" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N303" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O303" s="6"/>
     </row>
     <row r="304" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G304" s="3">
-        <v>45889</v>
+        <v>45903</v>
       </c>
       <c r="H304" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I304" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="J304" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="K304" s="5">
+      <c r="K304" s="8">
         <v>170</v>
       </c>
       <c r="L304" s="4" t="s">
@@ -9689,7 +9768,7 @@
         <v>8</v>
       </c>
       <c r="N304" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O304" s="6"/>
     </row>
@@ -9698,10 +9777,10 @@
         <v>45903</v>
       </c>
       <c r="H305" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I305" s="6" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="J305" s="4" t="s">
         <v>46</v>
@@ -9722,13 +9801,13 @@
     </row>
     <row r="306" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G306" s="3">
-        <v>45903</v>
+        <v>45910</v>
       </c>
       <c r="H306" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="I306" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="J306" s="4" t="s">
         <v>46</v>
@@ -9737,7 +9816,7 @@
         <v>170</v>
       </c>
       <c r="L306" s="4" t="s">
-        <v>48</v>
+        <v>214</v>
       </c>
       <c r="M306" s="4" t="s">
         <v>8</v>
@@ -9752,10 +9831,10 @@
         <v>45910</v>
       </c>
       <c r="H307" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I307" s="6" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="J307" s="4" t="s">
         <v>46</v>
@@ -9776,7 +9855,7 @@
     </row>
     <row r="308" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G308" s="3">
-        <v>45910</v>
+        <v>45924</v>
       </c>
       <c r="H308" s="4" t="s">
         <v>138</v>
@@ -9791,7 +9870,7 @@
         <v>170</v>
       </c>
       <c r="L308" s="4" t="s">
-        <v>214</v>
+        <v>48</v>
       </c>
       <c r="M308" s="4" t="s">
         <v>8</v>
@@ -9803,22 +9882,22 @@
     </row>
     <row r="309" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G309" s="3">
-        <v>45924</v>
+        <v>45931</v>
       </c>
       <c r="H309" s="4" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="I309" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J309" s="4" t="s">
-        <v>46</v>
+        <v>124</v>
+      </c>
+      <c r="J309" s="15" t="s">
+        <v>64</v>
       </c>
       <c r="K309" s="8">
-        <v>170</v>
+        <v>212</v>
       </c>
       <c r="L309" s="4" t="s">
-        <v>48</v>
+        <v>103</v>
       </c>
       <c r="M309" s="4" t="s">
         <v>8</v>
@@ -9830,22 +9909,22 @@
     </row>
     <row r="310" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G310" s="3">
-        <v>45931</v>
+        <v>45938</v>
       </c>
       <c r="H310" s="4" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I310" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J310" s="15" t="s">
-        <v>64</v>
+        <v>135</v>
+      </c>
+      <c r="J310" s="4" t="s">
+        <v>46</v>
       </c>
       <c r="K310" s="8">
-        <v>212</v>
+        <v>170</v>
       </c>
       <c r="L310" s="4" t="s">
-        <v>103</v>
+        <v>214</v>
       </c>
       <c r="M310" s="4" t="s">
         <v>8</v>
@@ -9860,10 +9939,10 @@
         <v>45938</v>
       </c>
       <c r="H311" s="4" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="I311" s="6" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="J311" s="4" t="s">
         <v>46</v>
@@ -9884,19 +9963,19 @@
     </row>
     <row r="312" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G312" s="3">
-        <v>45938</v>
+        <v>45945</v>
       </c>
       <c r="H312" s="4" t="s">
-        <v>155</v>
+        <v>138</v>
       </c>
       <c r="I312" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="J312" s="4" t="s">
         <v>46</v>
       </c>
       <c r="K312" s="8">
-        <v>170</v>
+        <v>230</v>
       </c>
       <c r="L312" s="4" t="s">
         <v>214</v>
@@ -9914,10 +9993,10 @@
         <v>45945</v>
       </c>
       <c r="H313" s="4" t="s">
-        <v>138</v>
+        <v>235</v>
       </c>
       <c r="I313" s="6" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="J313" s="4" t="s">
         <v>46</v>
@@ -9938,19 +10017,19 @@
     </row>
     <row r="314" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G314" s="3">
-        <v>45945</v>
+        <v>45952</v>
       </c>
       <c r="H314" s="4" t="s">
-        <v>235</v>
+        <v>138</v>
       </c>
       <c r="I314" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J314" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="J314" s="15" t="s">
         <v>46</v>
       </c>
       <c r="K314" s="8">
-        <v>230</v>
+        <v>170</v>
       </c>
       <c r="L314" s="4" t="s">
         <v>214</v>
@@ -9961,107 +10040,107 @@
       <c r="N314" s="6">
         <v>3</v>
       </c>
-      <c r="O314" s="6"/>
+      <c r="O314" s="25"/>
     </row>
     <row r="315" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G315" s="3">
-        <v>45952</v>
+        <v>45903</v>
       </c>
       <c r="H315" s="4" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I315" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J315" s="15" t="s">
-        <v>46</v>
+        <v>129</v>
+      </c>
+      <c r="J315" s="4" t="s">
+        <v>169</v>
       </c>
       <c r="K315" s="8">
+        <v>140</v>
+      </c>
+      <c r="L315" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="L315" s="4" t="s">
-        <v>214</v>
-      </c>
       <c r="M315" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N315" s="6">
-        <v>3</v>
-      </c>
-      <c r="O315" s="25"/>
+        <v>2</v>
+      </c>
+      <c r="O315" s="6"/>
     </row>
     <row r="316" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G316" s="3">
-        <v>45903</v>
+        <v>45952</v>
       </c>
       <c r="H316" s="4" t="s">
-        <v>143</v>
+        <v>198</v>
       </c>
       <c r="I316" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J316" s="4" t="s">
-        <v>169</v>
+        <v>46</v>
       </c>
       <c r="K316" s="8">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="L316" s="4" t="s">
-        <v>170</v>
+        <v>214</v>
       </c>
       <c r="M316" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N316" s="6">
-        <v>2</v>
-      </c>
-      <c r="O316" s="6"/>
+        <v>3</v>
+      </c>
+      <c r="O316" s="25"/>
     </row>
     <row r="317" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G317" s="3">
-        <v>45952</v>
+        <v>45895</v>
       </c>
       <c r="H317" s="4" t="s">
-        <v>198</v>
+        <v>156</v>
       </c>
       <c r="I317" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="J317" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="K317" s="8">
-        <v>170</v>
+        <v>13</v>
+      </c>
+      <c r="K317" s="5">
+        <v>200</v>
       </c>
       <c r="L317" s="4" t="s">
-        <v>214</v>
+        <v>12</v>
       </c>
       <c r="M317" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N317" s="6">
-        <v>3</v>
-      </c>
-      <c r="O317" s="25"/>
+        <v>2</v>
+      </c>
+      <c r="O317" s="6"/>
     </row>
     <row r="318" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G318" s="3">
-        <v>45895</v>
+        <v>45918</v>
       </c>
       <c r="H318" s="4" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="I318" s="6" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="J318" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K318" s="5">
+      <c r="K318" s="8">
         <v>200</v>
       </c>
       <c r="L318" s="4" t="s">
-        <v>12</v>
+        <v>185</v>
       </c>
       <c r="M318" s="4" t="s">
         <v>8</v>
@@ -10073,45 +10152,45 @@
     </row>
     <row r="319" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G319" s="3">
-        <v>45918</v>
+        <v>45873</v>
       </c>
       <c r="H319" s="4" t="s">
-        <v>158</v>
+        <v>138</v>
       </c>
       <c r="I319" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J319" s="4" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="K319" s="8">
-        <v>200</v>
+        <v>74.900000000000006</v>
       </c>
       <c r="L319" s="4" t="s">
-        <v>185</v>
+        <v>89</v>
       </c>
       <c r="M319" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N319" s="6">
+        <v>7</v>
+      </c>
+      <c r="N319" s="4">
         <v>2</v>
       </c>
       <c r="O319" s="6"/>
     </row>
     <row r="320" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G320" s="3">
-        <v>45873</v>
+        <v>45876</v>
       </c>
       <c r="H320" s="4" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="I320" s="6" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="J320" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K320" s="8">
+      <c r="K320" s="9">
         <v>74.900000000000006</v>
       </c>
       <c r="L320" s="4" t="s">
@@ -10120,25 +10199,25 @@
       <c r="M320" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="N320" s="4">
+      <c r="N320" s="6">
         <v>2</v>
       </c>
       <c r="O320" s="6"/>
     </row>
     <row r="321" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G321" s="3">
-        <v>45876</v>
+        <v>45880</v>
       </c>
       <c r="H321" s="4" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="I321" s="6" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="J321" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K321" s="9">
+      <c r="K321" s="5">
         <v>74.900000000000006</v>
       </c>
       <c r="L321" s="4" t="s">
@@ -10154,19 +10233,19 @@
     </row>
     <row r="322" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G322" s="3">
-        <v>45880</v>
+        <v>45883</v>
       </c>
       <c r="H322" s="4" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="I322" s="6" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="J322" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K322" s="5">
-        <v>74.900000000000006</v>
+        <v>129</v>
       </c>
       <c r="L322" s="4" t="s">
         <v>89</v>
@@ -10184,22 +10263,22 @@
         <v>45883</v>
       </c>
       <c r="H323" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="I323" s="6" t="s">
-        <v>132</v>
+        <v>120</v>
       </c>
       <c r="J323" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K323" s="5">
-        <v>129</v>
+        <v>149</v>
       </c>
       <c r="L323" s="4" t="s">
         <v>89</v>
       </c>
       <c r="M323" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N323" s="6">
         <v>2</v>
@@ -10208,13 +10287,13 @@
     </row>
     <row r="324" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G324" s="3">
-        <v>45883</v>
+        <v>45887</v>
       </c>
       <c r="H324" s="4" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="I324" s="6" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="J324" s="4" t="s">
         <v>24</v>
@@ -10226,7 +10305,7 @@
         <v>89</v>
       </c>
       <c r="M324" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N324" s="6">
         <v>2</v>
@@ -10235,19 +10314,19 @@
     </row>
     <row r="325" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G325" s="3">
-        <v>45887</v>
+        <v>45890</v>
       </c>
       <c r="H325" s="4" t="s">
         <v>149</v>
       </c>
       <c r="I325" s="6" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="J325" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K325" s="5">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="L325" s="4" t="s">
         <v>89</v>
@@ -10262,7 +10341,7 @@
     </row>
     <row r="326" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G326" s="3">
-        <v>45890</v>
+        <v>45894</v>
       </c>
       <c r="H326" s="4" t="s">
         <v>149</v>
@@ -10274,13 +10353,13 @@
         <v>24</v>
       </c>
       <c r="K326" s="5">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="L326" s="4" t="s">
         <v>89</v>
       </c>
       <c r="M326" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N326" s="6">
         <v>2</v>
@@ -10289,10 +10368,10 @@
     </row>
     <row r="327" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G327" s="3">
-        <v>45894</v>
+        <v>45897</v>
       </c>
       <c r="H327" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="I327" s="6" t="s">
         <v>121</v>
@@ -10300,8 +10379,8 @@
       <c r="J327" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K327" s="5">
-        <v>149</v>
+      <c r="K327" s="8">
+        <v>209</v>
       </c>
       <c r="L327" s="4" t="s">
         <v>89</v>
@@ -10316,10 +10395,10 @@
     </row>
     <row r="328" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G328" s="3">
-        <v>45897</v>
+        <v>45901</v>
       </c>
       <c r="H328" s="4" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="I328" s="6" t="s">
         <v>121</v>
@@ -10343,15 +10422,15 @@
     </row>
     <row r="329" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G329" s="3">
-        <v>45901</v>
+        <v>45904</v>
       </c>
       <c r="H329" s="4" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="I329" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="J329" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="J329" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K329" s="8">
@@ -10370,19 +10449,19 @@
     </row>
     <row r="330" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G330" s="3">
-        <v>45904</v>
+        <v>45908</v>
       </c>
       <c r="H330" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I330" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="J330" s="15" t="s">
+      <c r="I330" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="J330" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K330" s="8">
-        <v>209</v>
+        <v>159</v>
       </c>
       <c r="L330" s="4" t="s">
         <v>89</v>
@@ -10390,26 +10469,26 @@
       <c r="M330" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N330" s="6">
+      <c r="N330" s="4">
         <v>2</v>
       </c>
       <c r="O330" s="6"/>
     </row>
     <row r="331" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G331" s="3">
-        <v>45908</v>
+        <v>45911</v>
       </c>
       <c r="H331" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="I331" s="4" t="s">
+      <c r="I331" s="6" t="s">
         <v>121</v>
       </c>
       <c r="J331" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K331" s="8">
-        <v>159</v>
+        <v>209</v>
       </c>
       <c r="L331" s="4" t="s">
         <v>89</v>
@@ -10417,14 +10496,14 @@
       <c r="M331" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N331" s="4">
+      <c r="N331" s="6">
         <v>2</v>
       </c>
       <c r="O331" s="6"/>
     </row>
     <row r="332" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G332" s="3">
-        <v>45911</v>
+        <v>45915</v>
       </c>
       <c r="H332" s="4" t="s">
         <v>156</v>
@@ -10454,16 +10533,16 @@
         <v>45915</v>
       </c>
       <c r="H333" s="4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="I333" s="6" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="J333" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K333" s="8">
-        <v>209</v>
+        <v>259</v>
       </c>
       <c r="L333" s="4" t="s">
         <v>89</v>
@@ -10472,25 +10551,25 @@
         <v>8</v>
       </c>
       <c r="N333" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O333" s="6"/>
     </row>
     <row r="334" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G334" s="3">
-        <v>45915</v>
+        <v>45918</v>
       </c>
       <c r="H334" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="I334" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="J334" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K334" s="8">
-        <v>259</v>
+        <v>159</v>
       </c>
       <c r="L334" s="4" t="s">
         <v>89</v>
@@ -10499,13 +10578,13 @@
         <v>8</v>
       </c>
       <c r="N334" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O334" s="6"/>
     </row>
     <row r="335" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G335" s="3">
-        <v>45918</v>
+        <v>45922</v>
       </c>
       <c r="H335" s="4" t="s">
         <v>156</v>
@@ -10517,7 +10596,7 @@
         <v>24</v>
       </c>
       <c r="K335" s="8">
-        <v>159</v>
+        <v>209</v>
       </c>
       <c r="L335" s="4" t="s">
         <v>89</v>
@@ -10532,13 +10611,13 @@
     </row>
     <row r="336" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G336" s="3">
-        <v>45922</v>
+        <v>45925</v>
       </c>
       <c r="H336" s="4" t="s">
         <v>156</v>
       </c>
       <c r="I336" s="6" t="s">
-        <v>121</v>
+        <v>192</v>
       </c>
       <c r="J336" s="4" t="s">
         <v>24</v>
@@ -10559,7 +10638,7 @@
     </row>
     <row r="337" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G337" s="3">
-        <v>45925</v>
+        <v>45929</v>
       </c>
       <c r="H337" s="4" t="s">
         <v>156</v>
@@ -10567,7 +10646,7 @@
       <c r="I337" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="J337" s="4" t="s">
+      <c r="J337" s="15" t="s">
         <v>24</v>
       </c>
       <c r="K337" s="8">
@@ -10586,22 +10665,22 @@
     </row>
     <row r="338" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G338" s="3">
-        <v>45929</v>
+        <v>45957</v>
       </c>
       <c r="H338" s="4" t="s">
-        <v>156</v>
+        <v>256</v>
       </c>
       <c r="I338" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="J338" s="15" t="s">
-        <v>24</v>
+        <v>130</v>
+      </c>
+      <c r="J338" s="4" t="s">
+        <v>260</v>
       </c>
       <c r="K338" s="8">
-        <v>209</v>
+        <v>140</v>
       </c>
       <c r="L338" s="4" t="s">
-        <v>89</v>
+        <v>259</v>
       </c>
       <c r="M338" s="4" t="s">
         <v>8</v>
@@ -10609,25 +10688,25 @@
       <c r="N338" s="6">
         <v>2</v>
       </c>
-      <c r="O338" s="6"/>
+      <c r="O338" s="25"/>
     </row>
     <row r="339" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G339" s="3">
-        <v>45957</v>
+        <v>45959</v>
       </c>
       <c r="H339" s="4" t="s">
-        <v>256</v>
+        <v>148</v>
       </c>
       <c r="I339" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="J339" s="4" t="s">
-        <v>260</v>
-      </c>
-      <c r="K339" s="8">
+        <v>176</v>
+      </c>
+      <c r="J339" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="K339" s="10">
         <v>140</v>
       </c>
-      <c r="L339" s="4" t="s">
+      <c r="L339" s="1" t="s">
         <v>259</v>
       </c>
       <c r="M339" s="4" t="s">
@@ -10643,19 +10722,19 @@
         <v>45959</v>
       </c>
       <c r="H340" s="4" t="s">
-        <v>148</v>
+        <v>266</v>
       </c>
       <c r="I340" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="J340" s="1" t="s">
-        <v>270</v>
-      </c>
-      <c r="K340" s="10">
-        <v>140</v>
-      </c>
-      <c r="L340" s="1" t="s">
-        <v>259</v>
+        <v>130</v>
+      </c>
+      <c r="J340" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="K340" s="8">
+        <v>220</v>
+      </c>
+      <c r="L340" s="4" t="s">
+        <v>93</v>
       </c>
       <c r="M340" s="4" t="s">
         <v>8</v>
@@ -10667,22 +10746,22 @@
     </row>
     <row r="341" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G341" s="3">
-        <v>45959</v>
+        <v>45932</v>
       </c>
       <c r="H341" s="4" t="s">
-        <v>266</v>
+        <v>156</v>
       </c>
       <c r="I341" s="6" t="s">
-        <v>130</v>
+        <v>189</v>
       </c>
       <c r="J341" s="4" t="s">
-        <v>267</v>
+        <v>24</v>
       </c>
       <c r="K341" s="8">
-        <v>220</v>
+        <v>259</v>
       </c>
       <c r="L341" s="4" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="M341" s="4" t="s">
         <v>8</v>
@@ -10690,14 +10769,14 @@
       <c r="N341" s="6">
         <v>2</v>
       </c>
-      <c r="O341" s="25"/>
+      <c r="O341" s="6"/>
     </row>
     <row r="342" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G342" s="3">
-        <v>45932</v>
+        <v>45936</v>
       </c>
       <c r="H342" s="4" t="s">
-        <v>156</v>
+        <v>207</v>
       </c>
       <c r="I342" s="6" t="s">
         <v>189</v>
@@ -10721,7 +10800,7 @@
     </row>
     <row r="343" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G343" s="3">
-        <v>45936</v>
+        <v>45939</v>
       </c>
       <c r="H343" s="4" t="s">
         <v>207</v>
@@ -10733,10 +10812,10 @@
         <v>24</v>
       </c>
       <c r="K343" s="8">
-        <v>259</v>
+        <v>140</v>
       </c>
       <c r="L343" s="4" t="s">
-        <v>89</v>
+        <v>225</v>
       </c>
       <c r="M343" s="4" t="s">
         <v>8</v>
@@ -10748,19 +10827,19 @@
     </row>
     <row r="344" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G344" s="3">
-        <v>45939</v>
+        <v>45943</v>
       </c>
       <c r="H344" s="4" t="s">
-        <v>207</v>
+        <v>138</v>
       </c>
       <c r="I344" s="6" t="s">
-        <v>189</v>
+        <v>223</v>
       </c>
       <c r="J344" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K344" s="8">
-        <v>140</v>
+        <v>259</v>
       </c>
       <c r="L344" s="4" t="s">
         <v>225</v>
@@ -10775,22 +10854,22 @@
     </row>
     <row r="345" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G345" s="3">
-        <v>45943</v>
+        <v>45946</v>
       </c>
       <c r="H345" s="4" t="s">
-        <v>138</v>
+        <v>240</v>
       </c>
       <c r="I345" s="6" t="s">
-        <v>223</v>
+        <v>189</v>
       </c>
       <c r="J345" s="4" t="s">
         <v>24</v>
       </c>
       <c r="K345" s="8">
-        <v>259</v>
+        <v>159</v>
       </c>
       <c r="L345" s="4" t="s">
-        <v>225</v>
+        <v>89</v>
       </c>
       <c r="M345" s="4" t="s">
         <v>8</v>
@@ -10802,25 +10881,25 @@
     </row>
     <row r="346" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G346" s="3">
-        <v>45946</v>
+        <v>45896</v>
       </c>
       <c r="H346" s="4" t="s">
-        <v>240</v>
+        <v>143</v>
       </c>
       <c r="I346" s="6" t="s">
-        <v>189</v>
+        <v>129</v>
       </c>
       <c r="J346" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K346" s="8">
-        <v>159</v>
+        <v>108</v>
+      </c>
+      <c r="K346" s="5">
+        <v>55</v>
       </c>
       <c r="L346" s="4" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="M346" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N346" s="6">
         <v>2</v>
@@ -10829,7 +10908,7 @@
     </row>
     <row r="347" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G347" s="3">
-        <v>45896</v>
+        <v>45924</v>
       </c>
       <c r="H347" s="4" t="s">
         <v>143</v>
@@ -10840,85 +10919,85 @@
       <c r="J347" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="K347" s="5">
-        <v>55</v>
+      <c r="K347" s="8">
+        <v>110</v>
       </c>
       <c r="L347" s="4" t="s">
-        <v>111</v>
+        <v>191</v>
       </c>
       <c r="M347" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N347" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O347" s="6"/>
     </row>
     <row r="348" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G348" s="3">
-        <v>45924</v>
-      </c>
-      <c r="H348" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I348" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J348" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K348" s="8">
-        <v>110</v>
-      </c>
-      <c r="L348" s="4" t="s">
-        <v>191</v>
-      </c>
-      <c r="M348" s="4" t="s">
+      <c r="G348" s="17">
+        <v>45947</v>
+      </c>
+      <c r="H348" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="I348" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="J348" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="K348" s="20">
+        <v>259</v>
+      </c>
+      <c r="L348" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="M348" s="18" t="s">
         <v>8</v>
       </c>
       <c r="N348" s="6">
-        <v>3</v>
-      </c>
-      <c r="O348" s="6"/>
+        <v>1</v>
+      </c>
+      <c r="O348" s="6">
+        <v>1</v>
+      </c>
     </row>
     <row r="349" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G349" s="17">
-        <v>45947</v>
-      </c>
-      <c r="H349" s="18" t="s">
-        <v>240</v>
-      </c>
-      <c r="I349" s="19" t="s">
-        <v>189</v>
-      </c>
-      <c r="J349" s="18" t="s">
+      <c r="G349" s="3">
+        <v>45950</v>
+      </c>
+      <c r="H349" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="I349" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J349" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="K349" s="20">
-        <v>259</v>
-      </c>
-      <c r="L349" s="18" t="s">
+      <c r="K349" s="8">
+        <v>159</v>
+      </c>
+      <c r="L349" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="M349" s="18" t="s">
+      <c r="M349" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N349" s="6">
-        <v>1</v>
-      </c>
-      <c r="O349" s="6">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="O349" s="25"/>
     </row>
     <row r="350" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G350" s="3">
-        <v>45950</v>
+        <v>45957</v>
       </c>
       <c r="H350" s="4" t="s">
-        <v>149</v>
+        <v>207</v>
       </c>
       <c r="I350" s="6" t="s">
-        <v>124</v>
+        <v>189</v>
       </c>
       <c r="J350" s="4" t="s">
         <v>24</v>
@@ -10939,22 +11018,22 @@
     </row>
     <row r="351" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G351" s="3">
-        <v>45957</v>
+        <v>45931</v>
       </c>
       <c r="H351" s="4" t="s">
-        <v>207</v>
+        <v>143</v>
       </c>
       <c r="I351" s="6" t="s">
-        <v>189</v>
+        <v>129</v>
       </c>
       <c r="J351" s="4" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="K351" s="8">
-        <v>159</v>
+        <v>110</v>
       </c>
       <c r="L351" s="4" t="s">
-        <v>89</v>
+        <v>111</v>
       </c>
       <c r="M351" s="4" t="s">
         <v>8</v>
@@ -10962,29 +11041,29 @@
       <c r="N351" s="6">
         <v>2</v>
       </c>
-      <c r="O351" s="25"/>
+      <c r="O351" s="6"/>
     </row>
     <row r="352" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G352" s="3">
-        <v>45931</v>
+        <v>45889</v>
       </c>
       <c r="H352" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I352" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J352" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K352" s="8">
-        <v>110</v>
+        <v>241</v>
+      </c>
+      <c r="K352" s="5">
+        <v>130</v>
       </c>
       <c r="L352" s="4" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="M352" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N352" s="6">
         <v>2</v>
@@ -10993,7 +11072,7 @@
     </row>
     <row r="353" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G353" s="3">
-        <v>45889</v>
+        <v>45924</v>
       </c>
       <c r="H353" s="4" t="s">
         <v>146</v>
@@ -11004,53 +11083,53 @@
       <c r="J353" s="4" t="s">
         <v>241</v>
       </c>
-      <c r="K353" s="5">
-        <v>130</v>
+      <c r="K353" s="8">
+        <v>170</v>
       </c>
       <c r="L353" s="4" t="s">
-        <v>97</v>
+        <v>190</v>
       </c>
       <c r="M353" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N353" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O353" s="6"/>
     </row>
     <row r="354" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G354" s="3">
-        <v>45924</v>
+        <v>45938</v>
       </c>
       <c r="H354" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I354" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J354" s="4" t="s">
-        <v>241</v>
+        <v>108</v>
       </c>
       <c r="K354" s="8">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="L354" s="4" t="s">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="M354" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N354" s="6">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="O354" s="6"/>
     </row>
     <row r="355" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G355" s="3">
-        <v>45938</v>
+        <v>45945</v>
       </c>
       <c r="H355" s="4" t="s">
-        <v>143</v>
+        <v>237</v>
       </c>
       <c r="I355" s="6" t="s">
         <v>129</v>
@@ -11062,35 +11141,33 @@
         <v>160</v>
       </c>
       <c r="L355" s="4" t="s">
-        <v>215</v>
+        <v>239</v>
       </c>
       <c r="M355" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N355" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O355" s="6"/>
     </row>
     <row r="356" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G356" s="3">
-        <v>45945</v>
+        <v>45903</v>
       </c>
       <c r="H356" s="4" t="s">
-        <v>237</v>
+        <v>141</v>
       </c>
       <c r="I356" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J356" s="4" t="s">
-        <v>108</v>
+        <v>171</v>
       </c>
       <c r="K356" s="8">
-        <v>160</v>
-      </c>
-      <c r="L356" s="4" t="s">
-        <v>239</v>
-      </c>
+        <v>200</v>
+      </c>
+      <c r="L356" s="4"/>
       <c r="M356" s="4" t="s">
         <v>8</v>
       </c>
@@ -11101,7 +11178,7 @@
     </row>
     <row r="357" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G357" s="3">
-        <v>45903</v>
+        <v>45896</v>
       </c>
       <c r="H357" s="4" t="s">
         <v>141</v>
@@ -11110,131 +11187,133 @@
         <v>132</v>
       </c>
       <c r="J357" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="K357" s="8">
-        <v>200</v>
-      </c>
-      <c r="L357" s="4"/>
+        <v>106</v>
+      </c>
+      <c r="K357" s="5">
+        <v>120</v>
+      </c>
+      <c r="L357" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="M357" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N357" s="6">
         <v>2</v>
       </c>
-      <c r="O357" s="6"/>
+      <c r="O357"/>
     </row>
     <row r="358" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G358" s="3">
-        <v>45896</v>
+        <v>45952</v>
       </c>
       <c r="H358" s="4" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="I358" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J358" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="K358" s="5">
-        <v>120</v>
+        <v>108</v>
+      </c>
+      <c r="K358" s="8">
+        <v>160</v>
       </c>
       <c r="L358" s="4" t="s">
-        <v>109</v>
+        <v>215</v>
       </c>
       <c r="M358" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N358" s="6">
         <v>2</v>
       </c>
-      <c r="O358"/>
+      <c r="O358" s="25"/>
     </row>
     <row r="359" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G359" s="3">
-        <v>45952</v>
+        <v>45881</v>
       </c>
       <c r="H359" s="4" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="I359" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J359" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="K359" s="8">
+        <v>70</v>
+      </c>
+      <c r="K359" s="5">
         <v>160</v>
       </c>
       <c r="L359" s="4" t="s">
-        <v>215</v>
+        <v>69</v>
       </c>
       <c r="M359" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N359" s="6">
-        <v>2</v>
-      </c>
-      <c r="O359" s="25"/>
+        <v>3</v>
+      </c>
+      <c r="O359" s="6"/>
     </row>
     <row r="360" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G360" s="3">
         <v>45881</v>
       </c>
       <c r="H360" s="4" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="I360" s="6" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="J360" s="4" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="K360" s="5">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="L360" s="4" t="s">
-        <v>69</v>
+        <v>228</v>
       </c>
       <c r="M360" s="4" t="s">
         <v>7</v>
       </c>
       <c r="N360" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O360" s="6"/>
     </row>
     <row r="361" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G361" s="3">
-        <v>45881</v>
+        <v>45896</v>
       </c>
       <c r="H361" s="4" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="I361" s="6" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="J361" s="4" t="s">
         <v>107</v>
       </c>
       <c r="K361" s="5">
-        <v>150</v>
+        <v>230</v>
       </c>
       <c r="L361" s="4" t="s">
         <v>228</v>
       </c>
       <c r="M361" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N361" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O361" s="6"/>
     </row>
     <row r="362" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G362" s="3">
-        <v>45896</v>
+        <v>45903</v>
       </c>
       <c r="H362" s="4" t="s">
         <v>146</v>
@@ -11245,8 +11324,8 @@
       <c r="J362" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="K362" s="5">
-        <v>230</v>
+      <c r="K362" s="8">
+        <v>240</v>
       </c>
       <c r="L362" s="4" t="s">
         <v>228</v>
@@ -11276,7 +11355,7 @@
         <v>240</v>
       </c>
       <c r="L363" s="4" t="s">
-        <v>228</v>
+        <v>203</v>
       </c>
       <c r="M363" s="4" t="s">
         <v>8</v>
@@ -11288,7 +11367,7 @@
     </row>
     <row r="364" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G364" s="3">
-        <v>45903</v>
+        <v>45918</v>
       </c>
       <c r="H364" s="4" t="s">
         <v>146</v>
@@ -11303,7 +11382,7 @@
         <v>240</v>
       </c>
       <c r="L364" s="4" t="s">
-        <v>203</v>
+        <v>228</v>
       </c>
       <c r="M364" s="4" t="s">
         <v>8</v>
@@ -11311,11 +11390,11 @@
       <c r="N364" s="6">
         <v>1</v>
       </c>
-      <c r="O364" s="6"/>
+      <c r="O364" s="28"/>
     </row>
     <row r="365" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G365" s="3">
-        <v>45918</v>
+        <v>45925</v>
       </c>
       <c r="H365" s="4" t="s">
         <v>146</v>
@@ -11330,7 +11409,7 @@
         <v>240</v>
       </c>
       <c r="L365" s="4" t="s">
-        <v>228</v>
+        <v>195</v>
       </c>
       <c r="M365" s="4" t="s">
         <v>8</v>
@@ -11338,11 +11417,11 @@
       <c r="N365" s="6">
         <v>1</v>
       </c>
-      <c r="O365" s="28"/>
+      <c r="O365" s="6"/>
     </row>
     <row r="366" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G366" s="3">
-        <v>45925</v>
+        <v>45946</v>
       </c>
       <c r="H366" s="4" t="s">
         <v>146</v>
@@ -11351,13 +11430,13 @@
         <v>128</v>
       </c>
       <c r="J366" s="4" t="s">
-        <v>107</v>
+        <v>241</v>
       </c>
       <c r="K366" s="8">
-        <v>240</v>
+        <v>170</v>
       </c>
       <c r="L366" s="4" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="M366" s="4" t="s">
         <v>8</v>
@@ -11369,34 +11448,34 @@
     </row>
     <row r="367" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G367" s="3">
-        <v>45946</v>
+        <v>45882</v>
       </c>
       <c r="H367" s="4" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="I367" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J367" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="K367" s="8">
-        <v>170</v>
+        <v>77</v>
+      </c>
+      <c r="K367" s="5">
+        <v>175</v>
       </c>
       <c r="L367" s="4" t="s">
-        <v>190</v>
+        <v>78</v>
       </c>
       <c r="M367" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N367" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O367" s="6"/>
     </row>
     <row r="368" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G368" s="3">
-        <v>45882</v>
+        <v>45888</v>
       </c>
       <c r="H368" s="4" t="s">
         <v>140</v>
@@ -11423,7 +11502,7 @@
     </row>
     <row r="369" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G369" s="3">
-        <v>45888</v>
+        <v>45902</v>
       </c>
       <c r="H369" s="4" t="s">
         <v>140</v>
@@ -11434,7 +11513,7 @@
       <c r="J369" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="K369" s="5">
+      <c r="K369" s="8">
         <v>175</v>
       </c>
       <c r="L369" s="4" t="s">
@@ -11450,7 +11529,7 @@
     </row>
     <row r="370" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G370" s="3">
-        <v>45902</v>
+        <v>45909</v>
       </c>
       <c r="H370" s="4" t="s">
         <v>140</v>
@@ -11477,7 +11556,7 @@
     </row>
     <row r="371" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G371" s="3">
-        <v>45909</v>
+        <v>45924</v>
       </c>
       <c r="H371" s="4" t="s">
         <v>140</v>
@@ -11498,82 +11577,82 @@
         <v>7</v>
       </c>
       <c r="N371" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O371" s="6"/>
     </row>
     <row r="372" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G372" s="3">
-        <v>45924</v>
+        <v>45953</v>
       </c>
       <c r="H372" s="4" t="s">
-        <v>140</v>
+        <v>238</v>
       </c>
       <c r="I372" s="6" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="J372" s="4" t="s">
-        <v>77</v>
+        <v>241</v>
       </c>
       <c r="K372" s="8">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L372" s="4" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="M372" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N372" s="6">
         <v>1</v>
       </c>
-      <c r="O372" s="6"/>
+      <c r="O372" s="25"/>
     </row>
     <row r="373" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G373" s="3">
-        <v>45953</v>
+        <v>45957</v>
       </c>
       <c r="H373" s="4" t="s">
-        <v>238</v>
+        <v>148</v>
       </c>
       <c r="I373" s="6" t="s">
-        <v>128</v>
+        <v>176</v>
       </c>
       <c r="J373" s="4" t="s">
-        <v>241</v>
+        <v>257</v>
       </c>
       <c r="K373" s="8">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="L373" s="4" t="s">
-        <v>190</v>
+        <v>258</v>
       </c>
       <c r="M373" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N373" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O373" s="25"/>
     </row>
     <row r="374" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G374" s="3">
-        <v>45957</v>
+        <v>45939</v>
       </c>
       <c r="H374" s="4" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I374" s="6" t="s">
-        <v>176</v>
+        <v>128</v>
       </c>
       <c r="J374" s="4" t="s">
-        <v>257</v>
+        <v>107</v>
       </c>
       <c r="K374" s="8">
-        <v>175</v>
+        <v>230</v>
       </c>
       <c r="L374" s="4" t="s">
-        <v>258</v>
+        <v>228</v>
       </c>
       <c r="M374" s="4" t="s">
         <v>8</v>
@@ -11581,29 +11660,29 @@
       <c r="N374" s="6">
         <v>2</v>
       </c>
-      <c r="O374" s="25"/>
+      <c r="O374" s="6"/>
     </row>
     <row r="375" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G375" s="3">
-        <v>45939</v>
-      </c>
-      <c r="H375" s="4" t="s">
+        <v>45875</v>
+      </c>
+      <c r="H375" s="7" t="s">
         <v>146</v>
       </c>
       <c r="I375" s="6" t="s">
         <v>128</v>
       </c>
       <c r="J375" s="4" t="s">
-        <v>107</v>
+        <v>234</v>
       </c>
       <c r="K375" s="8">
-        <v>230</v>
+        <v>178</v>
       </c>
       <c r="L375" s="4" t="s">
-        <v>228</v>
+        <v>17</v>
       </c>
       <c r="M375" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N375" s="6">
         <v>2</v>
@@ -11612,9 +11691,9 @@
     </row>
     <row r="376" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G376" s="3">
-        <v>45875</v>
-      </c>
-      <c r="H376" s="7" t="s">
+        <v>45895</v>
+      </c>
+      <c r="H376" s="4" t="s">
         <v>146</v>
       </c>
       <c r="I376" s="6" t="s">
@@ -11623,7 +11702,7 @@
       <c r="J376" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="K376" s="8">
+      <c r="K376" s="5">
         <v>178</v>
       </c>
       <c r="L376" s="4" t="s">
@@ -11639,25 +11718,25 @@
     </row>
     <row r="377" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G377" s="3">
-        <v>45895</v>
+        <v>45938</v>
       </c>
       <c r="H377" s="4" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="I377" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J377" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="K377" s="5">
-        <v>178</v>
+        <v>77</v>
+      </c>
+      <c r="K377" s="8">
+        <v>200</v>
       </c>
       <c r="L377" s="4" t="s">
-        <v>17</v>
+        <v>216</v>
       </c>
       <c r="M377" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N377" s="6">
         <v>2</v>
@@ -11666,25 +11745,25 @@
     </row>
     <row r="378" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G378" s="3">
-        <v>45938</v>
+        <v>45876</v>
       </c>
       <c r="H378" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I378" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J378" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="K378" s="8">
-        <v>200</v>
+        <v>126</v>
+      </c>
+      <c r="J378" s="21" t="s">
+        <v>42</v>
+      </c>
+      <c r="K378" s="9">
+        <v>75</v>
       </c>
       <c r="L378" s="4" t="s">
-        <v>216</v>
+        <v>43</v>
       </c>
       <c r="M378" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N378" s="6">
         <v>2</v>
@@ -11693,18 +11772,18 @@
     </row>
     <row r="379" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G379" s="3">
-        <v>45876</v>
+        <v>45883</v>
       </c>
       <c r="H379" s="4" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="I379" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J379" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="J379" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K379" s="9">
+      <c r="K379" s="5">
         <v>75</v>
       </c>
       <c r="L379" s="4" t="s">
@@ -11723,10 +11802,10 @@
         <v>45883</v>
       </c>
       <c r="H380" s="4" t="s">
-        <v>149</v>
+        <v>138</v>
       </c>
       <c r="I380" s="6" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="J380" s="4" t="s">
         <v>42</v>
@@ -11747,13 +11826,13 @@
     </row>
     <row r="381" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G381" s="3">
-        <v>45883</v>
+        <v>45890</v>
       </c>
       <c r="H381" s="4" t="s">
-        <v>138</v>
+        <v>157</v>
       </c>
       <c r="I381" s="6" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="J381" s="4" t="s">
         <v>42</v>
@@ -11774,34 +11853,34 @@
     </row>
     <row r="382" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G382" s="3">
-        <v>45890</v>
+        <v>45897</v>
       </c>
       <c r="H382" s="4" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="I382" s="6" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="J382" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K382" s="5">
-        <v>75</v>
+      <c r="K382" s="8">
+        <v>140</v>
       </c>
       <c r="L382" s="4" t="s">
         <v>43</v>
       </c>
       <c r="M382" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N382" s="6">
         <v>2</v>
       </c>
-      <c r="O382" s="6"/>
+      <c r="O382" s="29"/>
     </row>
     <row r="383" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G383" s="3">
-        <v>45897</v>
+        <v>45918</v>
       </c>
       <c r="H383" s="4" t="s">
         <v>138</v>
@@ -11813,7 +11892,7 @@
         <v>42</v>
       </c>
       <c r="K383" s="8">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="L383" s="4" t="s">
         <v>43</v>
@@ -11824,11 +11903,11 @@
       <c r="N383" s="6">
         <v>2</v>
       </c>
-      <c r="O383" s="29"/>
+      <c r="O383" s="6"/>
     </row>
     <row r="384" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G384" s="3">
-        <v>45918</v>
+        <v>45925</v>
       </c>
       <c r="H384" s="4" t="s">
         <v>138</v>
@@ -11854,64 +11933,64 @@
       <c r="O384" s="6"/>
     </row>
     <row r="385" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G385" s="3">
-        <v>45925</v>
-      </c>
-      <c r="H385" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I385" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J385" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K385" s="8">
+      <c r="G385" s="17">
+        <v>45952</v>
+      </c>
+      <c r="H385" s="18" t="s">
+        <v>249</v>
+      </c>
+      <c r="I385" s="19" t="s">
+        <v>219</v>
+      </c>
+      <c r="J385" s="18" t="s">
+        <v>250</v>
+      </c>
+      <c r="K385" s="20">
         <v>150</v>
       </c>
-      <c r="L385" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="M385" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N385" s="6">
-        <v>2</v>
-      </c>
-      <c r="O385" s="6"/>
+      <c r="L385" s="18" t="s">
+        <v>251</v>
+      </c>
+      <c r="M385" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="N385" s="19">
+        <v>1</v>
+      </c>
+      <c r="O385" s="25" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="386" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G386" s="17">
-        <v>45952</v>
-      </c>
-      <c r="H386" s="18" t="s">
-        <v>249</v>
-      </c>
-      <c r="I386" s="19" t="s">
-        <v>219</v>
-      </c>
-      <c r="J386" s="18" t="s">
-        <v>250</v>
-      </c>
-      <c r="K386" s="20">
-        <v>150</v>
-      </c>
-      <c r="L386" s="18" t="s">
-        <v>251</v>
-      </c>
-      <c r="M386" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="N386" s="19">
-        <v>1</v>
-      </c>
-      <c r="O386" s="25" t="s">
-        <v>253</v>
-      </c>
+      <c r="G386" s="3">
+        <v>45951</v>
+      </c>
+      <c r="H386" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I386" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="J386" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="K386" s="8">
+        <v>270</v>
+      </c>
+      <c r="L386" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M386" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N386" s="6">
+        <v>3</v>
+      </c>
+      <c r="O386" s="25"/>
     </row>
     <row r="387" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G387" s="3">
-        <v>45951</v>
+        <v>45944</v>
       </c>
       <c r="H387" s="4" t="s">
         <v>146</v>
@@ -11920,7 +11999,7 @@
         <v>128</v>
       </c>
       <c r="J387" s="4" t="s">
-        <v>248</v>
+        <v>234</v>
       </c>
       <c r="K387" s="8">
         <v>270</v>
@@ -11934,56 +12013,56 @@
       <c r="N387" s="6">
         <v>3</v>
       </c>
-      <c r="O387" s="25"/>
+      <c r="O387" s="6"/>
     </row>
     <row r="388" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G388" s="3">
-        <v>45944</v>
+        <v>45932</v>
       </c>
       <c r="H388" s="4" t="s">
-        <v>146</v>
+        <v>200</v>
       </c>
       <c r="I388" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="J388" s="4" t="s">
-        <v>234</v>
+        <v>42</v>
       </c>
       <c r="K388" s="8">
-        <v>270</v>
+        <v>150</v>
       </c>
       <c r="L388" s="4" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="M388" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N388" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O388" s="6"/>
     </row>
     <row r="389" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G389" s="3">
-        <v>45932</v>
+        <v>45887</v>
       </c>
       <c r="H389" s="4" t="s">
-        <v>200</v>
+        <v>146</v>
       </c>
       <c r="I389" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="J389" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K389" s="8">
-        <v>150</v>
+        <v>91</v>
+      </c>
+      <c r="K389" s="5">
+        <v>135</v>
       </c>
       <c r="L389" s="4" t="s">
-        <v>43</v>
+        <v>92</v>
       </c>
       <c r="M389" s="4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N389" s="6">
         <v>2</v>
@@ -11992,22 +12071,22 @@
     </row>
     <row r="390" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G390" s="3">
-        <v>45887</v>
+        <v>45881</v>
       </c>
       <c r="H390" s="4" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="I390" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J390" s="4" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="K390" s="5">
-        <v>135</v>
+        <v>105</v>
       </c>
       <c r="L390" s="4" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="M390" s="4" t="s">
         <v>7</v>
@@ -12019,25 +12098,25 @@
     </row>
     <row r="391" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G391" s="3">
-        <v>45881</v>
+        <v>45939</v>
       </c>
       <c r="H391" s="4" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="I391" s="6" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="J391" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="K391" s="5">
-        <v>105</v>
+        <v>42</v>
+      </c>
+      <c r="K391" s="8">
+        <v>150</v>
       </c>
       <c r="L391" s="4" t="s">
-        <v>74</v>
+        <v>43</v>
       </c>
       <c r="M391" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N391" s="6">
         <v>2</v>
@@ -12046,23 +12125,17 @@
     </row>
     <row r="392" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G392" s="3">
-        <v>45939</v>
+        <v>45910</v>
       </c>
       <c r="H392" s="4" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="I392" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J392" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="K392" s="8">
-        <v>150</v>
-      </c>
-      <c r="L392" s="4" t="s">
-        <v>43</v>
-      </c>
+        <v>128</v>
+      </c>
+      <c r="J392" s="4"/>
+      <c r="K392" s="8"/>
+      <c r="L392" s="4"/>
       <c r="M392" s="4" t="s">
         <v>8</v>
       </c>
@@ -12073,13 +12146,13 @@
     </row>
     <row r="393" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G393" s="3">
-        <v>45910</v>
+        <v>45911</v>
       </c>
       <c r="H393" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="I393" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J393" s="4"/>
       <c r="K393" s="8"/>
@@ -12094,13 +12167,13 @@
     </row>
     <row r="394" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G394" s="3">
-        <v>45911</v>
+        <v>45918</v>
       </c>
       <c r="H394" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="I394" s="6" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="J394" s="4"/>
       <c r="K394" s="8"/>
@@ -12114,125 +12187,131 @@
       <c r="O394" s="6"/>
     </row>
     <row r="395" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G395" s="3">
-        <v>45918</v>
-      </c>
-      <c r="H395" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="I395" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J395" s="4"/>
-      <c r="K395" s="8"/>
-      <c r="L395" s="4"/>
-      <c r="M395" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N395" s="6">
-        <v>2</v>
-      </c>
-      <c r="O395" s="6"/>
+      <c r="G395" s="30">
+        <v>45946</v>
+      </c>
+      <c r="H395" s="31" t="s">
+        <v>157</v>
+      </c>
+      <c r="I395" s="29" t="s">
+        <v>126</v>
+      </c>
+      <c r="J395" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="K395" s="32">
+        <v>150</v>
+      </c>
+      <c r="L395" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="M395" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="N395" s="29">
+        <v>2</v>
+      </c>
+      <c r="O395" s="29"/>
     </row>
     <row r="396" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G396" s="30">
-        <v>45946</v>
-      </c>
-      <c r="H396" s="31" t="s">
-        <v>157</v>
-      </c>
-      <c r="I396" s="29" t="s">
+        <v>45953</v>
+      </c>
+      <c r="H396" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="I396" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J396" s="31" t="s">
+      <c r="J396" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K396" s="32">
+      <c r="K396" s="8">
         <v>150</v>
       </c>
       <c r="L396" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="M396" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="N396" s="29">
-        <v>2</v>
-      </c>
-      <c r="O396" s="29"/>
+      <c r="M396" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N396" s="6">
+        <v>2</v>
+      </c>
+      <c r="O396" s="25"/>
     </row>
     <row r="397" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G397" s="30">
-        <v>45953</v>
+        <v>45937</v>
       </c>
       <c r="H397" s="4" t="s">
-        <v>198</v>
+        <v>140</v>
       </c>
       <c r="I397" s="6" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="J397" s="4" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
       <c r="K397" s="8">
-        <v>150</v>
-      </c>
-      <c r="L397" s="31" t="s">
-        <v>43</v>
+        <v>140</v>
+      </c>
+      <c r="L397" s="4" t="s">
+        <v>212</v>
       </c>
       <c r="M397" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N397" s="6">
-        <v>2</v>
-      </c>
-      <c r="O397" s="25"/>
+        <v>3</v>
+      </c>
+      <c r="O397" s="6"/>
     </row>
     <row r="398" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G398" s="30">
-        <v>45937</v>
+        <v>45959</v>
       </c>
       <c r="H398" s="4" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="I398" s="6" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J398" s="4" t="s">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="K398" s="8">
-        <v>140</v>
+        <v>160</v>
       </c>
       <c r="L398" s="4" t="s">
-        <v>212</v>
+        <v>268</v>
       </c>
       <c r="M398" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N398" s="6">
-        <v>3</v>
-      </c>
-      <c r="O398" s="6"/>
+        <v>2</v>
+      </c>
+      <c r="O398" s="25"/>
     </row>
     <row r="399" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G399" s="30">
         <v>45959</v>
       </c>
       <c r="H399" s="4" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="I399" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J399" s="4" t="s">
-        <v>108</v>
+        <v>136</v>
+      </c>
+      <c r="J399" s="15" t="s">
+        <v>102</v>
       </c>
       <c r="K399" s="8">
-        <v>160</v>
+        <v>190</v>
       </c>
       <c r="L399" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M399" s="4" t="s">
         <v>8</v>
@@ -12247,25 +12326,25 @@
         <v>45959</v>
       </c>
       <c r="H400" s="4" t="s">
-        <v>140</v>
+        <v>262</v>
       </c>
       <c r="I400" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J400" s="15" t="s">
-        <v>102</v>
+        <v>263</v>
+      </c>
+      <c r="J400" s="4" t="s">
+        <v>21</v>
       </c>
       <c r="K400" s="8">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="L400" s="4" t="s">
-        <v>269</v>
+        <v>103</v>
       </c>
       <c r="M400" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N400" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O400" s="25"/>
     </row>
@@ -12274,19 +12353,19 @@
         <v>45959</v>
       </c>
       <c r="H401" s="4" t="s">
-        <v>262</v>
+        <v>165</v>
       </c>
       <c r="I401" s="6" t="s">
-        <v>263</v>
+        <v>174</v>
       </c>
       <c r="J401" s="4" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="K401" s="8">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="L401" s="4" t="s">
-        <v>103</v>
+        <v>236</v>
       </c>
       <c r="M401" s="4" t="s">
         <v>8</v>
@@ -12301,19 +12380,19 @@
         <v>45959</v>
       </c>
       <c r="H402" s="4" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="I402" s="6" t="s">
-        <v>174</v>
+        <v>126</v>
       </c>
       <c r="J402" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K402" s="8">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="L402" s="4" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="M402" s="4" t="s">
         <v>8</v>
@@ -12327,25 +12406,25 @@
       <c r="G403" s="30">
         <v>45959</v>
       </c>
-      <c r="H403" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="I403" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J403" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="K403" s="8">
-        <v>120</v>
-      </c>
-      <c r="L403" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="M403" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N403" s="6">
+      <c r="H403" s="31" t="s">
+        <v>264</v>
+      </c>
+      <c r="I403" s="29" t="s">
+        <v>265</v>
+      </c>
+      <c r="J403" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="K403" s="32">
+        <v>210</v>
+      </c>
+      <c r="L403" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="M403" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="N403" s="29">
         <v>3</v>
       </c>
       <c r="O403" s="25"/>
@@ -12354,58 +12433,70 @@
       <c r="G404" s="30">
         <v>45959</v>
       </c>
-      <c r="H404" s="31" t="s">
-        <v>264</v>
-      </c>
-      <c r="I404" s="29" t="s">
-        <v>265</v>
-      </c>
-      <c r="J404" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="K404" s="32">
-        <v>210</v>
-      </c>
-      <c r="L404" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="M404" s="31" t="s">
-        <v>8</v>
-      </c>
-      <c r="N404" s="29">
-        <v>3</v>
-      </c>
+      <c r="H404" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="I404" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J404" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="K404" s="8">
+        <v>280</v>
+      </c>
+      <c r="L404" s="4" t="s">
+        <v>261</v>
+      </c>
+      <c r="M404" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N404" s="6"/>
       <c r="O404" s="25"/>
     </row>
     <row r="405" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G405" s="30"/>
-      <c r="H405" s="4"/>
-      <c r="I405" s="6"/>
-      <c r="J405" s="4"/>
-      <c r="K405" s="8"/>
-      <c r="L405" s="4"/>
-      <c r="M405" s="4"/>
+      <c r="G405" s="30">
+        <v>45960</v>
+      </c>
+      <c r="H405" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="I405" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="J405" s="4" t="s">
+        <v>257</v>
+      </c>
+      <c r="K405" s="8">
+        <v>175</v>
+      </c>
+      <c r="L405" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="M405" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N405" s="6"/>
       <c r="O405" s="25"/>
     </row>
     <row r="406" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G406" s="30">
-        <v>45959</v>
+        <v>45960</v>
       </c>
       <c r="H406" s="4" t="s">
-        <v>198</v>
+        <v>131</v>
       </c>
       <c r="I406" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J406" s="4" t="s">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="K406" s="8">
-        <v>280</v>
+        <v>180</v>
       </c>
       <c r="L406" s="4" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="M406" s="4" t="s">
         <v>8</v>
@@ -12414,56 +12505,98 @@
       <c r="O406" s="25"/>
     </row>
     <row r="407" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G407" s="33"/>
-      <c r="H407" s="33"/>
-      <c r="I407" s="28"/>
-      <c r="J407" s="33"/>
-      <c r="K407" s="34"/>
-      <c r="L407" s="33"/>
-      <c r="M407" s="33"/>
-      <c r="N407" s="28"/>
+      <c r="G407" s="30">
+        <v>45960</v>
+      </c>
+      <c r="H407" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="I407" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="J407" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K407" s="8">
+        <v>198</v>
+      </c>
+      <c r="L407" s="4" t="s">
+        <v>272</v>
+      </c>
+      <c r="M407" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N407" s="6"/>
       <c r="O407" s="25"/>
     </row>
     <row r="408" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G408" s="4"/>
-      <c r="H408" s="4"/>
-      <c r="I408" s="6"/>
-      <c r="J408" s="4"/>
-      <c r="K408" s="8"/>
-      <c r="L408" s="4"/>
-      <c r="M408" s="4"/>
+      <c r="G408" s="30">
+        <v>45960</v>
+      </c>
+      <c r="H408" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I408" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J408" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="K408" s="8">
+        <v>180</v>
+      </c>
+      <c r="L408" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="M408" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N408" s="6"/>
       <c r="O408" s="25"/>
     </row>
     <row r="409" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G409" s="31"/>
-      <c r="H409" s="31"/>
-      <c r="I409" s="29"/>
-      <c r="J409" s="31"/>
-      <c r="K409" s="32"/>
-      <c r="L409" s="31"/>
-      <c r="M409" s="31"/>
-      <c r="N409" s="29"/>
+      <c r="G409" s="30">
+        <v>45960</v>
+      </c>
+      <c r="H409" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I409" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="J409" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K409" s="8">
+        <v>150</v>
+      </c>
+      <c r="L409" s="31" t="s">
+        <v>43</v>
+      </c>
+      <c r="M409" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N409" s="6"/>
       <c r="O409" s="25"/>
     </row>
     <row r="410" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G410" s="30">
         <v>45960</v>
       </c>
-      <c r="H410" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="I410" s="6" t="s">
-        <v>130</v>
+      <c r="H410" s="31" t="s">
+        <v>141</v>
+      </c>
+      <c r="I410" s="29" t="s">
+        <v>265</v>
       </c>
       <c r="J410" s="4" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="K410" s="8">
-        <v>175</v>
+        <v>220</v>
       </c>
       <c r="L410" s="4" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
       <c r="M410" s="4" t="s">
         <v>8</v>
@@ -12476,19 +12609,19 @@
         <v>45960</v>
       </c>
       <c r="H411" s="4" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="I411" s="6" t="s">
-        <v>129</v>
+        <v>219</v>
       </c>
       <c r="J411" s="4" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="K411" s="8">
-        <v>180</v>
+        <v>159</v>
       </c>
       <c r="L411" s="4" t="s">
-        <v>273</v>
+        <v>89</v>
       </c>
       <c r="M411" s="4" t="s">
         <v>8</v>
@@ -12501,19 +12634,19 @@
         <v>45960</v>
       </c>
       <c r="H412" s="4" t="s">
-        <v>262</v>
+        <v>158</v>
       </c>
       <c r="I412" s="6" t="s">
-        <v>263</v>
+        <v>122</v>
       </c>
       <c r="J412" s="4" t="s">
-        <v>86</v>
+        <v>13</v>
       </c>
       <c r="K412" s="8">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="L412" s="4" t="s">
-        <v>272</v>
+        <v>12</v>
       </c>
       <c r="M412" s="4" t="s">
         <v>8</v>
@@ -12526,19 +12659,19 @@
         <v>45960</v>
       </c>
       <c r="H413" s="4" t="s">
-        <v>165</v>
+        <v>151</v>
       </c>
       <c r="I413" s="6" t="s">
-        <v>174</v>
+        <v>271</v>
       </c>
       <c r="J413" s="4" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="K413" s="8">
-        <v>180</v>
+        <v>150</v>
       </c>
       <c r="L413" s="4" t="s">
-        <v>274</v>
+        <v>242</v>
       </c>
       <c r="M413" s="4" t="s">
         <v>8</v>
@@ -12547,23 +12680,23 @@
       <c r="O413" s="25"/>
     </row>
     <row r="414" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G414" s="30">
+      <c r="G414" s="3">
         <v>45960</v>
       </c>
       <c r="H414" s="4" t="s">
-        <v>155</v>
+        <v>247</v>
       </c>
       <c r="I414" s="6" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="J414" s="4" t="s">
-        <v>42</v>
+        <v>277</v>
       </c>
       <c r="K414" s="8">
-        <v>150</v>
-      </c>
-      <c r="L414" s="31" t="s">
-        <v>43</v>
+        <v>200</v>
+      </c>
+      <c r="L414" s="4" t="s">
+        <v>278</v>
       </c>
       <c r="M414" s="4" t="s">
         <v>8</v>
@@ -12572,23 +12705,23 @@
       <c r="O414" s="25"/>
     </row>
     <row r="415" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G415" s="30">
+      <c r="G415" s="3">
         <v>45960</v>
       </c>
-      <c r="H415" s="31" t="s">
-        <v>141</v>
-      </c>
-      <c r="I415" s="29" t="s">
-        <v>265</v>
+      <c r="H415" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I415" s="6" t="s">
+        <v>217</v>
       </c>
       <c r="J415" s="4" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="K415" s="8">
         <v>220</v>
       </c>
       <c r="L415" s="4" t="s">
-        <v>276</v>
+        <v>177</v>
       </c>
       <c r="M415" s="4" t="s">
         <v>8</v>
@@ -12597,23 +12730,23 @@
       <c r="O415" s="25"/>
     </row>
     <row r="416" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G416" s="30">
+      <c r="G416" s="3">
         <v>45960</v>
       </c>
       <c r="H416" s="4" t="s">
-        <v>240</v>
+        <v>146</v>
       </c>
       <c r="I416" s="6" t="s">
-        <v>219</v>
+        <v>128</v>
       </c>
       <c r="J416" s="4" t="s">
-        <v>70</v>
+        <v>164</v>
       </c>
       <c r="K416" s="8">
-        <v>159</v>
+        <v>179.9</v>
       </c>
       <c r="L416" s="4" t="s">
-        <v>89</v>
+        <v>213</v>
       </c>
       <c r="M416" s="4" t="s">
         <v>8</v>
@@ -12622,177 +12755,187 @@
       <c r="O416" s="25"/>
     </row>
     <row r="417" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G417" s="30">
-        <v>45960</v>
+      <c r="G417" s="3">
+        <v>45961</v>
       </c>
       <c r="H417" s="4" t="s">
-        <v>158</v>
+        <v>146</v>
       </c>
       <c r="I417" s="6" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="J417" s="4" t="s">
-        <v>13</v>
+        <v>327</v>
       </c>
       <c r="K417" s="8">
-        <v>200</v>
+        <v>253</v>
       </c>
       <c r="L417" s="4" t="s">
-        <v>12</v>
+        <v>328</v>
       </c>
       <c r="M417" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N417" s="6"/>
-      <c r="O417" s="25"/>
+      <c r="N417" s="6">
+        <v>1</v>
+      </c>
+      <c r="O417" s="25" t="s">
+        <v>253</v>
+      </c>
     </row>
     <row r="418" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G418" s="30">
-        <v>45960</v>
+      <c r="G418" s="3">
+        <v>45964</v>
       </c>
       <c r="H418" s="4" t="s">
-        <v>151</v>
+        <v>198</v>
       </c>
       <c r="I418" s="6" t="s">
-        <v>271</v>
+        <v>125</v>
       </c>
       <c r="J418" s="4" t="s">
-        <v>197</v>
+        <v>66</v>
       </c>
       <c r="K418" s="8">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="L418" s="4" t="s">
-        <v>242</v>
+        <v>337</v>
       </c>
       <c r="M418" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N418" s="6"/>
+      <c r="N418" s="6">
+        <v>2</v>
+      </c>
       <c r="O418" s="25"/>
     </row>
     <row r="419" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G419" s="3">
-        <v>45960</v>
+        <v>45964</v>
       </c>
       <c r="H419" s="4" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="I419" s="6" t="s">
-        <v>134</v>
+        <v>219</v>
       </c>
       <c r="J419" s="4" t="s">
-        <v>277</v>
+        <v>70</v>
       </c>
       <c r="K419" s="8">
-        <v>200</v>
+        <v>159</v>
       </c>
       <c r="L419" s="4" t="s">
-        <v>278</v>
+        <v>335</v>
       </c>
       <c r="M419" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N419" s="6"/>
+      <c r="N419" s="6">
+        <v>2</v>
+      </c>
       <c r="O419" s="25"/>
     </row>
     <row r="420" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G420" s="3">
-        <v>45960</v>
+        <v>45964</v>
       </c>
       <c r="H420" s="4" t="s">
-        <v>152</v>
+        <v>329</v>
       </c>
       <c r="I420" s="6" t="s">
-        <v>217</v>
+        <v>174</v>
       </c>
       <c r="J420" s="4" t="s">
-        <v>275</v>
+        <v>45</v>
       </c>
       <c r="K420" s="8">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="L420" s="4" t="s">
-        <v>177</v>
+        <v>236</v>
       </c>
       <c r="M420" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N420" s="6"/>
+      <c r="N420" s="6">
+        <v>2</v>
+      </c>
       <c r="O420" s="25"/>
     </row>
     <row r="421" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G421" s="3">
-        <v>45960</v>
+        <v>45964</v>
       </c>
       <c r="H421" s="4" t="s">
-        <v>146</v>
+        <v>330</v>
       </c>
       <c r="I421" s="6" t="s">
-        <v>128</v>
+        <v>176</v>
       </c>
       <c r="J421" s="4" t="s">
-        <v>164</v>
+        <v>230</v>
       </c>
       <c r="K421" s="8">
-        <v>179.9</v>
+        <v>220</v>
       </c>
       <c r="L421" s="4" t="s">
-        <v>213</v>
+        <v>93</v>
       </c>
       <c r="M421" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N421" s="6"/>
+      <c r="N421" s="6">
+        <v>2</v>
+      </c>
       <c r="O421" s="25"/>
     </row>
     <row r="422" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G422" s="3">
-        <v>45961</v>
+        <v>45964</v>
       </c>
       <c r="H422" s="4" t="s">
-        <v>146</v>
+        <v>331</v>
       </c>
       <c r="I422" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="J422" s="4" t="s">
-        <v>327</v>
+        <v>25</v>
       </c>
       <c r="K422" s="8">
-        <v>253</v>
+        <v>180</v>
       </c>
       <c r="L422" s="4" t="s">
-        <v>328</v>
+        <v>273</v>
       </c>
       <c r="M422" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N422" s="6">
-        <v>1</v>
-      </c>
-      <c r="O422" s="25" t="s">
-        <v>253</v>
-      </c>
+      <c r="N422" s="4">
+        <v>4</v>
+      </c>
+      <c r="O422" s="25"/>
     </row>
     <row r="423" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G423" s="3">
         <v>45964</v>
       </c>
       <c r="H423" s="4" t="s">
-        <v>198</v>
+        <v>152</v>
       </c>
       <c r="I423" s="6" t="s">
-        <v>125</v>
+        <v>217</v>
       </c>
       <c r="J423" s="4" t="s">
-        <v>66</v>
+        <v>334</v>
       </c>
       <c r="K423" s="8">
-        <v>160</v>
+        <v>175</v>
       </c>
       <c r="L423" s="4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M423" s="4" t="s">
         <v>8</v>
@@ -12807,73 +12950,73 @@
         <v>45964</v>
       </c>
       <c r="H424" s="4" t="s">
-        <v>240</v>
+        <v>262</v>
       </c>
       <c r="I424" s="6" t="s">
-        <v>219</v>
+        <v>263</v>
       </c>
       <c r="J424" s="4" t="s">
-        <v>70</v>
+        <v>332</v>
       </c>
       <c r="K424" s="8">
-        <v>159</v>
+        <v>200</v>
       </c>
       <c r="L424" s="4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="M424" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N424" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O424" s="25"/>
     </row>
     <row r="425" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G425" s="3">
-        <v>45964</v>
+        <v>45965</v>
       </c>
       <c r="H425" s="4" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="I425" s="6" t="s">
-        <v>174</v>
+        <v>136</v>
       </c>
       <c r="J425" s="4" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="K425" s="8">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="L425" s="4" t="s">
-        <v>236</v>
+        <v>101</v>
       </c>
       <c r="M425" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N425" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O425" s="25"/>
     </row>
     <row r="426" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G426" s="3">
-        <v>45964</v>
+        <v>45965</v>
       </c>
       <c r="H426" s="4" t="s">
-        <v>330</v>
+        <v>158</v>
       </c>
       <c r="I426" s="6" t="s">
-        <v>176</v>
+        <v>122</v>
       </c>
       <c r="J426" s="4" t="s">
-        <v>230</v>
+        <v>41</v>
       </c>
       <c r="K426" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L426" s="4" t="s">
-        <v>93</v>
+        <v>116</v>
       </c>
       <c r="M426" s="4" t="s">
         <v>8</v>
@@ -12885,49 +13028,49 @@
     </row>
     <row r="427" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G427" s="3">
-        <v>45964</v>
+        <v>45965</v>
       </c>
       <c r="H427" s="4" t="s">
-        <v>331</v>
+        <v>146</v>
       </c>
       <c r="I427" s="6" t="s">
-        <v>136</v>
+        <v>124</v>
       </c>
       <c r="J427" s="4" t="s">
-        <v>25</v>
+        <v>248</v>
       </c>
       <c r="K427" s="8">
-        <v>180</v>
+        <v>280</v>
       </c>
       <c r="L427" s="4" t="s">
-        <v>273</v>
+        <v>341</v>
       </c>
       <c r="M427" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N427" s="4">
-        <v>4</v>
+      <c r="N427" s="6">
+        <v>3</v>
       </c>
       <c r="O427" s="25"/>
     </row>
     <row r="428" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G428" s="3">
-        <v>45964</v>
+        <v>45965</v>
       </c>
       <c r="H428" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I428" s="6" t="s">
-        <v>217</v>
+        <v>338</v>
       </c>
       <c r="J428" s="4" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="K428" s="8">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="L428" s="4" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="M428" s="4" t="s">
         <v>8</v>
@@ -12939,85 +13082,101 @@
     </row>
     <row r="429" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G429" s="3">
-        <v>45964</v>
+        <v>45965</v>
       </c>
       <c r="H429" s="4" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
       <c r="I429" s="6" t="s">
-        <v>263</v>
+        <v>134</v>
       </c>
       <c r="J429" s="4" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="K429" s="8">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="L429" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="M429" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N429" s="6"/>
+        <v>261</v>
+      </c>
+      <c r="M429" s="4"/>
+      <c r="N429" s="6">
+        <v>2</v>
+      </c>
       <c r="O429" s="25"/>
     </row>
-    <row r="430" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G430" s="3"/>
-      <c r="H430" s="4"/>
-      <c r="I430" s="6"/>
-      <c r="J430" s="4"/>
-      <c r="K430" s="8"/>
-      <c r="L430" s="4"/>
-      <c r="M430" s="4"/>
-      <c r="N430" s="6"/>
+    <row r="430" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G430" s="3">
+        <v>45965</v>
+      </c>
+      <c r="H430" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="I430" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J430" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K430" s="8">
+        <v>160</v>
+      </c>
+      <c r="L430" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="M430" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N430" s="6">
+        <v>3</v>
+      </c>
       <c r="O430" s="25"/>
     </row>
-    <row r="431" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="431" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G431" s="3">
         <v>45965</v>
       </c>
       <c r="H431" s="4" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I431" s="6" t="s">
-        <v>136</v>
+        <v>176</v>
       </c>
       <c r="J431" s="4" t="s">
-        <v>25</v>
+        <v>257</v>
       </c>
       <c r="K431" s="8">
-        <v>180</v>
+        <v>205</v>
       </c>
       <c r="L431" s="4" t="s">
-        <v>101</v>
+        <v>258</v>
       </c>
       <c r="M431" s="4" t="s">
         <v>8</v>
       </c>
       <c r="N431" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O431" s="25"/>
     </row>
-    <row r="432" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="432" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G432" s="3">
-        <v>45965</v>
+        <v>45966</v>
       </c>
       <c r="H432" s="4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="I432" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="J432" s="4" t="s">
-        <v>41</v>
+        <v>230</v>
       </c>
       <c r="K432" s="8">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="L432" s="4" t="s">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="M432" s="4" t="s">
         <v>8</v>
@@ -13027,140 +13186,62 @@
       </c>
       <c r="O432" s="25"/>
     </row>
-    <row r="433" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G433" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H433" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="I433" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J433" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="K433" s="8">
-        <v>280</v>
-      </c>
-      <c r="L433" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="M433" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N433" s="6">
-        <v>3</v>
-      </c>
+    <row r="433" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G433" s="4"/>
+      <c r="H433" s="4"/>
+      <c r="I433" s="6"/>
+      <c r="J433" s="4"/>
+      <c r="K433" s="8"/>
+      <c r="L433" s="4"/>
+      <c r="M433" s="4"/>
+      <c r="N433" s="6"/>
       <c r="O433" s="25"/>
     </row>
-    <row r="434" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G434" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H434" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I434" s="6" t="s">
-        <v>338</v>
-      </c>
-      <c r="J434" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="K434" s="8">
-        <v>200</v>
-      </c>
-      <c r="L434" s="4" t="s">
-        <v>343</v>
-      </c>
-      <c r="M434" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N434" s="6">
-        <v>2</v>
-      </c>
+    <row r="434" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G434" s="4"/>
+      <c r="H434" s="4"/>
+      <c r="I434" s="6"/>
+      <c r="J434" s="4"/>
+      <c r="K434" s="8"/>
+      <c r="L434" s="4"/>
+      <c r="M434" s="4"/>
+      <c r="N434" s="6"/>
       <c r="O434" s="25"/>
     </row>
-    <row r="435" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G435" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H435" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="I435" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J435" s="4" t="s">
-        <v>344</v>
-      </c>
-      <c r="K435" s="8">
-        <v>280</v>
-      </c>
-      <c r="L435" s="4" t="s">
-        <v>261</v>
-      </c>
+    <row r="435" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G435" s="4"/>
+      <c r="H435" s="4"/>
+      <c r="I435" s="6"/>
+      <c r="J435" s="4"/>
+      <c r="K435" s="8"/>
+      <c r="L435" s="4"/>
       <c r="M435" s="4"/>
-      <c r="N435" s="6">
-        <v>2</v>
-      </c>
+      <c r="N435" s="6"/>
       <c r="O435" s="25"/>
     </row>
-    <row r="436" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G436" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H436" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="I436" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J436" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K436" s="8">
-        <v>160</v>
-      </c>
-      <c r="L436" s="4" t="s">
-        <v>340</v>
-      </c>
-      <c r="M436" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N436" s="6">
-        <v>3</v>
-      </c>
+    <row r="436" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G436" s="4"/>
+      <c r="H436" s="4"/>
+      <c r="I436" s="6"/>
+      <c r="J436" s="4"/>
+      <c r="K436" s="8"/>
+      <c r="L436" s="4"/>
+      <c r="M436" s="4"/>
+      <c r="N436" s="6"/>
       <c r="O436" s="25"/>
     </row>
-    <row r="437" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G437" s="3">
-        <v>45965</v>
-      </c>
-      <c r="H437" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="I437" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="J437" s="4" t="s">
-        <v>257</v>
-      </c>
-      <c r="K437" s="8">
-        <v>205</v>
-      </c>
-      <c r="L437" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="M437" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N437" s="6">
-        <v>1</v>
-      </c>
+    <row r="437" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G437" s="4"/>
+      <c r="H437" s="4"/>
+      <c r="I437" s="6"/>
+      <c r="J437" s="4"/>
+      <c r="K437" s="8"/>
+      <c r="L437" s="4"/>
+      <c r="M437" s="4"/>
+      <c r="N437" s="6"/>
       <c r="O437" s="25"/>
     </row>
-    <row r="438" spans="7:15" x14ac:dyDescent="0.25">
+    <row r="438" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
       <c r="G438" s="4"/>
       <c r="H438" s="4"/>
       <c r="I438" s="6"/>
@@ -13171,33 +13252,369 @@
       <c r="N438" s="6"/>
       <c r="O438" s="25"/>
     </row>
-    <row r="439" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G439" s="4"/>
-      <c r="H439" s="4"/>
-      <c r="I439" s="6"/>
-      <c r="J439" s="4"/>
-      <c r="K439" s="8"/>
-      <c r="L439" s="4"/>
+    <row r="439" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G439" s="3">
+        <v>45966</v>
+      </c>
+      <c r="H439" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="I439" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J439" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K439" s="8">
+        <v>170</v>
+      </c>
+      <c r="L439" s="4" t="s">
+        <v>346</v>
+      </c>
       <c r="M439" s="4"/>
-      <c r="N439" s="6"/>
+      <c r="N439" s="6">
+        <v>3</v>
+      </c>
       <c r="O439" s="25"/>
     </row>
-    <row r="440" spans="7:15" x14ac:dyDescent="0.25">
-      <c r="G440" s="4"/>
-      <c r="H440" s="4"/>
-      <c r="I440" s="6"/>
-      <c r="J440" s="4"/>
-      <c r="K440" s="8"/>
-      <c r="L440" s="4"/>
+    <row r="440" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G440" s="35">
+        <v>45966</v>
+      </c>
+      <c r="H440" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="I440" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J440" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K440" s="8">
+        <v>150</v>
+      </c>
+      <c r="L440" s="4" t="s">
+        <v>349</v>
+      </c>
       <c r="M440" s="4"/>
-      <c r="N440" s="6"/>
+      <c r="N440" s="6">
+        <v>2</v>
+      </c>
       <c r="O440" s="25"/>
     </row>
+    <row r="441" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G441" s="35">
+        <v>45966</v>
+      </c>
+      <c r="H441" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I441" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J441" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="K441" s="8">
+        <v>220</v>
+      </c>
+      <c r="L441" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="M441" s="4"/>
+      <c r="N441" s="6">
+        <v>2</v>
+      </c>
+      <c r="O441" s="25"/>
+    </row>
+    <row r="442" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G442" s="35">
+        <v>45966</v>
+      </c>
+      <c r="H442" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="I442" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J442" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="K442" s="8">
+        <v>160</v>
+      </c>
+      <c r="L442" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="M442" s="4"/>
+      <c r="N442" s="6">
+        <v>2</v>
+      </c>
+      <c r="O442" s="25"/>
+    </row>
+    <row r="443" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G443" s="35">
+        <v>45966</v>
+      </c>
+      <c r="H443" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="I443" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J443" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K443" s="8">
+        <v>200</v>
+      </c>
+      <c r="L443" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="M443" s="4"/>
+      <c r="N443" s="6">
+        <v>2</v>
+      </c>
+      <c r="O443" s="25"/>
+    </row>
+    <row r="444" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G444" s="3">
+        <v>45966</v>
+      </c>
+      <c r="H444" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I444" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="J444" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K444" s="8">
+        <v>170</v>
+      </c>
+      <c r="L444" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="M444" s="4"/>
+      <c r="N444" s="6">
+        <v>3</v>
+      </c>
+      <c r="O444" s="25"/>
+    </row>
+    <row r="445" spans="7:15" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G445" s="3">
+        <v>45966</v>
+      </c>
+      <c r="H445" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I445" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J445" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K445" s="8">
+        <v>170</v>
+      </c>
+      <c r="L445" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="M445" s="4"/>
+      <c r="N445" s="6">
+        <v>3</v>
+      </c>
+      <c r="O445" s="25"/>
+    </row>
+    <row r="446" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G446" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H446" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="I446" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J446" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="K446" s="8">
+        <v>200</v>
+      </c>
+      <c r="L446" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M446" s="4"/>
+      <c r="N446" s="6">
+        <v>2</v>
+      </c>
+      <c r="O446" s="25"/>
+    </row>
+    <row r="447" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G447" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H447" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I447" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J447" s="4"/>
+      <c r="K447" s="8"/>
+      <c r="L447" s="4"/>
+      <c r="M447" s="4"/>
+      <c r="N447" s="6">
+        <v>1</v>
+      </c>
+      <c r="O447" s="25"/>
+    </row>
+    <row r="448" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G448" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H448" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="I448" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J448" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K448" s="8">
+        <v>180</v>
+      </c>
+      <c r="L448" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M448" s="4"/>
+      <c r="N448" s="6">
+        <v>2</v>
+      </c>
+      <c r="O448" s="25"/>
+    </row>
+    <row r="449" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G449" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H449" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I449" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="J449" s="4"/>
+      <c r="K449" s="8"/>
+      <c r="L449" s="4"/>
+      <c r="M449" s="4"/>
+      <c r="N449" s="6">
+        <v>2</v>
+      </c>
+      <c r="O449" s="25"/>
+    </row>
+    <row r="450" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G450" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H450" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I450" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J450" s="4"/>
+      <c r="K450" s="8"/>
+      <c r="L450" s="4"/>
+      <c r="M450" s="4"/>
+      <c r="N450" s="6">
+        <v>2</v>
+      </c>
+      <c r="O450" s="25"/>
+    </row>
+    <row r="451" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G451" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H451" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="I451" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J451" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="K451" s="8">
+        <v>159</v>
+      </c>
+      <c r="L451" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M451" s="4"/>
+      <c r="N451" s="6"/>
+      <c r="O451" s="25"/>
+    </row>
+    <row r="452" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G452" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H452" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="I452" s="36" t="s">
+        <v>122</v>
+      </c>
+      <c r="J452" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K452" s="10">
+        <v>240</v>
+      </c>
+      <c r="L452" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="453" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G453" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H453" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="I453" s="36" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="454" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G454" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H454" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="I454" s="36" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="455" spans="7:15" x14ac:dyDescent="0.25">
+      <c r="G455" s="3">
+        <v>45967</v>
+      </c>
+      <c r="H455" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I455" s="36" t="s">
+        <v>217</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="G5:O437" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O455" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="4" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="6" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G67:O409">
@@ -13217,9 +13634,9 @@
   <dimension ref="B3:D50"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.5703125" style="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5703125" style="36" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="36" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" style="34" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5703125" style="34" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="34" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
@@ -13284,7 +13701,7 @@
       <c r="C8" s="7" t="s">
         <v>236</v>
       </c>
-      <c r="D8" s="35" t="s">
+      <c r="D8" s="33" t="s">
         <v>286</v>
       </c>
     </row>
@@ -13740,7 +14157,7 @@
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="B50" s="36" t="s">
+      <c r="B50" s="34" t="s">
         <v>70</v>
       </c>
       <c r="C50" s="7" t="s">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-12 17:18
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="874" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12A66445-C0BF-4136-AAC3-EE62DC0E1C6F}"/>
+  <xr:revisionPtr revIDLastSave="926" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FA197BF-71D0-4A41-8E1D-E322392815E6}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$496</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$482</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3027" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2954" uniqueCount="375">
   <si>
     <t>DATA</t>
   </si>
@@ -1155,6 +1155,15 @@
   </si>
   <si>
     <t>ABAETE PALACE</t>
+  </si>
+  <si>
+    <t>HOTEL AGUAS CLARAS</t>
+  </si>
+  <si>
+    <t>VIÇOSA</t>
+  </si>
+  <si>
+    <t>HOTEL CABANA</t>
   </si>
 </sst>
 </file>
@@ -1301,7 +1310,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1402,6 +1411,24 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -1741,7 +1768,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P509"/>
+  <dimension ref="G5:P495"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -1749,7 +1776,7 @@
     <col min="9" max="9" width="21" customWidth="1"/>
     <col min="10" max="10" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15" style="10" customWidth="1"/>
-    <col min="12" max="12" width="28.28515625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="36.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
     <col min="14" max="14" width="12.42578125" customWidth="1"/>
     <col min="15" max="15" width="20.140625" style="22" customWidth="1"/>
@@ -14537,22 +14564,22 @@
     </row>
     <row r="432" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G432" s="3">
-        <v>45964</v>
+        <v>45966</v>
       </c>
       <c r="H432" s="4" t="s">
-        <v>197</v>
+        <v>173</v>
       </c>
       <c r="I432" s="6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="J432" s="4" t="s">
-        <v>66</v>
+        <v>229</v>
       </c>
       <c r="K432" s="8">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="L432" s="4" t="s">
-        <v>335</v>
+        <v>93</v>
       </c>
       <c r="M432" s="4" t="s">
         <v>8</v>
@@ -14567,28 +14594,26 @@
     </row>
     <row r="433" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G433" s="3">
-        <v>45964</v>
+        <v>45966</v>
       </c>
       <c r="H433" s="4" t="s">
-        <v>239</v>
+        <v>343</v>
       </c>
       <c r="I433" s="6" t="s">
-        <v>218</v>
+        <v>135</v>
       </c>
       <c r="J433" s="4" t="s">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="K433" s="8">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="L433" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="M433" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="M433" s="4"/>
       <c r="N433" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O433" s="25"/>
       <c r="P433" t="s">
@@ -14596,27 +14621,25 @@
       </c>
     </row>
     <row r="434" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G434" s="3">
-        <v>45964</v>
+      <c r="G434" s="39">
+        <v>45966</v>
       </c>
       <c r="H434" s="4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I434" s="6" t="s">
-        <v>173</v>
+        <v>136</v>
       </c>
       <c r="J434" s="4" t="s">
-        <v>45</v>
+        <v>11</v>
       </c>
       <c r="K434" s="8">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="L434" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="M434" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>344</v>
+      </c>
+      <c r="M434" s="4"/>
       <c r="N434" s="6">
         <v>2</v>
       </c>
@@ -14626,27 +14649,25 @@
       </c>
     </row>
     <row r="435" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G435" s="3">
-        <v>45964</v>
+      <c r="G435" s="39">
+        <v>45966</v>
       </c>
       <c r="H435" s="4" t="s">
-        <v>328</v>
+        <v>146</v>
       </c>
       <c r="I435" s="6" t="s">
-        <v>175</v>
+        <v>124</v>
       </c>
       <c r="J435" s="4" t="s">
-        <v>229</v>
+        <v>345</v>
       </c>
       <c r="K435" s="8">
         <v>220</v>
       </c>
       <c r="L435" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M435" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>346</v>
+      </c>
+      <c r="M435" s="4"/>
       <c r="N435" s="6">
         <v>2</v>
       </c>
@@ -14656,29 +14677,27 @@
       </c>
     </row>
     <row r="436" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G436" s="3">
-        <v>45964</v>
+      <c r="G436" s="39">
+        <v>45966</v>
       </c>
       <c r="H436" s="4" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
       <c r="I436" s="6" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="J436" s="4" t="s">
-        <v>25</v>
+        <v>347</v>
       </c>
       <c r="K436" s="8">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="L436" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="M436" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N436" s="4">
-        <v>4</v>
+        <v>214</v>
+      </c>
+      <c r="M436" s="4"/>
+      <c r="N436" s="6">
+        <v>2</v>
       </c>
       <c r="O436" s="25"/>
       <c r="P436" t="s">
@@ -14686,27 +14705,25 @@
       </c>
     </row>
     <row r="437" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G437" s="3">
-        <v>45964</v>
+      <c r="G437" s="39">
+        <v>45966</v>
       </c>
       <c r="H437" s="4" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="I437" s="6" t="s">
-        <v>216</v>
+        <v>173</v>
       </c>
       <c r="J437" s="4" t="s">
-        <v>332</v>
+        <v>45</v>
       </c>
       <c r="K437" s="8">
-        <v>175</v>
+        <v>200</v>
       </c>
       <c r="L437" s="4" t="s">
-        <v>334</v>
-      </c>
-      <c r="M437" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>348</v>
+      </c>
+      <c r="M437" s="4"/>
       <c r="N437" s="6">
         <v>2</v>
       </c>
@@ -14717,26 +14734,24 @@
     </row>
     <row r="438" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G438" s="3">
-        <v>45964</v>
+        <v>45966</v>
       </c>
       <c r="H438" s="4" t="s">
-        <v>260</v>
+        <v>157</v>
       </c>
       <c r="I438" s="6" t="s">
-        <v>261</v>
+        <v>188</v>
       </c>
       <c r="J438" s="4" t="s">
-        <v>330</v>
+        <v>46</v>
       </c>
       <c r="K438" s="8">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="L438" s="4" t="s">
-        <v>331</v>
-      </c>
-      <c r="M438" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="M438" s="4"/>
       <c r="N438" s="6">
         <v>3</v>
       </c>
@@ -14747,26 +14762,24 @@
     </row>
     <row r="439" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G439" s="3">
-        <v>45965</v>
+        <v>45966</v>
       </c>
       <c r="H439" s="4" t="s">
-        <v>329</v>
+        <v>141</v>
       </c>
       <c r="I439" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J439" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K439" s="8">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="L439" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="M439" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>349</v>
+      </c>
+      <c r="M439" s="4"/>
       <c r="N439" s="6">
         <v>3</v>
       </c>
@@ -14777,26 +14790,24 @@
     </row>
     <row r="440" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G440" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H440" s="4" t="s">
-        <v>158</v>
+        <v>343</v>
       </c>
       <c r="I440" s="6" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="J440" s="4" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="K440" s="8">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="L440" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="M440" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="M440" s="4"/>
       <c r="N440" s="6">
         <v>2</v>
       </c>
@@ -14807,7 +14818,7 @@
     </row>
     <row r="441" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G441" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H441" s="4" t="s">
         <v>146</v>
@@ -14816,19 +14827,17 @@
         <v>124</v>
       </c>
       <c r="J441" s="4" t="s">
-        <v>246</v>
+        <v>350</v>
       </c>
       <c r="K441" s="8">
-        <v>280</v>
+        <v>240</v>
       </c>
       <c r="L441" s="4" t="s">
-        <v>339</v>
-      </c>
-      <c r="M441" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>194</v>
+      </c>
+      <c r="M441" s="4"/>
       <c r="N441" s="6">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="O441" s="25"/>
       <c r="P441" t="s">
@@ -14837,26 +14846,24 @@
     </row>
     <row r="442" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G442" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H442" s="4" t="s">
-        <v>151</v>
+        <v>337</v>
       </c>
       <c r="I442" s="6" t="s">
-        <v>336</v>
+        <v>129</v>
       </c>
       <c r="J442" s="4" t="s">
-        <v>340</v>
+        <v>25</v>
       </c>
       <c r="K442" s="8">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="L442" s="4" t="s">
-        <v>341</v>
-      </c>
-      <c r="M442" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="M442" s="4"/>
       <c r="N442" s="6">
         <v>2</v>
       </c>
@@ -14867,22 +14874,22 @@
     </row>
     <row r="443" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G443" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H443" s="4" t="s">
-        <v>245</v>
+        <v>157</v>
       </c>
       <c r="I443" s="6" t="s">
-        <v>134</v>
+        <v>188</v>
       </c>
       <c r="J443" s="4" t="s">
-        <v>342</v>
+        <v>42</v>
       </c>
       <c r="K443" s="8">
-        <v>280</v>
+        <v>150</v>
       </c>
       <c r="L443" s="4" t="s">
-        <v>259</v>
+        <v>351</v>
       </c>
       <c r="M443" s="4"/>
       <c r="N443" s="6">
@@ -14895,28 +14902,26 @@
     </row>
     <row r="444" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G444" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H444" s="4" t="s">
-        <v>337</v>
+        <v>141</v>
       </c>
       <c r="I444" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J444" s="4" t="s">
-        <v>14</v>
+        <v>106</v>
       </c>
       <c r="K444" s="8">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="L444" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="M444" s="4" t="s">
-        <v>8</v>
-      </c>
+        <v>352</v>
+      </c>
+      <c r="M444" s="4"/>
       <c r="N444" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O444" s="25"/>
       <c r="P444" t="s">
@@ -14925,29 +14930,25 @@
     </row>
     <row r="445" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G445" s="3">
-        <v>45965</v>
+        <v>45967</v>
       </c>
       <c r="H445" s="4" t="s">
-        <v>328</v>
+        <v>353</v>
       </c>
       <c r="I445" s="6" t="s">
-        <v>175</v>
+        <v>354</v>
       </c>
       <c r="J445" s="4" t="s">
-        <v>255</v>
+        <v>355</v>
       </c>
       <c r="K445" s="8">
-        <v>205</v>
+        <v>159</v>
       </c>
       <c r="L445" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="M445" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N445" s="6">
-        <v>1</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="M445" s="4"/>
+      <c r="N445" s="6"/>
       <c r="O445" s="25"/>
       <c r="P445" t="s">
         <v>358</v>
@@ -14955,29 +14956,25 @@
     </row>
     <row r="446" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G446" s="3">
-        <v>45966</v>
+        <v>45967</v>
       </c>
       <c r="H446" s="4" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="I446" s="6" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="J446" s="4" t="s">
-        <v>229</v>
+        <v>41</v>
       </c>
       <c r="K446" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L446" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M446" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N446" s="6">
-        <v>2</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="M446" s="4"/>
+      <c r="N446" s="6"/>
       <c r="O446" s="25"/>
       <c r="P446" t="s">
         <v>358</v>
@@ -14985,164 +14982,160 @@
     </row>
     <row r="447" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G447" s="3">
-        <v>45966</v>
+        <v>45967</v>
       </c>
       <c r="H447" s="4" t="s">
-        <v>343</v>
+        <v>245</v>
       </c>
       <c r="I447" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J447" s="4" t="s">
-        <v>46</v>
+        <v>356</v>
       </c>
       <c r="K447" s="8">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="L447" s="4" t="s">
-        <v>48</v>
+        <v>276</v>
       </c>
       <c r="M447" s="4"/>
-      <c r="N447" s="6">
-        <v>3</v>
-      </c>
+      <c r="N447" s="6"/>
       <c r="O447" s="25"/>
       <c r="P447" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="448" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G448" s="39">
-        <v>45966</v>
+      <c r="G448" s="3">
+        <v>45967</v>
       </c>
       <c r="H448" s="4" t="s">
-        <v>329</v>
+        <v>152</v>
       </c>
       <c r="I448" s="6" t="s">
-        <v>136</v>
+        <v>216</v>
       </c>
       <c r="J448" s="4" t="s">
-        <v>11</v>
+        <v>273</v>
       </c>
       <c r="K448" s="8">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="L448" s="4" t="s">
-        <v>344</v>
+        <v>176</v>
       </c>
       <c r="M448" s="4"/>
-      <c r="N448" s="6">
-        <v>2</v>
-      </c>
+      <c r="N448" s="6"/>
       <c r="O448" s="25"/>
       <c r="P448" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="449" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G449" s="39">
-        <v>45966</v>
+      <c r="G449" s="3">
+        <v>45967</v>
       </c>
       <c r="H449" s="4" t="s">
-        <v>146</v>
+        <v>329</v>
       </c>
       <c r="I449" s="6" t="s">
-        <v>124</v>
+        <v>136</v>
       </c>
       <c r="J449" s="4" t="s">
-        <v>345</v>
+        <v>102</v>
       </c>
       <c r="K449" s="8">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="L449" s="4" t="s">
-        <v>346</v>
+        <v>267</v>
       </c>
       <c r="M449" s="4"/>
-      <c r="N449" s="6">
-        <v>2</v>
-      </c>
+      <c r="N449" s="6"/>
       <c r="O449" s="25"/>
       <c r="P449" t="s">
         <v>358</v>
       </c>
     </row>
     <row r="450" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G450" s="39">
-        <v>45966</v>
-      </c>
-      <c r="H450" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="I450" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J450" s="4" t="s">
-        <v>347</v>
-      </c>
-      <c r="K450" s="8">
-        <v>160</v>
-      </c>
-      <c r="L450" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="M450" s="4"/>
-      <c r="N450" s="6">
-        <v>2</v>
-      </c>
-      <c r="O450" s="25"/>
+      <c r="G450" s="30">
+        <v>45967</v>
+      </c>
+      <c r="H450" s="31" t="s">
+        <v>164</v>
+      </c>
+      <c r="I450" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="J450" s="31" t="s">
+        <v>192</v>
+      </c>
+      <c r="K450" s="32">
+        <v>230</v>
+      </c>
+      <c r="L450" s="31" t="s">
+        <v>193</v>
+      </c>
+      <c r="M450" s="31"/>
+      <c r="N450" s="29"/>
+      <c r="O450" s="37"/>
       <c r="P450" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="451" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G451" s="39">
-        <v>45966</v>
+    <row r="451" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G451" s="3">
+        <v>45973</v>
       </c>
       <c r="H451" s="4" t="s">
-        <v>164</v>
+        <v>197</v>
       </c>
       <c r="I451" s="6" t="s">
-        <v>173</v>
+        <v>125</v>
       </c>
       <c r="J451" s="4" t="s">
-        <v>45</v>
+        <v>25</v>
       </c>
       <c r="K451" s="8">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="L451" s="4" t="s">
-        <v>348</v>
-      </c>
-      <c r="M451" s="4"/>
+        <v>101</v>
+      </c>
+      <c r="M451" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N451" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O451" s="25"/>
       <c r="P451" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="452" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="452" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G452" s="3">
-        <v>45966</v>
+        <v>45973</v>
       </c>
       <c r="H452" s="4" t="s">
-        <v>157</v>
+        <v>337</v>
       </c>
       <c r="I452" s="6" t="s">
-        <v>188</v>
+        <v>129</v>
       </c>
       <c r="J452" s="4" t="s">
-        <v>46</v>
+        <v>347</v>
       </c>
       <c r="K452" s="8">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="L452" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="M452" s="4"/>
+        <v>214</v>
+      </c>
+      <c r="M452" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N452" s="6">
         <v>3</v>
       </c>
@@ -15151,26 +15144,28 @@
         <v>358</v>
       </c>
     </row>
-    <row r="453" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="453" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G453" s="3">
-        <v>45966</v>
+        <v>45973</v>
       </c>
       <c r="H453" s="4" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="I453" s="6" t="s">
-        <v>132</v>
+        <v>359</v>
       </c>
       <c r="J453" s="4" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="K453" s="8">
         <v>170</v>
       </c>
       <c r="L453" s="4" t="s">
-        <v>349</v>
-      </c>
-      <c r="M453" s="4"/>
+        <v>48</v>
+      </c>
+      <c r="M453" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N453" s="6">
         <v>3</v>
       </c>
@@ -15179,43 +15174,45 @@
         <v>358</v>
       </c>
     </row>
-    <row r="454" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="454" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G454" s="3">
-        <v>45967</v>
+        <v>45973</v>
       </c>
       <c r="H454" s="4" t="s">
-        <v>343</v>
+        <v>142</v>
       </c>
       <c r="I454" s="6" t="s">
-        <v>135</v>
+        <v>188</v>
       </c>
       <c r="J454" s="4" t="s">
-        <v>86</v>
+        <v>373</v>
       </c>
       <c r="K454" s="8">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="L454" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="M454" s="4"/>
+        <v>374</v>
+      </c>
+      <c r="M454" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N454" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O454" s="25"/>
       <c r="P454" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="455" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G455" s="3">
-        <v>45967</v>
+        <v>45973</v>
       </c>
       <c r="H455" s="4" t="s">
         <v>146</v>
       </c>
       <c r="I455" s="6" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="J455" s="4" t="s">
         <v>350</v>
@@ -15226,74 +15223,80 @@
       <c r="L455" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="M455" s="4"/>
+      <c r="M455" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N455" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O455" s="25"/>
       <c r="P455" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="456" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G456" s="3">
-        <v>45967</v>
+        <v>45973</v>
       </c>
       <c r="H456" s="4" t="s">
-        <v>337</v>
+        <v>164</v>
       </c>
       <c r="I456" s="6" t="s">
-        <v>129</v>
+        <v>173</v>
       </c>
       <c r="J456" s="4" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="K456" s="8">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="L456" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="M456" s="4"/>
+        <v>372</v>
+      </c>
+      <c r="M456" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N456" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O456" s="25"/>
       <c r="P456" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="457" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G457" s="3">
-        <v>45967</v>
+        <v>45973</v>
       </c>
       <c r="H457" s="4" t="s">
         <v>157</v>
       </c>
       <c r="I457" s="6" t="s">
-        <v>188</v>
+        <v>208</v>
       </c>
       <c r="J457" s="4" t="s">
         <v>42</v>
       </c>
       <c r="K457" s="8">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="L457" s="4" t="s">
         <v>351</v>
       </c>
-      <c r="M457" s="4"/>
+      <c r="M457" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N457" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O457" s="25"/>
       <c r="P457" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="458" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G458" s="3">
-        <v>45967</v>
+        <v>45973</v>
       </c>
       <c r="H458" s="4" t="s">
         <v>141</v>
@@ -15302,471 +15305,530 @@
         <v>132</v>
       </c>
       <c r="J458" s="4" t="s">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="K458" s="8">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="L458" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="M458" s="4"/>
+        <v>22</v>
+      </c>
+      <c r="M458" s="4" t="s">
+        <v>8</v>
+      </c>
       <c r="N458" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O458" s="25"/>
       <c r="P458" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="459" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G459" s="3">
-        <v>45967</v>
-      </c>
-      <c r="H459" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="I459" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="J459" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="K459" s="8">
-        <v>159</v>
-      </c>
-      <c r="L459" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="M459" s="4"/>
-      <c r="N459" s="6"/>
-      <c r="O459" s="25"/>
+    <row r="459" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G459" s="30">
+        <v>45973</v>
+      </c>
+      <c r="H459" s="31" t="s">
+        <v>328</v>
+      </c>
+      <c r="I459" s="29" t="s">
+        <v>135</v>
+      </c>
+      <c r="J459" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="K459" s="32">
+        <v>220</v>
+      </c>
+      <c r="L459" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="M459" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="N459" s="29">
+        <v>3</v>
+      </c>
+      <c r="O459" s="37"/>
       <c r="P459" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="460" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G460" s="3">
-        <v>45967</v>
-      </c>
-      <c r="H460" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="I460" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="J460" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="K460" s="8">
-        <v>240</v>
-      </c>
-      <c r="L460" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="M460" s="4"/>
-      <c r="N460" s="6"/>
-      <c r="O460" s="25"/>
+    <row r="460" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G460" s="45">
+        <v>45973</v>
+      </c>
+      <c r="H460" s="46" t="s">
+        <v>361</v>
+      </c>
+      <c r="I460" s="47"/>
+      <c r="J460" s="46" t="s">
+        <v>65</v>
+      </c>
+      <c r="K460" s="48">
+        <v>100</v>
+      </c>
+      <c r="L460" s="46" t="s">
+        <v>252</v>
+      </c>
+      <c r="M460" s="46" t="s">
+        <v>8</v>
+      </c>
+      <c r="N460" s="47">
+        <v>1</v>
+      </c>
+      <c r="O460" s="49" t="s">
+        <v>251</v>
+      </c>
       <c r="P460" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="461" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G461" s="3">
-        <v>45967</v>
-      </c>
-      <c r="H461" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="I461" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J461" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="K461" s="8">
-        <v>200</v>
-      </c>
-      <c r="L461" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="M461" s="4"/>
-      <c r="N461" s="6"/>
-      <c r="O461" s="25"/>
-      <c r="P461" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="462" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G462" s="3">
-        <v>45967</v>
-      </c>
-      <c r="H462" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="I462" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="J462" s="4" t="s">
-        <v>273</v>
-      </c>
-      <c r="K462" s="8">
-        <v>220</v>
-      </c>
-      <c r="L462" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="M462" s="4"/>
-      <c r="N462" s="6"/>
-      <c r="O462" s="25"/>
-      <c r="P462" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="463" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G463" s="3">
-        <v>45967</v>
-      </c>
-      <c r="H463" s="4" t="s">
+    <row r="461" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="466" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G466" s="3">
+        <v>45972</v>
+      </c>
+      <c r="H466" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="I463" s="6" t="s">
+      <c r="I466" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="J463" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="K463" s="8">
-        <v>200</v>
-      </c>
-      <c r="L463" s="4" t="s">
-        <v>267</v>
-      </c>
-      <c r="M463" s="4"/>
-      <c r="N463" s="6"/>
-      <c r="O463" s="25"/>
-      <c r="P463" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="464" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G464" s="30">
-        <v>45967</v>
-      </c>
-      <c r="H464" s="31" t="s">
-        <v>164</v>
-      </c>
-      <c r="I464" s="29" t="s">
-        <v>173</v>
-      </c>
-      <c r="J464" s="31" t="s">
-        <v>192</v>
-      </c>
-      <c r="K464" s="32">
-        <v>230</v>
-      </c>
-      <c r="L464" s="31" t="s">
-        <v>193</v>
-      </c>
-      <c r="M464" s="31"/>
-      <c r="N464" s="29"/>
-      <c r="O464" s="37"/>
-      <c r="P464" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="465" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G465" s="3">
-        <v>45973</v>
-      </c>
-      <c r="H465" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="I465" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J465" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K465" s="8">
-        <v>180</v>
-      </c>
-      <c r="L465" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="M465" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N465" s="6">
-        <v>3</v>
-      </c>
-      <c r="O465" s="25"/>
-      <c r="P465" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="466" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G466" s="3">
-        <v>45973</v>
-      </c>
-      <c r="H466" s="4" t="s">
-        <v>337</v>
-      </c>
-      <c r="I466" s="6" t="s">
-        <v>129</v>
-      </c>
       <c r="J466" s="4" t="s">
-        <v>347</v>
+        <v>11</v>
       </c>
       <c r="K466" s="8">
         <v>160</v>
       </c>
       <c r="L466" s="4" t="s">
-        <v>214</v>
+        <v>364</v>
       </c>
       <c r="M466" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N466" s="6">
-        <v>3</v>
-      </c>
+      <c r="N466" s="6"/>
       <c r="O466" s="25"/>
       <c r="P466" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="467" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="467" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G467" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H467" s="4" t="s">
-        <v>138</v>
+        <v>158</v>
       </c>
       <c r="I467" s="6" t="s">
-        <v>359</v>
+        <v>122</v>
       </c>
       <c r="J467" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="K467" s="8">
-        <v>170</v>
+        <v>240</v>
       </c>
       <c r="L467" s="4" t="s">
-        <v>48</v>
+        <v>116</v>
       </c>
       <c r="M467" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N467" s="6">
-        <v>3</v>
-      </c>
+      <c r="N467" s="6"/>
       <c r="O467" s="25"/>
       <c r="P467" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="468" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="468" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G468" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H468" s="4" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="I468" s="6" t="s">
-        <v>188</v>
+        <v>134</v>
       </c>
       <c r="J468" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="K468" s="8"/>
-      <c r="L468" s="4"/>
+        <v>163</v>
+      </c>
+      <c r="K468" s="8">
+        <v>220</v>
+      </c>
+      <c r="L468" s="4" t="s">
+        <v>346</v>
+      </c>
       <c r="M468" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N468" s="6">
-        <v>3</v>
-      </c>
+      <c r="N468" s="6"/>
       <c r="O468" s="25"/>
       <c r="P468" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="469" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="469" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G469" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H469" s="4" t="s">
-        <v>197</v>
+        <v>131</v>
       </c>
       <c r="I469" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J469" s="4"/>
-      <c r="K469" s="8"/>
-      <c r="L469" s="4"/>
+        <v>130</v>
+      </c>
+      <c r="J469" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K469" s="8">
+        <v>266</v>
+      </c>
+      <c r="L469" s="4" t="s">
+        <v>365</v>
+      </c>
       <c r="M469" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N469" s="6">
-        <v>3</v>
-      </c>
+      <c r="N469" s="6"/>
       <c r="O469" s="25"/>
       <c r="P469" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="470" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="470" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G470" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H470" s="4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="I470" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J470" s="4"/>
-      <c r="K470" s="8"/>
-      <c r="L470" s="4"/>
+        <v>222</v>
+      </c>
+      <c r="J470" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="K470" s="8">
+        <v>200</v>
+      </c>
+      <c r="L470" s="4" t="s">
+        <v>162</v>
+      </c>
       <c r="M470" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N470" s="6">
-        <v>2</v>
-      </c>
+      <c r="N470" s="6"/>
       <c r="O470" s="25"/>
       <c r="P470" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="471" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="471" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G471" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H471" s="4" t="s">
-        <v>164</v>
+        <v>245</v>
       </c>
       <c r="I471" s="6" t="s">
-        <v>173</v>
+        <v>360</v>
       </c>
       <c r="J471" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K471" s="8"/>
-      <c r="L471" s="4"/>
+        <v>342</v>
+      </c>
+      <c r="K471" s="8">
+        <v>280</v>
+      </c>
+      <c r="L471" s="4" t="s">
+        <v>259</v>
+      </c>
       <c r="M471" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N471" s="6">
-        <v>3</v>
-      </c>
+      <c r="N471" s="6"/>
       <c r="O471" s="25"/>
       <c r="P471" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="472" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="472" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G472" s="3">
-        <v>45973</v>
+        <v>45972</v>
       </c>
       <c r="H472" s="4" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="I472" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="J472" s="4"/>
-      <c r="K472" s="8"/>
-      <c r="L472" s="4"/>
+        <v>129</v>
+      </c>
+      <c r="J472" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K472" s="8">
+        <v>160</v>
+      </c>
+      <c r="L472" s="4" t="s">
+        <v>338</v>
+      </c>
       <c r="M472" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="N472" s="6">
-        <v>3</v>
-      </c>
+      <c r="N472" s="6"/>
       <c r="O472" s="25"/>
       <c r="P472" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="473" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G473" s="3">
-        <v>45973</v>
-      </c>
-      <c r="H473" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="I473" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="J473" s="4"/>
-      <c r="K473" s="8"/>
-      <c r="L473" s="4"/>
-      <c r="M473" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N473" s="6">
-        <v>3</v>
-      </c>
-      <c r="O473" s="25"/>
-      <c r="P473" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="474" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G474" s="3">
-        <v>45973</v>
-      </c>
-      <c r="H474" s="4" t="s">
+    <row r="473" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G473" s="17">
+        <v>45972</v>
+      </c>
+      <c r="H473" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="I473" s="19"/>
+      <c r="J473" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="K473" s="20">
+        <v>110</v>
+      </c>
+      <c r="L473" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="M473" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="N473" s="19"/>
+      <c r="O473" s="41" t="s">
+        <v>251</v>
+      </c>
+      <c r="P473" s="38" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="474" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G474" s="17">
+        <v>45972</v>
+      </c>
+      <c r="H474" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="I474" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="J474" s="18" t="s">
+        <v>366</v>
+      </c>
+      <c r="K474" s="20">
+        <v>180</v>
+      </c>
+      <c r="L474" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="M474" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="N474" s="19"/>
+      <c r="O474" s="41" t="s">
+        <v>251</v>
+      </c>
+      <c r="P474" s="38" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="475" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G475" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H475" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I475" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J475" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="K475" s="8">
+        <v>150</v>
+      </c>
+      <c r="L475" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="M475" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N475" s="6"/>
+      <c r="O475" s="25"/>
+      <c r="P475" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="476" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G476" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H476" s="4" t="s">
+        <v>368</v>
+      </c>
+      <c r="I476" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="J476" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="K476" s="8">
+        <v>159</v>
+      </c>
+      <c r="L476" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="M476" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N476" s="6"/>
+      <c r="O476" s="25"/>
+      <c r="P476" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="477" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G477" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H477" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I477" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J477" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K477" s="8">
+        <v>170</v>
+      </c>
+      <c r="L477" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M477" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N477" s="6"/>
+      <c r="O477" s="25"/>
+      <c r="P477" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="478" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G478" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H478" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="I478" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J478" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="K478" s="8">
+        <v>220</v>
+      </c>
+      <c r="L478" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="M478" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N478" s="6"/>
+      <c r="O478" s="25"/>
+      <c r="P478" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="479" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G479" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H479" s="4" t="s">
         <v>328</v>
       </c>
-      <c r="I474" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J474" s="4" t="s">
+      <c r="I479" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="J479" s="4" t="s">
         <v>229</v>
       </c>
-      <c r="K474" s="8">
+      <c r="K479" s="8">
         <v>220</v>
       </c>
-      <c r="L474" s="4" t="s">
+      <c r="L479" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="M474" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N474" s="6">
-        <v>3</v>
-      </c>
-      <c r="O474" s="25"/>
-      <c r="P474" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="475" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="476" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="477" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="478" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="479" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="480" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+      <c r="M479" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N479" s="6"/>
+      <c r="O479" s="25"/>
+      <c r="P479" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="480" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G480" s="3">
+        <v>45971</v>
+      </c>
+      <c r="H480" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="I480" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J480" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K480" s="8">
+        <v>180</v>
+      </c>
+      <c r="L480" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M480" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N480" s="6"/>
+      <c r="O480" s="25"/>
+      <c r="P480" t="s">
+        <v>358</v>
+      </c>
+    </row>
     <row r="481" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G481" s="3">
-        <v>45972</v>
+        <v>45971</v>
       </c>
       <c r="H481" s="4" t="s">
-        <v>329</v>
+        <v>152</v>
       </c>
       <c r="I481" s="6" t="s">
-        <v>136</v>
+        <v>216</v>
       </c>
       <c r="J481" s="4" t="s">
-        <v>11</v>
+        <v>332</v>
       </c>
       <c r="K481" s="8">
-        <v>160</v>
+        <v>215</v>
       </c>
       <c r="L481" s="4" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="M481" s="4" t="s">
         <v>8</v>
@@ -15777,593 +15839,172 @@
         <v>358</v>
       </c>
     </row>
-    <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G482" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H482" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="I482" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="J482" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="K482" s="8">
-        <v>240</v>
-      </c>
-      <c r="L482" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="M482" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N482" s="6"/>
-      <c r="O482" s="25"/>
-      <c r="P482" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="483" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G483" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H483" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="I483" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J483" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="K483" s="8">
-        <v>220</v>
-      </c>
-      <c r="L483" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="M483" s="4" t="s">
-        <v>8</v>
-      </c>
+    <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="483" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G483" s="4"/>
+      <c r="H483" s="4"/>
+      <c r="I483" s="6"/>
+      <c r="J483" s="4"/>
+      <c r="K483" s="8"/>
+      <c r="L483" s="4"/>
+      <c r="M483" s="4"/>
       <c r="N483" s="6"/>
       <c r="O483" s="25"/>
-      <c r="P483" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="484" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G484" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H484" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="I484" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="J484" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="K484" s="8">
-        <v>266</v>
-      </c>
-      <c r="L484" s="4" t="s">
-        <v>365</v>
-      </c>
-      <c r="M484" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P483" s="6"/>
+    </row>
+    <row r="484" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G484" s="4"/>
+      <c r="H484" s="4"/>
+      <c r="I484" s="6"/>
+      <c r="J484" s="4"/>
+      <c r="K484" s="8"/>
+      <c r="L484" s="4"/>
+      <c r="M484" s="4"/>
       <c r="N484" s="6"/>
       <c r="O484" s="25"/>
-      <c r="P484" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="485" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G485" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H485" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I485" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="J485" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="K485" s="8">
-        <v>200</v>
-      </c>
-      <c r="L485" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="M485" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N485" s="6"/>
-      <c r="O485" s="25"/>
-      <c r="P485" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="486" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G486" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H486" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="I486" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="J486" s="4" t="s">
-        <v>342</v>
-      </c>
-      <c r="K486" s="8">
-        <v>280</v>
-      </c>
-      <c r="L486" s="4" t="s">
-        <v>259</v>
-      </c>
-      <c r="M486" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P484" s="6"/>
+    </row>
+    <row r="485" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G485" s="42"/>
+      <c r="H485" s="42"/>
+      <c r="I485" s="28"/>
+      <c r="J485" s="42"/>
+      <c r="K485" s="43"/>
+      <c r="L485" s="42"/>
+      <c r="M485" s="42"/>
+      <c r="N485" s="28"/>
+      <c r="O485" s="44"/>
+      <c r="P485" s="28"/>
+    </row>
+    <row r="486" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G486" s="4"/>
+      <c r="H486" s="4"/>
+      <c r="I486" s="6"/>
+      <c r="J486" s="4"/>
+      <c r="K486" s="8"/>
+      <c r="L486" s="4"/>
+      <c r="M486" s="4"/>
       <c r="N486" s="6"/>
       <c r="O486" s="25"/>
-      <c r="P486" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="487" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G487" s="3">
-        <v>45972</v>
-      </c>
-      <c r="H487" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="I487" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J487" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K487" s="8">
-        <v>160</v>
-      </c>
-      <c r="L487" s="4" t="s">
-        <v>338</v>
-      </c>
-      <c r="M487" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P486" s="6"/>
+    </row>
+    <row r="487" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G487" s="4"/>
+      <c r="H487" s="4"/>
+      <c r="I487" s="6"/>
+      <c r="J487" s="4"/>
+      <c r="K487" s="8"/>
+      <c r="L487" s="4"/>
+      <c r="M487" s="4"/>
       <c r="N487" s="6"/>
       <c r="O487" s="25"/>
-      <c r="P487" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="488" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G488" s="17">
-        <v>45972</v>
-      </c>
-      <c r="H488" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="I488" s="19"/>
-      <c r="J488" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="K488" s="20">
-        <v>110</v>
-      </c>
-      <c r="L488" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="M488" s="18" t="s">
-        <v>7</v>
-      </c>
-      <c r="N488" s="19"/>
-      <c r="O488" s="41" t="s">
-        <v>251</v>
-      </c>
-      <c r="P488" s="38" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="489" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G489" s="17">
-        <v>45972</v>
-      </c>
-      <c r="H489" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="I489" s="19" t="s">
-        <v>175</v>
-      </c>
-      <c r="J489" s="18" t="s">
-        <v>366</v>
-      </c>
-      <c r="K489" s="20">
-        <v>180</v>
-      </c>
-      <c r="L489" s="18" t="s">
-        <v>367</v>
-      </c>
-      <c r="M489" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="N489" s="19"/>
-      <c r="O489" s="41" t="s">
-        <v>251</v>
-      </c>
-      <c r="P489" s="38" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="490" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G490" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H490" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="I490" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J490" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="K490" s="8">
-        <v>150</v>
-      </c>
-      <c r="L490" s="4" t="s">
-        <v>370</v>
-      </c>
-      <c r="M490" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P487" s="6"/>
+    </row>
+    <row r="488" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G488" s="4"/>
+      <c r="H488" s="4"/>
+      <c r="I488" s="6"/>
+      <c r="J488" s="4"/>
+      <c r="K488" s="8"/>
+      <c r="L488" s="4"/>
+      <c r="M488" s="4"/>
+      <c r="N488" s="6"/>
+      <c r="O488" s="25"/>
+      <c r="P488" s="6"/>
+    </row>
+    <row r="489" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G489" s="4"/>
+      <c r="H489" s="4"/>
+      <c r="I489" s="6"/>
+      <c r="J489" s="4"/>
+      <c r="K489" s="8"/>
+      <c r="L489" s="4"/>
+      <c r="M489" s="4"/>
+      <c r="N489" s="6"/>
+      <c r="O489" s="25"/>
+      <c r="P489" s="6"/>
+    </row>
+    <row r="490" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G490" s="4"/>
+      <c r="H490" s="4"/>
+      <c r="I490" s="6"/>
+      <c r="J490" s="4"/>
+      <c r="K490" s="8"/>
+      <c r="L490" s="4"/>
+      <c r="M490" s="4"/>
       <c r="N490" s="6"/>
       <c r="O490" s="25"/>
-      <c r="P490" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="491" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G491" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H491" s="4" t="s">
-        <v>368</v>
-      </c>
-      <c r="I491" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="J491" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="K491" s="8">
-        <v>159</v>
-      </c>
-      <c r="L491" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="M491" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P490" s="6"/>
+    </row>
+    <row r="491" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G491" s="4"/>
+      <c r="H491" s="4"/>
+      <c r="I491" s="6"/>
+      <c r="J491" s="4"/>
+      <c r="K491" s="8"/>
+      <c r="L491" s="4"/>
+      <c r="M491" s="4"/>
       <c r="N491" s="6"/>
       <c r="O491" s="25"/>
-      <c r="P491" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="492" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G492" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H492" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="I492" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="J492" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K492" s="8">
-        <v>170</v>
-      </c>
-      <c r="L492" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="M492" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P491" s="6"/>
+    </row>
+    <row r="492" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G492" s="4"/>
+      <c r="H492" s="4"/>
+      <c r="I492" s="6"/>
+      <c r="J492" s="4"/>
+      <c r="K492" s="8"/>
+      <c r="L492" s="4"/>
+      <c r="M492" s="4"/>
       <c r="N492" s="6"/>
       <c r="O492" s="25"/>
-      <c r="P492" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="493" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G493" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H493" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="I493" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="J493" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="K493" s="8">
-        <v>220</v>
-      </c>
-      <c r="L493" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M493" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P492" s="6"/>
+    </row>
+    <row r="493" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G493" s="4"/>
+      <c r="H493" s="4"/>
+      <c r="I493" s="6"/>
+      <c r="J493" s="4"/>
+      <c r="K493" s="8"/>
+      <c r="L493" s="4"/>
+      <c r="M493" s="4"/>
       <c r="N493" s="6"/>
       <c r="O493" s="25"/>
-      <c r="P493" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="494" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G494" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H494" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="I494" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="J494" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="K494" s="8">
-        <v>220</v>
-      </c>
-      <c r="L494" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="M494" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P493" s="6"/>
+    </row>
+    <row r="494" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G494" s="4"/>
+      <c r="H494" s="4"/>
+      <c r="I494" s="6"/>
+      <c r="J494" s="4"/>
+      <c r="K494" s="8"/>
+      <c r="L494" s="4"/>
+      <c r="M494" s="4"/>
       <c r="N494" s="6"/>
       <c r="O494" s="25"/>
-      <c r="P494" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="495" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G495" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H495" s="4" t="s">
-        <v>369</v>
-      </c>
-      <c r="I495" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J495" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K495" s="8">
-        <v>180</v>
-      </c>
-      <c r="L495" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="M495" s="4" t="s">
-        <v>8</v>
-      </c>
+      <c r="P494" s="6"/>
+    </row>
+    <row r="495" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G495" s="4"/>
+      <c r="H495" s="4"/>
+      <c r="I495" s="6"/>
+      <c r="J495" s="4"/>
+      <c r="K495" s="8"/>
+      <c r="L495" s="4"/>
+      <c r="M495" s="4"/>
       <c r="N495" s="6"/>
       <c r="O495" s="25"/>
-      <c r="P495" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="496" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G496" s="3">
-        <v>45971</v>
-      </c>
-      <c r="H496" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="I496" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="J496" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="K496" s="8">
-        <v>215</v>
-      </c>
-      <c r="L496" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="M496" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N496" s="6"/>
-      <c r="O496" s="25"/>
-      <c r="P496" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="497" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G497" s="3"/>
-      <c r="H497" s="4"/>
-      <c r="I497" s="6"/>
-      <c r="J497" s="4"/>
-      <c r="K497" s="8"/>
-      <c r="L497" s="4"/>
-      <c r="M497" s="4"/>
-      <c r="N497" s="6"/>
-      <c r="O497" s="25"/>
-      <c r="P497" s="6"/>
-    </row>
-    <row r="498" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G498" s="4"/>
-      <c r="H498" s="4"/>
-      <c r="I498" s="6"/>
-      <c r="J498" s="4"/>
-      <c r="K498" s="8"/>
-      <c r="L498" s="4"/>
-      <c r="M498" s="4"/>
-      <c r="N498" s="6"/>
-      <c r="O498" s="25"/>
-      <c r="P498" s="6"/>
-    </row>
-    <row r="499" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G499" s="4"/>
-      <c r="H499" s="4"/>
-      <c r="I499" s="6"/>
-      <c r="J499" s="4"/>
-      <c r="K499" s="8"/>
-      <c r="L499" s="4"/>
-      <c r="M499" s="4"/>
-      <c r="N499" s="6"/>
-      <c r="O499" s="25"/>
-      <c r="P499" s="6"/>
-    </row>
-    <row r="500" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G500" s="4"/>
-      <c r="H500" s="4"/>
-      <c r="I500" s="6"/>
-      <c r="J500" s="4"/>
-      <c r="K500" s="8"/>
-      <c r="L500" s="4"/>
-      <c r="M500" s="4"/>
-      <c r="N500" s="6"/>
-      <c r="O500" s="25"/>
-      <c r="P500" s="6"/>
-    </row>
-    <row r="501" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G501" s="4"/>
-      <c r="H501" s="4"/>
-      <c r="I501" s="6"/>
-      <c r="J501" s="4"/>
-      <c r="K501" s="8"/>
-      <c r="L501" s="4"/>
-      <c r="M501" s="4"/>
-      <c r="N501" s="6"/>
-      <c r="O501" s="25"/>
-      <c r="P501" s="6"/>
-    </row>
-    <row r="502" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G502" s="4"/>
-      <c r="H502" s="4"/>
-      <c r="I502" s="6"/>
-      <c r="J502" s="4"/>
-      <c r="K502" s="8"/>
-      <c r="L502" s="4"/>
-      <c r="M502" s="4"/>
-      <c r="N502" s="6"/>
-      <c r="O502" s="25"/>
-      <c r="P502" s="6"/>
-    </row>
-    <row r="503" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G503" s="4"/>
-      <c r="H503" s="4"/>
-      <c r="I503" s="6"/>
-      <c r="J503" s="4"/>
-      <c r="K503" s="8"/>
-      <c r="L503" s="4"/>
-      <c r="M503" s="4"/>
-      <c r="N503" s="6"/>
-      <c r="O503" s="25"/>
-      <c r="P503" s="6"/>
-    </row>
-    <row r="504" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G504" s="4"/>
-      <c r="H504" s="4"/>
-      <c r="I504" s="6"/>
-      <c r="J504" s="4"/>
-      <c r="K504" s="8"/>
-      <c r="L504" s="4"/>
-      <c r="M504" s="4"/>
-      <c r="N504" s="6"/>
-      <c r="O504" s="25"/>
-      <c r="P504" s="6"/>
-    </row>
-    <row r="505" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G505" s="4"/>
-      <c r="H505" s="4"/>
-      <c r="I505" s="6"/>
-      <c r="J505" s="4"/>
-      <c r="K505" s="8"/>
-      <c r="L505" s="4"/>
-      <c r="M505" s="4"/>
-      <c r="N505" s="6"/>
-      <c r="O505" s="25"/>
-      <c r="P505" s="6"/>
-    </row>
-    <row r="506" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G506" s="4"/>
-      <c r="H506" s="4"/>
-      <c r="I506" s="6"/>
-      <c r="J506" s="4"/>
-      <c r="K506" s="8"/>
-      <c r="L506" s="4"/>
-      <c r="M506" s="4"/>
-      <c r="N506" s="6"/>
-      <c r="O506" s="25"/>
-      <c r="P506" s="6"/>
-    </row>
-    <row r="507" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G507" s="4"/>
-      <c r="H507" s="4"/>
-      <c r="I507" s="6"/>
-      <c r="J507" s="4"/>
-      <c r="K507" s="8"/>
-      <c r="L507" s="4"/>
-      <c r="M507" s="4"/>
-      <c r="N507" s="6"/>
-      <c r="O507" s="25"/>
-      <c r="P507" s="6"/>
-    </row>
-    <row r="508" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G508" s="4"/>
-      <c r="H508" s="4"/>
-      <c r="I508" s="6"/>
-      <c r="J508" s="4"/>
-      <c r="K508" s="8"/>
-      <c r="L508" s="4"/>
-      <c r="M508" s="4"/>
-      <c r="N508" s="6"/>
-      <c r="O508" s="25"/>
-      <c r="P508" s="6"/>
-    </row>
-    <row r="509" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G509" s="4"/>
-      <c r="H509" s="4"/>
-      <c r="I509" s="6"/>
-      <c r="J509" s="4"/>
-      <c r="K509" s="8"/>
-      <c r="L509" s="4"/>
-      <c r="M509" s="4"/>
-      <c r="N509" s="6"/>
-      <c r="O509" s="25"/>
-      <c r="P509" s="6"/>
+      <c r="P495" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O496" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O482" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2025" month="11" day="12" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O437">
-      <sortCondition ref="G5:G437"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
+      <sortCondition ref="G5:G431"/>
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G6:N339">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-14  9:10
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="926" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FA197BF-71D0-4A41-8E1D-E322392815E6}"/>
+  <xr:revisionPtr revIDLastSave="1017" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBFD530D-67CB-4D10-A3D9-714120DAB40F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$482</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$495</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2954" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3021" uniqueCount="387">
   <si>
     <t>DATA</t>
   </si>
@@ -1164,6 +1164,42 @@
   </si>
   <si>
     <t>HOTEL CABANA</t>
+  </si>
+  <si>
+    <t>PEDRO</t>
+  </si>
+  <si>
+    <t>MARCOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRISTIANO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">POUSADA RESIDENCIAL </t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>HOTEL STELATI</t>
+  </si>
+  <si>
+    <t>Jaguariúna, SP</t>
+  </si>
+  <si>
+    <t>TRES MARIAS</t>
+  </si>
+  <si>
+    <t>POUSADA AMERICA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ITBIRA </t>
+  </si>
+  <si>
+    <t>HOTEL CHACARÁ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POUSADA PADRE CICERO </t>
   </si>
 </sst>
 </file>
@@ -1310,7 +1346,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1429,6 +1465,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -1768,7 +1805,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P495"/>
+  <dimension ref="G5:P498"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -15084,7 +15121,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="451" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="451" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G451" s="3">
         <v>45973</v>
       </c>
@@ -15114,7 +15151,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="452" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="452" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G452" s="3">
         <v>45973</v>
       </c>
@@ -15144,7 +15181,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="453" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="453" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G453" s="3">
         <v>45973</v>
       </c>
@@ -15174,7 +15211,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="454" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="454" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G454" s="3">
         <v>45973</v>
       </c>
@@ -15204,7 +15241,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="455" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="455" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G455" s="3">
         <v>45973</v>
       </c>
@@ -15234,7 +15271,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="456" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="456" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G456" s="3">
         <v>45973</v>
       </c>
@@ -15264,7 +15301,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="457" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="457" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G457" s="3">
         <v>45973</v>
       </c>
@@ -15294,7 +15331,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="458" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="458" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G458" s="3">
         <v>45973</v>
       </c>
@@ -15324,7 +15361,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="459" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="459" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G459" s="30">
         <v>45973</v>
       </c>
@@ -15354,7 +15391,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="460" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="460" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G460" s="45">
         <v>45973</v>
       </c>
@@ -15841,166 +15878,414 @@
     </row>
     <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="483" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G483" s="4"/>
-      <c r="H483" s="4"/>
-      <c r="I483" s="6"/>
-      <c r="J483" s="4"/>
-      <c r="K483" s="8"/>
-      <c r="L483" s="4"/>
+      <c r="G483" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H483" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I483" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J483" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="K483" s="8">
+        <v>150</v>
+      </c>
+      <c r="L483" s="4" t="s">
+        <v>383</v>
+      </c>
       <c r="M483" s="4"/>
-      <c r="N483" s="6"/>
+      <c r="N483" s="6">
+        <v>2</v>
+      </c>
       <c r="O483" s="25"/>
-      <c r="P483" s="6"/>
+      <c r="P483" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="484" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G484" s="4"/>
-      <c r="H484" s="4"/>
-      <c r="I484" s="6"/>
-      <c r="J484" s="4"/>
-      <c r="K484" s="8"/>
-      <c r="L484" s="4"/>
-      <c r="M484" s="4"/>
-      <c r="N484" s="6"/>
+      <c r="G484" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H484" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I484" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J484" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K484" s="8">
+        <v>180</v>
+      </c>
+      <c r="L484" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="M484" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="N484" s="6">
+        <v>2</v>
+      </c>
       <c r="O484" s="25"/>
-      <c r="P484" s="6"/>
+      <c r="P484" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="485" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G485" s="42"/>
-      <c r="H485" s="42"/>
-      <c r="I485" s="28"/>
-      <c r="J485" s="42"/>
-      <c r="K485" s="43"/>
-      <c r="L485" s="42"/>
+      <c r="G485" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H485" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="I485" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="J485" s="42" t="s">
+        <v>46</v>
+      </c>
+      <c r="K485" s="43">
+        <v>170</v>
+      </c>
+      <c r="L485" s="42" t="s">
+        <v>48</v>
+      </c>
       <c r="M485" s="42"/>
-      <c r="N485" s="28"/>
+      <c r="N485" s="6">
+        <v>2</v>
+      </c>
       <c r="O485" s="44"/>
-      <c r="P485" s="28"/>
+      <c r="P485" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="486" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G486" s="4"/>
-      <c r="H486" s="4"/>
-      <c r="I486" s="6"/>
-      <c r="J486" s="4"/>
-      <c r="K486" s="8"/>
-      <c r="L486" s="4"/>
+      <c r="G486" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H486" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I486" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="J486" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="K486" s="8">
+        <v>160</v>
+      </c>
+      <c r="L486" s="4" t="s">
+        <v>365</v>
+      </c>
       <c r="M486" s="4"/>
-      <c r="N486" s="6"/>
+      <c r="N486" s="6">
+        <v>2</v>
+      </c>
       <c r="O486" s="25"/>
-      <c r="P486" s="6"/>
+      <c r="P486" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="487" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G487" s="4"/>
-      <c r="H487" s="4"/>
-      <c r="I487" s="6"/>
-      <c r="J487" s="4"/>
-      <c r="K487" s="8"/>
-      <c r="L487" s="4"/>
+      <c r="G487" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H487" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I487" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J487" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="K487" s="8">
+        <v>230</v>
+      </c>
+      <c r="L487" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="M487" s="4"/>
-      <c r="N487" s="6"/>
+      <c r="N487" s="6">
+        <v>2</v>
+      </c>
       <c r="O487" s="25"/>
-      <c r="P487" s="6"/>
+      <c r="P487" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="488" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G488" s="4"/>
-      <c r="H488" s="4"/>
-      <c r="I488" s="6"/>
-      <c r="J488" s="4"/>
-      <c r="K488" s="8"/>
-      <c r="L488" s="4"/>
+      <c r="G488" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H488" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I488" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="J488" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="K488" s="8">
+        <v>180</v>
+      </c>
+      <c r="L488" s="4" t="s">
+        <v>386</v>
+      </c>
       <c r="M488" s="4"/>
-      <c r="N488" s="6"/>
+      <c r="N488" s="6">
+        <v>2</v>
+      </c>
       <c r="O488" s="25"/>
-      <c r="P488" s="6"/>
+      <c r="P488" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="489" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G489" s="4"/>
-      <c r="H489" s="4"/>
-      <c r="I489" s="6"/>
-      <c r="J489" s="4"/>
-      <c r="K489" s="8"/>
-      <c r="L489" s="4"/>
+      <c r="G489" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H489" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I489" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J489" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K489" s="8">
+        <v>200</v>
+      </c>
+      <c r="L489" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="M489" s="4"/>
-      <c r="N489" s="6"/>
+      <c r="N489" s="6">
+        <v>2</v>
+      </c>
       <c r="O489" s="25"/>
-      <c r="P489" s="6"/>
+      <c r="P489" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="490" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G490" s="4"/>
-      <c r="H490" s="4"/>
-      <c r="I490" s="6"/>
-      <c r="J490" s="4"/>
-      <c r="K490" s="8"/>
-      <c r="L490" s="4"/>
+      <c r="G490" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H490" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="I490" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J490" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K490" s="8">
+        <v>159</v>
+      </c>
+      <c r="L490" s="4" t="s">
+        <v>89</v>
+      </c>
       <c r="M490" s="4"/>
-      <c r="N490" s="6"/>
+      <c r="N490" s="6">
+        <v>2</v>
+      </c>
       <c r="O490" s="25"/>
-      <c r="P490" s="6"/>
+      <c r="P490" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="491" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G491" s="4"/>
-      <c r="H491" s="4"/>
-      <c r="I491" s="6"/>
-      <c r="J491" s="4"/>
-      <c r="K491" s="8"/>
-      <c r="L491" s="4"/>
+      <c r="G491" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H491" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I491" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="J491" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K491" s="8">
+        <v>240</v>
+      </c>
+      <c r="L491" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="M491" s="4"/>
-      <c r="N491" s="6"/>
+      <c r="N491" s="6">
+        <v>2</v>
+      </c>
       <c r="O491" s="25"/>
-      <c r="P491" s="6"/>
+      <c r="P491" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="492" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G492" s="4"/>
-      <c r="H492" s="4"/>
-      <c r="I492" s="6"/>
-      <c r="J492" s="4"/>
-      <c r="K492" s="8"/>
-      <c r="L492" s="4"/>
+      <c r="G492" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H492" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I492" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="J492" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="K492" s="10">
+        <v>180</v>
+      </c>
+      <c r="L492" s="4" t="s">
+        <v>241</v>
+      </c>
       <c r="M492" s="4"/>
-      <c r="N492" s="6"/>
+      <c r="N492" s="6">
+        <v>2</v>
+      </c>
       <c r="O492" s="25"/>
-      <c r="P492" s="6"/>
+      <c r="P492" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="493" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G493" s="4"/>
-      <c r="H493" s="4"/>
-      <c r="I493" s="6"/>
-      <c r="J493" s="4"/>
-      <c r="K493" s="8"/>
-      <c r="L493" s="4"/>
+      <c r="G493" s="30">
+        <v>45974</v>
+      </c>
+      <c r="H493" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="I493" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="J493" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="K493" s="8">
+        <v>200</v>
+      </c>
+      <c r="L493" s="4" t="s">
+        <v>385</v>
+      </c>
       <c r="M493" s="4"/>
-      <c r="N493" s="6"/>
+      <c r="N493" s="6">
+        <v>2</v>
+      </c>
       <c r="O493" s="25"/>
-      <c r="P493" s="6"/>
+      <c r="P493" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="494" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G494" s="4"/>
-      <c r="H494" s="4"/>
-      <c r="I494" s="6"/>
-      <c r="J494" s="4"/>
-      <c r="K494" s="8"/>
-      <c r="L494" s="4"/>
-      <c r="M494" s="4"/>
-      <c r="N494" s="6"/>
-      <c r="O494" s="25"/>
-      <c r="P494" s="6"/>
+      <c r="G494" s="45">
+        <v>45974</v>
+      </c>
+      <c r="H494" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="I494" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="J494" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="K494" s="20">
+        <v>255</v>
+      </c>
+      <c r="L494" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="M494" s="18"/>
+      <c r="N494" s="19">
+        <v>2</v>
+      </c>
+      <c r="O494" s="41" t="s">
+        <v>251</v>
+      </c>
+      <c r="P494" s="19" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="495" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G495" s="4"/>
-      <c r="H495" s="4"/>
-      <c r="I495" s="6"/>
-      <c r="J495" s="4"/>
-      <c r="K495" s="8"/>
-      <c r="L495" s="4"/>
+      <c r="G495" s="3">
+        <v>45974</v>
+      </c>
+      <c r="H495" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I495" s="50" t="s">
+        <v>216</v>
+      </c>
+      <c r="J495" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="K495" s="8">
+        <v>220</v>
+      </c>
+      <c r="L495" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="M495" s="4"/>
-      <c r="N495" s="6"/>
+      <c r="N495" s="6">
+        <v>2</v>
+      </c>
       <c r="O495" s="25"/>
-      <c r="P495" s="6"/>
+      <c r="P495" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="496" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G496" s="4"/>
+      <c r="H496" s="4"/>
+      <c r="I496" s="6"/>
+      <c r="J496" s="4"/>
+      <c r="K496" s="8"/>
+      <c r="L496" s="4"/>
+      <c r="M496" s="4"/>
+      <c r="N496" s="6"/>
+      <c r="O496" s="25"/>
+      <c r="P496" s="6"/>
+    </row>
+    <row r="497" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G497" s="3"/>
+      <c r="H497" s="4"/>
+      <c r="I497" s="6"/>
+      <c r="J497" s="4"/>
+      <c r="K497" s="8"/>
+      <c r="L497" s="4"/>
+      <c r="M497" s="4"/>
+      <c r="N497" s="6"/>
+      <c r="O497" s="25"/>
+      <c r="P497" s="6"/>
+    </row>
+    <row r="498" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G498" s="4"/>
+      <c r="H498" s="4"/>
+      <c r="I498" s="6"/>
+      <c r="J498" s="4"/>
+      <c r="K498" s="8"/>
+      <c r="L498" s="4"/>
+      <c r="M498" s="4"/>
+      <c r="N498" s="6"/>
+      <c r="O498" s="25"/>
+      <c r="P498" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O482" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O496" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="12" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="13" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
@@ -16011,7 +16296,7 @@
     <sortCondition ref="G6:G339"/>
   </sortState>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="39" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-14 10:39
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1017" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBFD530D-67CB-4D10-A3D9-714120DAB40F}"/>
+  <xr:revisionPtr revIDLastSave="1018" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78E4521E-4E7C-4665-BBFD-824294B8D2C4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$495</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$496</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -1346,7 +1346,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1465,7 +1465,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -14825,7 +14824,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="440" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="440" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G440" s="3">
         <v>45967</v>
       </c>
@@ -14853,7 +14852,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="441" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="441" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G441" s="3">
         <v>45967</v>
       </c>
@@ -14881,7 +14880,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="442" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="442" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G442" s="3">
         <v>45967</v>
       </c>
@@ -14909,7 +14908,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="443" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="443" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G443" s="3">
         <v>45967</v>
       </c>
@@ -14937,7 +14936,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="444" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="444" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G444" s="3">
         <v>45967</v>
       </c>
@@ -14965,7 +14964,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="445" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="445" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G445" s="3">
         <v>45967</v>
       </c>
@@ -14991,7 +14990,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="446" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="446" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G446" s="3">
         <v>45967</v>
       </c>
@@ -15017,7 +15016,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="447" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="447" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G447" s="3">
         <v>45967</v>
       </c>
@@ -15043,7 +15042,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="448" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="448" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G448" s="3">
         <v>45967</v>
       </c>
@@ -15069,7 +15068,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="449" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="449" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G449" s="3">
         <v>45967</v>
       </c>
@@ -15095,7 +15094,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="450" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="450" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G450" s="30">
         <v>45967</v>
       </c>
@@ -16224,7 +16223,7 @@
       <c r="H495" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="I495" s="50" t="s">
+      <c r="I495" s="6" t="s">
         <v>216</v>
       </c>
       <c r="J495" s="4" t="s">
@@ -16245,7 +16244,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="496" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="496" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G496" s="4"/>
       <c r="H496" s="4"/>
       <c r="I496" s="6"/>
@@ -16285,6 +16284,7 @@
   <autoFilter ref="G5:O496" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
+        <dateGroupItem year="2025" month="11" day="6" dateTimeGrouping="day"/>
         <dateGroupItem year="2025" month="11" day="13" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-19 17:32
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1018" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78E4521E-4E7C-4665-BBFD-824294B8D2C4}"/>
+  <xr:revisionPtr revIDLastSave="1274" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACE9DC15-78EC-43F8-9B35-2AD03F257109}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$496</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$521</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3021" uniqueCount="387">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3162" uniqueCount="409">
   <si>
     <t>DATA</t>
   </si>
@@ -1200,6 +1200,72 @@
   </si>
   <si>
     <t xml:space="preserve">POUSADA PADRE CICERO </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PAULO </t>
+  </si>
+  <si>
+    <t>EDR</t>
+  </si>
+  <si>
+    <t>MATEUS SE</t>
+  </si>
+  <si>
+    <t>LUCAS</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MARLON</t>
+  </si>
+  <si>
+    <t>DOUGLAS RO</t>
+  </si>
+  <si>
+    <t>DOUGLAS.A</t>
+  </si>
+  <si>
+    <t>GUNHAES</t>
+  </si>
+  <si>
+    <t>POUSADA SANTOS DRUMMONT</t>
+  </si>
+  <si>
+    <t>MORADA NOVA</t>
+  </si>
+  <si>
+    <t>HOTEL MARAJA</t>
+  </si>
+  <si>
+    <t>POUSADA VILLA DA SERRA</t>
+  </si>
+  <si>
+    <t>MARIO CAMPOS</t>
+  </si>
+  <si>
+    <t>DIONISIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FRANCIS </t>
+  </si>
+  <si>
+    <t>JOÃO</t>
+  </si>
+  <si>
+    <t>PONTE NOVA</t>
+  </si>
+  <si>
+    <t>HOTEL PARAISO</t>
+  </si>
+  <si>
+    <t>AGUAS CLARAS</t>
+  </si>
+  <si>
+    <t>HOTEL CARMEN VIEIRA</t>
+  </si>
+  <si>
+    <t>carmo do paranaiba</t>
+  </si>
+  <si>
+    <t>carmo palace</t>
   </si>
 </sst>
 </file>
@@ -1804,7 +1870,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P498"/>
+  <dimension ref="G5:P522"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -14824,7 +14890,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="440" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="440" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G440" s="3">
         <v>45967</v>
       </c>
@@ -14852,7 +14918,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="441" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="441" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G441" s="3">
         <v>45967</v>
       </c>
@@ -14880,7 +14946,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="442" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="442" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G442" s="3">
         <v>45967</v>
       </c>
@@ -14908,7 +14974,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="443" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="443" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G443" s="3">
         <v>45967</v>
       </c>
@@ -14936,7 +15002,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="444" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="444" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G444" s="3">
         <v>45967</v>
       </c>
@@ -14964,7 +15030,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="445" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="445" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G445" s="3">
         <v>45967</v>
       </c>
@@ -14990,7 +15056,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="446" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="446" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G446" s="3">
         <v>45967</v>
       </c>
@@ -15016,7 +15082,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="447" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="447" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G447" s="3">
         <v>45967</v>
       </c>
@@ -15042,7 +15108,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="448" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="448" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G448" s="3">
         <v>45967</v>
       </c>
@@ -15068,7 +15134,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="449" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="449" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G449" s="3">
         <v>45967</v>
       </c>
@@ -15094,7 +15160,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="450" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="450" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G450" s="30">
         <v>45967</v>
       </c>
@@ -15876,7 +15942,7 @@
       </c>
     </row>
     <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="483" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="483" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G483" s="30">
         <v>45974</v>
       </c>
@@ -15904,7 +15970,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="484" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="484" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G484" s="30">
         <v>45974</v>
       </c>
@@ -15934,7 +16000,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="485" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="485" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G485" s="30">
         <v>45974</v>
       </c>
@@ -15962,7 +16028,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="486" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="486" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G486" s="30">
         <v>45974</v>
       </c>
@@ -15990,7 +16056,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="487" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="487" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G487" s="30">
         <v>45974</v>
       </c>
@@ -16018,7 +16084,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="488" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="488" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G488" s="30">
         <v>45974</v>
       </c>
@@ -16046,7 +16112,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="489" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="489" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G489" s="30">
         <v>45974</v>
       </c>
@@ -16074,7 +16140,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="490" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="490" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G490" s="30">
         <v>45974</v>
       </c>
@@ -16102,7 +16168,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="491" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="491" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G491" s="30">
         <v>45974</v>
       </c>
@@ -16130,7 +16196,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="492" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="492" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G492" s="30">
         <v>45974</v>
       </c>
@@ -16158,7 +16224,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="493" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="493" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G493" s="30">
         <v>45974</v>
       </c>
@@ -16186,7 +16252,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="494" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="494" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G494" s="45">
         <v>45974</v>
       </c>
@@ -16216,7 +16282,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="495" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="495" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G495" s="3">
         <v>45974</v>
       </c>
@@ -16254,38 +16320,738 @@
       <c r="M496" s="4"/>
       <c r="N496" s="6"/>
       <c r="O496" s="25"/>
-      <c r="P496" s="6"/>
-    </row>
-    <row r="497" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G497" s="3"/>
-      <c r="H497" s="4"/>
-      <c r="I497" s="6"/>
-      <c r="J497" s="4"/>
-      <c r="K497" s="8"/>
-      <c r="L497" s="4"/>
-      <c r="M497" s="4"/>
-      <c r="N497" s="6"/>
+      <c r="P496" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="497" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G497" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H497" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="I497" s="6" t="s">
+        <v>388</v>
+      </c>
+      <c r="J497" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="K497" s="8">
+        <v>220</v>
+      </c>
+      <c r="L497" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="M497" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N497" s="6">
+        <v>2</v>
+      </c>
       <c r="O497" s="25"/>
-      <c r="P497" s="6"/>
-    </row>
-    <row r="498" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G498" s="4"/>
-      <c r="H498" s="4"/>
-      <c r="I498" s="6"/>
-      <c r="J498" s="4"/>
-      <c r="K498" s="8"/>
-      <c r="L498" s="4"/>
-      <c r="M498" s="4"/>
-      <c r="N498" s="6"/>
-      <c r="O498" s="25"/>
-      <c r="P498" s="6"/>
+      <c r="P497" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="498" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G498" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H498" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="I498" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="J498" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="K498" s="8">
+        <v>170</v>
+      </c>
+      <c r="L498" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="M498" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N498" s="6">
+        <v>2</v>
+      </c>
+      <c r="O498" s="4"/>
+      <c r="P498" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="499" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G499" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H499" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="I499" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="J499" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K499" s="8">
+        <v>159</v>
+      </c>
+      <c r="L499" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="M499" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N499" s="4">
+        <v>2</v>
+      </c>
+      <c r="O499" s="4"/>
+      <c r="P499" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="500" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G500" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H500" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I500" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="J500" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K500" s="8">
+        <v>200</v>
+      </c>
+      <c r="L500" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="M500" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N500" s="4">
+        <v>2</v>
+      </c>
+      <c r="O500" s="4"/>
+      <c r="P500" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="501" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G501" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H501" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="I501" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="J501" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K501" s="8">
+        <v>180</v>
+      </c>
+      <c r="L501" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M501" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N501" s="4">
+        <v>3</v>
+      </c>
+      <c r="O501" s="4"/>
+      <c r="P501" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="502" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G502" s="3">
+        <v>45978</v>
+      </c>
+      <c r="H502" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I502" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="J502" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K502" s="8">
+        <v>220</v>
+      </c>
+      <c r="L502" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="M502" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N502" s="4">
+        <v>2</v>
+      </c>
+      <c r="O502" s="4"/>
+      <c r="P502" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="503" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G503" s="17">
+        <v>45978</v>
+      </c>
+      <c r="H503" s="18" t="s">
+        <v>393</v>
+      </c>
+      <c r="I503" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="J503" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="K503" s="20">
+        <v>220</v>
+      </c>
+      <c r="L503" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="M503" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="N503" s="18">
+        <v>1</v>
+      </c>
+      <c r="O503" s="18">
+        <v>1</v>
+      </c>
+      <c r="P503" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="504" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G504" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H504" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="I504" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="J504" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K504" s="8">
+        <v>150</v>
+      </c>
+      <c r="L504" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="M504" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N504" s="4">
+        <v>2</v>
+      </c>
+      <c r="O504" s="4"/>
+      <c r="P504" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="505" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G505" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H505" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I505" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="J505" s="4" t="s">
+        <v>396</v>
+      </c>
+      <c r="K505" s="8">
+        <v>260</v>
+      </c>
+      <c r="L505" s="4" t="s">
+        <v>397</v>
+      </c>
+      <c r="M505" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N505" s="4"/>
+      <c r="O505" s="4"/>
+      <c r="P505" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="506" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G506" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H506" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="I506" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="J506" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K506" s="8">
+        <v>159</v>
+      </c>
+      <c r="L506" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M506" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N506" s="4"/>
+      <c r="O506" s="4"/>
+      <c r="P506" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="507" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G507" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H507" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I507" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="J507" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K507" s="8">
+        <v>240</v>
+      </c>
+      <c r="L507" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="M507" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N507" s="4">
+        <v>2</v>
+      </c>
+      <c r="O507" s="4"/>
+      <c r="P507" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="508" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G508" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H508" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I508" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J508" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="K508" s="8">
+        <v>280</v>
+      </c>
+      <c r="L508" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M508" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N508" s="4">
+        <v>3</v>
+      </c>
+      <c r="O508" s="4"/>
+      <c r="P508" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="509" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G509" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H509" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I509" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="J509" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="K509" s="8">
+        <v>200</v>
+      </c>
+      <c r="L509" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="M509" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N509" s="4">
+        <v>2</v>
+      </c>
+      <c r="O509" s="4"/>
+      <c r="P509" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="510" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G510" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H510" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I510" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J510" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="K510" s="8">
+        <v>160</v>
+      </c>
+      <c r="L510" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="M510" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N510" s="6"/>
+      <c r="O510" s="25"/>
+      <c r="P510" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="511" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G511" s="3">
+        <v>45979</v>
+      </c>
+      <c r="H511" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="I511" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="J511" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="K511" s="8">
+        <v>180</v>
+      </c>
+      <c r="L511" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="M511" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N511" s="6">
+        <v>1</v>
+      </c>
+      <c r="O511" s="25"/>
+      <c r="P511" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="512" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G512" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H512" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I512" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J512" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="K512" s="8">
+        <v>240</v>
+      </c>
+      <c r="L512" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="M512" s="4"/>
+      <c r="N512" s="6">
+        <v>2</v>
+      </c>
+      <c r="O512" s="25"/>
+      <c r="P512" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="513" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G513" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H513" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I513" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J513" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="K513" s="8">
+        <v>160</v>
+      </c>
+      <c r="L513" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="M513" s="4"/>
+      <c r="N513" s="6">
+        <v>2</v>
+      </c>
+      <c r="O513" s="25"/>
+      <c r="P513" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="514" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G514" s="17">
+        <v>45980</v>
+      </c>
+      <c r="H514" s="18" t="s">
+        <v>145</v>
+      </c>
+      <c r="I514" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="J514" s="18" t="s">
+        <v>407</v>
+      </c>
+      <c r="K514" s="20">
+        <v>159</v>
+      </c>
+      <c r="L514" s="18" t="s">
+        <v>408</v>
+      </c>
+      <c r="M514" s="18"/>
+      <c r="N514" s="19"/>
+      <c r="O514" s="41" t="s">
+        <v>251</v>
+      </c>
+      <c r="P514" s="19" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="515" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G515" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H515" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I515" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J515" s="4" t="s">
+        <v>399</v>
+      </c>
+      <c r="K515" s="8">
+        <v>290</v>
+      </c>
+      <c r="L515" s="4" t="s">
+        <v>398</v>
+      </c>
+      <c r="M515" s="4"/>
+      <c r="N515" s="6">
+        <v>2</v>
+      </c>
+      <c r="O515" s="25"/>
+      <c r="P515" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="516" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G516" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H516" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="I516" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J516" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K516" s="8">
+        <v>200</v>
+      </c>
+      <c r="L516" s="4" t="s">
+        <v>405</v>
+      </c>
+      <c r="M516" s="4"/>
+      <c r="N516" s="6">
+        <v>3</v>
+      </c>
+      <c r="O516" s="25"/>
+      <c r="P516" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="517" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G517" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H517" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="I517" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="J517" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K517" s="8">
+        <v>150</v>
+      </c>
+      <c r="L517" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="M517" s="4"/>
+      <c r="N517" s="6">
+        <v>3</v>
+      </c>
+      <c r="O517" s="25"/>
+      <c r="P517" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="518" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G518" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H518" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I518" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J518" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K518" s="8">
+        <v>170</v>
+      </c>
+      <c r="L518" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M518" s="4"/>
+      <c r="N518" s="6">
+        <v>3</v>
+      </c>
+      <c r="O518" s="25"/>
+      <c r="P518" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="519" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G519" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H519" s="4" t="s">
+        <v>387</v>
+      </c>
+      <c r="I519" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="J519" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="K519" s="8">
+        <v>220</v>
+      </c>
+      <c r="L519" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="M519" s="4"/>
+      <c r="N519" s="6">
+        <v>2</v>
+      </c>
+      <c r="O519" s="25"/>
+      <c r="P519" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="520" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G520" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H520" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="I520" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J520" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="K520" s="8">
+        <v>280</v>
+      </c>
+      <c r="L520" s="4" t="s">
+        <v>406</v>
+      </c>
+      <c r="M520" s="4"/>
+      <c r="N520" s="6">
+        <v>2</v>
+      </c>
+      <c r="O520" s="25"/>
+      <c r="P520" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="521" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="522" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G522" s="3">
+        <v>45980</v>
+      </c>
+      <c r="H522" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="I522" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="J522" s="4" t="s">
+        <v>403</v>
+      </c>
+      <c r="K522" s="8">
+        <v>180</v>
+      </c>
+      <c r="L522" s="4" t="s">
+        <v>404</v>
+      </c>
+      <c r="M522" s="4"/>
+      <c r="N522" s="6"/>
+      <c r="O522" s="25"/>
+      <c r="P522" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O496" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O521" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="6" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="11" day="13" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="19" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-21  9:13
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1274" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ACE9DC15-78EC-43F8-9B35-2AD03F257109}"/>
+  <xr:revisionPtr revIDLastSave="1373" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF3CEE5A-BB45-4B96-A2F3-F9753A73F0B0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,9 +17,10 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$521</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$534</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3162" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3227" uniqueCount="420">
   <si>
     <t>DATA</t>
   </si>
@@ -1250,12 +1251,6 @@
     <t>JOÃO</t>
   </si>
   <si>
-    <t>PONTE NOVA</t>
-  </si>
-  <si>
-    <t>HOTEL PARAISO</t>
-  </si>
-  <si>
     <t>AGUAS CLARAS</t>
   </si>
   <si>
@@ -1266,6 +1261,45 @@
   </si>
   <si>
     <t>carmo palace</t>
+  </si>
+  <si>
+    <t>RYCHARD</t>
+  </si>
+  <si>
+    <t>HOTEL GIRASOL</t>
+  </si>
+  <si>
+    <t>CAMPINAS SP</t>
+  </si>
+  <si>
+    <t>HOTEL PRIMEIN</t>
+  </si>
+  <si>
+    <t>Abaete</t>
+  </si>
+  <si>
+    <t>TRêS CORAÇÕES</t>
+  </si>
+  <si>
+    <t>CASTELO</t>
+  </si>
+  <si>
+    <t>JOÃO MONLEVADE</t>
+  </si>
+  <si>
+    <t>Douglas.r</t>
+  </si>
+  <si>
+    <t>SÃO JOÃO DEL REI</t>
+  </si>
+  <si>
+    <t>hotel rotor</t>
+  </si>
+  <si>
+    <t>OURO BRANCO</t>
+  </si>
+  <si>
+    <t>MAXX HOTEL</t>
   </si>
 </sst>
 </file>
@@ -1412,7 +1446,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1531,6 +1565,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -1870,7 +1905,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P522"/>
+  <dimension ref="G5:P535"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -16770,7 +16805,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="512" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="512" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G512" s="3">
         <v>45980</v>
       </c>
@@ -16798,7 +16833,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="513" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="513" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G513" s="3">
         <v>45980</v>
       </c>
@@ -16826,7 +16861,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="514" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="514" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G514" s="17">
         <v>45980</v>
       </c>
@@ -16837,13 +16872,13 @@
         <v>216</v>
       </c>
       <c r="J514" s="18" t="s">
-        <v>407</v>
+        <v>405</v>
       </c>
       <c r="K514" s="20">
         <v>159</v>
       </c>
       <c r="L514" s="18" t="s">
-        <v>408</v>
+        <v>406</v>
       </c>
       <c r="M514" s="18"/>
       <c r="N514" s="19"/>
@@ -16854,7 +16889,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="515" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="515" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G515" s="3">
         <v>45980</v>
       </c>
@@ -16882,7 +16917,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="516" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="516" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G516" s="3">
         <v>45980</v>
       </c>
@@ -16899,7 +16934,7 @@
         <v>200</v>
       </c>
       <c r="L516" s="4" t="s">
-        <v>405</v>
+        <v>403</v>
       </c>
       <c r="M516" s="4"/>
       <c r="N516" s="6">
@@ -16910,7 +16945,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="517" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="517" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G517" s="3">
         <v>45980</v>
       </c>
@@ -16938,7 +16973,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="518" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="518" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G518" s="3">
         <v>45980</v>
       </c>
@@ -16966,7 +17001,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="519" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="519" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G519" s="3">
         <v>45980</v>
       </c>
@@ -16994,7 +17029,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="520" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="520" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G520" s="3">
         <v>45980</v>
       </c>
@@ -17011,7 +17046,7 @@
         <v>280</v>
       </c>
       <c r="L520" s="4" t="s">
-        <v>406</v>
+        <v>404</v>
       </c>
       <c r="M520" s="4"/>
       <c r="N520" s="6">
@@ -17023,7 +17058,7 @@
       </c>
     </row>
     <row r="521" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="522" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="522" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G522" s="3">
         <v>45980</v>
       </c>
@@ -17033,25 +17068,381 @@
       <c r="I522" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="J522" s="4" t="s">
-        <v>403</v>
-      </c>
-      <c r="K522" s="8">
+      <c r="J522" s="4"/>
+      <c r="K522" s="8"/>
+      <c r="L522" s="4"/>
+      <c r="M522" s="4"/>
+      <c r="N522" s="6">
+        <v>2</v>
+      </c>
+      <c r="O522" s="25"/>
+      <c r="P522" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="523" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G523" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H523" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="I523" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J523" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="K523" s="8">
+        <v>210</v>
+      </c>
+      <c r="L523" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="M523" s="4"/>
+      <c r="N523" s="6">
+        <v>2</v>
+      </c>
+      <c r="O523" s="25"/>
+      <c r="P523" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="524" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G524" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H524" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="I524" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="J524" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K524" s="8">
+        <v>190</v>
+      </c>
+      <c r="L524" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="M524" s="4"/>
+      <c r="N524" s="6">
+        <v>2</v>
+      </c>
+      <c r="O524" s="25"/>
+      <c r="P524" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="525" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G525" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H525" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I525" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J525" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K525" s="8">
+        <v>200</v>
+      </c>
+      <c r="L525" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="M525" s="4"/>
+      <c r="N525" s="6">
+        <v>2</v>
+      </c>
+      <c r="O525" s="25"/>
+      <c r="P525" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="526" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G526" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H526" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I526" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J526" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="K526" s="8">
+        <v>250</v>
+      </c>
+      <c r="L526" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="M526" s="4"/>
+      <c r="N526" s="6">
+        <v>2</v>
+      </c>
+      <c r="O526" s="25"/>
+      <c r="P526" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="527" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G527" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H527" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="I527" s="6" t="s">
+        <v>407</v>
+      </c>
+      <c r="J527" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="K527" s="8">
+        <v>159</v>
+      </c>
+      <c r="L527" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="M527" s="4"/>
+      <c r="N527" s="6">
+        <v>2</v>
+      </c>
+      <c r="O527" s="25"/>
+      <c r="P527" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="528" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G528" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H528" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I528" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="J528" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K528" s="8">
+        <v>240</v>
+      </c>
+      <c r="L528" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M528" s="4"/>
+      <c r="N528" s="6">
+        <v>2</v>
+      </c>
+      <c r="O528" s="25"/>
+      <c r="P528" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="529" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G529" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H529" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="I529" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J529" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K529" s="8">
+        <v>280</v>
+      </c>
+      <c r="L529" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="M529" s="4"/>
+      <c r="N529" s="6">
+        <v>2</v>
+      </c>
+      <c r="O529" s="25"/>
+      <c r="P529" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="530" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G530" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H530" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I530" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J530" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="K530" s="8">
+        <v>175</v>
+      </c>
+      <c r="L530" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M530" s="4"/>
+      <c r="N530" s="6">
+        <v>2</v>
+      </c>
+      <c r="O530" s="25"/>
+      <c r="P530" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="531" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G531" s="17">
+        <v>45981</v>
+      </c>
+      <c r="H531" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="I531" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="J531" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="K531" s="20">
+        <v>259.38</v>
+      </c>
+      <c r="L531" s="18" t="s">
+        <v>410</v>
+      </c>
+      <c r="M531" s="18"/>
+      <c r="N531" s="19">
+        <v>2</v>
+      </c>
+      <c r="O531" s="41" t="s">
+        <v>251</v>
+      </c>
+      <c r="P531" s="19" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="532" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G532" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H532" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I532" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J532" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="K532" s="8">
+        <v>240</v>
+      </c>
+      <c r="L532" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="M532" s="4"/>
+      <c r="N532" s="6"/>
+      <c r="O532" s="25"/>
+      <c r="P532" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="533" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G533" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H533" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I533" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J533" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K533" s="8">
         <v>180</v>
       </c>
-      <c r="L522" s="4" t="s">
-        <v>404</v>
-      </c>
-      <c r="M522" s="4"/>
-      <c r="N522" s="6"/>
-      <c r="O522" s="25"/>
-      <c r="P522" s="6"/>
+      <c r="L533" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M533" s="4"/>
+      <c r="N533" s="6"/>
+      <c r="O533" s="25"/>
+      <c r="P533" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="534" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G534" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H534" s="4" t="s">
+        <v>401</v>
+      </c>
+      <c r="I534" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="J534" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="K534" s="8">
+        <v>198</v>
+      </c>
+      <c r="L534" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M534" s="4"/>
+      <c r="N534" s="6"/>
+      <c r="O534" s="25"/>
+      <c r="P534" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="535" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G535" s="3">
+        <v>45981</v>
+      </c>
+      <c r="H535" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="I535" s="50" t="s">
+        <v>218</v>
+      </c>
+      <c r="J535" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K535" s="8">
+        <v>266</v>
+      </c>
+      <c r="L535" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="M535" s="4"/>
+      <c r="N535" s="6"/>
+      <c r="O535" s="25"/>
+      <c r="P535" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O521" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O535" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="19" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="20" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-26  9:07
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1402" documentId="14_{26B40267-1D17-4F43-A747-F3AF1361A198}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FE58BAB1-5454-449B-B8A2-219F1A743771}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$536</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$553</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3241" uniqueCount="420">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3304" uniqueCount="430">
   <si>
     <t>DATA</t>
   </si>
@@ -1299,6 +1299,36 @@
   </si>
   <si>
     <t>MAXX HOTEL</t>
+  </si>
+  <si>
+    <t>DOUGLAS.a</t>
+  </si>
+  <si>
+    <t>hotel santos drummont</t>
+  </si>
+  <si>
+    <t>hotel piracema</t>
+  </si>
+  <si>
+    <t>HOTEL REAL</t>
+  </si>
+  <si>
+    <t>HOTEL JOAZINHO</t>
+  </si>
+  <si>
+    <t>Hotel chacara</t>
+  </si>
+  <si>
+    <t>POUSADA AMÉRICA</t>
+  </si>
+  <si>
+    <t>HOTEL CAFÉ PALACE</t>
+  </si>
+  <si>
+    <t>PIUMNHI</t>
+  </si>
+  <si>
+    <t>HOTEL CANDIDEZ</t>
   </si>
 </sst>
 </file>
@@ -1903,7 +1933,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P544"/>
+  <dimension ref="G5:P553"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -16569,7 +16599,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="504" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="504" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G504" s="3">
         <v>45979</v>
       </c>
@@ -16599,7 +16629,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="505" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="505" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G505" s="3">
         <v>45979</v>
       </c>
@@ -16627,7 +16657,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="506" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="506" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G506" s="3">
         <v>45979</v>
       </c>
@@ -16655,7 +16685,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="507" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="507" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G507" s="3">
         <v>45979</v>
       </c>
@@ -16685,7 +16715,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="508" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="508" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G508" s="3">
         <v>45979</v>
       </c>
@@ -16715,7 +16745,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="509" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="509" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G509" s="3">
         <v>45979</v>
       </c>
@@ -16745,7 +16775,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="510" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="510" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G510" s="3">
         <v>45979</v>
       </c>
@@ -16773,7 +16803,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="511" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="511" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G511" s="3">
         <v>45979</v>
       </c>
@@ -16803,7 +16833,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="512" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="512" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G512" s="3">
         <v>45980</v>
       </c>
@@ -16831,7 +16861,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="513" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="513" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G513" s="3">
         <v>45980</v>
       </c>
@@ -16859,7 +16889,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="514" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="514" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G514" s="17">
         <v>45980</v>
       </c>
@@ -16887,7 +16917,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="515" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="515" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G515" s="3">
         <v>45980</v>
       </c>
@@ -16915,7 +16945,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="516" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="516" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G516" s="3">
         <v>45980</v>
       </c>
@@ -16943,7 +16973,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="517" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="517" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G517" s="3">
         <v>45980</v>
       </c>
@@ -16971,7 +17001,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="518" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="518" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G518" s="3">
         <v>45980</v>
       </c>
@@ -16999,7 +17029,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="519" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="519" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G519" s="3">
         <v>45980</v>
       </c>
@@ -17027,7 +17057,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="520" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="520" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G520" s="3">
         <v>45980</v>
       </c>
@@ -17056,7 +17086,7 @@
       </c>
     </row>
     <row r="521" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="522" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="522" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G522" s="3">
         <v>45980</v>
       </c>
@@ -17078,7 +17108,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="523" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="523" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G523" s="3">
         <v>45981</v>
       </c>
@@ -17106,7 +17136,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="524" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="524" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G524" s="3">
         <v>45981</v>
       </c>
@@ -17134,7 +17164,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="525" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="525" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G525" s="3">
         <v>45981</v>
       </c>
@@ -17162,7 +17192,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="526" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="526" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G526" s="3">
         <v>45981</v>
       </c>
@@ -17190,7 +17220,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="527" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="527" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G527" s="3">
         <v>45981</v>
       </c>
@@ -17218,7 +17248,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="528" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="528" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G528" s="3">
         <v>45981</v>
       </c>
@@ -17246,7 +17276,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="529" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="529" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G529" s="3">
         <v>45981</v>
       </c>
@@ -17274,7 +17304,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="530" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="530" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G530" s="3">
         <v>45981</v>
       </c>
@@ -17302,7 +17332,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="531" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="531" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G531" s="17">
         <v>45981</v>
       </c>
@@ -17332,7 +17362,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="532" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="532" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G532" s="3">
         <v>45981</v>
       </c>
@@ -17358,7 +17388,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="533" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="533" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G533" s="3">
         <v>45981</v>
       </c>
@@ -17384,7 +17414,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="534" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="534" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G534" s="3">
         <v>45981</v>
       </c>
@@ -17410,7 +17440,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="535" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="535" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G535" s="3">
         <v>45981</v>
       </c>
@@ -17438,7 +17468,7 @@
     </row>
     <row r="536" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G536" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H536" s="4" t="s">
         <v>197</v>
@@ -17446,39 +17476,55 @@
       <c r="I536" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="J536" s="4"/>
-      <c r="K536" s="8"/>
-      <c r="L536" s="4"/>
+      <c r="J536" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="K536" s="8">
+        <v>170</v>
+      </c>
+      <c r="L536" s="4" t="s">
+        <v>422</v>
+      </c>
       <c r="M536" s="4"/>
       <c r="N536" s="6">
         <v>2</v>
       </c>
       <c r="O536" s="25"/>
-      <c r="P536" s="6"/>
+      <c r="P536" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="537" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G537" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H537" s="4" t="s">
-        <v>156</v>
+        <v>420</v>
       </c>
       <c r="I537" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="J537" s="4"/>
-      <c r="K537" s="8"/>
-      <c r="L537" s="4"/>
+      <c r="J537" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="K537" s="8">
+        <v>159</v>
+      </c>
+      <c r="L537" s="4" t="s">
+        <v>89</v>
+      </c>
       <c r="M537" s="4"/>
       <c r="N537" s="6">
         <v>2</v>
       </c>
       <c r="O537" s="25"/>
-      <c r="P537" s="6"/>
+      <c r="P537" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="538" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G538" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H538" s="4" t="s">
         <v>137</v>
@@ -17486,19 +17532,27 @@
       <c r="I538" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="J538" s="4"/>
-      <c r="K538" s="8"/>
-      <c r="L538" s="4"/>
+      <c r="J538" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="K538" s="8">
+        <v>240</v>
+      </c>
+      <c r="L538" s="4" t="s">
+        <v>423</v>
+      </c>
       <c r="M538" s="4"/>
       <c r="N538" s="6">
         <v>2</v>
       </c>
       <c r="O538" s="25"/>
-      <c r="P538" s="6"/>
+      <c r="P538" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="539" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G539" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H539" s="4" t="s">
         <v>131</v>
@@ -17506,19 +17560,27 @@
       <c r="I539" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="J539" s="4"/>
-      <c r="K539" s="8"/>
-      <c r="L539" s="4"/>
+      <c r="J539" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="K539" s="8">
+        <v>220</v>
+      </c>
+      <c r="L539" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="M539" s="4"/>
       <c r="N539" s="6">
         <v>2</v>
       </c>
       <c r="O539" s="25"/>
-      <c r="P539" s="6"/>
+      <c r="P539" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="540" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G540" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H540" s="4" t="s">
         <v>329</v>
@@ -17526,19 +17588,27 @@
       <c r="I540" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="J540" s="4"/>
-      <c r="K540" s="8"/>
-      <c r="L540" s="4"/>
+      <c r="J540" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K540" s="8">
+        <v>160</v>
+      </c>
+      <c r="L540" s="4" t="s">
+        <v>421</v>
+      </c>
       <c r="M540" s="4"/>
       <c r="N540" s="6">
         <v>3</v>
       </c>
       <c r="O540" s="25"/>
-      <c r="P540" s="6"/>
+      <c r="P540" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="541" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G541" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H541" s="4" t="s">
         <v>145</v>
@@ -17546,19 +17616,27 @@
       <c r="I541" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="J541" s="4"/>
-      <c r="K541" s="8"/>
-      <c r="L541" s="4"/>
+      <c r="J541" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="K541" s="10">
+        <v>180</v>
+      </c>
+      <c r="L541" s="1" t="s">
+        <v>101</v>
+      </c>
       <c r="M541" s="4"/>
       <c r="N541" s="6">
         <v>2</v>
       </c>
       <c r="O541" s="25"/>
-      <c r="P541" s="6"/>
+      <c r="P541" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="542" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G542" s="3">
-        <v>45982</v>
+        <v>45985</v>
       </c>
       <c r="H542" s="4" t="s">
         <v>152</v>
@@ -17566,45 +17644,297 @@
       <c r="I542" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="J542" s="4"/>
-      <c r="K542" s="8"/>
-      <c r="L542" s="4"/>
+      <c r="J542" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="K542" s="8">
+        <v>175</v>
+      </c>
+      <c r="L542" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="M542" s="4"/>
       <c r="N542" s="6">
         <v>2</v>
       </c>
       <c r="O542" s="25"/>
-      <c r="P542" s="6"/>
+      <c r="P542" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="543" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G543" s="3"/>
-      <c r="H543" s="4"/>
-      <c r="I543" s="6"/>
-      <c r="J543" s="4"/>
-      <c r="K543" s="8"/>
-      <c r="L543" s="4"/>
+      <c r="G543" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H543" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="I543" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J543" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="K543" s="8">
+        <v>200</v>
+      </c>
+      <c r="L543" s="4" t="s">
+        <v>426</v>
+      </c>
       <c r="M543" s="4"/>
-      <c r="N543" s="6"/>
+      <c r="N543" s="6">
+        <v>2</v>
+      </c>
       <c r="O543" s="25"/>
-      <c r="P543" s="6"/>
+      <c r="P543" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
     <row r="544" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G544" s="3"/>
-      <c r="H544" s="4"/>
-      <c r="I544" s="6"/>
-      <c r="J544" s="4"/>
-      <c r="K544" s="8"/>
-      <c r="L544" s="4"/>
+      <c r="G544" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H544" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I544" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="J544" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K544" s="8">
+        <v>240</v>
+      </c>
+      <c r="L544" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="M544" s="4"/>
-      <c r="N544" s="6"/>
+      <c r="N544" s="6">
+        <v>2</v>
+      </c>
       <c r="O544" s="25"/>
-      <c r="P544" s="6"/>
+      <c r="P544" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="545" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G545" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H545" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I545" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J545" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="K545" s="8">
+        <v>280</v>
+      </c>
+      <c r="L545" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="M545" s="4"/>
+      <c r="N545" s="6">
+        <v>3</v>
+      </c>
+      <c r="O545" s="25"/>
+      <c r="P545" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="546" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G546" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H546" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I546" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="J546" s="4" t="s">
+        <v>428</v>
+      </c>
+      <c r="K546" s="8">
+        <v>210</v>
+      </c>
+      <c r="L546" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="M546" s="4"/>
+      <c r="N546" s="6">
+        <v>2</v>
+      </c>
+      <c r="O546" s="25"/>
+      <c r="P546" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="547" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G547" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H547" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="I547" s="6" t="s">
+        <v>402</v>
+      </c>
+      <c r="J547" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K547" s="8">
+        <v>200</v>
+      </c>
+      <c r="L547" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="M547" s="4"/>
+      <c r="N547" s="6">
+        <v>2</v>
+      </c>
+      <c r="O547" s="25"/>
+      <c r="P547" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="548" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G548" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H548" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I548" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J548" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K548" s="8">
+        <v>180</v>
+      </c>
+      <c r="L548" s="4" t="s">
+        <v>424</v>
+      </c>
+      <c r="M548" s="4"/>
+      <c r="N548" s="6">
+        <v>3</v>
+      </c>
+      <c r="O548" s="25"/>
+      <c r="P548" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="549" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G549" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H549" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="I549" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="J549" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K549" s="8">
+        <v>266</v>
+      </c>
+      <c r="L549" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="M549" s="4"/>
+      <c r="N549" s="6">
+        <v>2</v>
+      </c>
+      <c r="O549" s="25"/>
+      <c r="P549" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="550" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G550" s="3"/>
+      <c r="H550" s="4"/>
+      <c r="I550" s="6"/>
+      <c r="J550" s="4"/>
+      <c r="K550" s="8"/>
+      <c r="L550" s="4"/>
+      <c r="M550" s="4"/>
+      <c r="N550" s="6"/>
+      <c r="O550" s="25"/>
+      <c r="P550" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="551" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G551" s="3"/>
+      <c r="H551" s="4"/>
+      <c r="I551" s="6"/>
+      <c r="J551" s="4"/>
+      <c r="K551" s="8"/>
+      <c r="L551" s="4"/>
+      <c r="M551" s="4"/>
+      <c r="N551" s="6"/>
+      <c r="O551" s="25"/>
+      <c r="P551" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="552" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G552" s="3"/>
+      <c r="H552" s="4"/>
+      <c r="I552" s="6"/>
+      <c r="J552" s="4"/>
+      <c r="K552" s="8"/>
+      <c r="L552" s="4"/>
+      <c r="M552" s="4"/>
+      <c r="N552" s="6"/>
+      <c r="O552" s="25"/>
+      <c r="P552" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="553" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G553" s="3">
+        <v>45986</v>
+      </c>
+      <c r="H553" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I553" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="J553" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K553" s="8">
+        <v>180</v>
+      </c>
+      <c r="L553" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="M553" s="4"/>
+      <c r="N553" s="6">
+        <v>1</v>
+      </c>
+      <c r="O553" s="25"/>
+      <c r="P553" s="6"/>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O536" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O553" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="21" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="18" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="19" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="20" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="24" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="25" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-26 11:01
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA1241C0-EBE5-42EC-9649-5D61227AEF66}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$553</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$561</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3304" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3333" uniqueCount="431">
   <si>
     <t>DATA</t>
   </si>
@@ -1329,6 +1329,9 @@
   </si>
   <si>
     <t>HOTEL CANDIDEZ</t>
+  </si>
+  <si>
+    <t>HOTEL CAMPEAO</t>
   </si>
 </sst>
 </file>
@@ -1933,7 +1936,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P553"/>
+  <dimension ref="G5:P563"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -16599,7 +16602,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="504" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="504" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G504" s="3">
         <v>45979</v>
       </c>
@@ -16629,7 +16632,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="505" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="505" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G505" s="3">
         <v>45979</v>
       </c>
@@ -16657,7 +16660,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="506" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="506" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G506" s="3">
         <v>45979</v>
       </c>
@@ -16685,7 +16688,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="507" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="507" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G507" s="3">
         <v>45979</v>
       </c>
@@ -16715,7 +16718,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="508" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="508" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G508" s="3">
         <v>45979</v>
       </c>
@@ -16745,7 +16748,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="509" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="509" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G509" s="3">
         <v>45979</v>
       </c>
@@ -16775,7 +16778,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="510" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="510" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G510" s="3">
         <v>45979</v>
       </c>
@@ -16803,7 +16806,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="511" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="511" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G511" s="3">
         <v>45979</v>
       </c>
@@ -16833,7 +16836,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="512" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="512" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G512" s="3">
         <v>45980</v>
       </c>
@@ -16861,7 +16864,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="513" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="513" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G513" s="3">
         <v>45980</v>
       </c>
@@ -16889,7 +16892,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="514" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="514" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G514" s="17">
         <v>45980</v>
       </c>
@@ -16917,7 +16920,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="515" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="515" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G515" s="3">
         <v>45980</v>
       </c>
@@ -16945,7 +16948,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="516" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="516" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G516" s="3">
         <v>45980</v>
       </c>
@@ -16973,7 +16976,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="517" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="517" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G517" s="3">
         <v>45980</v>
       </c>
@@ -17001,7 +17004,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="518" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="518" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G518" s="3">
         <v>45980</v>
       </c>
@@ -17029,7 +17032,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="519" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="519" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G519" s="3">
         <v>45980</v>
       </c>
@@ -17057,7 +17060,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="520" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="520" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G520" s="3">
         <v>45980</v>
       </c>
@@ -17086,7 +17089,7 @@
       </c>
     </row>
     <row r="521" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="522" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="522" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G522" s="3">
         <v>45980</v>
       </c>
@@ -17108,7 +17111,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="523" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="523" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G523" s="3">
         <v>45981</v>
       </c>
@@ -17136,7 +17139,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="524" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="524" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G524" s="3">
         <v>45981</v>
       </c>
@@ -17164,7 +17167,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="525" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="525" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G525" s="3">
         <v>45981</v>
       </c>
@@ -17192,7 +17195,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="526" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="526" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G526" s="3">
         <v>45981</v>
       </c>
@@ -17220,7 +17223,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="527" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="527" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G527" s="3">
         <v>45981</v>
       </c>
@@ -17248,7 +17251,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="528" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="528" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G528" s="3">
         <v>45981</v>
       </c>
@@ -17276,7 +17279,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="529" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="529" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G529" s="3">
         <v>45981</v>
       </c>
@@ -17304,7 +17307,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="530" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="530" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G530" s="3">
         <v>45981</v>
       </c>
@@ -17332,7 +17335,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="531" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="531" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G531" s="17">
         <v>45981</v>
       </c>
@@ -17362,7 +17365,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="532" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="532" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G532" s="3">
         <v>45981</v>
       </c>
@@ -17388,7 +17391,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="533" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="533" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G533" s="3">
         <v>45981</v>
       </c>
@@ -17414,7 +17417,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="534" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="534" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G534" s="3">
         <v>45981</v>
       </c>
@@ -17440,7 +17443,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="535" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="535" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G535" s="3">
         <v>45981</v>
       </c>
@@ -17466,7 +17469,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="536" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="536" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G536" s="3">
         <v>45985</v>
       </c>
@@ -17494,7 +17497,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="537" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="537" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G537" s="3">
         <v>45985</v>
       </c>
@@ -17522,7 +17525,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="538" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="538" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G538" s="3">
         <v>45985</v>
       </c>
@@ -17550,7 +17553,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="539" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="539" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G539" s="3">
         <v>45985</v>
       </c>
@@ -17578,7 +17581,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="540" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="540" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G540" s="3">
         <v>45985</v>
       </c>
@@ -17606,7 +17609,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="541" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="541" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G541" s="3">
         <v>45985</v>
       </c>
@@ -17634,7 +17637,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="542" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="542" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G542" s="3">
         <v>45985</v>
       </c>
@@ -17662,7 +17665,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="543" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="543" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G543" s="3">
         <v>45986</v>
       </c>
@@ -17690,7 +17693,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="544" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="544" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G544" s="3">
         <v>45986</v>
       </c>
@@ -17718,7 +17721,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="545" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="545" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G545" s="3">
         <v>45986</v>
       </c>
@@ -17746,7 +17749,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="546" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="546" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G546" s="3">
         <v>45986</v>
       </c>
@@ -17774,7 +17777,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="547" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="547" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G547" s="3">
         <v>45986</v>
       </c>
@@ -17802,7 +17805,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="548" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="548" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G548" s="3">
         <v>45986</v>
       </c>
@@ -17830,7 +17833,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="549" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="549" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G549" s="3">
         <v>45986</v>
       </c>
@@ -17900,7 +17903,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="553" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="553" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G553" s="3">
         <v>45986</v>
       </c>
@@ -17924,17 +17927,225 @@
         <v>1</v>
       </c>
       <c r="O553" s="25"/>
-      <c r="P553" s="6"/>
+      <c r="P553" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="554" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G554" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H554" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="I554" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J554" s="4"/>
+      <c r="K554" s="8"/>
+      <c r="L554" s="4"/>
+      <c r="M554" s="4"/>
+      <c r="N554" s="6">
+        <v>2</v>
+      </c>
+      <c r="O554" s="25"/>
+      <c r="P554" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="555" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G555" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H555" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I555" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J555" s="4"/>
+      <c r="K555" s="8"/>
+      <c r="L555" s="4"/>
+      <c r="M555" s="4"/>
+      <c r="N555" s="6">
+        <v>2</v>
+      </c>
+      <c r="O555" s="25"/>
+      <c r="P555" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="556" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G556" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H556" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I556" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="J556" s="4"/>
+      <c r="K556" s="8"/>
+      <c r="L556" s="4"/>
+      <c r="M556" s="4"/>
+      <c r="N556" s="6">
+        <v>2</v>
+      </c>
+      <c r="O556" s="25"/>
+      <c r="P556" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="557" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G557" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H557" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="I557" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J557" s="4"/>
+      <c r="K557" s="8"/>
+      <c r="L557" s="4"/>
+      <c r="M557" s="4"/>
+      <c r="N557" s="6">
+        <v>3</v>
+      </c>
+      <c r="O557" s="25"/>
+      <c r="P557" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="558" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G558" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H558" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="I558" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J558" s="4"/>
+      <c r="K558" s="8"/>
+      <c r="L558" s="4"/>
+      <c r="M558" s="4"/>
+      <c r="N558" s="6">
+        <v>3</v>
+      </c>
+      <c r="O558" s="25"/>
+      <c r="P558" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="559" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G559" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H559" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="I559" s="6" t="s">
+        <v>359</v>
+      </c>
+      <c r="J559" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K559" s="8">
+        <v>150</v>
+      </c>
+      <c r="L559" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="M559" s="4"/>
+      <c r="N559" s="6">
+        <v>3</v>
+      </c>
+      <c r="O559" s="25"/>
+      <c r="P559" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="560" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G560" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H560" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="I560" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="J560" s="4"/>
+      <c r="K560" s="8"/>
+      <c r="L560" s="4"/>
+      <c r="M560" s="4"/>
+      <c r="N560" s="6">
+        <v>3</v>
+      </c>
+      <c r="O560" s="25"/>
+      <c r="P560" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="561" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G561" s="3">
+        <v>45987</v>
+      </c>
+      <c r="H561" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I561" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J561" s="4"/>
+      <c r="K561" s="8"/>
+      <c r="L561" s="4"/>
+      <c r="M561" s="4"/>
+      <c r="N561" s="6">
+        <v>2</v>
+      </c>
+      <c r="O561" s="25"/>
+      <c r="P561" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="562" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G562" s="4"/>
+      <c r="H562" s="4"/>
+      <c r="I562" s="6"/>
+      <c r="J562" s="4"/>
+      <c r="K562" s="8"/>
+      <c r="L562" s="4"/>
+      <c r="M562" s="4"/>
+      <c r="N562" s="6"/>
+      <c r="O562" s="25"/>
+      <c r="P562" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="563" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G563" s="4"/>
+      <c r="H563" s="4"/>
+      <c r="I563" s="6"/>
+      <c r="J563" s="4"/>
+      <c r="K563" s="8"/>
+      <c r="L563" s="4"/>
+      <c r="M563" s="4"/>
+      <c r="N563" s="6"/>
+      <c r="O563" s="25"/>
+      <c r="P563" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O553" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O561" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" day="18" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="11" day="19" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="11" day="20" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="11" day="24" dateTimeGrouping="day"/>
-        <dateGroupItem year="2025" month="11" day="25" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="11" day="26" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-27 16:56
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="144" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89E1D078-6F64-4C80-AFB5-8BDB354BFB6D}"/>
+  <xr:revisionPtr revIDLastSave="150" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{798A6908-6661-461F-899E-4C8E931253DD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3406" uniqueCount="439">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3410" uniqueCount="440">
   <si>
     <t>DATA</t>
   </si>
@@ -1356,6 +1356,9 @@
   </si>
   <si>
     <t>são joão del rey</t>
+  </si>
+  <si>
+    <t>IBIA</t>
   </si>
 </sst>
 </file>
@@ -18301,9 +18304,15 @@
       <c r="I566" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="J566" s="4"/>
-      <c r="K566" s="8"/>
-      <c r="L566" s="4"/>
+      <c r="J566" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="K566" s="8">
+        <v>200</v>
+      </c>
+      <c r="L566" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="M566" s="4"/>
       <c r="N566" s="6">
         <v>2</v>
@@ -18407,9 +18416,15 @@
       <c r="I570" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="J570" s="4"/>
-      <c r="K570" s="8"/>
-      <c r="L570" s="4"/>
+      <c r="J570" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="K570" s="8">
+        <v>160</v>
+      </c>
+      <c r="L570" s="4" t="s">
+        <v>118</v>
+      </c>
       <c r="M570" s="4"/>
       <c r="N570" s="6">
         <v>2</v>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-27 17:42
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="150" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{798A6908-6661-461F-899E-4C8E931253DD}"/>
+  <xr:revisionPtr revIDLastSave="161" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8E3251F5-B7B9-4AAE-A1F6-60CB42A44D61}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3410" uniqueCount="440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3417" uniqueCount="441">
   <si>
     <t>DATA</t>
   </si>
@@ -1359,6 +1359,9 @@
   </si>
   <si>
     <t>IBIA</t>
+  </si>
+  <si>
+    <t>HIPOCRATES</t>
   </si>
 </sst>
 </file>
@@ -1963,7 +1966,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P574"/>
+  <dimension ref="G5:P575"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
@@ -18543,6 +18546,38 @@
       </c>
       <c r="O574" s="25"/>
       <c r="P574" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="575" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G575" s="3">
+        <v>45988</v>
+      </c>
+      <c r="H575" s="4" t="s">
+        <v>440</v>
+      </c>
+      <c r="I575" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="J575" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="K575" s="8">
+        <v>175</v>
+      </c>
+      <c r="L575" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M575" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="N575" s="6">
+        <v>1</v>
+      </c>
+      <c r="O575" s="25" t="s">
+        <v>251</v>
+      </c>
+      <c r="P575" s="6" t="s">
         <v>358</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-02 14:32
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="234" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{223BE3DA-800E-4D9C-8725-9F56499C2653}"/>
+  <xr:revisionPtr revIDLastSave="297" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E7C4BE95-6C56-4AB3-B4B6-2D6E5FD8083C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="NÚMERO DE HOTEIS" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$584</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS!$G$5:$O$593</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3460" uniqueCount="443">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3484" uniqueCount="443">
   <si>
     <t>DATA</t>
   </si>
@@ -1972,18 +1972,18 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P586"/>
+  <dimension ref="G5:P593"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="7" max="7" width="13.28515625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="20.28515625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="27.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15" style="10" customWidth="1"/>
-    <col min="12" max="12" width="36.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.28515625" style="1" customWidth="1"/>
-    <col min="14" max="14" width="12.42578125" customWidth="1"/>
-    <col min="15" max="15" width="20.140625" style="22" customWidth="1"/>
+    <col min="11" max="11" width="12.7109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.7109375" style="22" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="12.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -18583,7 +18583,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="576" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="576" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G576" s="3">
         <v>45992</v>
       </c>
@@ -18611,7 +18611,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="577" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="577" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G577" s="3">
         <v>45992</v>
       </c>
@@ -18639,7 +18639,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="578" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="578" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G578" s="3">
         <v>45992</v>
       </c>
@@ -18667,7 +18667,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="579" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="579" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G579" s="3">
         <v>45992</v>
       </c>
@@ -18695,7 +18695,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="580" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="580" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G580" s="3">
         <v>45992</v>
       </c>
@@ -18723,7 +18723,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="581" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="581" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G581" s="3">
         <v>45992</v>
       </c>
@@ -18751,7 +18751,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="582" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="582" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G582" s="3">
         <v>45992</v>
       </c>
@@ -18779,7 +18779,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="583" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="583" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G583" s="3">
         <v>45992</v>
       </c>
@@ -18807,7 +18807,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="584" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="584" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G584" s="3">
         <v>45992</v>
       </c>
@@ -18834,9 +18834,15 @@
       </c>
     </row>
     <row r="585" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G585" s="4"/>
-      <c r="H585" s="4"/>
-      <c r="I585" s="6"/>
+      <c r="G585" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H585" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="I585" s="6" t="s">
+        <v>407</v>
+      </c>
       <c r="J585" s="4"/>
       <c r="K585" s="8"/>
       <c r="L585" s="4"/>
@@ -18846,9 +18852,15 @@
       <c r="P585" s="6"/>
     </row>
     <row r="586" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G586" s="4"/>
-      <c r="H586" s="4"/>
-      <c r="I586" s="6"/>
+      <c r="G586" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H586" s="4" t="s">
+        <v>437</v>
+      </c>
+      <c r="I586" s="6" t="s">
+        <v>173</v>
+      </c>
       <c r="J586" s="4"/>
       <c r="K586" s="8"/>
       <c r="L586" s="4"/>
@@ -18857,11 +18869,169 @@
       <c r="O586" s="25"/>
       <c r="P586" s="6"/>
     </row>
+    <row r="587" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G587" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H587" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="I587" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="J587" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="K587" s="8">
+        <v>200</v>
+      </c>
+      <c r="L587" s="4" t="s">
+        <v>426</v>
+      </c>
+      <c r="M587" s="4"/>
+      <c r="N587" s="6">
+        <v>2</v>
+      </c>
+      <c r="O587" s="25"/>
+      <c r="P587" s="6"/>
+    </row>
+    <row r="588" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G588" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H588" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I588" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="J588" s="4"/>
+      <c r="K588" s="8"/>
+      <c r="L588" s="4"/>
+      <c r="M588" s="4"/>
+      <c r="N588" s="6">
+        <v>2</v>
+      </c>
+      <c r="O588" s="25"/>
+      <c r="P588" s="6"/>
+    </row>
+    <row r="589" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G589" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H589" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="I589" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J589" s="4"/>
+      <c r="K589" s="8"/>
+      <c r="L589" s="4"/>
+      <c r="M589" s="4"/>
+      <c r="N589" s="6">
+        <v>3</v>
+      </c>
+      <c r="O589" s="25"/>
+      <c r="P589" s="6"/>
+    </row>
+    <row r="590" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G590" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H590" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="I590" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="J590" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K590" s="8">
+        <v>240</v>
+      </c>
+      <c r="L590" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M590" s="4"/>
+      <c r="N590" s="6">
+        <v>2</v>
+      </c>
+      <c r="O590" s="25"/>
+      <c r="P590" s="6"/>
+    </row>
+    <row r="591" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G591" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H591" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="I591" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="J591" s="4"/>
+      <c r="K591" s="8"/>
+      <c r="L591" s="4"/>
+      <c r="M591" s="4"/>
+      <c r="N591" s="6">
+        <v>2</v>
+      </c>
+      <c r="O591" s="25"/>
+      <c r="P591" s="6"/>
+    </row>
+    <row r="592" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G592" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H592" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="I592" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J592" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K592" s="8">
+        <v>200</v>
+      </c>
+      <c r="L592" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="M592" s="4"/>
+      <c r="N592" s="6">
+        <v>3</v>
+      </c>
+      <c r="O592" s="25"/>
+      <c r="P592" s="6"/>
+    </row>
+    <row r="593" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G593" s="3">
+        <v>45993</v>
+      </c>
+      <c r="H593" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="I593" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="J593" s="4"/>
+      <c r="K593" s="8"/>
+      <c r="L593" s="4"/>
+      <c r="M593" s="4"/>
+      <c r="N593" s="6">
+        <v>2</v>
+      </c>
+      <c r="O593" s="25"/>
+      <c r="P593" s="6"/>
+    </row>
   </sheetData>
-  <autoFilter ref="G5:O584" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O596" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="12" dateTimeGrouping="month"/>
+        <dateGroupItem year="2025" month="12" day="2" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-04 10:04
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="493" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{350AB99D-6FA2-4550-9A2A-436196A6901B}"/>
+  <xr:revisionPtr revIDLastSave="510" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38972DE8-45AA-45B4-9435-A3DD891BCFF4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3586" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3611" uniqueCount="450">
   <si>
     <t>DATA</t>
   </si>
@@ -14558,7 +14558,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="424" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="424" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G424" s="17">
         <v>45964</v>
       </c>
@@ -14796,7 +14796,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="432" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="432" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G432" s="17">
         <v>45966</v>
       </c>
@@ -14856,7 +14856,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="434" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="434" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G434" s="51">
         <v>45966</v>
       </c>
@@ -15054,7 +15054,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="441" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="441" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G441" s="17">
         <v>45967</v>
       </c>
@@ -15272,7 +15272,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="449" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="449" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G449" s="17">
         <v>45967</v>
       </c>
@@ -15326,7 +15326,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="451" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="451" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G451" s="17">
         <v>45973</v>
       </c>
@@ -15596,7 +15596,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="460" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="460" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G460" s="45">
         <v>45973</v>
       </c>
@@ -15715,7 +15715,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="469" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="469" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G469" s="17">
         <v>45972</v>
       </c>
@@ -15829,7 +15829,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="473" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="473" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G473" s="17">
         <v>45972</v>
       </c>
@@ -15857,7 +15857,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="474" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="474" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G474" s="17">
         <v>45972</v>
       </c>
@@ -15973,7 +15973,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="478" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="478" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G478" s="17">
         <v>45971</v>
       </c>
@@ -16088,7 +16088,7 @@
       </c>
     </row>
     <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="483" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="483" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G483" s="45">
         <v>45974</v>
       </c>
@@ -16400,7 +16400,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="494" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="494" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G494" s="45">
         <v>45974</v>
       </c>
@@ -16652,7 +16652,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="503" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="503" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G503" s="17">
         <v>45978</v>
       </c>
@@ -16742,7 +16742,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="506" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="506" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G506" s="17">
         <v>45979</v>
       </c>
@@ -16890,7 +16890,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="511" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="511" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G511" s="17">
         <v>45979</v>
       </c>
@@ -16978,7 +16978,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="514" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="514" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G514" s="17">
         <v>45980</v>
       </c>
@@ -17006,7 +17006,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="515" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="515" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G515" s="17">
         <v>45980</v>
       </c>
@@ -17423,7 +17423,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="531" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="531" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G531" s="17">
         <v>45981</v>
       </c>
@@ -17453,7 +17453,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="532" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="532" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G532" s="17">
         <v>45981</v>
       </c>
@@ -17533,7 +17533,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="535" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="535" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G535" s="17">
         <v>45981</v>
       </c>
@@ -17645,7 +17645,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="539" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="539" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G539" s="17">
         <v>45985</v>
       </c>
@@ -17703,7 +17703,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="541" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="541" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G541" s="17">
         <v>45985</v>
       </c>
@@ -17929,7 +17929,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="549" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="549" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G549" s="17">
         <v>45986</v>
       </c>
@@ -18001,7 +18001,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="553" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="553" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G553" s="17">
         <v>45986</v>
       </c>
@@ -18087,7 +18087,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="556" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="556" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G556" s="17">
         <v>45987</v>
       </c>
@@ -18229,7 +18229,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="561" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="561" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G561" s="17">
         <v>45987</v>
       </c>
@@ -18259,7 +18259,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="562" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="562" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G562" s="17">
         <v>45987</v>
       </c>
@@ -18401,7 +18401,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="567" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="567" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G567" s="17">
         <v>45988</v>
       </c>
@@ -18623,7 +18623,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="575" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="575" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G575" s="17">
         <v>45988</v>
       </c>
@@ -18655,7 +18655,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="576" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="576" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G576" s="3">
         <v>45992</v>
       </c>
@@ -18683,7 +18683,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="577" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="577" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G577" s="3">
         <v>45992</v>
       </c>
@@ -18711,7 +18711,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="578" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="578" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G578" s="3">
         <v>45992</v>
       </c>
@@ -18739,7 +18739,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="579" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="579" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G579" s="3">
         <v>45992</v>
       </c>
@@ -18767,7 +18767,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="580" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="580" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G580" s="3">
         <v>45992</v>
       </c>
@@ -18795,7 +18795,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="581" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="581" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G581" s="3">
         <v>45992</v>
       </c>
@@ -18823,7 +18823,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="582" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="582" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G582" s="3">
         <v>45992</v>
       </c>
@@ -18851,7 +18851,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="583" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="583" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G583" s="3">
         <v>45992</v>
       </c>
@@ -18879,7 +18879,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="584" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="584" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G584" s="3">
         <v>45992</v>
       </c>
@@ -18905,7 +18905,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="585" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="585" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G585" s="3">
         <v>45993</v>
       </c>
@@ -18933,7 +18933,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="586" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="586" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G586" s="3">
         <v>45993</v>
       </c>
@@ -18961,7 +18961,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="587" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="587" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G587" s="3">
         <v>45993</v>
       </c>
@@ -18989,7 +18989,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="588" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="588" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G588" s="3">
         <v>45993</v>
       </c>
@@ -19017,7 +19017,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="589" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="589" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G589" s="3">
         <v>45993</v>
       </c>
@@ -19045,7 +19045,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="590" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="590" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G590" s="3">
         <v>45993</v>
       </c>
@@ -19073,7 +19073,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="591" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="591" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G591" s="3">
         <v>45993</v>
       </c>
@@ -19105,7 +19105,7 @@
     <row r="593" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="594" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="595" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="596" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="596" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G596" s="3">
         <v>45993</v>
       </c>
@@ -19132,7 +19132,7 @@
       </c>
     </row>
     <row r="597" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="598" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="598" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G598" s="3">
         <v>45994</v>
       </c>
@@ -19156,9 +19156,11 @@
         <v>2</v>
       </c>
       <c r="O598" s="25"/>
-      <c r="P598" s="6"/>
-    </row>
-    <row r="599" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P598" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="599" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G599" s="3">
         <v>45994</v>
       </c>
@@ -19182,9 +19184,11 @@
         <v>2</v>
       </c>
       <c r="O599" s="25"/>
-      <c r="P599" s="6"/>
-    </row>
-    <row r="600" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P599" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="600" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G600" s="3">
         <v>45994</v>
       </c>
@@ -19208,9 +19212,11 @@
         <v>2</v>
       </c>
       <c r="O600" s="25"/>
-      <c r="P600" s="6"/>
-    </row>
-    <row r="601" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P600" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="601" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G601" s="3">
         <v>45994</v>
       </c>
@@ -19234,9 +19240,11 @@
         <v>3</v>
       </c>
       <c r="O601" s="25"/>
-      <c r="P601" s="6"/>
-    </row>
-    <row r="602" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P601" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="602" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G602" s="3">
         <v>45994</v>
       </c>
@@ -19260,9 +19268,11 @@
         <v>2</v>
       </c>
       <c r="O602" s="25"/>
-      <c r="P602" s="6"/>
-    </row>
-    <row r="603" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P602" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="603" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G603" s="3">
         <v>45994</v>
       </c>
@@ -19286,9 +19296,11 @@
         <v>3</v>
       </c>
       <c r="O603" s="25"/>
-      <c r="P603" s="6"/>
-    </row>
-    <row r="604" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P603" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="604" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G604" s="3">
         <v>45994</v>
       </c>
@@ -19312,9 +19324,11 @@
         <v>3</v>
       </c>
       <c r="O604" s="25"/>
-      <c r="P604" s="6"/>
-    </row>
-    <row r="605" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P604" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="605" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G605" s="3">
         <v>45994</v>
       </c>
@@ -19338,9 +19352,11 @@
         <v>2</v>
       </c>
       <c r="O605" s="25"/>
-      <c r="P605" s="6"/>
-    </row>
-    <row r="606" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P605" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="606" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G606" s="3">
         <v>45994</v>
       </c>
@@ -19364,9 +19380,11 @@
         <v>2</v>
       </c>
       <c r="O606" s="25"/>
-      <c r="P606" s="6"/>
-    </row>
-    <row r="607" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P606" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="607" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G607" s="3">
         <v>45995</v>
       </c>
@@ -19382,9 +19400,11 @@
       <c r="M607" s="4"/>
       <c r="N607" s="6"/>
       <c r="O607" s="25"/>
-      <c r="P607" s="6"/>
-    </row>
-    <row r="608" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P607" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="608" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G608" s="3">
         <v>45995</v>
       </c>
@@ -19400,9 +19420,11 @@
       <c r="M608" s="4"/>
       <c r="N608" s="6"/>
       <c r="O608" s="25"/>
-      <c r="P608" s="6"/>
-    </row>
-    <row r="609" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P608" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="609" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G609" s="3">
         <v>45995</v>
       </c>
@@ -19412,15 +19434,21 @@
       <c r="I609" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="J609" s="4"/>
+      <c r="J609" s="4" t="s">
+        <v>192</v>
+      </c>
       <c r="K609" s="8"/>
-      <c r="L609" s="4"/>
+      <c r="L609" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="M609" s="4"/>
       <c r="N609" s="6"/>
       <c r="O609" s="25"/>
-      <c r="P609" s="6"/>
-    </row>
-    <row r="610" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P609" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="610" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G610" s="3">
         <v>45995</v>
       </c>
@@ -19436,9 +19464,11 @@
       <c r="M610" s="4"/>
       <c r="N610" s="6"/>
       <c r="O610" s="25"/>
-      <c r="P610" s="6"/>
-    </row>
-    <row r="611" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P610" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="611" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G611" s="3">
         <v>45995</v>
       </c>
@@ -19454,9 +19484,11 @@
       <c r="M611" s="4"/>
       <c r="N611" s="6"/>
       <c r="O611" s="25"/>
-      <c r="P611" s="6"/>
-    </row>
-    <row r="612" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P611" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="612" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G612" s="3">
         <v>45995</v>
       </c>
@@ -19472,9 +19504,11 @@
       <c r="M612" s="4"/>
       <c r="N612" s="6"/>
       <c r="O612" s="25"/>
-      <c r="P612" s="6"/>
-    </row>
-    <row r="613" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P612" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="613" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G613" s="3">
         <v>45995</v>
       </c>
@@ -19490,9 +19524,11 @@
       <c r="M613" s="4"/>
       <c r="N613" s="6"/>
       <c r="O613" s="25"/>
-      <c r="P613" s="6"/>
-    </row>
-    <row r="614" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P613" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="614" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G614" s="3">
         <v>45995</v>
       </c>
@@ -19508,9 +19544,11 @@
       <c r="M614" s="4"/>
       <c r="N614" s="6"/>
       <c r="O614" s="25"/>
-      <c r="P614" s="6"/>
-    </row>
-    <row r="615" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P614" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="615" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G615" s="3">
         <v>45995</v>
       </c>
@@ -19526,9 +19564,11 @@
       <c r="M615" s="4"/>
       <c r="N615" s="6"/>
       <c r="O615" s="25"/>
-      <c r="P615" s="6"/>
-    </row>
-    <row r="616" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P615" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="616" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G616" s="3">
         <v>45995</v>
       </c>
@@ -19544,9 +19584,11 @@
       <c r="M616" s="4"/>
       <c r="N616" s="6"/>
       <c r="O616" s="25"/>
-      <c r="P616" s="6"/>
-    </row>
-    <row r="617" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P616" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="617" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G617" s="3">
         <v>45995</v>
       </c>
@@ -19562,9 +19604,11 @@
       <c r="M617" s="4"/>
       <c r="N617" s="6"/>
       <c r="O617" s="25"/>
-      <c r="P617" s="6"/>
-    </row>
-    <row r="618" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P617" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="618" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G618" s="3">
         <v>45995</v>
       </c>
@@ -19580,9 +19624,11 @@
       <c r="M618" s="4"/>
       <c r="N618" s="6"/>
       <c r="O618" s="25"/>
-      <c r="P618" s="6"/>
-    </row>
-    <row r="619" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P618" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="619" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G619" s="3">
         <v>45995</v>
       </c>
@@ -19598,9 +19644,11 @@
       <c r="M619" s="4"/>
       <c r="N619" s="6"/>
       <c r="O619" s="25"/>
-      <c r="P619" s="6"/>
-    </row>
-    <row r="620" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P619" s="6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="620" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G620" s="3">
         <v>45995</v>
       </c>
@@ -19616,19 +19664,16 @@
       <c r="M620" s="4"/>
       <c r="N620" s="6"/>
       <c r="O620" s="25"/>
-      <c r="P620" s="6"/>
+      <c r="P620" s="6" t="s">
+        <v>358</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="G5:O620" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="11" dateTimeGrouping="month"/>
+        <dateGroupItem year="2025" month="12" dateTimeGrouping="month"/>
       </filters>
-    </filterColumn>
-    <filterColumn colId="8">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
       <sortCondition ref="G5:G431"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-04 10:10
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="510" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{38972DE8-45AA-45B4-9435-A3DD891BCFF4}"/>
+  <xr:revisionPtr revIDLastSave="511" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDC5F5DE-4970-4068-B053-0924CAD98608}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3611" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3612" uniqueCount="450">
   <si>
     <t>DATA</t>
   </si>
@@ -19638,7 +19638,9 @@
       <c r="I619" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="J619" s="4"/>
+      <c r="J619" s="4" t="s">
+        <v>258</v>
+      </c>
       <c r="K619" s="8"/>
       <c r="L619" s="4"/>
       <c r="M619" s="4"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-04 16:44
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="511" documentId="8_{73A0EBB2-ADEE-482F-AD69-A855E6A79730}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDC5F5DE-4970-4068-B053-0924CAD98608}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="13_ncr:1_{34E05656-CA77-4071-9A18-1B40738BA650}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DF5FA9B-6616-4597-A2BF-7D56A48EED63}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3612" uniqueCount="450">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3632" uniqueCount="458">
   <si>
     <t>DATA</t>
   </si>
@@ -1389,6 +1389,30 @@
   </si>
   <si>
     <t>JOSE</t>
+  </si>
+  <si>
+    <t>hotel casa nova</t>
+  </si>
+  <si>
+    <t>HOTEL GIRA SOL</t>
+  </si>
+  <si>
+    <t>dores do indaia</t>
+  </si>
+  <si>
+    <t>SABINOPOLIS</t>
+  </si>
+  <si>
+    <t>HOTEL SÃO JOAQUIM</t>
+  </si>
+  <si>
+    <t>joão monlevade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRÊS CORAÇÔES </t>
+  </si>
+  <si>
+    <t>HOTEL VALE DAS PRIMAVERA</t>
   </si>
 </sst>
 </file>
@@ -1535,7 +1559,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1661,6 +1685,7 @@
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -2000,7 +2025,7 @@
   <sheetPr codeName="Planilha1" filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="G5:P620"/>
+  <dimension ref="F5:P620"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="10.42578125" style="1" bestFit="1" customWidth="1"/>
@@ -18655,7 +18680,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="576" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="576" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G576" s="3">
         <v>45992</v>
       </c>
@@ -18683,7 +18708,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="577" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="577" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G577" s="3">
         <v>45992</v>
       </c>
@@ -18711,7 +18736,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="578" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="578" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G578" s="3">
         <v>45992</v>
       </c>
@@ -18739,7 +18764,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="579" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="579" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G579" s="3">
         <v>45992</v>
       </c>
@@ -18767,7 +18792,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="580" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="580" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G580" s="3">
         <v>45992</v>
       </c>
@@ -18795,7 +18820,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="581" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="581" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G581" s="3">
         <v>45992</v>
       </c>
@@ -18823,7 +18848,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="582" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="582" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G582" s="3">
         <v>45992</v>
       </c>
@@ -18851,7 +18876,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="583" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="583" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G583" s="3">
         <v>45992</v>
       </c>
@@ -18879,7 +18904,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="584" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="584" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G584" s="3">
         <v>45992</v>
       </c>
@@ -18905,7 +18930,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="585" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="585" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G585" s="3">
         <v>45993</v>
       </c>
@@ -18933,7 +18958,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="586" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="586" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G586" s="3">
         <v>45993</v>
       </c>
@@ -18961,7 +18986,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="587" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="587" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G587" s="3">
         <v>45993</v>
       </c>
@@ -18989,7 +19014,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="588" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="588" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G588" s="3">
         <v>45993</v>
       </c>
@@ -19017,7 +19042,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="589" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="589" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G589" s="3">
         <v>45993</v>
       </c>
@@ -19045,7 +19070,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="590" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="590" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G590" s="3">
         <v>45993</v>
       </c>
@@ -19073,7 +19098,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="591" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="591" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G591" s="3">
         <v>45993</v>
       </c>
@@ -19105,7 +19130,7 @@
     <row r="593" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="594" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="595" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="596" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="596" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G596" s="3">
         <v>45993</v>
       </c>
@@ -19132,7 +19157,7 @@
       </c>
     </row>
     <row r="597" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="598" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="598" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G598" s="3">
         <v>45994</v>
       </c>
@@ -19160,7 +19185,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="599" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="599" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G599" s="3">
         <v>45994</v>
       </c>
@@ -19188,7 +19213,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="600" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="600" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G600" s="3">
         <v>45994</v>
       </c>
@@ -19216,7 +19241,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="601" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="601" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G601" s="3">
         <v>45994</v>
       </c>
@@ -19244,7 +19269,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="602" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="602" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G602" s="3">
         <v>45994</v>
       </c>
@@ -19272,7 +19297,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="603" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="603" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G603" s="3">
         <v>45994</v>
       </c>
@@ -19300,7 +19325,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="604" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="604" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G604" s="3">
         <v>45994</v>
       </c>
@@ -19328,7 +19353,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="605" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="605" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G605" s="3">
         <v>45994</v>
       </c>
@@ -19356,7 +19381,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="606" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="606" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G606" s="3">
         <v>45994</v>
       </c>
@@ -19370,7 +19395,7 @@
         <v>229</v>
       </c>
       <c r="K606" s="8">
-        <v>280</v>
+        <v>240</v>
       </c>
       <c r="L606" s="4" t="s">
         <v>93</v>
@@ -19394,9 +19419,15 @@
       <c r="I607" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="J607" s="4"/>
-      <c r="K607" s="8"/>
-      <c r="L607" s="4"/>
+      <c r="J607" s="4" t="s">
+        <v>453</v>
+      </c>
+      <c r="K607" s="8">
+        <v>200</v>
+      </c>
+      <c r="L607" s="4" t="s">
+        <v>454</v>
+      </c>
       <c r="M607" s="4"/>
       <c r="N607" s="6"/>
       <c r="O607" s="25"/>
@@ -19409,14 +19440,20 @@
         <v>45995</v>
       </c>
       <c r="H608" s="4" t="s">
-        <v>329</v>
+        <v>164</v>
       </c>
       <c r="I608" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="J608" s="4"/>
-      <c r="K608" s="8"/>
-      <c r="L608" s="4"/>
+        <v>173</v>
+      </c>
+      <c r="J608" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="K608" s="8">
+        <v>230</v>
+      </c>
+      <c r="L608" s="4" t="s">
+        <v>193</v>
+      </c>
       <c r="M608" s="4"/>
       <c r="N608" s="6"/>
       <c r="O608" s="25"/>
@@ -19424,22 +19461,24 @@
         <v>358</v>
       </c>
     </row>
-    <row r="609" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="609" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G609" s="3">
         <v>45995</v>
       </c>
       <c r="H609" s="4" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="I609" s="6" t="s">
-        <v>173</v>
+        <v>124</v>
       </c>
       <c r="J609" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="K609" s="8"/>
+        <v>373</v>
+      </c>
+      <c r="K609" s="8">
+        <v>198</v>
+      </c>
       <c r="L609" s="4" t="s">
-        <v>193</v>
+        <v>30</v>
       </c>
       <c r="M609" s="4"/>
       <c r="N609" s="6"/>
@@ -19448,19 +19487,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="610" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="610" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G610" s="3">
         <v>45995</v>
       </c>
       <c r="H610" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="I610" s="6" t="s">
-        <v>359</v>
-      </c>
-      <c r="J610" s="4"/>
-      <c r="K610" s="8"/>
-      <c r="L610" s="4"/>
+        <v>126</v>
+      </c>
+      <c r="J610" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K610" s="8">
+        <v>190</v>
+      </c>
+      <c r="L610" s="4" t="s">
+        <v>451</v>
+      </c>
       <c r="M610" s="4"/>
       <c r="N610" s="6"/>
       <c r="O610" s="25"/>
@@ -19468,19 +19513,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="611" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="611" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G611" s="3">
         <v>45995</v>
       </c>
       <c r="H611" s="4" t="s">
-        <v>153</v>
+        <v>141</v>
       </c>
       <c r="I611" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J611" s="4"/>
-      <c r="K611" s="8"/>
-      <c r="L611" s="4"/>
+        <v>132</v>
+      </c>
+      <c r="J611" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="K611" s="8">
+        <v>200</v>
+      </c>
+      <c r="L611" s="4" t="s">
+        <v>252</v>
+      </c>
       <c r="M611" s="4"/>
       <c r="N611" s="6"/>
       <c r="O611" s="25"/>
@@ -19488,19 +19539,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="612" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="612" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G612" s="3">
         <v>45995</v>
       </c>
       <c r="H612" s="4" t="s">
-        <v>138</v>
+        <v>197</v>
       </c>
       <c r="I612" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J612" s="4"/>
-      <c r="K612" s="8"/>
-      <c r="L612" s="4"/>
+        <v>188</v>
+      </c>
+      <c r="J612" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="K612" s="8">
+        <v>220</v>
+      </c>
+      <c r="L612" s="4" t="s">
+        <v>93</v>
+      </c>
       <c r="M612" s="4"/>
       <c r="N612" s="6"/>
       <c r="O612" s="25"/>
@@ -19508,19 +19565,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="613" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="613" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G613" s="3">
         <v>45995</v>
       </c>
       <c r="H613" s="4" t="s">
-        <v>141</v>
+        <v>206</v>
       </c>
       <c r="I613" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="J613" s="4"/>
-      <c r="K613" s="8"/>
-      <c r="L613" s="4"/>
+        <v>134</v>
+      </c>
+      <c r="J613" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="K613" s="8">
+        <v>276</v>
+      </c>
+      <c r="L613" s="4" t="s">
+        <v>457</v>
+      </c>
       <c r="M613" s="4"/>
       <c r="N613" s="6"/>
       <c r="O613" s="25"/>
@@ -19528,19 +19591,28 @@
         <v>358</v>
       </c>
     </row>
-    <row r="614" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="614" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F614">
+        <v>1</v>
+      </c>
       <c r="G614" s="3">
         <v>45995</v>
       </c>
       <c r="H614" s="4" t="s">
-        <v>197</v>
+        <v>393</v>
       </c>
       <c r="I614" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="J614" s="4"/>
-      <c r="K614" s="8"/>
-      <c r="L614" s="4"/>
+        <v>407</v>
+      </c>
+      <c r="J614" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="K614" s="8">
+        <v>159</v>
+      </c>
+      <c r="L614" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="M614" s="4"/>
       <c r="N614" s="6"/>
       <c r="O614" s="25"/>
@@ -19548,19 +19620,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="615" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="615" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G615" s="3">
         <v>45995</v>
       </c>
       <c r="H615" s="4" t="s">
-        <v>206</v>
+        <v>158</v>
       </c>
       <c r="I615" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="J615" s="4"/>
-      <c r="K615" s="8"/>
-      <c r="L615" s="4"/>
+        <v>360</v>
+      </c>
+      <c r="J615" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K615" s="8">
+        <v>240</v>
+      </c>
+      <c r="L615" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="M615" s="4"/>
       <c r="N615" s="6"/>
       <c r="O615" s="25"/>
@@ -19568,19 +19646,28 @@
         <v>358</v>
       </c>
     </row>
-    <row r="616" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="616" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F616">
+        <v>1</v>
+      </c>
       <c r="G616" s="3">
         <v>45995</v>
       </c>
       <c r="H616" s="4" t="s">
-        <v>393</v>
+        <v>449</v>
       </c>
       <c r="I616" s="6" t="s">
-        <v>407</v>
-      </c>
-      <c r="J616" s="4"/>
-      <c r="K616" s="8"/>
-      <c r="L616" s="4"/>
+        <v>222</v>
+      </c>
+      <c r="J616" s="4" t="s">
+        <v>455</v>
+      </c>
+      <c r="K616" s="8">
+        <v>280</v>
+      </c>
+      <c r="L616" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="M616" s="4"/>
       <c r="N616" s="6"/>
       <c r="O616" s="25"/>
@@ -19588,19 +19675,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="617" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="617" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G617" s="3">
         <v>45995</v>
       </c>
       <c r="H617" s="4" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
       <c r="I617" s="6" t="s">
-        <v>360</v>
-      </c>
-      <c r="J617" s="4"/>
-      <c r="K617" s="8"/>
-      <c r="L617" s="4"/>
+        <v>175</v>
+      </c>
+      <c r="J617" s="4" t="s">
+        <v>258</v>
+      </c>
+      <c r="K617" s="8">
+        <v>266</v>
+      </c>
+      <c r="L617" s="4" t="s">
+        <v>450</v>
+      </c>
       <c r="M617" s="4"/>
       <c r="N617" s="6"/>
       <c r="O617" s="25"/>
@@ -19608,19 +19701,25 @@
         <v>358</v>
       </c>
     </row>
-    <row r="618" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="618" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G618" s="3">
         <v>45995</v>
       </c>
       <c r="H618" s="4" t="s">
-        <v>449</v>
+        <v>152</v>
       </c>
       <c r="I618" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="J618" s="4"/>
-      <c r="K618" s="8"/>
-      <c r="L618" s="4"/>
+        <v>135</v>
+      </c>
+      <c r="J618" s="4" t="s">
+        <v>452</v>
+      </c>
+      <c r="K618" s="8">
+        <v>220</v>
+      </c>
+      <c r="L618" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="M618" s="4"/>
       <c r="N618" s="6"/>
       <c r="O618" s="25"/>
@@ -19628,41 +19727,26 @@
         <v>358</v>
       </c>
     </row>
-    <row r="619" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G619" s="3">
-        <v>45995</v>
-      </c>
-      <c r="H619" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="I619" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="J619" s="4" t="s">
-        <v>258</v>
-      </c>
-      <c r="K619" s="8"/>
-      <c r="L619" s="4"/>
-      <c r="M619" s="4"/>
-      <c r="N619" s="6"/>
-      <c r="O619" s="25"/>
-      <c r="P619" s="6" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="620" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="619" spans="6:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="620" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G620" s="3">
         <v>45995</v>
       </c>
       <c r="H620" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="I620" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J620" s="4"/>
-      <c r="K620" s="8"/>
-      <c r="L620" s="4"/>
+        <v>151</v>
+      </c>
+      <c r="I620" s="53" t="s">
+        <v>390</v>
+      </c>
+      <c r="J620" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="K620" s="8">
+        <v>160</v>
+      </c>
+      <c r="L620" s="4" t="s">
+        <v>118</v>
+      </c>
       <c r="M620" s="4"/>
       <c r="N620" s="6"/>
       <c r="O620" s="25"/>
@@ -19674,7 +19758,7 @@
   <autoFilter ref="G5:O620" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="12" dateTimeGrouping="month"/>
+        <dateGroupItem year="2025" month="12" day="4" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-06 11:27
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="810" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7CA14F9-DD1D-403E-9D70-F0BE104A3A96}"/>
+  <xr:revisionPtr revIDLastSave="854" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAA663B4-30EB-4C3B-906E-A125612CDD0F}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4113" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4144" uniqueCount="486">
   <si>
     <t>DATA</t>
   </si>
@@ -1490,6 +1490,15 @@
   </si>
   <si>
     <t xml:space="preserve">HOTEL MARIO ARMANDO </t>
+  </si>
+  <si>
+    <t>DOUGLAS AL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">JOSE </t>
+  </si>
+  <si>
+    <t>POUSADA BOUGAVILLIA</t>
   </si>
 </sst>
 </file>
@@ -1636,7 +1645,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1760,6 +1769,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -22470,6 +22482,177 @@
         <v>351</v>
       </c>
     </row>
+    <row r="6" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G6" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="I6" t="s">
+        <v>354</v>
+      </c>
+      <c r="N6">
+        <v>2</v>
+      </c>
+      <c r="P6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="7" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G7" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="I7" t="s">
+        <v>133</v>
+      </c>
+      <c r="N7">
+        <v>3</v>
+      </c>
+      <c r="P7" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="8" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G8" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="I8" t="s">
+        <v>129</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>426</v>
+      </c>
+      <c r="K8" s="10">
+        <v>260</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="N8">
+        <v>2</v>
+      </c>
+      <c r="P8" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="9" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G9" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="I9" t="s">
+        <v>213</v>
+      </c>
+      <c r="N9">
+        <v>2</v>
+      </c>
+      <c r="P9" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="10" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G10" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I10" t="s">
+        <v>126</v>
+      </c>
+      <c r="N10">
+        <v>2</v>
+      </c>
+      <c r="P10" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="11" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G11" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="I11" t="s">
+        <v>325</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="10">
+        <v>160</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="N11">
+        <v>3</v>
+      </c>
+      <c r="P11" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G12" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="I12" t="s">
+        <v>395</v>
+      </c>
+      <c r="N12">
+        <v>2</v>
+      </c>
+      <c r="P12" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="13" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G13" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="I13" t="s">
+        <v>206</v>
+      </c>
+      <c r="N13">
+        <v>2</v>
+      </c>
+      <c r="P13" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="14" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G14" s="53">
+        <v>45663</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="I14" t="s">
+        <v>353</v>
+      </c>
+      <c r="N14">
+        <v>2</v>
+      </c>
+      <c r="P14" t="s">
+        <v>352</v>
+      </c>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-06 15:34
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="854" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAA663B4-30EB-4C3B-906E-A125612CDD0F}"/>
+  <xr:revisionPtr revIDLastSave="878" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFC07C10-84C8-465C-9FA9-DBA2722FFD0B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4144" uniqueCount="486">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4153" uniqueCount="490">
   <si>
     <t>DATA</t>
   </si>
@@ -1499,6 +1499,18 @@
   </si>
   <si>
     <t>POUSADA BOUGAVILLIA</t>
+  </si>
+  <si>
+    <t>PIUMHI</t>
+  </si>
+  <si>
+    <t>HOTEL STALO</t>
+  </si>
+  <si>
+    <t>HOTEL MONZA COMFORT</t>
+  </si>
+  <si>
+    <t>HOTEL NOVO</t>
   </si>
 </sst>
 </file>
@@ -10153,7 +10165,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="272" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="272" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G272" s="3">
         <v>45875</v>
       </c>
@@ -10183,7 +10195,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="273" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="273" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G273" s="3">
         <v>45881</v>
       </c>
@@ -10213,7 +10225,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="274" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="274" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G274" s="3">
         <v>45883</v>
       </c>
@@ -10243,7 +10255,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="275" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="275" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G275" s="3">
         <v>45883</v>
       </c>
@@ -10273,7 +10285,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="276" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="276" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G276" s="3">
         <v>45890</v>
       </c>
@@ -10303,7 +10315,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="277" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="277" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G277" s="3">
         <v>45895</v>
       </c>
@@ -10333,7 +10345,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="278" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="278" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G278" s="3">
         <v>45897</v>
       </c>
@@ -10363,7 +10375,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="279" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="279" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G279" s="3">
         <v>45904</v>
       </c>
@@ -10374,7 +10386,7 @@
         <v>129</v>
       </c>
       <c r="J279" s="4" t="s">
-        <v>5</v>
+        <v>226</v>
       </c>
       <c r="K279" s="8">
         <v>220</v>
@@ -15739,6 +15751,11 @@
         <v>352</v>
       </c>
     </row>
+    <row r="461" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="462" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="463" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="464" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="465" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="466" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G466" s="3">
         <v>45972</v>
@@ -16195,6 +16212,7 @@
         <v>352</v>
       </c>
     </row>
+    <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="483" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G483" s="45">
         <v>45974</v>
@@ -16565,7 +16583,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="496" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="496" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G496" s="4"/>
       <c r="H496" s="4"/>
       <c r="I496" s="6"/>
@@ -17281,6 +17299,7 @@
         <v>352</v>
       </c>
     </row>
+    <row r="521" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="522" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G522" s="3">
         <v>45980</v>
@@ -18063,7 +18082,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="550" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="550" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G550" s="3"/>
       <c r="H550" s="4"/>
       <c r="I550" s="6"/>
@@ -18075,7 +18094,7 @@
       <c r="O550" s="25"/>
       <c r="P550" s="6"/>
     </row>
-    <row r="551" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="551" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G551" s="3"/>
       <c r="H551" s="4"/>
       <c r="I551" s="6"/>
@@ -18087,7 +18106,7 @@
       <c r="O551" s="25"/>
       <c r="P551" s="6"/>
     </row>
-    <row r="552" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="552" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G552" s="3"/>
       <c r="H552" s="4"/>
       <c r="I552" s="6"/>
@@ -19199,6 +19218,10 @@
         <v>352</v>
       </c>
     </row>
+    <row r="592" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="593" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="594" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="595" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="596" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G596" s="3">
         <v>45993</v>
@@ -19225,6 +19248,7 @@
         <v>352</v>
       </c>
     </row>
+    <row r="597" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="598" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G598" s="3">
         <v>45994</v>
@@ -19789,6 +19813,7 @@
         <v>352</v>
       </c>
     </row>
+    <row r="619" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="620" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G620" s="3">
         <v>45995</v>
@@ -21113,7 +21138,8 @@
         <v>352</v>
       </c>
     </row>
-    <row r="668" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="667" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="668" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G668" s="3"/>
       <c r="H668" s="4"/>
       <c r="I668" s="6"/>
@@ -22019,7 +22045,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="702" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="702" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G702" s="3">
         <v>46013</v>
       </c>
@@ -22047,7 +22073,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="703" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="703" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G703" s="3">
         <v>46013</v>
       </c>
@@ -22073,7 +22099,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="704" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="704" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G704" s="3">
         <v>46013</v>
       </c>
@@ -22099,7 +22125,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="705" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="705" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G705" s="3">
         <v>46013</v>
       </c>
@@ -22125,7 +22151,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="706" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="706" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G706" s="3">
         <v>46013</v>
       </c>
@@ -22151,7 +22177,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="707" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="707" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G707" s="3">
         <v>46013</v>
       </c>
@@ -22177,7 +22203,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="708" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="708" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G708" s="3">
         <v>46013</v>
       </c>
@@ -22203,7 +22229,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="709" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="709" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G709" s="3">
         <v>46013</v>
       </c>
@@ -22229,7 +22255,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="710" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="710" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G710" s="3">
         <v>46013</v>
       </c>
@@ -22255,7 +22281,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="711" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="711" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G711" s="3">
         <v>46013</v>
       </c>
@@ -22281,7 +22307,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="712" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="712" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G712" s="3">
         <v>46013</v>
       </c>
@@ -22307,7 +22333,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="713" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="713" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G713" s="3">
         <v>46013</v>
       </c>
@@ -22333,7 +22359,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="714" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="714" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G714" s="3">
         <v>46013</v>
       </c>
@@ -22359,7 +22385,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="715" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="715" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G715" s="3">
         <v>46013</v>
       </c>
@@ -22385,7 +22411,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="716" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="716" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G716" s="3">
         <v>46013</v>
       </c>
@@ -22413,9 +22439,9 @@
     </row>
   </sheetData>
   <autoFilter ref="G5:O716" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-    <filterColumn colId="0">
-      <filters blank="1">
-        <dateGroupItem year="2025" month="12" day="22" dateTimeGrouping="day"/>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="PEDRO LEOPOLDO"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
@@ -22492,6 +22518,15 @@
       <c r="I6" t="s">
         <v>354</v>
       </c>
+      <c r="J6" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K6" s="10">
+        <v>240</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>115</v>
+      </c>
       <c r="N6">
         <v>2</v>
       </c>
@@ -22509,6 +22544,15 @@
       <c r="I7" t="s">
         <v>133</v>
       </c>
+      <c r="J7" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="K7" s="10">
+        <v>179.9</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>210</v>
+      </c>
       <c r="N7">
         <v>3</v>
       </c>
@@ -22552,6 +22596,15 @@
       <c r="I9" t="s">
         <v>213</v>
       </c>
+      <c r="J9" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="K9" s="10">
+        <v>280</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>487</v>
+      </c>
       <c r="N9">
         <v>2</v>
       </c>
@@ -22569,6 +22622,15 @@
       <c r="I10" t="s">
         <v>126</v>
       </c>
+      <c r="J10" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="K10" s="10">
+        <v>280</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>488</v>
+      </c>
       <c r="N10">
         <v>2</v>
       </c>
@@ -22612,6 +22674,15 @@
       <c r="I12" t="s">
         <v>395</v>
       </c>
+      <c r="J12" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="K12" s="10">
+        <v>180</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>489</v>
+      </c>
       <c r="N12">
         <v>2</v>
       </c>
@@ -22629,6 +22700,15 @@
       <c r="I13" t="s">
         <v>206</v>
       </c>
+      <c r="J13" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="K13" s="10">
+        <v>200</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>92</v>
+      </c>
       <c r="N13">
         <v>2</v>
       </c>
@@ -22637,21 +22717,7 @@
       </c>
     </row>
     <row r="14" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G14" s="53">
-        <v>45663</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>478</v>
-      </c>
-      <c r="I14" t="s">
-        <v>353</v>
-      </c>
-      <c r="N14">
-        <v>2</v>
-      </c>
-      <c r="P14" t="s">
-        <v>352</v>
-      </c>
+      <c r="G14" s="53"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-07 16:20
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="878" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BFC07C10-84C8-465C-9FA9-DBA2722FFD0B}"/>
+  <xr:revisionPtr revIDLastSave="944" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FDE43C2-75F6-439D-8709-38A01634D64E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$25</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4153" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4193" uniqueCount="495">
   <si>
     <t>DATA</t>
   </si>
@@ -1511,6 +1511,21 @@
   </si>
   <si>
     <t>HOTEL NOVO</t>
+  </si>
+  <si>
+    <t>LUCAS AP</t>
+  </si>
+  <si>
+    <t>WESLEY ANT</t>
+  </si>
+  <si>
+    <t>WESLEY LU</t>
+  </si>
+  <si>
+    <t>são joao evangelista</t>
+  </si>
+  <si>
+    <t>hotel medieval 1</t>
   </si>
 </sst>
 </file>
@@ -1657,7 +1672,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1783,9 +1798,22 @@
     <xf numFmtId="44" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -10165,7 +10193,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="272" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="272" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G272" s="3">
         <v>45875</v>
       </c>
@@ -10195,7 +10223,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="273" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="273" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G273" s="3">
         <v>45881</v>
       </c>
@@ -10225,7 +10253,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="274" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="274" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G274" s="3">
         <v>45883</v>
       </c>
@@ -10255,7 +10283,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="275" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="275" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G275" s="3">
         <v>45883</v>
       </c>
@@ -10285,7 +10313,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="276" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="276" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G276" s="3">
         <v>45890</v>
       </c>
@@ -10315,7 +10343,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="277" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="277" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G277" s="3">
         <v>45895</v>
       </c>
@@ -10345,7 +10373,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="278" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="278" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G278" s="3">
         <v>45897</v>
       </c>
@@ -10375,7 +10403,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="279" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="279" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G279" s="3">
         <v>45904</v>
       </c>
@@ -22045,7 +22073,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="702" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="702" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G702" s="3">
         <v>46013</v>
       </c>
@@ -22073,7 +22101,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="703" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="703" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G703" s="3">
         <v>46013</v>
       </c>
@@ -22099,7 +22127,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="704" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="704" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G704" s="3">
         <v>46013</v>
       </c>
@@ -22125,7 +22153,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="705" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="705" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G705" s="3">
         <v>46013</v>
       </c>
@@ -22151,7 +22179,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="706" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="706" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G706" s="3">
         <v>46013</v>
       </c>
@@ -22177,7 +22205,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="707" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="707" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G707" s="3">
         <v>46013</v>
       </c>
@@ -22203,7 +22231,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="708" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="708" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G708" s="3">
         <v>46013</v>
       </c>
@@ -22229,7 +22257,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="709" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="709" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G709" s="3">
         <v>46013</v>
       </c>
@@ -22255,7 +22283,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="710" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="710" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G710" s="3">
         <v>46013</v>
       </c>
@@ -22281,7 +22309,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="711" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="711" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G711" s="3">
         <v>46013</v>
       </c>
@@ -22307,7 +22335,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="712" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="712" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G712" s="3">
         <v>46013</v>
       </c>
@@ -22333,7 +22361,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="713" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="713" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G713" s="3">
         <v>46013</v>
       </c>
@@ -22359,7 +22387,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="714" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="714" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G714" s="3">
         <v>46013</v>
       </c>
@@ -22385,7 +22413,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="715" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="715" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G715" s="3">
         <v>46013</v>
       </c>
@@ -22411,7 +22439,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="716" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="716" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G716" s="3">
         <v>46013</v>
       </c>
@@ -22439,9 +22467,9 @@
     </row>
   </sheetData>
   <autoFilter ref="G5:O716" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-    <filterColumn colId="3">
+    <filterColumn colId="0">
       <filters>
-        <filter val="PEDRO LEOPOLDO"/>
+        <dateGroupItem year="2025" month="12" day="22" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
@@ -22477,31 +22505,31 @@
   </cols>
   <sheetData>
     <row r="5" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="53" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="53" t="s">
         <v>138</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="54" t="s">
         <v>118</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="L5" s="2" t="s">
+      <c r="K5" s="55" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="2" t="s">
+      <c r="M5" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="O5" s="24" t="s">
+      <c r="O5" s="56" t="s">
         <v>247</v>
       </c>
       <c r="P5" s="40" t="s">
@@ -22509,215 +22537,448 @@
       </c>
     </row>
     <row r="6" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G6" s="53">
+      <c r="G6" s="3">
         <v>45663</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="J6" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="K6" s="10">
+      <c r="K6" s="8">
         <v>240</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="L6" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="N6">
-        <v>2</v>
-      </c>
-      <c r="P6" t="s">
+      <c r="M6" s="4"/>
+      <c r="N6" s="6">
+        <v>2</v>
+      </c>
+      <c r="O6" s="25"/>
+      <c r="P6" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="7" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G7" s="53">
+      <c r="G7" s="3">
         <v>45663</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="4" t="s">
         <v>145</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="4" t="s">
         <v>162</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="8">
         <v>179.9</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="N7">
+      <c r="M7" s="4"/>
+      <c r="N7" s="6">
         <v>3</v>
       </c>
-      <c r="P7" t="s">
+      <c r="O7" s="25"/>
+      <c r="P7" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="8" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G8" s="53">
+      <c r="G8" s="3">
         <v>45663</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="4" t="s">
         <v>426</v>
       </c>
-      <c r="K8" s="10">
+      <c r="K8" s="8">
         <v>260</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="L8" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="N8">
-        <v>2</v>
-      </c>
-      <c r="P8" t="s">
+      <c r="M8" s="4"/>
+      <c r="N8" s="6">
+        <v>2</v>
+      </c>
+      <c r="O8" s="25"/>
+      <c r="P8" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="9" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G9" s="53">
+      <c r="G9" s="3">
         <v>45663</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="H9" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="J9" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="8">
         <v>280</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="L9" s="4" t="s">
         <v>487</v>
       </c>
-      <c r="N9">
-        <v>2</v>
-      </c>
-      <c r="P9" t="s">
+      <c r="M9" s="4"/>
+      <c r="N9" s="6">
+        <v>2</v>
+      </c>
+      <c r="O9" s="25"/>
+      <c r="P9" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="10" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G10" s="53">
+      <c r="G10" s="3">
         <v>45663</v>
       </c>
-      <c r="H10" s="1" t="s">
+      <c r="H10" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="J10" s="1" t="s">
+      <c r="J10" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="8">
         <v>280</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="L10" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="N10">
-        <v>2</v>
-      </c>
-      <c r="P10" t="s">
+      <c r="M10" s="4"/>
+      <c r="N10" s="6">
+        <v>2</v>
+      </c>
+      <c r="O10" s="25"/>
+      <c r="P10" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="11" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G11" s="53">
+      <c r="G11" s="3">
         <v>45663</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="H11" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="J11" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="K11" s="10">
+      <c r="K11" s="8">
         <v>160</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="4" t="s">
         <v>459</v>
       </c>
-      <c r="N11">
+      <c r="M11" s="4"/>
+      <c r="N11" s="6">
         <v>3</v>
       </c>
-      <c r="P11" t="s">
+      <c r="O11" s="25"/>
+      <c r="P11" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="12" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G12" s="53">
+      <c r="G12" s="3">
         <v>45663</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="H12" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="J12" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="K12" s="10">
+      <c r="K12" s="8">
         <v>180</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="L12" s="4" t="s">
         <v>489</v>
       </c>
-      <c r="N12">
-        <v>2</v>
-      </c>
-      <c r="P12" t="s">
+      <c r="M12" s="4"/>
+      <c r="N12" s="6">
+        <v>2</v>
+      </c>
+      <c r="O12" s="25"/>
+      <c r="P12" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="13" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G13" s="53">
+      <c r="G13" s="3">
         <v>45663</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="H13" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="J13" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="K13" s="10">
+      <c r="K13" s="8">
         <v>200</v>
       </c>
-      <c r="L13" s="1" t="s">
+      <c r="L13" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="N13">
-        <v>2</v>
-      </c>
-      <c r="P13" t="s">
+      <c r="M13" s="4"/>
+      <c r="N13" s="6">
+        <v>2</v>
+      </c>
+      <c r="O13" s="25"/>
+      <c r="P13" s="6" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="14" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G14" s="53"/>
+      <c r="G14" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K14" s="8">
+        <v>230</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="M14" s="4"/>
+      <c r="N14" s="6"/>
+      <c r="O14" s="25"/>
+      <c r="P14" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="15" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G15" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="K15" s="8">
+        <v>150</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="M15" s="4"/>
+      <c r="N15" s="6"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="16" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G16" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="K16" s="8">
+        <v>260</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M16" s="4"/>
+      <c r="N16" s="6"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="17" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G17" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K17" s="8">
+        <v>200</v>
+      </c>
+      <c r="L17" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M17" s="4"/>
+      <c r="N17" s="6"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="18" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G18" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H18" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K18" s="8">
+        <v>115</v>
+      </c>
+      <c r="L18" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M18" s="4"/>
+      <c r="N18" s="6"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="19" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G19" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H19" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K19" s="8">
+        <v>85</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M19" s="4"/>
+      <c r="N19" s="6"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="20" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G20" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K20" s="8">
+        <v>190</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M20" s="4"/>
+      <c r="N20" s="6"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="21" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G21" s="3">
+        <v>45664</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K21" s="8">
+        <v>180</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>489</v>
+      </c>
+      <c r="M21" s="4"/>
+      <c r="N21" s="6"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="24" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G24" s="57"/>
+      <c r="H24" s="57"/>
+      <c r="I24" s="58"/>
+      <c r="J24" s="57"/>
+      <c r="K24" s="59"/>
+      <c r="L24" s="57"/>
+      <c r="M24" s="57"/>
+      <c r="N24" s="58"/>
+      <c r="O24" s="60"/>
+      <c r="P24" s="58"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -22750,7 +23011,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O5" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:O25" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="39" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-08 08:48
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="944" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FDE43C2-75F6-439D-8709-38A01634D64E}"/>
+  <xr:revisionPtr revIDLastSave="969" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AB2D066-DA92-4DBE-A2C4-8AD22D823FF3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$29</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4193" uniqueCount="495">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4235" uniqueCount="496">
   <si>
     <t>DATA</t>
   </si>
@@ -1526,6 +1526,9 @@
   </si>
   <si>
     <t>hotel medieval 1</t>
+  </si>
+  <si>
+    <t>JOSE ANT</t>
   </si>
 </sst>
 </file>
@@ -1672,7 +1675,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1806,14 +1809,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -22486,7 +22482,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC7C7783-563A-4FF7-A8A1-9637FFE5F054}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="F5:P682"/>
@@ -22536,7 +22532,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="6" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>45663</v>
       </c>
@@ -22564,7 +22560,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="7" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>45663</v>
       </c>
@@ -22592,7 +22588,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>45663</v>
       </c>
@@ -22620,7 +22616,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="9" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>45663</v>
       </c>
@@ -22648,7 +22644,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="10" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>45663</v>
       </c>
@@ -22676,7 +22672,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="11" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>45663</v>
       </c>
@@ -22704,7 +22700,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>45663</v>
       </c>
@@ -22732,7 +22728,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="13" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>45663</v>
       </c>
@@ -22760,7 +22756,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="14" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>45664</v>
       </c>
@@ -22780,13 +22776,15 @@
         <v>494</v>
       </c>
       <c r="M14" s="4"/>
-      <c r="N14" s="6"/>
+      <c r="N14" s="6">
+        <v>2</v>
+      </c>
       <c r="O14" s="25"/>
       <c r="P14" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="15" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>45664</v>
       </c>
@@ -22812,7 +22810,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="16" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>45664</v>
       </c>
@@ -22838,7 +22836,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="17" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>45664</v>
       </c>
@@ -22864,7 +22862,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="18" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>45664</v>
       </c>
@@ -22890,7 +22888,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="19" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>45664</v>
       </c>
@@ -22916,7 +22914,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>45664</v>
       </c>
@@ -22942,7 +22940,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="21" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>45664</v>
       </c>
@@ -22968,17 +22966,297 @@
         <v>352</v>
       </c>
     </row>
+    <row r="22" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G22" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J22" s="4"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="6"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="23" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G23" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J23" s="4"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="4"/>
+      <c r="M23" s="4"/>
+      <c r="N23" s="6"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
     <row r="24" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G24" s="57"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="58"/>
-      <c r="J24" s="57"/>
-      <c r="K24" s="59"/>
-      <c r="L24" s="57"/>
-      <c r="M24" s="57"/>
-      <c r="N24" s="58"/>
-      <c r="O24" s="60"/>
-      <c r="P24" s="58"/>
+      <c r="G24" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="J24" s="4"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="4"/>
+      <c r="M24" s="4"/>
+      <c r="N24" s="6"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="25" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G25" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="J25" s="4"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="4"/>
+      <c r="M25" s="4"/>
+      <c r="N25" s="6"/>
+      <c r="O25" s="25"/>
+      <c r="P25" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="26" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G26" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J26" s="4"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="4"/>
+      <c r="M26" s="4"/>
+      <c r="N26" s="6"/>
+      <c r="O26" s="25"/>
+      <c r="P26" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="27" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G27" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J27" s="4"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="4"/>
+      <c r="M27" s="4"/>
+      <c r="N27" s="6"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G28" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J28" s="4"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="6"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="29" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G29" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J29" s="4"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="4"/>
+      <c r="M29" s="4"/>
+      <c r="N29" s="6"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="30" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G30" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="I30" s="57" t="s">
+        <v>395</v>
+      </c>
+      <c r="J30" s="4"/>
+      <c r="K30" s="8"/>
+      <c r="L30" s="4"/>
+      <c r="M30" s="4"/>
+      <c r="N30" s="6">
+        <v>2</v>
+      </c>
+      <c r="O30" s="25"/>
+      <c r="P30" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="31" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G31" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I31" s="57" t="s">
+        <v>354</v>
+      </c>
+      <c r="J31" s="4"/>
+      <c r="K31" s="8"/>
+      <c r="L31" s="4"/>
+      <c r="M31" s="4"/>
+      <c r="N31" s="6">
+        <v>2</v>
+      </c>
+      <c r="O31" s="25"/>
+      <c r="P31" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="32" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G32" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="I32" s="57" t="s">
+        <v>215</v>
+      </c>
+      <c r="J32" s="4"/>
+      <c r="K32" s="8"/>
+      <c r="L32" s="4"/>
+      <c r="M32" s="4"/>
+      <c r="N32" s="6">
+        <v>2</v>
+      </c>
+      <c r="O32" s="25"/>
+      <c r="P32" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="33" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G33" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="I33" s="57" t="s">
+        <v>126</v>
+      </c>
+      <c r="J33" s="4"/>
+      <c r="K33" s="8"/>
+      <c r="L33" s="4"/>
+      <c r="M33" s="4"/>
+      <c r="N33" s="6">
+        <v>2</v>
+      </c>
+      <c r="O33" s="25"/>
+      <c r="P33" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="34" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G34" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I34" s="57" t="s">
+        <v>129</v>
+      </c>
+      <c r="J34" s="4"/>
+      <c r="K34" s="8"/>
+      <c r="L34" s="4"/>
+      <c r="M34" s="4"/>
+      <c r="N34" s="6">
+        <v>2</v>
+      </c>
+      <c r="O34" s="25"/>
+      <c r="P34" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="35" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G35" s="3">
+        <v>45665</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I35" s="57" t="s">
+        <v>213</v>
+      </c>
+      <c r="J35" s="4"/>
+      <c r="K35" s="8"/>
+      <c r="L35" s="4"/>
+      <c r="M35" s="4"/>
+      <c r="N35" s="6">
+        <v>2</v>
+      </c>
+      <c r="O35" s="25"/>
+      <c r="P35" s="6" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -23011,7 +23289,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O25" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:O29" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+    <filterColumn colId="0">
+      <filters>
+        <dateGroupItem year="2025" month="1" day="8" dateTimeGrouping="day"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="39" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-09 11:55
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="969" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4AB2D066-DA92-4DBE-A2C4-8AD22D823FF3}"/>
+  <xr:revisionPtr revIDLastSave="1008" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92AD4577-2E2E-420D-BB2D-FDDBA51E55D4}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4235" uniqueCount="496">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4251" uniqueCount="499">
   <si>
     <t>DATA</t>
   </si>
@@ -1529,6 +1529,15 @@
   </si>
   <si>
     <t>JOSE ANT</t>
+  </si>
+  <si>
+    <t>HOTEL GIRASOL</t>
+  </si>
+  <si>
+    <t>HOTEL VITORIA</t>
+  </si>
+  <si>
+    <t>SÃO JOAO DEL REI</t>
   </si>
 </sst>
 </file>
@@ -1675,7 +1684,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1809,7 +1818,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -22971,14 +22979,20 @@
         <v>45665</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="J22" s="4"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="4"/>
+        <v>325</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K22" s="8">
+        <v>180</v>
+      </c>
+      <c r="L22" s="4" t="s">
+        <v>100</v>
+      </c>
       <c r="M22" s="4"/>
       <c r="N22" s="6"/>
       <c r="O22" s="25"/>
@@ -22991,14 +23005,20 @@
         <v>45665</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="J23" s="4"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="4"/>
+        <v>127</v>
+      </c>
+      <c r="J23" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="K23" s="8">
+        <v>260</v>
+      </c>
+      <c r="L23" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="M23" s="4"/>
       <c r="N23" s="6"/>
       <c r="O23" s="25"/>
@@ -23011,14 +23031,20 @@
         <v>45665</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>152</v>
+        <v>490</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="J24" s="4"/>
-      <c r="K24" s="8"/>
-      <c r="L24" s="4"/>
+        <v>172</v>
+      </c>
+      <c r="J24" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K24" s="8">
+        <v>230</v>
+      </c>
+      <c r="L24" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="M24" s="4"/>
       <c r="N24" s="6"/>
       <c r="O24" s="25"/>
@@ -23031,14 +23057,20 @@
         <v>45665</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="J25" s="4"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="4"/>
+        <v>125</v>
+      </c>
+      <c r="J25" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K25" s="8">
+        <v>190</v>
+      </c>
+      <c r="L25" s="4" t="s">
+        <v>496</v>
+      </c>
       <c r="M25" s="4"/>
       <c r="N25" s="6"/>
       <c r="O25" s="25"/>
@@ -23051,14 +23083,20 @@
         <v>45665</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>491</v>
+        <v>325</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J26" s="4"/>
-      <c r="K26" s="8"/>
-      <c r="L26" s="4"/>
+        <v>135</v>
+      </c>
+      <c r="J26" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K26" s="8">
+        <v>150</v>
+      </c>
+      <c r="L26" s="4" t="s">
+        <v>497</v>
+      </c>
       <c r="M26" s="4"/>
       <c r="N26" s="6"/>
       <c r="O26" s="25"/>
@@ -23071,14 +23109,20 @@
         <v>45665</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>325</v>
+        <v>492</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J27" s="4"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="4"/>
+        <v>131</v>
+      </c>
+      <c r="J27" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K27" s="8">
+        <v>200</v>
+      </c>
+      <c r="L27" s="4" t="s">
+        <v>249</v>
+      </c>
       <c r="M27" s="4"/>
       <c r="N27" s="6"/>
       <c r="O27" s="25"/>
@@ -23091,16 +23135,24 @@
         <v>45665</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>492</v>
+        <v>483</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="J28" s="4"/>
-      <c r="K28" s="8"/>
-      <c r="L28" s="4"/>
+        <v>395</v>
+      </c>
+      <c r="J28" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="K28" s="8">
+        <v>209</v>
+      </c>
+      <c r="L28" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="M28" s="4"/>
-      <c r="N28" s="6"/>
+      <c r="N28" s="6">
+        <v>2</v>
+      </c>
       <c r="O28" s="25"/>
       <c r="P28" s="6" t="s">
         <v>352</v>
@@ -23111,16 +23163,24 @@
         <v>45665</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>478</v>
+        <v>157</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="8"/>
-      <c r="L29" s="4"/>
+        <v>354</v>
+      </c>
+      <c r="J29" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K29" s="8">
+        <v>240</v>
+      </c>
+      <c r="L29" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M29" s="4"/>
-      <c r="N29" s="6"/>
+      <c r="N29" s="6">
+        <v>2</v>
+      </c>
       <c r="O29" s="25"/>
       <c r="P29" s="6" t="s">
         <v>352</v>
@@ -23131,14 +23191,20 @@
         <v>45665</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>483</v>
-      </c>
-      <c r="I30" s="57" t="s">
-        <v>395</v>
-      </c>
-      <c r="J30" s="4"/>
-      <c r="K30" s="8"/>
-      <c r="L30" s="4"/>
+        <v>495</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="J30" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="K30" s="8">
+        <v>210</v>
+      </c>
+      <c r="L30" s="4" t="s">
+        <v>412</v>
+      </c>
       <c r="M30" s="4"/>
       <c r="N30" s="6">
         <v>2</v>
@@ -23153,14 +23219,20 @@
         <v>45665</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I31" s="57" t="s">
-        <v>354</v>
-      </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="4"/>
+        <v>242</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="J31" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="K31" s="8">
+        <v>300</v>
+      </c>
+      <c r="L31" s="4" t="s">
+        <v>54</v>
+      </c>
       <c r="M31" s="4"/>
       <c r="N31" s="6">
         <v>2</v>
@@ -23175,14 +23247,20 @@
         <v>45665</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>495</v>
-      </c>
-      <c r="I32" s="57" t="s">
-        <v>215</v>
-      </c>
-      <c r="J32" s="4"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="4"/>
+        <v>147</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K32" s="8">
+        <v>175</v>
+      </c>
+      <c r="L32" s="4" t="s">
+        <v>253</v>
+      </c>
       <c r="M32" s="4"/>
       <c r="N32" s="6">
         <v>2</v>
@@ -23197,10 +23275,10 @@
         <v>45665</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="I33" s="57" t="s">
-        <v>126</v>
+        <v>144</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>213</v>
       </c>
       <c r="J33" s="4"/>
       <c r="K33" s="8"/>
@@ -23211,50 +23289,6 @@
       </c>
       <c r="O33" s="25"/>
       <c r="P33" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="34" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G34" s="3">
-        <v>45665</v>
-      </c>
-      <c r="H34" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="I34" s="57" t="s">
-        <v>129</v>
-      </c>
-      <c r="J34" s="4"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
-      <c r="N34" s="6">
-        <v>2</v>
-      </c>
-      <c r="O34" s="25"/>
-      <c r="P34" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="35" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G35" s="3">
-        <v>45665</v>
-      </c>
-      <c r="H35" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I35" s="57" t="s">
-        <v>213</v>
-      </c>
-      <c r="J35" s="4"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="4"/>
-      <c r="M35" s="4"/>
-      <c r="N35" s="6">
-        <v>2</v>
-      </c>
-      <c r="O35" s="25"/>
-      <c r="P35" s="6" t="s">
         <v>352</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-12 16:17
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1008" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{92AD4577-2E2E-420D-BB2D-FDDBA51E55D4}"/>
+  <xr:revisionPtr revIDLastSave="1066" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E99F9725-D94C-48A0-AD25-72900AFE284E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$40</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4251" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4282" uniqueCount="503">
   <si>
     <t>DATA</t>
   </si>
@@ -1538,6 +1538,18 @@
   </si>
   <si>
     <t>SÃO JOAO DEL REI</t>
+  </si>
+  <si>
+    <t>MATEUS SEVE</t>
+  </si>
+  <si>
+    <t>DOUGLAS ALB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MATHEUS </t>
+  </si>
+  <si>
+    <t>CARMOPOLIS</t>
   </si>
 </sst>
 </file>
@@ -22542,7 +22554,7 @@
     </row>
     <row r="6" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H6" s="4" t="s">
         <v>157</v>
@@ -22570,7 +22582,7 @@
     </row>
     <row r="7" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H7" s="4" t="s">
         <v>145</v>
@@ -22598,7 +22610,7 @@
     </row>
     <row r="8" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H8" s="4" t="s">
         <v>147</v>
@@ -22626,7 +22638,7 @@
     </row>
     <row r="9" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>144</v>
@@ -22654,7 +22666,7 @@
     </row>
     <row r="10" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H10" s="4" t="s">
         <v>242</v>
@@ -22682,7 +22694,7 @@
     </row>
     <row r="11" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H11" s="4" t="s">
         <v>142</v>
@@ -22710,7 +22722,7 @@
     </row>
     <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>483</v>
@@ -22738,7 +22750,7 @@
     </row>
     <row r="13" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
-        <v>45663</v>
+        <v>46028</v>
       </c>
       <c r="H13" s="4" t="s">
         <v>484</v>
@@ -22766,7 +22778,7 @@
     </row>
     <row r="14" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>145</v>
@@ -22794,7 +22806,7 @@
     </row>
     <row r="15" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>142</v>
@@ -22820,7 +22832,7 @@
     </row>
     <row r="16" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>152</v>
@@ -22846,7 +22858,7 @@
     </row>
     <row r="17" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>490</v>
@@ -22872,7 +22884,7 @@
     </row>
     <row r="18" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>491</v>
@@ -22898,7 +22910,7 @@
     </row>
     <row r="19" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>325</v>
@@ -22924,7 +22936,7 @@
     </row>
     <row r="20" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>492</v>
@@ -22950,7 +22962,7 @@
     </row>
     <row r="21" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
-        <v>45664</v>
+        <v>46029</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>478</v>
@@ -22974,9 +22986,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="22" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>142</v>
@@ -23000,9 +23012,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="23" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H23" s="4" t="s">
         <v>152</v>
@@ -23026,9 +23038,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="24" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H24" s="4" t="s">
         <v>490</v>
@@ -23052,9 +23064,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="25" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H25" s="4" t="s">
         <v>491</v>
@@ -23078,9 +23090,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="26" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>325</v>
@@ -23104,9 +23116,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="27" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>492</v>
@@ -23130,9 +23142,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>483</v>
@@ -23158,9 +23170,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="29" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>157</v>
@@ -23186,9 +23198,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="30" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>495</v>
@@ -23214,9 +23226,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="31" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H31" s="4" t="s">
         <v>242</v>
@@ -23242,9 +23254,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="32" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H32" s="4" t="s">
         <v>147</v>
@@ -23270,9 +23282,9 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
-        <v>45665</v>
+        <v>46030</v>
       </c>
       <c r="H33" s="4" t="s">
         <v>144</v>
@@ -23292,6 +23304,226 @@
         <v>352</v>
       </c>
     </row>
+    <row r="34" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G34" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K34" s="8">
+        <v>175</v>
+      </c>
+      <c r="L34" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="M34" s="4"/>
+      <c r="N34" s="6">
+        <v>2</v>
+      </c>
+      <c r="O34" s="25"/>
+      <c r="P34" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="35" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G35" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="K35" s="8">
+        <v>220</v>
+      </c>
+      <c r="L35" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="M35" s="4"/>
+      <c r="N35" s="6">
+        <v>2</v>
+      </c>
+      <c r="O35" s="25"/>
+      <c r="P35" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="36" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G36" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="K36" s="8">
+        <v>159</v>
+      </c>
+      <c r="L36" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="M36" s="4"/>
+      <c r="N36" s="6">
+        <v>2</v>
+      </c>
+      <c r="O36" s="25"/>
+      <c r="P36" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="37" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G37" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="J37" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K37" s="8">
+        <v>200</v>
+      </c>
+      <c r="L37" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M37" s="4"/>
+      <c r="N37" s="6">
+        <v>2</v>
+      </c>
+      <c r="O37" s="25"/>
+      <c r="P37" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="38" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G38" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J38" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K38" s="8">
+        <v>180</v>
+      </c>
+      <c r="L38" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M38" s="4"/>
+      <c r="N38" s="6">
+        <v>2</v>
+      </c>
+      <c r="O38" s="25"/>
+      <c r="P38" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="39" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G39" s="3">
+        <v>46034</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>501</v>
+      </c>
+      <c r="I39" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J39" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K39" s="8">
+        <v>190</v>
+      </c>
+      <c r="L39" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M39" s="4"/>
+      <c r="N39" s="6">
+        <v>2</v>
+      </c>
+      <c r="O39" s="25"/>
+      <c r="P39" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="40" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G40" s="3"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="6"/>
+      <c r="J40" s="4"/>
+      <c r="K40" s="8"/>
+      <c r="L40" s="4"/>
+      <c r="M40" s="4"/>
+      <c r="N40" s="6">
+        <v>2</v>
+      </c>
+      <c r="O40" s="25"/>
+      <c r="P40" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="41" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G41" s="4"/>
+      <c r="H41" s="4"/>
+      <c r="I41" s="6"/>
+      <c r="J41" s="4"/>
+      <c r="K41" s="8"/>
+      <c r="L41" s="4"/>
+      <c r="M41" s="4"/>
+      <c r="N41" s="6"/>
+      <c r="O41" s="25"/>
+      <c r="P41" s="6"/>
+    </row>
+    <row r="42" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G42" s="4"/>
+      <c r="H42" s="4"/>
+      <c r="I42" s="6"/>
+      <c r="J42" s="4"/>
+      <c r="K42" s="8"/>
+      <c r="L42" s="4"/>
+      <c r="M42" s="4"/>
+      <c r="N42" s="6"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="6"/>
+    </row>
+    <row r="43" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G43" s="4"/>
+      <c r="H43" s="4"/>
+      <c r="I43" s="6"/>
+      <c r="J43" s="4"/>
+      <c r="K43" s="8"/>
+      <c r="L43" s="4"/>
+      <c r="M43" s="4"/>
+      <c r="N43" s="6"/>
+      <c r="O43" s="25"/>
+      <c r="P43" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -23323,10 +23555,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O29" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O40" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="1" day="8" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="1" day="12" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-13 15:36
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1094" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1B03678-379A-426E-9B12-566A7EBFF2FB}"/>
+  <xr:revisionPtr revIDLastSave="1128" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B9A2478-E1A1-47EF-82D9-18D006B8A76E}"/>
   <bookViews>
-    <workbookView xWindow="7560" yWindow="3555" windowWidth="18345" windowHeight="11295" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
   <sheets>
     <sheet name="HOTEIS2025" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4317" uniqueCount="505">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4312" uniqueCount="506">
   <si>
     <t>DATA</t>
   </si>
@@ -1556,6 +1556,9 @@
   </si>
   <si>
     <t>ROGERIO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAGO DOS ENCANTOS </t>
   </si>
 </sst>
 </file>
@@ -19100,7 +19103,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="586" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="586" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G586" s="3">
         <v>45993</v>
       </c>
@@ -20196,7 +20199,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="632" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="632" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G632" s="3">
         <v>46000</v>
       </c>
@@ -21319,7 +21322,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="673" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="673" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G673" s="3">
         <v>46007</v>
       </c>
@@ -22095,7 +22098,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="702" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="702" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G702" s="3">
         <v>46013</v>
       </c>
@@ -22123,7 +22126,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="703" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="703" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G703" s="3">
         <v>46013</v>
       </c>
@@ -22149,7 +22152,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="704" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="704" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G704" s="3">
         <v>46013</v>
       </c>
@@ -22201,7 +22204,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="706" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="706" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G706" s="3">
         <v>46013</v>
       </c>
@@ -22227,7 +22230,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="707" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="707" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G707" s="3">
         <v>46013</v>
       </c>
@@ -22253,7 +22256,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="708" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="708" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G708" s="3">
         <v>46013</v>
       </c>
@@ -22279,7 +22282,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="709" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="709" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G709" s="3">
         <v>46013</v>
       </c>
@@ -22305,7 +22308,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="710" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="710" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G710" s="3">
         <v>46013</v>
       </c>
@@ -22331,7 +22334,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="711" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="711" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G711" s="3">
         <v>46013</v>
       </c>
@@ -22357,7 +22360,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="712" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="712" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G712" s="3">
         <v>46013</v>
       </c>
@@ -22383,7 +22386,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="713" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="713" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G713" s="3">
         <v>46013</v>
       </c>
@@ -22409,7 +22412,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="714" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="714" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G714" s="3">
         <v>46013</v>
       </c>
@@ -22435,7 +22438,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="715" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="715" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G715" s="3">
         <v>46013</v>
       </c>
@@ -22461,7 +22464,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="716" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="716" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G716" s="3">
         <v>46013</v>
       </c>
@@ -22491,7 +22494,12 @@
   <autoFilter ref="G5:O716" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="12" day="22" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="12" dateTimeGrouping="month"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="5">
+      <filters>
+        <filter val="POUSADA OASIS"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
@@ -23499,14 +23507,20 @@
         <v>46035</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>147</v>
+        <v>490</v>
       </c>
       <c r="I41" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J41" s="4"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="4"/>
+        <v>172</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K41" s="8">
+        <v>170</v>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>32</v>
+      </c>
       <c r="M41" s="4"/>
       <c r="N41" s="6"/>
       <c r="O41" s="25"/>
@@ -23519,16 +23533,24 @@
         <v>46035</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>499</v>
+        <v>157</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J42" s="4"/>
-      <c r="K42" s="8"/>
-      <c r="L42" s="4"/>
+        <v>354</v>
+      </c>
+      <c r="J42" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" s="8">
+        <v>220</v>
+      </c>
+      <c r="L42" s="4" t="s">
+        <v>12</v>
+      </c>
       <c r="M42" s="4"/>
-      <c r="N42" s="6"/>
+      <c r="N42" s="6">
+        <v>2</v>
+      </c>
       <c r="O42" s="25"/>
       <c r="P42" s="6" t="s">
         <v>352</v>
@@ -23539,16 +23561,24 @@
         <v>46035</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>500</v>
+        <v>145</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>395</v>
-      </c>
-      <c r="J43" s="4"/>
-      <c r="K43" s="8"/>
-      <c r="L43" s="4"/>
+        <v>133</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="K43" s="8">
+        <v>240</v>
+      </c>
+      <c r="L43" s="4" t="s">
+        <v>505</v>
+      </c>
       <c r="M43" s="4"/>
-      <c r="N43" s="6"/>
+      <c r="N43" s="6">
+        <v>3</v>
+      </c>
       <c r="O43" s="25"/>
       <c r="P43" s="6" t="s">
         <v>352</v>
@@ -23559,16 +23589,24 @@
         <v>46035</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>490</v>
+        <v>495</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="J44" s="4"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="4"/>
+        <v>215</v>
+      </c>
+      <c r="J44" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K44" s="8">
+        <v>200</v>
+      </c>
+      <c r="L44" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="M44" s="4"/>
-      <c r="N44" s="6"/>
+      <c r="N44" s="6">
+        <v>2</v>
+      </c>
       <c r="O44" s="25"/>
       <c r="P44" s="6" t="s">
         <v>352</v>
@@ -23579,16 +23617,24 @@
         <v>46035</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>325</v>
+        <v>503</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J45" s="4"/>
-      <c r="K45" s="8"/>
-      <c r="L45" s="4"/>
+        <v>504</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="K45" s="8">
+        <v>280</v>
+      </c>
+      <c r="L45" s="4" t="s">
+        <v>256</v>
+      </c>
       <c r="M45" s="4"/>
-      <c r="N45" s="6"/>
+      <c r="N45" s="6">
+        <v>2</v>
+      </c>
       <c r="O45" s="25"/>
       <c r="P45" s="6" t="s">
         <v>352</v>
@@ -23599,134 +23645,26 @@
         <v>46035</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>501</v>
+        <v>142</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J46" s="4"/>
-      <c r="K46" s="8"/>
-      <c r="L46" s="4"/>
+        <v>325</v>
+      </c>
+      <c r="J46" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K46" s="8">
+        <v>160</v>
+      </c>
+      <c r="L46" s="4" t="s">
+        <v>459</v>
+      </c>
       <c r="M46" s="4"/>
-      <c r="N46" s="6"/>
+      <c r="N46" s="6">
+        <v>3</v>
+      </c>
       <c r="O46" s="25"/>
       <c r="P46" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="47" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G47" s="3">
-        <v>46035</v>
-      </c>
-      <c r="H47" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I47" s="6" t="s">
-        <v>354</v>
-      </c>
-      <c r="J47" s="4"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="4"/>
-      <c r="M47" s="4"/>
-      <c r="N47" s="6">
-        <v>2</v>
-      </c>
-      <c r="O47" s="25"/>
-      <c r="P47" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="48" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G48" s="3">
-        <v>46035</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="I48" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="J48" s="4"/>
-      <c r="K48" s="8"/>
-      <c r="L48" s="4"/>
-      <c r="M48" s="4"/>
-      <c r="N48" s="6">
-        <v>3</v>
-      </c>
-      <c r="O48" s="25"/>
-      <c r="P48" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="49" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G49" s="3">
-        <v>46035</v>
-      </c>
-      <c r="H49" s="4" t="s">
-        <v>495</v>
-      </c>
-      <c r="I49" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="J49" s="4"/>
-      <c r="K49" s="8"/>
-      <c r="L49" s="4"/>
-      <c r="M49" s="4"/>
-      <c r="N49" s="6">
-        <v>2</v>
-      </c>
-      <c r="O49" s="25"/>
-      <c r="P49" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="50" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G50" s="3">
-        <v>46035</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>503</v>
-      </c>
-      <c r="I50" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="J50" s="4"/>
-      <c r="K50" s="8"/>
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="6">
-        <v>2</v>
-      </c>
-      <c r="O50" s="25"/>
-      <c r="P50" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="51" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G51" s="3">
-        <v>46035</v>
-      </c>
-      <c r="H51" s="4" t="s">
-        <v>142</v>
-      </c>
-      <c r="I51" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="J51" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="K51" s="8">
-        <v>160</v>
-      </c>
-      <c r="L51" s="4" t="s">
-        <v>459</v>
-      </c>
-      <c r="M51" s="4"/>
-      <c r="N51" s="6">
-        <v>3</v>
-      </c>
-      <c r="O51" s="25"/>
-      <c r="P51" s="6" t="s">
         <v>352</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-19 11:49
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1332" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA2DF416-C17A-4975-A42D-E485D091D028}"/>
+  <xr:revisionPtr revIDLastSave="1336" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0624558-D589-4FDD-AB05-D56E82FCFA54}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4424" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="513">
   <si>
     <t>DATA</t>
   </si>
@@ -1726,7 +1726,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1869,7 +1869,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -22547,7 +22546,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC7C7783-563A-4FF7-A8A1-9637FFE5F054}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="F5:P682"/>
@@ -22597,7 +22596,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="6" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>46028</v>
       </c>
@@ -22625,7 +22624,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="7" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>46028</v>
       </c>
@@ -22653,7 +22652,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>46028</v>
       </c>
@@ -22681,7 +22680,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="9" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>46028</v>
       </c>
@@ -22709,7 +22708,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="10" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>46028</v>
       </c>
@@ -22737,7 +22736,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="11" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>46028</v>
       </c>
@@ -22765,7 +22764,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>46028</v>
       </c>
@@ -22793,7 +22792,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="13" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>46028</v>
       </c>
@@ -22821,7 +22820,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="14" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>46029</v>
       </c>
@@ -22849,7 +22848,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="15" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>46029</v>
       </c>
@@ -22875,7 +22874,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="16" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>46029</v>
       </c>
@@ -22901,7 +22900,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="17" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>46029</v>
       </c>
@@ -22927,7 +22926,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="18" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>46029</v>
       </c>
@@ -22953,7 +22952,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="19" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>46029</v>
       </c>
@@ -22979,7 +22978,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>46029</v>
       </c>
@@ -23005,7 +23004,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="21" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>46029</v>
       </c>
@@ -23031,7 +23030,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="22" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
         <v>46030</v>
       </c>
@@ -23057,7 +23056,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="23" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
         <v>46030</v>
       </c>
@@ -23083,7 +23082,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="24" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
         <v>46030</v>
       </c>
@@ -23109,7 +23108,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="25" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
         <v>46030</v>
       </c>
@@ -23135,7 +23134,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="26" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
         <v>46030</v>
       </c>
@@ -23161,7 +23160,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="27" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
         <v>46030</v>
       </c>
@@ -23187,7 +23186,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="28" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>46030</v>
       </c>
@@ -23215,7 +23214,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="29" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
         <v>46030</v>
       </c>
@@ -23243,7 +23242,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="30" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
         <v>46030</v>
       </c>
@@ -23271,7 +23270,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="31" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
         <v>46030</v>
       </c>
@@ -23299,7 +23298,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="32" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
         <v>46030</v>
       </c>
@@ -23327,7 +23326,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
         <v>46030</v>
       </c>
@@ -23349,7 +23348,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="34" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G34" s="3">
         <v>46034</v>
       </c>
@@ -23377,7 +23376,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="35" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G35" s="3">
         <v>46034</v>
       </c>
@@ -23405,7 +23404,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="36" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>46034</v>
       </c>
@@ -23433,7 +23432,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="37" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G37" s="3">
         <v>46034</v>
       </c>
@@ -23461,7 +23460,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="38" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G38" s="3">
         <v>46034</v>
       </c>
@@ -23489,7 +23488,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="39" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G39" s="3">
         <v>46034</v>
       </c>
@@ -23533,7 +23532,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="41" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G41" s="59">
         <v>46035</v>
       </c>
@@ -23559,7 +23558,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="42" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G42" s="3">
         <v>46035</v>
       </c>
@@ -23587,7 +23586,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="43" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G43" s="3">
         <v>46035</v>
       </c>
@@ -23615,7 +23614,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="44" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G44" s="3">
         <v>46035</v>
       </c>
@@ -23643,7 +23642,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="45" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G45" s="3">
         <v>46035</v>
       </c>
@@ -23671,7 +23670,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="46" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G46" s="3">
         <v>46035</v>
       </c>
@@ -23699,7 +23698,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="47" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G47" s="3">
         <v>46036</v>
       </c>
@@ -23721,9 +23720,11 @@
       <c r="M47" s="4"/>
       <c r="N47" s="6"/>
       <c r="O47" s="25"/>
-      <c r="P47" s="6"/>
-    </row>
-    <row r="48" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P47" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="48" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G48" s="3">
         <v>46036</v>
       </c>
@@ -23745,9 +23746,11 @@
       <c r="M48" s="4"/>
       <c r="N48" s="6"/>
       <c r="O48" s="25"/>
-      <c r="P48" s="6"/>
-    </row>
-    <row r="49" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P48" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="49" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G49" s="3">
         <v>46036</v>
       </c>
@@ -23769,9 +23772,11 @@
       <c r="M49" s="4"/>
       <c r="N49" s="6"/>
       <c r="O49" s="25"/>
-      <c r="P49" s="6"/>
-    </row>
-    <row r="50" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P49" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="50" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G50" s="3">
         <v>46036</v>
       </c>
@@ -23789,9 +23794,11 @@
         <v>2</v>
       </c>
       <c r="O50" s="25"/>
-      <c r="P50" s="6"/>
-    </row>
-    <row r="51" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P50" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="51" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G51" s="3">
         <v>46036</v>
       </c>
@@ -23815,9 +23822,11 @@
         <v>3</v>
       </c>
       <c r="O51" s="25"/>
-      <c r="P51" s="6"/>
-    </row>
-    <row r="52" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P51" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="52" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G52" s="3">
         <v>46036</v>
       </c>
@@ -23841,9 +23850,11 @@
         <v>3</v>
       </c>
       <c r="O52" s="25"/>
-      <c r="P52" s="6"/>
-    </row>
-    <row r="53" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P52" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="53" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G53" s="3">
         <v>46036</v>
       </c>
@@ -23867,9 +23878,11 @@
         <v>3</v>
       </c>
       <c r="O53" s="25"/>
-      <c r="P53" s="6"/>
-    </row>
-    <row r="54" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P53" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="54" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G54" s="3">
         <v>46036</v>
       </c>
@@ -23893,9 +23906,11 @@
         <v>2</v>
       </c>
       <c r="O54" s="25"/>
-      <c r="P54" s="6"/>
-    </row>
-    <row r="55" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P54" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="55" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G55" s="3">
         <v>46036</v>
       </c>
@@ -23917,9 +23932,11 @@
       <c r="M55" s="31"/>
       <c r="N55" s="29"/>
       <c r="O55" s="37"/>
-      <c r="P55" s="29"/>
-    </row>
-    <row r="56" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P55" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="56" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G56" s="3">
         <v>46037</v>
       </c>
@@ -23941,9 +23958,11 @@
       <c r="M56" s="4"/>
       <c r="N56" s="6"/>
       <c r="O56" s="25"/>
-      <c r="P56" s="6"/>
-    </row>
-    <row r="57" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P56" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="57" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G57" s="3">
         <v>46037</v>
       </c>
@@ -23953,8 +23972,11 @@
       <c r="I57" s="50" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="58" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P57" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="58" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G58" s="3">
         <v>46037</v>
       </c>
@@ -23976,9 +23998,11 @@
       <c r="M58" s="4"/>
       <c r="N58" s="6"/>
       <c r="O58" s="25"/>
-      <c r="P58" s="6"/>
-    </row>
-    <row r="59" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P58" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="59" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G59" s="3">
         <v>46037</v>
       </c>
@@ -24002,9 +24026,11 @@
         <v>1</v>
       </c>
       <c r="O59" s="25"/>
-      <c r="P59" s="6"/>
-    </row>
-    <row r="60" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P59" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="60" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G60" s="3">
         <v>46037</v>
       </c>
@@ -24026,9 +24052,11 @@
       <c r="M60" s="4"/>
       <c r="N60" s="6"/>
       <c r="O60" s="25"/>
-      <c r="P60" s="6"/>
-    </row>
-    <row r="61" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P60" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="61" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G61" s="3">
         <v>46037</v>
       </c>
@@ -24050,9 +24078,11 @@
       <c r="M61" s="4"/>
       <c r="N61" s="6"/>
       <c r="O61" s="25"/>
-      <c r="P61" s="6"/>
-    </row>
-    <row r="62" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P61" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="62" spans="6:16" x14ac:dyDescent="0.25">
       <c r="F62">
         <v>1</v>
       </c>
@@ -24077,9 +24107,11 @@
       <c r="M62" s="4"/>
       <c r="N62" s="6"/>
       <c r="O62" s="25"/>
-      <c r="P62" s="6"/>
-    </row>
-    <row r="63" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P62" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="63" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>46037</v>
       </c>
@@ -24101,9 +24133,11 @@
       <c r="M63" s="4"/>
       <c r="N63" s="6"/>
       <c r="O63" s="25"/>
-      <c r="P63" s="6"/>
-    </row>
-    <row r="64" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P63" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="64" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G64" s="3">
         <v>46037</v>
       </c>
@@ -24127,9 +24161,11 @@
         <v>2</v>
       </c>
       <c r="O64" s="25"/>
-      <c r="P64" s="6"/>
-    </row>
-    <row r="65" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P64" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="65" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G65" s="3">
         <v>46037</v>
       </c>
@@ -24153,9 +24189,11 @@
         <v>2</v>
       </c>
       <c r="O65" s="25"/>
-      <c r="P65" s="6"/>
-    </row>
-    <row r="66" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P65" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="66" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G66" s="3">
         <v>46037</v>
       </c>
@@ -24179,9 +24217,11 @@
         <v>2</v>
       </c>
       <c r="O66" s="25"/>
-      <c r="P66" s="6"/>
-    </row>
-    <row r="67" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P66" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="67" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G67" s="3">
         <v>46037</v>
       </c>
@@ -24205,9 +24245,11 @@
         <v>2</v>
       </c>
       <c r="O67" s="25"/>
-      <c r="P67" s="6"/>
-    </row>
-    <row r="68" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P67" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="68" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G68" s="3">
         <v>46037</v>
       </c>
@@ -24231,9 +24273,11 @@
         <v>2</v>
       </c>
       <c r="O68" s="25"/>
-      <c r="P68" s="6"/>
-    </row>
-    <row r="69" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="P68" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="69" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G69" s="3">
         <v>46037</v>
       </c>
@@ -24255,7 +24299,9 @@
       <c r="M69" s="4"/>
       <c r="N69" s="6"/>
       <c r="O69" s="25"/>
-      <c r="P69" s="6"/>
+      <c r="P69" s="6" t="s">
+        <v>352</v>
+      </c>
     </row>
     <row r="70" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G70" s="3">
@@ -24264,7 +24310,7 @@
       <c r="H70" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="I70" s="60" t="s">
+      <c r="I70" s="6" t="s">
         <v>125</v>
       </c>
       <c r="J70" s="4" t="s">
@@ -24440,13 +24486,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O77" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
-    <filterColumn colId="0">
-      <filters blank="1">
-        <dateGroupItem year="2026" month="1" day="19" dateTimeGrouping="day"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="G5:O77" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="39" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-23 09:03
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1336" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0624558-D589-4FDD-AB05-D56E82FCFA54}"/>
+  <xr:revisionPtr revIDLastSave="1589" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{878BD0F2-71A8-4B5E-A00F-CD4CF396BCCD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$105</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="513">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="525">
   <si>
     <t>DATA</t>
   </si>
@@ -1580,6 +1580,42 @@
   </si>
   <si>
     <t>BOM JESUS</t>
+  </si>
+  <si>
+    <t>BARAO DE COCAIS</t>
+  </si>
+  <si>
+    <t>POUSADA JOAOZINHO</t>
+  </si>
+  <si>
+    <t>POUSADA BARAO DE COCAIS</t>
+  </si>
+  <si>
+    <t>COQUEIRAL</t>
+  </si>
+  <si>
+    <t>BELA VISTA COQUEIRAL</t>
+  </si>
+  <si>
+    <t>JOAO HELIO</t>
+  </si>
+  <si>
+    <t>BRUMADINHO</t>
+  </si>
+  <si>
+    <t>POUSADA TAMBORIL</t>
+  </si>
+  <si>
+    <t>HOTEL ROSA DAS GERAIS</t>
+  </si>
+  <si>
+    <t>HOTEL SANTA RITA</t>
+  </si>
+  <si>
+    <t>TERÊS CORAÇÕES</t>
+  </si>
+  <si>
+    <t>HOTEL TRIANGULO</t>
   </si>
 </sst>
 </file>
@@ -1726,7 +1762,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1863,12 +1899,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -19133,7 +19168,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="586" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="586" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G586" s="3">
         <v>45993</v>
       </c>
@@ -20229,7 +20264,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="632" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="632" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G632" s="3">
         <v>46000</v>
       </c>
@@ -20397,7 +20432,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="638" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="638" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G638" s="3">
         <v>46001</v>
       </c>
@@ -21352,7 +21387,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="673" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="673" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G673" s="3">
         <v>46007</v>
       </c>
@@ -22208,7 +22243,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="705" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="705" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G705" s="3">
         <v>46013</v>
       </c>
@@ -22524,12 +22559,15 @@
   <autoFilter ref="G5:O716" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2025" month="12" dateTimeGrouping="month"/>
+        <dateGroupItem year="2025" month="12" day="8" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="12" day="9" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="12" day="10" dateTimeGrouping="day"/>
+        <dateGroupItem year="2025" month="12" day="11" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
     <filterColumn colId="5">
       <filters>
-        <filter val="POUSADA OASIS"/>
+        <filter val="HOTEL COSTA E FILHO"/>
       </filters>
     </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G16:O431">
@@ -22546,7 +22584,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC7C7783-563A-4FF7-A8A1-9637FFE5F054}">
-  <sheetPr>
+  <sheetPr filterMode="1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="F5:P682"/>
@@ -22596,7 +22634,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="6" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="6" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G6" s="3">
         <v>46028</v>
       </c>
@@ -22624,7 +22662,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="7" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="7" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G7" s="3">
         <v>46028</v>
       </c>
@@ -22652,7 +22690,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="8" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="8" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G8" s="3">
         <v>46028</v>
       </c>
@@ -22680,7 +22718,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="9" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="9" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G9" s="3">
         <v>46028</v>
       </c>
@@ -22708,7 +22746,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="10" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G10" s="3">
         <v>46028</v>
       </c>
@@ -22736,7 +22774,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="11" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="11" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G11" s="3">
         <v>46028</v>
       </c>
@@ -22764,7 +22802,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>46028</v>
       </c>
@@ -22792,7 +22830,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="13" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="13" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G13" s="3">
         <v>46028</v>
       </c>
@@ -22820,7 +22858,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="14" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="14" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G14" s="3">
         <v>46029</v>
       </c>
@@ -22848,7 +22886,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="15" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="15" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G15" s="3">
         <v>46029</v>
       </c>
@@ -22874,7 +22912,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="16" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="16" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G16" s="3">
         <v>46029</v>
       </c>
@@ -22900,7 +22938,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="17" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G17" s="3">
         <v>46029</v>
       </c>
@@ -22926,7 +22964,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="18" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G18" s="3">
         <v>46029</v>
       </c>
@@ -22952,7 +22990,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="19" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G19" s="3">
         <v>46029</v>
       </c>
@@ -22978,7 +23016,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="20" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G20" s="3">
         <v>46029</v>
       </c>
@@ -23004,7 +23042,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="21" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G21" s="3">
         <v>46029</v>
       </c>
@@ -23030,7 +23068,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="22" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G22" s="3">
         <v>46030</v>
       </c>
@@ -23056,7 +23094,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="23" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G23" s="3">
         <v>46030</v>
       </c>
@@ -23082,7 +23120,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="24" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G24" s="3">
         <v>46030</v>
       </c>
@@ -23108,7 +23146,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="25" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G25" s="3">
         <v>46030</v>
       </c>
@@ -23134,7 +23172,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="26" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G26" s="3">
         <v>46030</v>
       </c>
@@ -23160,7 +23198,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="27" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G27" s="3">
         <v>46030</v>
       </c>
@@ -23186,7 +23224,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>46030</v>
       </c>
@@ -23214,7 +23252,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="29" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G29" s="3">
         <v>46030</v>
       </c>
@@ -23242,7 +23280,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="30" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="30" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G30" s="3">
         <v>46030</v>
       </c>
@@ -23270,7 +23308,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="31" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="31" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G31" s="3">
         <v>46030</v>
       </c>
@@ -23298,7 +23336,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="32" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="32" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G32" s="3">
         <v>46030</v>
       </c>
@@ -23326,7 +23364,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="33" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="33" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G33" s="3">
         <v>46030</v>
       </c>
@@ -23348,7 +23386,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="34" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="34" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G34" s="3">
         <v>46034</v>
       </c>
@@ -23376,7 +23414,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="35" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="35" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G35" s="3">
         <v>46034</v>
       </c>
@@ -23404,7 +23442,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="36" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>46034</v>
       </c>
@@ -23432,7 +23470,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="37" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="37" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G37" s="3">
         <v>46034</v>
       </c>
@@ -23460,7 +23498,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="38" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="38" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G38" s="3">
         <v>46034</v>
       </c>
@@ -23488,7 +23526,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="39" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="39" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G39" s="3">
         <v>46034</v>
       </c>
@@ -23516,122 +23554,134 @@
         <v>352</v>
       </c>
     </row>
-    <row r="40" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G40" s="3"/>
-      <c r="H40" s="4"/>
-      <c r="I40" s="6"/>
-      <c r="J40" s="4"/>
-      <c r="K40" s="8"/>
-      <c r="L40" s="4"/>
-      <c r="M40" s="4"/>
-      <c r="N40" s="6">
-        <v>2</v>
-      </c>
-      <c r="O40" s="25"/>
-      <c r="P40" s="6" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="41" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G41" s="59">
+    <row r="40" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G40" s="58">
         <v>46035</v>
       </c>
-      <c r="H41" s="42" t="s">
+      <c r="H40" s="42" t="s">
         <v>490</v>
       </c>
-      <c r="I41" s="28" t="s">
+      <c r="I40" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="J41" s="42" t="s">
+      <c r="J40" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="K41" s="43">
+      <c r="K40" s="43">
         <v>170</v>
       </c>
-      <c r="L41" s="42" t="s">
+      <c r="L40" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="M41" s="42"/>
-      <c r="N41" s="28"/>
-      <c r="O41" s="44"/>
-      <c r="P41" s="28" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="42" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="M40" s="42"/>
+      <c r="N40" s="28"/>
+      <c r="O40" s="44"/>
+      <c r="P40" s="28" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="41" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G41" s="3">
+        <v>46035</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I41" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K41" s="8">
+        <v>220</v>
+      </c>
+      <c r="L41" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M41" s="4"/>
+      <c r="N41" s="6">
+        <v>2</v>
+      </c>
+      <c r="O41" s="25"/>
+      <c r="P41" s="6" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="42" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G42" s="3">
         <v>46035</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="I42" s="6" t="s">
-        <v>354</v>
+        <v>133</v>
       </c>
       <c r="J42" s="4" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="K42" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L42" s="4" t="s">
-        <v>12</v>
+        <v>505</v>
       </c>
       <c r="M42" s="4"/>
       <c r="N42" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O42" s="25"/>
       <c r="P42" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="43" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="43" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G43" s="3">
         <v>46035</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>145</v>
+        <v>495</v>
       </c>
       <c r="I43" s="6" t="s">
-        <v>133</v>
+        <v>215</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="K43" s="8">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="L43" s="4" t="s">
-        <v>505</v>
+        <v>161</v>
       </c>
       <c r="M43" s="4"/>
       <c r="N43" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O43" s="25"/>
       <c r="P43" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="44" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="44" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G44" s="3">
         <v>46035</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="I44" s="6" t="s">
-        <v>215</v>
+        <v>504</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>95</v>
+        <v>400</v>
       </c>
       <c r="K44" s="8">
-        <v>200</v>
+        <v>300</v>
       </c>
       <c r="L44" s="4" t="s">
-        <v>161</v>
+        <v>256</v>
       </c>
       <c r="M44" s="4"/>
       <c r="N44" s="6">
@@ -23642,80 +23692,78 @@
         <v>352</v>
       </c>
     </row>
-    <row r="45" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="45" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G45" s="3">
         <v>46035</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>503</v>
+        <v>142</v>
       </c>
       <c r="I45" s="6" t="s">
-        <v>504</v>
+        <v>325</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>400</v>
+        <v>14</v>
       </c>
       <c r="K45" s="8">
-        <v>300</v>
+        <v>160</v>
       </c>
       <c r="L45" s="4" t="s">
-        <v>256</v>
+        <v>459</v>
       </c>
       <c r="M45" s="4"/>
       <c r="N45" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O45" s="25"/>
       <c r="P45" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="46" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="46" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G46" s="3">
-        <v>46035</v>
+        <v>46036</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>142</v>
+        <v>325</v>
       </c>
       <c r="I46" s="6" t="s">
-        <v>325</v>
+        <v>135</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="K46" s="8">
         <v>160</v>
       </c>
       <c r="L46" s="4" t="s">
-        <v>459</v>
+        <v>506</v>
       </c>
       <c r="M46" s="4"/>
-      <c r="N46" s="6">
-        <v>3</v>
-      </c>
+      <c r="N46" s="6"/>
       <c r="O46" s="25"/>
       <c r="P46" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="47" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="47" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G47" s="3">
         <v>46036</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>325</v>
+        <v>145</v>
       </c>
       <c r="I47" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J47" s="4" t="s">
-        <v>11</v>
+        <v>106</v>
       </c>
       <c r="K47" s="8">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="L47" s="4" t="s">
-        <v>506</v>
+        <v>224</v>
       </c>
       <c r="M47" s="4"/>
       <c r="N47" s="6"/>
@@ -23724,24 +23772,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="48" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="48" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G48" s="3">
         <v>46036</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="I48" s="6" t="s">
-        <v>133</v>
+        <v>325</v>
       </c>
       <c r="J48" s="4" t="s">
-        <v>106</v>
+        <v>432</v>
       </c>
       <c r="K48" s="8">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="L48" s="4" t="s">
-        <v>224</v>
+        <v>433</v>
       </c>
       <c r="M48" s="4"/>
       <c r="N48" s="6"/>
@@ -23750,72 +23798,74 @@
         <v>352</v>
       </c>
     </row>
-    <row r="49" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="49" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G49" s="3">
         <v>46036</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I49" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="J49" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="K49" s="8">
-        <v>200</v>
-      </c>
-      <c r="L49" s="4" t="s">
-        <v>433</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="J49" s="4"/>
+      <c r="K49" s="8"/>
+      <c r="L49" s="4"/>
       <c r="M49" s="4"/>
-      <c r="N49" s="6"/>
+      <c r="N49" s="6">
+        <v>2</v>
+      </c>
       <c r="O49" s="25"/>
       <c r="P49" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="50" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="50" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G50" s="3">
         <v>46036</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>147</v>
+        <v>507</v>
       </c>
       <c r="I50" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="J50" s="4"/>
-      <c r="K50" s="8"/>
-      <c r="L50" s="4"/>
+        <v>213</v>
+      </c>
+      <c r="J50" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K50" s="8">
+        <v>190</v>
+      </c>
+      <c r="L50" s="4" t="s">
+        <v>464</v>
+      </c>
       <c r="M50" s="4"/>
       <c r="N50" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O50" s="25"/>
       <c r="P50" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="51" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="51" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G51" s="3">
         <v>46036</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I51" s="6" t="s">
-        <v>213</v>
+        <v>172</v>
       </c>
       <c r="J51" s="4" t="s">
-        <v>414</v>
+        <v>45</v>
       </c>
       <c r="K51" s="8">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="L51" s="4" t="s">
-        <v>464</v>
+        <v>454</v>
       </c>
       <c r="M51" s="4"/>
       <c r="N51" s="6">
@@ -23826,24 +23876,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="52" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="52" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G52" s="3">
         <v>46036</v>
       </c>
       <c r="H52" s="4" t="s">
-        <v>508</v>
+        <v>491</v>
       </c>
       <c r="I52" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J52" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K52" s="8">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="L52" s="4" t="s">
-        <v>454</v>
+        <v>413</v>
       </c>
       <c r="M52" s="4"/>
       <c r="N52" s="6">
@@ -23854,200 +23904,198 @@
         <v>352</v>
       </c>
     </row>
-    <row r="53" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="53" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G53" s="3">
         <v>46036</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>491</v>
+        <v>205</v>
       </c>
       <c r="I53" s="6" t="s">
-        <v>174</v>
+        <v>126</v>
       </c>
       <c r="J53" s="4" t="s">
-        <v>46</v>
+        <v>359</v>
       </c>
       <c r="K53" s="8">
-        <v>170</v>
+        <v>290</v>
       </c>
       <c r="L53" s="4" t="s">
-        <v>413</v>
+        <v>510</v>
       </c>
       <c r="M53" s="4"/>
       <c r="N53" s="6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O53" s="25"/>
       <c r="P53" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="54" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="54" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G54" s="3">
         <v>46036</v>
       </c>
-      <c r="H54" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="I54" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J54" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="K54" s="8">
-        <v>290</v>
-      </c>
-      <c r="L54" s="4" t="s">
-        <v>510</v>
-      </c>
-      <c r="M54" s="4"/>
-      <c r="N54" s="6">
-        <v>2</v>
-      </c>
-      <c r="O54" s="25"/>
+      <c r="H54" s="31" t="s">
+        <v>509</v>
+      </c>
+      <c r="I54" s="29" t="s">
+        <v>131</v>
+      </c>
+      <c r="J54" s="31" t="s">
+        <v>21</v>
+      </c>
+      <c r="K54" s="32">
+        <v>230</v>
+      </c>
+      <c r="L54" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="M54" s="31"/>
+      <c r="N54" s="29"/>
+      <c r="O54" s="37"/>
       <c r="P54" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="55" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="55" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G55" s="3">
-        <v>46036</v>
-      </c>
-      <c r="H55" s="31" t="s">
-        <v>509</v>
-      </c>
-      <c r="I55" s="29" t="s">
-        <v>131</v>
-      </c>
-      <c r="J55" s="31" t="s">
-        <v>21</v>
-      </c>
-      <c r="K55" s="32">
-        <v>230</v>
-      </c>
-      <c r="L55" s="31" t="s">
-        <v>22</v>
-      </c>
-      <c r="M55" s="31"/>
-      <c r="N55" s="29"/>
-      <c r="O55" s="37"/>
+        <v>46037</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K55" s="8">
+        <v>180</v>
+      </c>
+      <c r="L55" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="M55" s="4"/>
+      <c r="N55" s="6"/>
+      <c r="O55" s="25"/>
       <c r="P55" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="56" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="56" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G56" s="3">
         <v>46037</v>
       </c>
-      <c r="H56" s="4" t="s">
-        <v>325</v>
-      </c>
-      <c r="I56" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="J56" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="K56" s="8">
-        <v>180</v>
-      </c>
-      <c r="L56" s="4" t="s">
-        <v>511</v>
-      </c>
-      <c r="M56" s="4"/>
-      <c r="N56" s="6"/>
-      <c r="O56" s="25"/>
+      <c r="H56" s="57" t="s">
+        <v>145</v>
+      </c>
+      <c r="I56" s="50" t="s">
+        <v>133</v>
+      </c>
       <c r="P56" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="57" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="57" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G57" s="3">
         <v>46037</v>
       </c>
-      <c r="H57" s="57" t="s">
-        <v>145</v>
-      </c>
-      <c r="I57" s="50" t="s">
-        <v>133</v>
-      </c>
+      <c r="H57" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K57" s="8">
+        <v>180</v>
+      </c>
+      <c r="L57" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M57" s="4"/>
+      <c r="N57" s="6"/>
+      <c r="O57" s="25"/>
       <c r="P57" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="58" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="58" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G58" s="3">
         <v>46037</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="I58" s="6" t="s">
-        <v>325</v>
+        <v>129</v>
       </c>
       <c r="J58" s="4" t="s">
-        <v>25</v>
+        <v>226</v>
       </c>
       <c r="K58" s="8">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="L58" s="4" t="s">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="M58" s="4"/>
-      <c r="N58" s="6"/>
+      <c r="N58" s="6">
+        <v>1</v>
+      </c>
       <c r="O58" s="25"/>
       <c r="P58" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="59" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="59" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G59" s="3">
         <v>46037</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>147</v>
+        <v>507</v>
       </c>
       <c r="I59" s="6" t="s">
-        <v>129</v>
+        <v>213</v>
       </c>
       <c r="J59" s="4" t="s">
-        <v>226</v>
+        <v>364</v>
       </c>
       <c r="K59" s="8">
         <v>220</v>
       </c>
       <c r="L59" s="4" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="M59" s="4"/>
-      <c r="N59" s="6">
-        <v>1</v>
-      </c>
+      <c r="N59" s="6"/>
       <c r="O59" s="25"/>
       <c r="P59" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="60" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="60" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G60" s="3">
         <v>46037</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="I60" s="6" t="s">
-        <v>213</v>
+        <v>172</v>
       </c>
       <c r="J60" s="4" t="s">
-        <v>364</v>
+        <v>31</v>
       </c>
       <c r="K60" s="8">
-        <v>220</v>
+        <v>170</v>
       </c>
       <c r="L60" s="4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M60" s="4"/>
       <c r="N60" s="6"/>
@@ -24056,24 +24104,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="61" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="61" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G61" s="3">
         <v>46037</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>508</v>
+        <v>491</v>
       </c>
       <c r="I61" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J61" s="4" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="K61" s="8">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="L61" s="4" t="s">
-        <v>32</v>
+        <v>496</v>
       </c>
       <c r="M61" s="4"/>
       <c r="N61" s="6"/>
@@ -24082,7 +24130,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="62" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="62" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="F62">
         <v>1</v>
       </c>
@@ -24090,19 +24138,19 @@
         <v>46037</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>491</v>
+        <v>509</v>
       </c>
       <c r="I62" s="6" t="s">
-        <v>174</v>
+        <v>131</v>
       </c>
       <c r="J62" s="4" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="K62" s="8">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="L62" s="4" t="s">
-        <v>496</v>
+        <v>249</v>
       </c>
       <c r="M62" s="4"/>
       <c r="N62" s="6"/>
@@ -24111,50 +24159,52 @@
         <v>352</v>
       </c>
     </row>
-    <row r="63" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>46037</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>509</v>
+        <v>500</v>
       </c>
       <c r="I63" s="6" t="s">
-        <v>131</v>
+        <v>395</v>
       </c>
       <c r="J63" s="4" t="s">
-        <v>65</v>
+        <v>498</v>
       </c>
       <c r="K63" s="8">
-        <v>240</v>
+        <v>209</v>
       </c>
       <c r="L63" s="4" t="s">
-        <v>249</v>
+        <v>88</v>
       </c>
       <c r="M63" s="4"/>
-      <c r="N63" s="6"/>
+      <c r="N63" s="6">
+        <v>2</v>
+      </c>
       <c r="O63" s="25"/>
       <c r="P63" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="64" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="64" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G64" s="3">
         <v>46037</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>500</v>
+        <v>157</v>
       </c>
       <c r="I64" s="6" t="s">
-        <v>395</v>
+        <v>354</v>
       </c>
       <c r="J64" s="4" t="s">
-        <v>498</v>
+        <v>41</v>
       </c>
       <c r="K64" s="8">
-        <v>209</v>
+        <v>240</v>
       </c>
       <c r="L64" s="4" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="M64" s="4"/>
       <c r="N64" s="6">
@@ -24165,24 +24215,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="65" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="65" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G65" s="3">
         <v>46037</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>157</v>
+        <v>495</v>
       </c>
       <c r="I65" s="6" t="s">
-        <v>354</v>
+        <v>215</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>41</v>
+        <v>486</v>
       </c>
       <c r="K65" s="8">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="L65" s="4" t="s">
-        <v>115</v>
+        <v>412</v>
       </c>
       <c r="M65" s="4"/>
       <c r="N65" s="6">
@@ -24193,24 +24243,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="66" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="66" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G66" s="3">
         <v>46037</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>495</v>
+        <v>503</v>
       </c>
       <c r="I66" s="6" t="s">
-        <v>215</v>
+        <v>504</v>
       </c>
       <c r="J66" s="4" t="s">
-        <v>486</v>
+        <v>10</v>
       </c>
       <c r="K66" s="8">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="L66" s="4" t="s">
-        <v>412</v>
+        <v>9</v>
       </c>
       <c r="M66" s="4"/>
       <c r="N66" s="6">
@@ -24221,24 +24271,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="67" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="67" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G67" s="3">
         <v>46037</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>503</v>
+        <v>478</v>
       </c>
       <c r="I67" s="6" t="s">
-        <v>504</v>
+        <v>127</v>
       </c>
       <c r="J67" s="4" t="s">
-        <v>10</v>
+        <v>359</v>
       </c>
       <c r="K67" s="8">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="L67" s="4" t="s">
-        <v>9</v>
+        <v>360</v>
       </c>
       <c r="M67" s="4"/>
       <c r="N67" s="6">
@@ -24249,76 +24299,78 @@
         <v>352</v>
       </c>
     </row>
-    <row r="68" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="68" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G68" s="3">
         <v>46037</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>478</v>
+        <v>490</v>
       </c>
       <c r="I68" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J68" s="4" t="s">
-        <v>359</v>
+        <v>270</v>
       </c>
       <c r="K68" s="8">
-        <v>180</v>
+        <v>220</v>
       </c>
       <c r="L68" s="4" t="s">
-        <v>360</v>
+        <v>175</v>
       </c>
       <c r="M68" s="4"/>
-      <c r="N68" s="6">
-        <v>2</v>
-      </c>
+      <c r="N68" s="6"/>
       <c r="O68" s="25"/>
       <c r="P68" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="69" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="69" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G69" s="3">
-        <v>46037</v>
+        <v>46041</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>490</v>
+        <v>508</v>
       </c>
       <c r="I69" s="6" t="s">
         <v>125</v>
       </c>
       <c r="J69" s="4" t="s">
-        <v>270</v>
+        <v>328</v>
       </c>
       <c r="K69" s="8">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="L69" s="4" t="s">
-        <v>175</v>
+        <v>55</v>
       </c>
       <c r="M69" s="4"/>
-      <c r="N69" s="6"/>
+      <c r="N69" s="6">
+        <v>2</v>
+      </c>
       <c r="O69" s="25"/>
       <c r="P69" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="70" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="70" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G70" s="3">
         <v>46041</v>
       </c>
       <c r="H70" s="4" t="s">
-        <v>508</v>
+        <v>325</v>
       </c>
       <c r="I70" s="6" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="J70" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="K70" s="8"/>
+        <v>25</v>
+      </c>
+      <c r="K70" s="8">
+        <v>180</v>
+      </c>
       <c r="L70" s="4" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="M70" s="4"/>
       <c r="N70" s="6">
@@ -24329,24 +24381,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="71" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="71" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G71" s="3">
         <v>46041</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>325</v>
+        <v>147</v>
       </c>
       <c r="I71" s="6" t="s">
-        <v>135</v>
+        <v>174</v>
       </c>
       <c r="J71" s="4" t="s">
-        <v>25</v>
+        <v>252</v>
       </c>
       <c r="K71" s="8">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="L71" s="4" t="s">
-        <v>100</v>
+        <v>512</v>
       </c>
       <c r="M71" s="4"/>
       <c r="N71" s="6">
@@ -24357,22 +24409,24 @@
         <v>352</v>
       </c>
     </row>
-    <row r="72" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>46041</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I72" s="6" t="s">
-        <v>174</v>
+        <v>395</v>
       </c>
       <c r="J72" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="K72" s="8"/>
+        <v>227</v>
+      </c>
+      <c r="K72" s="8">
+        <v>190</v>
+      </c>
       <c r="L72" s="4" t="s">
-        <v>512</v>
+        <v>250</v>
       </c>
       <c r="M72" s="4"/>
       <c r="N72" s="6">
@@ -24383,19 +24437,25 @@
         <v>352</v>
       </c>
     </row>
-    <row r="73" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="73" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G73" s="3">
         <v>46041</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>144</v>
+        <v>490</v>
       </c>
       <c r="I73" s="6" t="s">
-        <v>395</v>
-      </c>
-      <c r="J73" s="4"/>
-      <c r="K73" s="8"/>
-      <c r="L73" s="4"/>
+        <v>213</v>
+      </c>
+      <c r="J73" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K73" s="8">
+        <v>200</v>
+      </c>
+      <c r="L73" s="4" t="s">
+        <v>481</v>
+      </c>
       <c r="M73" s="4"/>
       <c r="N73" s="6">
         <v>2</v>
@@ -24405,19 +24465,25 @@
         <v>352</v>
       </c>
     </row>
-    <row r="74" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="74" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G74" s="3">
         <v>46041</v>
       </c>
       <c r="H74" s="4" t="s">
-        <v>490</v>
+        <v>379</v>
       </c>
       <c r="I74" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="J74" s="4"/>
-      <c r="K74" s="8"/>
-      <c r="L74" s="4"/>
+        <v>124</v>
+      </c>
+      <c r="J74" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K74" s="8">
+        <v>170</v>
+      </c>
+      <c r="L74" s="4" t="s">
+        <v>363</v>
+      </c>
       <c r="M74" s="4"/>
       <c r="N74" s="6">
         <v>2</v>
@@ -24427,33 +24493,719 @@
         <v>352</v>
       </c>
     </row>
-    <row r="75" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="75" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G75" s="3">
-        <v>46041</v>
+        <v>46042</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>379</v>
+        <v>325</v>
       </c>
       <c r="I75" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J75" s="4"/>
-      <c r="K75" s="8"/>
-      <c r="L75" s="4"/>
+        <v>135</v>
+      </c>
+      <c r="J75" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K75" s="8">
+        <v>250</v>
+      </c>
+      <c r="L75" s="4" t="s">
+        <v>506</v>
+      </c>
       <c r="M75" s="4"/>
-      <c r="N75" s="6">
-        <v>2</v>
-      </c>
+      <c r="N75" s="6"/>
       <c r="O75" s="25"/>
       <c r="P75" s="6" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="76" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G76" s="58"/>
-    </row>
-    <row r="77" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G77" s="58"/>
+    <row r="76" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G76" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I76" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J76" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="K76" s="8">
+        <v>240</v>
+      </c>
+      <c r="L76" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="M76" s="4"/>
+      <c r="N76" s="6">
+        <v>3</v>
+      </c>
+      <c r="O76" s="25"/>
+      <c r="P76" s="6"/>
+    </row>
+    <row r="77" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G77" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="J77" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="K77" s="8">
+        <v>160</v>
+      </c>
+      <c r="L77" s="4" t="s">
+        <v>517</v>
+      </c>
+      <c r="M77" s="4"/>
+      <c r="N77" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="78" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G78" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J78" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K78" s="8">
+        <v>205</v>
+      </c>
+      <c r="L78" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="M78" s="4"/>
+      <c r="N78" s="6">
+        <v>2</v>
+      </c>
+      <c r="O78" s="25"/>
+      <c r="P78" s="6"/>
+    </row>
+    <row r="79" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G79" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="J79" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K79" s="8">
+        <v>200</v>
+      </c>
+      <c r="L79" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="M79" s="4"/>
+      <c r="N79" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="80" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G80" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="I80" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="J80" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="K80" s="8">
+        <v>220</v>
+      </c>
+      <c r="L80" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="M80" s="4"/>
+      <c r="N80" s="6">
+        <v>3</v>
+      </c>
+      <c r="O80" s="25"/>
+      <c r="P80" s="6"/>
+    </row>
+    <row r="81" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G81" s="3">
+        <v>46042</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I81" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J81" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K81" s="8">
+        <v>160</v>
+      </c>
+      <c r="L81" s="4" t="s">
+        <v>514</v>
+      </c>
+      <c r="M81" s="4"/>
+      <c r="N81" s="6"/>
+      <c r="O81" s="25"/>
+      <c r="P81" s="6"/>
+    </row>
+    <row r="82" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G82" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K82" s="8">
+        <v>180</v>
+      </c>
+      <c r="L82" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="M82" s="4"/>
+      <c r="N82" s="6"/>
+      <c r="O82" s="25"/>
+      <c r="P82" s="6"/>
+    </row>
+    <row r="83" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G83" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I83" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J83" s="4" t="s">
+        <v>493</v>
+      </c>
+      <c r="K83" s="8">
+        <v>180</v>
+      </c>
+      <c r="L83" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="M83" s="4"/>
+      <c r="N83" s="6"/>
+      <c r="O83" s="25"/>
+      <c r="P83" s="6"/>
+    </row>
+    <row r="84" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G84" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H84" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I84" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J84" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="K84" s="8">
+        <v>240</v>
+      </c>
+      <c r="L84" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="M84" s="4"/>
+      <c r="N84" s="6"/>
+      <c r="O84" s="25"/>
+      <c r="P84" s="6"/>
+    </row>
+    <row r="85" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G85" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H85" s="31" t="s">
+        <v>147</v>
+      </c>
+      <c r="I85" s="29" t="s">
+        <v>124</v>
+      </c>
+      <c r="J85" s="31" t="s">
+        <v>226</v>
+      </c>
+      <c r="K85" s="32">
+        <v>240</v>
+      </c>
+      <c r="L85" s="31" t="s">
+        <v>92</v>
+      </c>
+      <c r="M85" s="4"/>
+      <c r="N85" s="6"/>
+      <c r="O85" s="25"/>
+      <c r="P85" s="6"/>
+    </row>
+    <row r="86" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G86" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="I86" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J86" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K86" s="8">
+        <v>230</v>
+      </c>
+      <c r="L86" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M86" s="4"/>
+      <c r="N86" s="6"/>
+      <c r="O86" s="25"/>
+      <c r="P86" s="6"/>
+    </row>
+    <row r="87" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G87" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="I87" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="J87" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="K87" s="8">
+        <v>280</v>
+      </c>
+      <c r="L87" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="M87" s="4"/>
+      <c r="N87" s="6"/>
+      <c r="O87" s="25"/>
+      <c r="P87" s="6"/>
+    </row>
+    <row r="88" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G88" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I88" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J88" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K88" s="8">
+        <v>170</v>
+      </c>
+      <c r="L88" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M88" s="4"/>
+      <c r="N88" s="6"/>
+      <c r="O88" s="25"/>
+      <c r="P88" s="6"/>
+    </row>
+    <row r="89" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G89" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I89" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J89" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K89" s="8">
+        <v>200</v>
+      </c>
+      <c r="L89" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="M89" s="31"/>
+      <c r="N89" s="29"/>
+    </row>
+    <row r="90" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G90" s="3">
+        <v>46043</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I90" s="6" t="s">
+        <v>518</v>
+      </c>
+      <c r="J90" s="31" t="s">
+        <v>414</v>
+      </c>
+      <c r="K90" s="32">
+        <v>190</v>
+      </c>
+      <c r="L90" s="31" t="s">
+        <v>464</v>
+      </c>
+      <c r="M90" s="31"/>
+      <c r="N90" s="29"/>
+      <c r="O90" s="37"/>
+      <c r="P90" s="29"/>
+    </row>
+    <row r="91" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G91" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="I91" s="60" t="s">
+        <v>504</v>
+      </c>
+      <c r="J91" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="K91" s="8">
+        <v>300</v>
+      </c>
+      <c r="L91" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M91" s="4"/>
+      <c r="N91" s="6"/>
+      <c r="O91" s="25"/>
+      <c r="P91" s="6"/>
+    </row>
+    <row r="92" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G92" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="I92" s="60" t="s">
+        <v>174</v>
+      </c>
+      <c r="J92" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K92" s="8">
+        <v>175</v>
+      </c>
+      <c r="L92" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="M92" s="4"/>
+      <c r="N92" s="6"/>
+      <c r="O92" s="25"/>
+      <c r="P92" s="6"/>
+    </row>
+    <row r="93" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G93" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H93" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="I93" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="J93" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="K93" s="8">
+        <v>220</v>
+      </c>
+      <c r="L93" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="M93" s="4"/>
+      <c r="N93" s="6"/>
+      <c r="O93" s="25"/>
+      <c r="P93" s="6"/>
+    </row>
+    <row r="94" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G94" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H94" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I94" s="60" t="s">
+        <v>354</v>
+      </c>
+      <c r="J94" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K94" s="8">
+        <v>240</v>
+      </c>
+      <c r="L94" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="M94" s="4"/>
+      <c r="N94" s="6"/>
+      <c r="O94" s="25"/>
+      <c r="P94" s="6"/>
+    </row>
+    <row r="95" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G95" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H95" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="I95" s="60" t="s">
+        <v>134</v>
+      </c>
+      <c r="J95" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K95" s="8">
+        <v>190</v>
+      </c>
+      <c r="L95" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="M95" s="4"/>
+      <c r="N95" s="6"/>
+      <c r="O95" s="25"/>
+      <c r="P95" s="6"/>
+    </row>
+    <row r="96" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G96" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H96" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="I96" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="J96" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="K96" s="8">
+        <v>216</v>
+      </c>
+      <c r="L96" s="4" t="s">
+        <v>524</v>
+      </c>
+      <c r="M96" s="4"/>
+      <c r="N96" s="6"/>
+      <c r="O96" s="25"/>
+      <c r="P96" s="6"/>
+    </row>
+    <row r="97" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H97" s="1" t="s">
+        <v>491</v>
+      </c>
+      <c r="I97" s="59" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="98" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H98" s="1" t="s">
+        <v>490</v>
+      </c>
+      <c r="I98" s="59" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="99" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="H99" s="1" t="s">
+        <v>507</v>
+      </c>
+      <c r="I99" s="59" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="100" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G100" s="3"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="6"/>
+      <c r="J100" s="4"/>
+      <c r="K100" s="8"/>
+      <c r="L100" s="4"/>
+      <c r="M100" s="4"/>
+      <c r="N100" s="6"/>
+      <c r="O100" s="25"/>
+      <c r="P100" s="6"/>
+    </row>
+    <row r="101" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G101" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H101" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I101" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J101" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K101" s="8">
+        <v>180</v>
+      </c>
+      <c r="L101" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M101" s="4"/>
+      <c r="N101" s="6"/>
+      <c r="O101" s="25"/>
+      <c r="P101" s="6"/>
+    </row>
+    <row r="102" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G102" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H102" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I102" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J102" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="K102" s="8">
+        <v>240</v>
+      </c>
+      <c r="L102" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="M102" s="4"/>
+      <c r="N102" s="6"/>
+      <c r="O102" s="25"/>
+      <c r="P102" s="6"/>
+    </row>
+    <row r="103" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G103" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H103" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I103" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J103" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K103" s="8">
+        <v>170</v>
+      </c>
+      <c r="L103" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="M103" s="4"/>
+      <c r="N103" s="6"/>
+      <c r="O103" s="25"/>
+      <c r="P103" s="6"/>
+    </row>
+    <row r="104" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G104" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H104" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I104" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J104" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K104" s="8">
+        <v>190</v>
+      </c>
+      <c r="L104" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="M104" s="4"/>
+      <c r="N104" s="6"/>
+      <c r="O104" s="25"/>
+      <c r="P104" s="6"/>
+    </row>
+    <row r="105" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G105" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H105" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I105" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J105" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K105" s="8">
+        <v>230</v>
+      </c>
+      <c r="L105" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="M105" s="4"/>
+      <c r="N105" s="6"/>
+      <c r="O105" s="25"/>
+      <c r="P105" s="6"/>
+    </row>
+    <row r="106" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G106" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H106" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I106" s="60" t="s">
+        <v>215</v>
+      </c>
+      <c r="J106" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="K106" s="8">
+        <v>240</v>
+      </c>
+      <c r="L106" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="M106" s="4"/>
+      <c r="N106" s="6"/>
+      <c r="O106" s="25"/>
+      <c r="P106" s="6"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -24486,7 +25238,13 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O77" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}"/>
+  <autoFilter ref="G5:O105" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+    <filterColumn colId="0">
+      <filters>
+        <dateGroupItem year="2026" month="1" day="22" dateTimeGrouping="day"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="39" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-27 08:21
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1589" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{878BD0F2-71A8-4B5E-A00F-CD4CF396BCCD}"/>
+  <xr:revisionPtr revIDLastSave="1662" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{864D2873-A6E0-44B9-A773-BEB57E0F0714}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$120</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="525">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4611" uniqueCount="528">
   <si>
     <t>DATA</t>
   </si>
@@ -1616,6 +1616,15 @@
   </si>
   <si>
     <t>HOTEL TRIANGULO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LUIS </t>
+  </si>
+  <si>
+    <t>HOTEL PANORAMIC</t>
+  </si>
+  <si>
+    <t>HOTEL SANTA TEREZINHA</t>
   </si>
 </sst>
 </file>
@@ -1762,7 +1771,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1902,8 +1911,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -24883,14 +24890,14 @@
       <c r="O90" s="37"/>
       <c r="P90" s="29"/>
     </row>
-    <row r="91" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="91" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G91" s="3">
         <v>46044</v>
       </c>
       <c r="H91" s="4" t="s">
         <v>242</v>
       </c>
-      <c r="I91" s="60" t="s">
+      <c r="I91" s="6" t="s">
         <v>504</v>
       </c>
       <c r="J91" s="4" t="s">
@@ -24907,14 +24914,14 @@
       <c r="O91" s="25"/>
       <c r="P91" s="6"/>
     </row>
-    <row r="92" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="92" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G92" s="3">
         <v>46044</v>
       </c>
       <c r="H92" s="4" t="s">
         <v>468</v>
       </c>
-      <c r="I92" s="60" t="s">
+      <c r="I92" s="6" t="s">
         <v>174</v>
       </c>
       <c r="J92" s="4" t="s">
@@ -24931,14 +24938,14 @@
       <c r="O92" s="25"/>
       <c r="P92" s="6"/>
     </row>
-    <row r="93" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="93" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G93" s="3">
         <v>46044</v>
       </c>
       <c r="H93" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="I93" s="60" t="s">
+      <c r="I93" s="6" t="s">
         <v>125</v>
       </c>
       <c r="J93" s="4" t="s">
@@ -24955,14 +24962,14 @@
       <c r="O93" s="25"/>
       <c r="P93" s="6"/>
     </row>
-    <row r="94" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="94" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G94" s="3">
         <v>46044</v>
       </c>
       <c r="H94" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="I94" s="60" t="s">
+      <c r="I94" s="6" t="s">
         <v>354</v>
       </c>
       <c r="J94" s="4" t="s">
@@ -24979,14 +24986,14 @@
       <c r="O94" s="25"/>
       <c r="P94" s="6"/>
     </row>
-    <row r="95" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="95" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G95" s="3">
         <v>46044</v>
       </c>
       <c r="H95" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="I95" s="60" t="s">
+      <c r="I95" s="6" t="s">
         <v>134</v>
       </c>
       <c r="J95" s="4" t="s">
@@ -25003,14 +25010,14 @@
       <c r="O95" s="25"/>
       <c r="P95" s="6"/>
     </row>
-    <row r="96" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="96" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G96" s="3">
         <v>46044</v>
       </c>
       <c r="H96" s="4" t="s">
         <v>509</v>
       </c>
-      <c r="I96" s="60" t="s">
+      <c r="I96" s="6" t="s">
         <v>131</v>
       </c>
       <c r="J96" s="4" t="s">
@@ -25031,7 +25038,7 @@
       <c r="H97" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="I97" s="59" t="s">
+      <c r="I97" s="50" t="s">
         <v>195</v>
       </c>
     </row>
@@ -25039,7 +25046,7 @@
       <c r="H98" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="I98" s="59" t="s">
+      <c r="I98" s="50" t="s">
         <v>213</v>
       </c>
     </row>
@@ -25047,7 +25054,7 @@
       <c r="H99" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="I99" s="59" t="s">
+      <c r="I99" s="50" t="s">
         <v>518</v>
       </c>
     </row>
@@ -25063,7 +25070,7 @@
       <c r="O100" s="25"/>
       <c r="P100" s="6"/>
     </row>
-    <row r="101" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="101" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G101" s="3">
         <v>46044</v>
       </c>
@@ -25087,7 +25094,7 @@
       <c r="O101" s="25"/>
       <c r="P101" s="6"/>
     </row>
-    <row r="102" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="102" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G102" s="3">
         <v>46044</v>
       </c>
@@ -25111,7 +25118,7 @@
       <c r="O102" s="25"/>
       <c r="P102" s="6"/>
     </row>
-    <row r="103" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="103" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G103" s="3">
         <v>46044</v>
       </c>
@@ -25135,7 +25142,7 @@
       <c r="O103" s="25"/>
       <c r="P103" s="6"/>
     </row>
-    <row r="104" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="104" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G104" s="3">
         <v>46044</v>
       </c>
@@ -25159,7 +25166,7 @@
       <c r="O104" s="25"/>
       <c r="P104" s="6"/>
     </row>
-    <row r="105" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="105" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G105" s="3">
         <v>46044</v>
       </c>
@@ -25183,14 +25190,14 @@
       <c r="O105" s="25"/>
       <c r="P105" s="6"/>
     </row>
-    <row r="106" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="106" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G106" s="3">
         <v>46044</v>
       </c>
       <c r="H106" s="4" t="s">
         <v>144</v>
       </c>
-      <c r="I106" s="60" t="s">
+      <c r="I106" s="6" t="s">
         <v>215</v>
       </c>
       <c r="J106" s="4" t="s">
@@ -25207,6 +25214,294 @@
       <c r="O106" s="25"/>
       <c r="P106" s="6"/>
     </row>
+    <row r="107" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G107" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H107" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I107" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J107" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K107" s="8">
+        <v>200</v>
+      </c>
+      <c r="L107" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M107" s="4"/>
+      <c r="N107" s="6"/>
+      <c r="O107" s="25"/>
+      <c r="P107" s="6"/>
+    </row>
+    <row r="108" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G108" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H108" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="I108" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J108" s="4" t="s">
+        <v>502</v>
+      </c>
+      <c r="K108" s="8">
+        <v>240</v>
+      </c>
+      <c r="L108" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="M108" s="4"/>
+      <c r="N108" s="6"/>
+      <c r="O108" s="25"/>
+      <c r="P108" s="6"/>
+    </row>
+    <row r="109" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G109" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H109" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="I109" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="J109" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K109" s="8">
+        <v>190</v>
+      </c>
+      <c r="L109" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="M109" s="4"/>
+      <c r="N109" s="6"/>
+      <c r="O109" s="25"/>
+      <c r="P109" s="6"/>
+    </row>
+    <row r="110" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G110" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H110" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="I110" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J110" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K110" s="8">
+        <v>220</v>
+      </c>
+      <c r="L110" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="M110" s="4"/>
+      <c r="N110" s="6"/>
+      <c r="O110" s="25"/>
+      <c r="P110" s="6"/>
+    </row>
+    <row r="111" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G111" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H111" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="I111" s="6" t="s">
+        <v>525</v>
+      </c>
+      <c r="J111" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="K111" s="8">
+        <v>175</v>
+      </c>
+      <c r="L111" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="M111" s="4"/>
+      <c r="N111" s="6"/>
+      <c r="O111" s="25"/>
+      <c r="P111" s="6"/>
+    </row>
+    <row r="112" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G112" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H112" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I112" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J112" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K112" s="8">
+        <v>180</v>
+      </c>
+      <c r="L112" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M112" s="4"/>
+      <c r="N112" s="6"/>
+      <c r="O112" s="25"/>
+      <c r="P112" s="6"/>
+    </row>
+    <row r="113" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G113" s="3">
+        <v>46048</v>
+      </c>
+      <c r="H113" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="I113" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J113" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="K113" s="8">
+        <v>220</v>
+      </c>
+      <c r="L113" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="M113" s="4"/>
+      <c r="N113" s="6"/>
+      <c r="O113" s="25"/>
+      <c r="P113" s="6"/>
+    </row>
+    <row r="114" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G114" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H114" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I114" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J114" s="4"/>
+      <c r="K114" s="8"/>
+      <c r="L114" s="4"/>
+      <c r="M114" s="4"/>
+      <c r="N114" s="6"/>
+      <c r="O114" s="25"/>
+      <c r="P114" s="6"/>
+    </row>
+    <row r="115" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G115" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H115" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I115" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J115" s="4"/>
+      <c r="K115" s="8"/>
+      <c r="L115" s="4"/>
+      <c r="M115" s="4"/>
+      <c r="N115" s="6"/>
+      <c r="O115" s="25"/>
+      <c r="P115" s="6"/>
+    </row>
+    <row r="116" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G116" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H116" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I116" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J116" s="4"/>
+      <c r="K116" s="8"/>
+      <c r="L116" s="4"/>
+      <c r="M116" s="4"/>
+      <c r="N116" s="6"/>
+      <c r="O116" s="25"/>
+      <c r="P116" s="6"/>
+    </row>
+    <row r="117" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G117" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H117" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="I117" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="J117" s="4"/>
+      <c r="K117" s="8"/>
+      <c r="L117" s="4"/>
+      <c r="M117" s="4"/>
+      <c r="N117" s="6"/>
+      <c r="O117" s="25"/>
+      <c r="P117" s="6"/>
+    </row>
+    <row r="118" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G118" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H118" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I118" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="J118" s="4"/>
+      <c r="K118" s="8"/>
+      <c r="L118" s="4"/>
+      <c r="M118" s="4"/>
+      <c r="N118" s="6"/>
+      <c r="O118" s="25"/>
+      <c r="P118" s="6"/>
+    </row>
+    <row r="119" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G119" s="3">
+        <v>46049</v>
+      </c>
+      <c r="H119" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I119" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J119" s="4"/>
+      <c r="K119" s="8"/>
+      <c r="L119" s="4"/>
+      <c r="M119" s="4"/>
+      <c r="N119" s="6"/>
+      <c r="O119" s="25"/>
+      <c r="P119" s="6"/>
+    </row>
+    <row r="120" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G120" s="3"/>
+      <c r="H120" s="4"/>
+      <c r="I120" s="6"/>
+      <c r="J120" s="4"/>
+      <c r="K120" s="8"/>
+      <c r="L120" s="4"/>
+      <c r="M120" s="4"/>
+      <c r="N120" s="6"/>
+      <c r="O120" s="25"/>
+      <c r="P120" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -25238,10 +25533,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O105" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O120" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="1" day="22" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="1" day="27" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-02 15:17
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1944" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1CA4E53E-F98E-4790-B4EC-597246D4782D}"/>
+  <xr:revisionPtr revIDLastSave="1960" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5ACA4CC-4A4C-425A-8370-E852FA72CBD1}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4742" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4751" uniqueCount="544">
   <si>
     <t>DATA</t>
   </si>
@@ -26292,9 +26292,15 @@
       <c r="I152" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J152" s="4"/>
-      <c r="K152" s="8"/>
-      <c r="L152" s="4"/>
+      <c r="J152" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K152" s="8">
+        <v>200</v>
+      </c>
+      <c r="L152" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="M152" s="4"/>
       <c r="N152" s="6"/>
       <c r="O152" s="25"/>
@@ -26344,9 +26350,15 @@
         <v>543</v>
       </c>
       <c r="I155" s="6"/>
-      <c r="J155" s="4"/>
-      <c r="K155" s="8"/>
-      <c r="L155" s="4"/>
+      <c r="J155" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K155" s="8">
+        <v>100</v>
+      </c>
+      <c r="L155" s="4" t="s">
+        <v>100</v>
+      </c>
       <c r="M155" s="4"/>
       <c r="N155" s="6"/>
       <c r="O155" s="25"/>
@@ -26362,8 +26374,12 @@
       <c r="I156" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="J156" s="4"/>
-      <c r="K156" s="8"/>
+      <c r="J156" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K156" s="8">
+        <v>200</v>
+      </c>
       <c r="L156" s="4"/>
       <c r="M156" s="4"/>
       <c r="N156" s="6"/>
@@ -26371,12 +26387,24 @@
       <c r="P156" s="6"/>
     </row>
     <row r="157" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G157" s="4"/>
-      <c r="H157" s="4"/>
-      <c r="I157" s="6"/>
-      <c r="J157" s="4"/>
-      <c r="K157" s="8"/>
-      <c r="L157" s="4"/>
+      <c r="G157" s="3">
+        <v>46055</v>
+      </c>
+      <c r="H157" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="I157" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J157" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="K157" s="8">
+        <v>220</v>
+      </c>
+      <c r="L157" s="4" t="s">
+        <v>175</v>
+      </c>
       <c r="M157" s="4"/>
       <c r="N157" s="6"/>
       <c r="O157" s="25"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-03 11:18
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1960" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5ACA4CC-4A4C-425A-8370-E852FA72CBD1}"/>
+  <xr:revisionPtr revIDLastSave="1977" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0CF3005-2139-4991-BF27-B16F2B83E16D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$157</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4751" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4771" uniqueCount="544">
   <si>
     <t>DATA</t>
   </si>
@@ -26248,7 +26248,7 @@
         <v>226</v>
       </c>
       <c r="K150" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L150" s="4" t="s">
         <v>92</v>
@@ -26316,9 +26316,15 @@
       <c r="I153" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="J153" s="4"/>
-      <c r="K153" s="8"/>
-      <c r="L153" s="4"/>
+      <c r="J153" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K153" s="8">
+        <v>190</v>
+      </c>
+      <c r="L153" s="4" t="s">
+        <v>250</v>
+      </c>
       <c r="M153" s="4"/>
       <c r="N153" s="6"/>
       <c r="O153" s="25"/>
@@ -26334,9 +26340,15 @@
       <c r="I154" s="6" t="s">
         <v>534</v>
       </c>
-      <c r="J154" s="4"/>
-      <c r="K154" s="8"/>
-      <c r="L154" s="4"/>
+      <c r="J154" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K154" s="8">
+        <v>240</v>
+      </c>
+      <c r="L154" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="M154" s="4"/>
       <c r="N154" s="6"/>
       <c r="O154" s="25"/>
@@ -26380,7 +26392,9 @@
       <c r="K156" s="8">
         <v>200</v>
       </c>
-      <c r="L156" s="4"/>
+      <c r="L156" s="4" t="s">
+        <v>100</v>
+      </c>
       <c r="M156" s="4"/>
       <c r="N156" s="6"/>
       <c r="O156" s="25"/>
@@ -26411,9 +26425,15 @@
       <c r="P157" s="6"/>
     </row>
     <row r="158" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G158" s="4"/>
-      <c r="H158" s="4"/>
-      <c r="I158" s="6"/>
+      <c r="G158" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H158" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I158" s="6" t="s">
+        <v>174</v>
+      </c>
       <c r="J158" s="4"/>
       <c r="K158" s="8"/>
       <c r="L158" s="4"/>
@@ -26423,9 +26443,15 @@
       <c r="P158" s="6"/>
     </row>
     <row r="159" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G159" s="4"/>
-      <c r="H159" s="4"/>
-      <c r="I159" s="6"/>
+      <c r="G159" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H159" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I159" s="6" t="s">
+        <v>129</v>
+      </c>
       <c r="J159" s="4"/>
       <c r="K159" s="8"/>
       <c r="L159" s="4"/>
@@ -26435,9 +26461,15 @@
       <c r="P159" s="6"/>
     </row>
     <row r="160" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G160" s="4"/>
-      <c r="H160" s="4"/>
-      <c r="I160" s="6"/>
+      <c r="G160" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H160" s="4" t="s">
+        <v>541</v>
+      </c>
+      <c r="I160" s="6" t="s">
+        <v>124</v>
+      </c>
       <c r="J160" s="4"/>
       <c r="K160" s="8"/>
       <c r="L160" s="4"/>
@@ -26447,9 +26479,15 @@
       <c r="P160" s="6"/>
     </row>
     <row r="161" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G161" s="4"/>
-      <c r="H161" s="4"/>
-      <c r="I161" s="6"/>
+      <c r="G161" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H161" s="4" t="s">
+        <v>483</v>
+      </c>
+      <c r="I161" s="6" t="s">
+        <v>395</v>
+      </c>
       <c r="J161" s="4"/>
       <c r="K161" s="8"/>
       <c r="L161" s="4"/>
@@ -26458,6 +26496,100 @@
       <c r="O161" s="25"/>
       <c r="P161" s="6"/>
     </row>
+    <row r="162" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G162" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H162" s="4" t="s">
+        <v>542</v>
+      </c>
+      <c r="I162" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="J162" s="4"/>
+      <c r="K162" s="8"/>
+      <c r="L162" s="4"/>
+      <c r="M162" s="4"/>
+      <c r="N162" s="6"/>
+      <c r="O162" s="25"/>
+      <c r="P162" s="6"/>
+    </row>
+    <row r="163" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G163" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H163" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="I163" s="6"/>
+      <c r="J163" s="4"/>
+      <c r="K163" s="8"/>
+      <c r="L163" s="4"/>
+      <c r="M163" s="4"/>
+      <c r="N163" s="6"/>
+      <c r="O163" s="25"/>
+      <c r="P163" s="6"/>
+    </row>
+    <row r="164" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G164" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H164" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="I164" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J164" s="4"/>
+      <c r="K164" s="8"/>
+      <c r="L164" s="4"/>
+      <c r="M164" s="4"/>
+      <c r="N164" s="6"/>
+      <c r="O164" s="25"/>
+      <c r="P164" s="6"/>
+    </row>
+    <row r="165" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G165" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H165" s="4" t="s">
+        <v>533</v>
+      </c>
+      <c r="I165" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J165" s="4"/>
+      <c r="K165" s="8"/>
+      <c r="L165" s="4"/>
+      <c r="M165" s="4"/>
+      <c r="N165" s="6"/>
+      <c r="O165" s="25"/>
+      <c r="P165" s="6"/>
+    </row>
+    <row r="166" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G166" s="4"/>
+      <c r="H166" s="4"/>
+      <c r="I166" s="6"/>
+      <c r="J166" s="4"/>
+      <c r="K166" s="8"/>
+      <c r="L166" s="4"/>
+      <c r="M166" s="4"/>
+      <c r="N166" s="6"/>
+      <c r="O166" s="25"/>
+      <c r="P166" s="6"/>
+    </row>
+    <row r="167" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G167" s="4"/>
+      <c r="H167" s="4"/>
+      <c r="I167" s="6"/>
+      <c r="J167" s="4"/>
+      <c r="K167" s="8"/>
+      <c r="L167" s="4"/>
+      <c r="M167" s="4"/>
+      <c r="N167" s="6"/>
+      <c r="O167" s="25"/>
+      <c r="P167" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -26489,7 +26621,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O156" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O157" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2026" month="2" dateTimeGrouping="month"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-03 11:53
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1977" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0CF3005-2139-4991-BF27-B16F2B83E16D}"/>
+  <xr:revisionPtr revIDLastSave="1999" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B52CF7E-4928-4DB7-8E0A-9D4D2808EF00}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
+    <workbookView minimized="1" xWindow="10455" yWindow="4185" windowWidth="18345" windowHeight="11295" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
   <sheets>
     <sheet name="HOTEIS2025" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$157</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$171</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4771" uniqueCount="544">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4787" uniqueCount="550">
   <si>
     <t>DATA</t>
   </si>
@@ -1673,6 +1673,24 @@
   </si>
   <si>
     <t>RICARDO DE OLIVEIRA</t>
+  </si>
+  <si>
+    <t>jose ant</t>
+  </si>
+  <si>
+    <t>elder</t>
+  </si>
+  <si>
+    <t>geraldo</t>
+  </si>
+  <si>
+    <t>marcelo</t>
+  </si>
+  <si>
+    <t>lucas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jose </t>
   </si>
 </sst>
 </file>
@@ -1819,7 +1837,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1959,6 +1977,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -26234,7 +26253,7 @@
       <c r="O149" s="25"/>
       <c r="P149" s="6"/>
     </row>
-    <row r="150" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="150" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G150" s="3">
         <v>46055</v>
       </c>
@@ -26258,7 +26277,7 @@
       <c r="O150" s="25"/>
       <c r="P150" s="6"/>
     </row>
-    <row r="151" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="151" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G151" s="3">
         <v>46055</v>
       </c>
@@ -26282,7 +26301,7 @@
       <c r="O151" s="25"/>
       <c r="P151" s="6"/>
     </row>
-    <row r="152" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="152" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G152" s="3">
         <v>46055</v>
       </c>
@@ -26306,7 +26325,7 @@
       <c r="O152" s="25"/>
       <c r="P152" s="6"/>
     </row>
-    <row r="153" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>46055</v>
       </c>
@@ -26330,7 +26349,7 @@
       <c r="O153" s="25"/>
       <c r="P153" s="6"/>
     </row>
-    <row r="154" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="154" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G154" s="3">
         <v>46055</v>
       </c>
@@ -26354,7 +26373,7 @@
       <c r="O154" s="25"/>
       <c r="P154" s="6"/>
     </row>
-    <row r="155" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="155" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G155" s="3">
         <v>46055</v>
       </c>
@@ -26376,7 +26395,7 @@
       <c r="O155" s="25"/>
       <c r="P155" s="6"/>
     </row>
-    <row r="156" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>46055</v>
       </c>
@@ -26400,7 +26419,7 @@
       <c r="O156" s="25"/>
       <c r="P156" s="6"/>
     </row>
-    <row r="157" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="157" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G157" s="3">
         <v>46055</v>
       </c>
@@ -26434,9 +26453,13 @@
       <c r="I158" s="6" t="s">
         <v>174</v>
       </c>
-      <c r="J158" s="4"/>
+      <c r="J158" s="4" t="s">
+        <v>226</v>
+      </c>
       <c r="K158" s="8"/>
-      <c r="L158" s="4"/>
+      <c r="L158" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="M158" s="4"/>
       <c r="N158" s="6"/>
       <c r="O158" s="25"/>
@@ -26567,21 +26590,39 @@
       <c r="P165" s="6"/>
     </row>
     <row r="166" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G166" s="4"/>
-      <c r="H166" s="4"/>
-      <c r="I166" s="6"/>
-      <c r="J166" s="4"/>
-      <c r="K166" s="8"/>
-      <c r="L166" s="4"/>
+      <c r="G166" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H166" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I166" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J166" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K166" s="8">
+        <v>240</v>
+      </c>
+      <c r="L166" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M166" s="4"/>
       <c r="N166" s="6"/>
       <c r="O166" s="25"/>
       <c r="P166" s="6"/>
     </row>
     <row r="167" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G167" s="4"/>
-      <c r="H167" s="4"/>
-      <c r="I167" s="6"/>
+      <c r="G167" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H167" s="4" t="s">
+        <v>544</v>
+      </c>
+      <c r="I167" s="6" t="s">
+        <v>545</v>
+      </c>
       <c r="J167" s="4"/>
       <c r="K167" s="8"/>
       <c r="L167" s="4"/>
@@ -26590,6 +26631,78 @@
       <c r="O167" s="25"/>
       <c r="P167" s="6"/>
     </row>
+    <row r="168" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G168" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H168" s="4" t="s">
+        <v>546</v>
+      </c>
+      <c r="I168" s="59" t="s">
+        <v>547</v>
+      </c>
+      <c r="J168" s="4"/>
+      <c r="K168" s="8"/>
+      <c r="L168" s="4"/>
+      <c r="M168" s="4"/>
+      <c r="N168" s="6"/>
+      <c r="O168" s="25"/>
+      <c r="P168" s="6"/>
+    </row>
+    <row r="169" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G169" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H169" s="4" t="s">
+        <v>532</v>
+      </c>
+      <c r="I169" s="59" t="s">
+        <v>548</v>
+      </c>
+      <c r="J169" s="4"/>
+      <c r="K169" s="8"/>
+      <c r="L169" s="4"/>
+      <c r="M169" s="4"/>
+      <c r="N169" s="6"/>
+      <c r="O169" s="25"/>
+      <c r="P169" s="6"/>
+    </row>
+    <row r="170" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G170" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H170" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="I170" s="59" t="s">
+        <v>504</v>
+      </c>
+      <c r="J170" s="4"/>
+      <c r="K170" s="8"/>
+      <c r="L170" s="4"/>
+      <c r="M170" s="4"/>
+      <c r="N170" s="6"/>
+      <c r="O170" s="25"/>
+      <c r="P170" s="6"/>
+    </row>
+    <row r="171" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G171" s="3">
+        <v>46056</v>
+      </c>
+      <c r="H171" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="I171" s="59" t="s">
+        <v>325</v>
+      </c>
+      <c r="J171" s="4"/>
+      <c r="K171" s="8"/>
+      <c r="L171" s="4"/>
+      <c r="M171" s="4"/>
+      <c r="N171" s="6"/>
+      <c r="O171" s="25"/>
+      <c r="P171" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -26621,10 +26734,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O157" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O171" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="2" dateTimeGrouping="month"/>
+        <dateGroupItem year="2026" month="2" day="3" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-03 15:27
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1999" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B52CF7E-4928-4DB7-8E0A-9D4D2808EF00}"/>
+  <xr:revisionPtr revIDLastSave="2020" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95FB586B-16F0-4E85-B5AE-534A064B7775}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="10455" yWindow="4185" windowWidth="18345" windowHeight="11295" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
   <sheets>
     <sheet name="HOTEIS2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4787" uniqueCount="550">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4789" uniqueCount="552">
   <si>
     <t>DATA</t>
   </si>
@@ -1691,6 +1691,12 @@
   </si>
   <si>
     <t xml:space="preserve">jose </t>
+  </si>
+  <si>
+    <t>hotel santos dummont</t>
+  </si>
+  <si>
+    <t>santa barbara</t>
   </si>
 </sst>
 </file>
@@ -1837,7 +1843,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1977,7 +1983,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -26456,7 +26461,9 @@
       <c r="J158" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="K158" s="8"/>
+      <c r="K158" s="8">
+        <v>220</v>
+      </c>
       <c r="L158" s="4" t="s">
         <v>92</v>
       </c>
@@ -26475,9 +26482,15 @@
       <c r="I159" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="J159" s="4"/>
-      <c r="K159" s="8"/>
-      <c r="L159" s="4"/>
+      <c r="J159" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K159" s="8">
+        <v>230</v>
+      </c>
+      <c r="L159" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="M159" s="4"/>
       <c r="N159" s="6"/>
       <c r="O159" s="25"/>
@@ -26488,14 +26501,20 @@
         <v>46056</v>
       </c>
       <c r="H160" s="4" t="s">
-        <v>541</v>
+        <v>362</v>
       </c>
       <c r="I160" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J160" s="4"/>
-      <c r="K160" s="8"/>
-      <c r="L160" s="4"/>
+        <v>195</v>
+      </c>
+      <c r="J160" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K160" s="8">
+        <v>170</v>
+      </c>
+      <c r="L160" s="4" t="s">
+        <v>550</v>
+      </c>
       <c r="M160" s="4"/>
       <c r="N160" s="6"/>
       <c r="O160" s="25"/>
@@ -26506,10 +26525,10 @@
         <v>46056</v>
       </c>
       <c r="H161" s="4" t="s">
-        <v>483</v>
+        <v>533</v>
       </c>
       <c r="I161" s="6" t="s">
-        <v>395</v>
+        <v>125</v>
       </c>
       <c r="J161" s="4"/>
       <c r="K161" s="8"/>
@@ -26524,14 +26543,20 @@
         <v>46056</v>
       </c>
       <c r="H162" s="4" t="s">
-        <v>542</v>
+        <v>157</v>
       </c>
       <c r="I162" s="6" t="s">
-        <v>534</v>
-      </c>
-      <c r="J162" s="4"/>
-      <c r="K162" s="8"/>
-      <c r="L162" s="4"/>
+        <v>354</v>
+      </c>
+      <c r="J162" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K162" s="8">
+        <v>240</v>
+      </c>
+      <c r="L162" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M162" s="4"/>
       <c r="N162" s="6"/>
       <c r="O162" s="25"/>
@@ -26542,12 +26567,20 @@
         <v>46056</v>
       </c>
       <c r="H163" s="4" t="s">
-        <v>543</v>
-      </c>
-      <c r="I163" s="6"/>
-      <c r="J163" s="4"/>
-      <c r="K163" s="8"/>
-      <c r="L163" s="4"/>
+        <v>544</v>
+      </c>
+      <c r="I163" s="6" t="s">
+        <v>545</v>
+      </c>
+      <c r="J163" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="K163" s="8">
+        <v>296</v>
+      </c>
+      <c r="L163" s="4" t="s">
+        <v>410</v>
+      </c>
       <c r="M163" s="4"/>
       <c r="N163" s="6"/>
       <c r="O163" s="25"/>
@@ -26558,10 +26591,10 @@
         <v>46056</v>
       </c>
       <c r="H164" s="4" t="s">
-        <v>362</v>
+        <v>546</v>
       </c>
       <c r="I164" s="6" t="s">
-        <v>195</v>
+        <v>547</v>
       </c>
       <c r="J164" s="4"/>
       <c r="K164" s="8"/>
@@ -26576,14 +26609,20 @@
         <v>46056</v>
       </c>
       <c r="H165" s="4" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="I165" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J165" s="4"/>
-      <c r="K165" s="8"/>
-      <c r="L165" s="4"/>
+        <v>548</v>
+      </c>
+      <c r="J165" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K165" s="8">
+        <v>200</v>
+      </c>
+      <c r="L165" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="M165" s="4"/>
       <c r="N165" s="6"/>
       <c r="O165" s="25"/>
@@ -26594,20 +26633,16 @@
         <v>46056</v>
       </c>
       <c r="H166" s="4" t="s">
-        <v>157</v>
+        <v>549</v>
       </c>
       <c r="I166" s="6" t="s">
-        <v>354</v>
+        <v>504</v>
       </c>
       <c r="J166" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="K166" s="8">
-        <v>240</v>
-      </c>
-      <c r="L166" s="4" t="s">
-        <v>115</v>
-      </c>
+        <v>551</v>
+      </c>
+      <c r="K166" s="8"/>
+      <c r="L166" s="4"/>
       <c r="M166" s="4"/>
       <c r="N166" s="6"/>
       <c r="O166" s="25"/>
@@ -26618,10 +26653,10 @@
         <v>46056</v>
       </c>
       <c r="H167" s="4" t="s">
-        <v>544</v>
+        <v>333</v>
       </c>
       <c r="I167" s="6" t="s">
-        <v>545</v>
+        <v>325</v>
       </c>
       <c r="J167" s="4"/>
       <c r="K167" s="8"/>
@@ -26632,72 +26667,24 @@
       <c r="P167" s="6"/>
     </row>
     <row r="168" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G168" s="3">
-        <v>46056</v>
-      </c>
-      <c r="H168" s="4" t="s">
-        <v>546</v>
-      </c>
-      <c r="I168" s="59" t="s">
-        <v>547</v>
-      </c>
-      <c r="J168" s="4"/>
-      <c r="K168" s="8"/>
-      <c r="L168" s="4"/>
       <c r="M168" s="4"/>
       <c r="N168" s="6"/>
       <c r="O168" s="25"/>
       <c r="P168" s="6"/>
     </row>
     <row r="169" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G169" s="3">
-        <v>46056</v>
-      </c>
-      <c r="H169" s="4" t="s">
-        <v>532</v>
-      </c>
-      <c r="I169" s="59" t="s">
-        <v>548</v>
-      </c>
-      <c r="J169" s="4"/>
-      <c r="K169" s="8"/>
-      <c r="L169" s="4"/>
       <c r="M169" s="4"/>
       <c r="N169" s="6"/>
       <c r="O169" s="25"/>
       <c r="P169" s="6"/>
     </row>
     <row r="170" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G170" s="3">
-        <v>46056</v>
-      </c>
-      <c r="H170" s="4" t="s">
-        <v>549</v>
-      </c>
-      <c r="I170" s="59" t="s">
-        <v>504</v>
-      </c>
-      <c r="J170" s="4"/>
-      <c r="K170" s="8"/>
-      <c r="L170" s="4"/>
       <c r="M170" s="4"/>
       <c r="N170" s="6"/>
       <c r="O170" s="25"/>
       <c r="P170" s="6"/>
     </row>
     <row r="171" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G171" s="3">
-        <v>46056</v>
-      </c>
-      <c r="H171" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="I171" s="59" t="s">
-        <v>325</v>
-      </c>
-      <c r="J171" s="4"/>
-      <c r="K171" s="8"/>
-      <c r="L171" s="4"/>
       <c r="M171" s="4"/>
       <c r="N171" s="6"/>
       <c r="O171" s="25"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-04 10:19
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2020" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{95FB586B-16F0-4E85-B5AE-534A064B7775}"/>
+  <xr:revisionPtr revIDLastSave="2032" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B5D256D-7FD5-4D93-936D-C5E29CB9CEDC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4789" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4796" uniqueCount="552">
   <si>
     <t>DATA</t>
   </si>
@@ -1696,7 +1696,7 @@
     <t>hotel santos dummont</t>
   </si>
   <si>
-    <t>santa barbara</t>
+    <t xml:space="preserve">HOTEL POUSADA DA SERRA </t>
   </si>
 </sst>
 </file>
@@ -22873,7 +22873,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>46028</v>
       </c>
@@ -23295,7 +23295,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="28" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>46030</v>
       </c>
@@ -23513,7 +23513,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="36" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>46034</v>
       </c>
@@ -24230,7 +24230,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="63" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>46037</v>
       </c>
@@ -24480,7 +24480,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="72" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>46041</v>
       </c>
@@ -24860,7 +24860,7 @@
       <c r="O86" s="25"/>
       <c r="P86" s="6"/>
     </row>
-    <row r="87" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G87" s="3">
         <v>46043</v>
       </c>
@@ -25311,7 +25311,7 @@
       <c r="O108" s="25"/>
       <c r="P108" s="6"/>
     </row>
-    <row r="109" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G109" s="3">
         <v>46048</v>
       </c>
@@ -26234,7 +26234,7 @@
       <c r="O148" s="25"/>
       <c r="P148" s="6"/>
     </row>
-    <row r="149" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="149" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
         <v>46051</v>
       </c>
@@ -26330,7 +26330,7 @@
       <c r="O152" s="25"/>
       <c r="P152" s="6"/>
     </row>
-    <row r="153" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>46055</v>
       </c>
@@ -26448,7 +26448,7 @@
       <c r="O157" s="25"/>
       <c r="P157" s="6"/>
     </row>
-    <row r="158" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="158" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G158" s="3">
         <v>46056</v>
       </c>
@@ -26472,7 +26472,7 @@
       <c r="O158" s="25"/>
       <c r="P158" s="6"/>
     </row>
-    <row r="159" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="159" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G159" s="3">
         <v>46056</v>
       </c>
@@ -26496,7 +26496,7 @@
       <c r="O159" s="25"/>
       <c r="P159" s="6"/>
     </row>
-    <row r="160" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>46056</v>
       </c>
@@ -26520,7 +26520,7 @@
       <c r="O160" s="25"/>
       <c r="P160" s="6"/>
     </row>
-    <row r="161" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="161" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G161" s="3">
         <v>46056</v>
       </c>
@@ -26530,15 +26530,21 @@
       <c r="I161" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="J161" s="4"/>
-      <c r="K161" s="8"/>
-      <c r="L161" s="4"/>
+      <c r="J161" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K161" s="8">
+        <v>190</v>
+      </c>
+      <c r="L161" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="M161" s="4"/>
       <c r="N161" s="6"/>
       <c r="O161" s="25"/>
       <c r="P161" s="6"/>
     </row>
-    <row r="162" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="162" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G162" s="3">
         <v>46056</v>
       </c>
@@ -26562,7 +26568,7 @@
       <c r="O162" s="25"/>
       <c r="P162" s="6"/>
     </row>
-    <row r="163" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="163" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G163" s="3">
         <v>46056</v>
       </c>
@@ -26586,7 +26592,7 @@
       <c r="O163" s="25"/>
       <c r="P163" s="6"/>
     </row>
-    <row r="164" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="164" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G164" s="3">
         <v>46056</v>
       </c>
@@ -26596,15 +26602,21 @@
       <c r="I164" s="6" t="s">
         <v>547</v>
       </c>
-      <c r="J164" s="4"/>
-      <c r="K164" s="8"/>
-      <c r="L164" s="4"/>
+      <c r="J164" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K164" s="8">
+        <v>220</v>
+      </c>
+      <c r="L164" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="M164" s="4"/>
       <c r="N164" s="6"/>
       <c r="O164" s="25"/>
       <c r="P164" s="6"/>
     </row>
-    <row r="165" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="165" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G165" s="3">
         <v>46056</v>
       </c>
@@ -26628,7 +26640,7 @@
       <c r="O165" s="25"/>
       <c r="P165" s="6"/>
     </row>
-    <row r="166" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="166" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G166" s="3">
         <v>46056</v>
       </c>
@@ -26639,16 +26651,20 @@
         <v>504</v>
       </c>
       <c r="J166" s="4" t="s">
+        <v>513</v>
+      </c>
+      <c r="K166" s="8">
+        <v>200</v>
+      </c>
+      <c r="L166" s="4" t="s">
         <v>551</v>
       </c>
-      <c r="K166" s="8"/>
-      <c r="L166" s="4"/>
       <c r="M166" s="4"/>
       <c r="N166" s="6"/>
       <c r="O166" s="25"/>
       <c r="P166" s="6"/>
     </row>
-    <row r="167" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="167" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G167" s="3">
         <v>46056</v>
       </c>
@@ -26658,33 +26674,39 @@
       <c r="I167" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="J167" s="4"/>
-      <c r="K167" s="8"/>
-      <c r="L167" s="4"/>
+      <c r="J167" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="K167" s="8">
+        <v>160</v>
+      </c>
+      <c r="L167" s="4" t="s">
+        <v>459</v>
+      </c>
       <c r="M167" s="4"/>
       <c r="N167" s="6"/>
       <c r="O167" s="25"/>
       <c r="P167" s="6"/>
     </row>
-    <row r="168" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="168" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="M168" s="4"/>
       <c r="N168" s="6"/>
       <c r="O168" s="25"/>
       <c r="P168" s="6"/>
     </row>
-    <row r="169" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="169" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="M169" s="4"/>
       <c r="N169" s="6"/>
       <c r="O169" s="25"/>
       <c r="P169" s="6"/>
     </row>
-    <row r="170" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="170" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="M170" s="4"/>
       <c r="N170" s="6"/>
       <c r="O170" s="25"/>
       <c r="P170" s="6"/>
     </row>
-    <row r="171" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="171" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="M171" s="4"/>
       <c r="N171" s="6"/>
       <c r="O171" s="25"/>
@@ -26723,8 +26745,13 @@
   </sheetData>
   <autoFilter ref="G5:O171" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
+      <customFilters>
+        <customFilter operator="notEqual" val=" "/>
+      </customFilters>
+    </filterColumn>
+    <filterColumn colId="2">
       <filters>
-        <dateGroupItem year="2026" month="2" day="3" dateTimeGrouping="day"/>
+        <filter val="RYCHARD"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-05 11:40
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2032" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B5D256D-7FD5-4D93-936D-C5E29CB9CEDC}"/>
+  <xr:revisionPtr revIDLastSave="2126" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69C8073F-0053-44F2-A7D3-4A6B3B567D1C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$171</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$180</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4796" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4852" uniqueCount="561">
   <si>
     <t>DATA</t>
   </si>
@@ -1697,6 +1697,33 @@
   </si>
   <si>
     <t xml:space="preserve">HOTEL POUSADA DA SERRA </t>
+  </si>
+  <si>
+    <t>wesley ant</t>
+  </si>
+  <si>
+    <t>ricardo</t>
+  </si>
+  <si>
+    <t>matheus motorista</t>
+  </si>
+  <si>
+    <t>JOAO VITOR</t>
+  </si>
+  <si>
+    <t>BRUNO</t>
+  </si>
+  <si>
+    <t>CARMO DO PARANAIBA</t>
+  </si>
+  <si>
+    <t>CARMO PALACE HOTEL</t>
+  </si>
+  <si>
+    <t>LUCAS APA</t>
+  </si>
+  <si>
+    <t>JOSE ARILD</t>
   </si>
 </sst>
 </file>
@@ -22873,7 +22900,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="12" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="12" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G12" s="3">
         <v>46028</v>
       </c>
@@ -23295,7 +23322,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="28" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G28" s="3">
         <v>46030</v>
       </c>
@@ -23513,7 +23540,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="36" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="36" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G36" s="3">
         <v>46034</v>
       </c>
@@ -24230,7 +24257,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="63" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="63" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G63" s="3">
         <v>46037</v>
       </c>
@@ -24480,7 +24507,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="72" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="72" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G72" s="3">
         <v>46041</v>
       </c>
@@ -24860,7 +24887,7 @@
       <c r="O86" s="25"/>
       <c r="P86" s="6"/>
     </row>
-    <row r="87" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="87" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G87" s="3">
         <v>46043</v>
       </c>
@@ -25311,7 +25338,7 @@
       <c r="O108" s="25"/>
       <c r="P108" s="6"/>
     </row>
-    <row r="109" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="109" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G109" s="3">
         <v>46048</v>
       </c>
@@ -26234,7 +26261,7 @@
       <c r="O148" s="25"/>
       <c r="P148" s="6"/>
     </row>
-    <row r="149" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="149" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
         <v>46051</v>
       </c>
@@ -26330,7 +26357,7 @@
       <c r="O152" s="25"/>
       <c r="P152" s="6"/>
     </row>
-    <row r="153" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="153" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
         <v>46055</v>
       </c>
@@ -26462,7 +26489,7 @@
         <v>226</v>
       </c>
       <c r="K158" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L158" s="4" t="s">
         <v>92</v>
@@ -26606,7 +26633,7 @@
         <v>226</v>
       </c>
       <c r="K164" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L164" s="4" t="s">
         <v>92</v>
@@ -26707,10 +26734,396 @@
       <c r="P170" s="6"/>
     </row>
     <row r="171" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="M171" s="4"/>
-      <c r="N171" s="6"/>
-      <c r="O171" s="25"/>
-      <c r="P171" s="6"/>
+      <c r="M171" s="31"/>
+      <c r="N171" s="29"/>
+      <c r="O171" s="37"/>
+      <c r="P171" s="29"/>
+    </row>
+    <row r="172" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G172" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H172" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="I172" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J172" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="K172" s="8">
+        <v>200</v>
+      </c>
+      <c r="L172" s="4" t="s">
+        <v>511</v>
+      </c>
+      <c r="M172" s="4"/>
+      <c r="N172" s="6"/>
+      <c r="O172" s="25"/>
+      <c r="P172" s="6"/>
+    </row>
+    <row r="173" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G173" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H173" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="I173" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="J173" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K173" s="8">
+        <v>265</v>
+      </c>
+      <c r="L173" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M173" s="4"/>
+      <c r="N173" s="6"/>
+      <c r="O173" s="25"/>
+      <c r="P173" s="6"/>
+    </row>
+    <row r="174" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G174" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H174" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="I174" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J174" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="K174" s="8">
+        <v>180</v>
+      </c>
+      <c r="L174" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="M174" s="4"/>
+      <c r="N174" s="6"/>
+      <c r="O174" s="25"/>
+      <c r="P174" s="6"/>
+    </row>
+    <row r="175" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G175" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H175" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="I175" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="J175" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K175" s="8">
+        <v>220</v>
+      </c>
+      <c r="L175" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M175" s="4"/>
+      <c r="N175" s="6"/>
+      <c r="O175" s="25"/>
+      <c r="P175" s="6"/>
+    </row>
+    <row r="176" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G176" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H176" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="I176" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="J176" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="K176" s="8">
+        <v>280</v>
+      </c>
+      <c r="L176" s="4" t="s">
+        <v>520</v>
+      </c>
+      <c r="M176" s="4"/>
+      <c r="N176" s="6"/>
+      <c r="O176" s="25"/>
+      <c r="P176" s="6"/>
+    </row>
+    <row r="177" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G177" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H177" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I177" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="J177" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K177" s="8">
+        <v>245</v>
+      </c>
+      <c r="L177" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="M177" s="4"/>
+      <c r="N177" s="6"/>
+      <c r="O177" s="25"/>
+      <c r="P177" s="6"/>
+    </row>
+    <row r="178" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G178" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H178" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="I178" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J178" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K178" s="8">
+        <v>250</v>
+      </c>
+      <c r="L178" s="4" t="s">
+        <v>408</v>
+      </c>
+      <c r="M178" s="4"/>
+      <c r="N178" s="6"/>
+      <c r="O178" s="25"/>
+      <c r="P178" s="6"/>
+    </row>
+    <row r="179" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G179" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H179" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="I179" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J179" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="K179" s="8">
+        <v>179</v>
+      </c>
+      <c r="L179" s="4" t="s">
+        <v>558</v>
+      </c>
+      <c r="M179" s="4"/>
+      <c r="N179" s="6"/>
+      <c r="O179" s="25"/>
+      <c r="P179" s="6"/>
+    </row>
+    <row r="180" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G180" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H180" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="I180" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J180" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K180" s="8">
+        <v>234.9</v>
+      </c>
+      <c r="L180" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M180" s="4"/>
+      <c r="N180" s="6"/>
+      <c r="O180" s="25"/>
+      <c r="P180" s="6"/>
+    </row>
+    <row r="181" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G181" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H181" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I181" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J181" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K181" s="8">
+        <v>240</v>
+      </c>
+      <c r="L181" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M181" s="4"/>
+      <c r="N181" s="6"/>
+      <c r="O181" s="25"/>
+      <c r="P181" s="6"/>
+    </row>
+    <row r="182" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G182" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H182" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I182" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J182" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K182" s="8">
+        <v>240</v>
+      </c>
+      <c r="L182" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M182" s="4"/>
+      <c r="N182" s="6"/>
+      <c r="O182" s="25"/>
+      <c r="P182" s="6"/>
+    </row>
+    <row r="183" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G183" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H183" s="4" t="s">
+        <v>500</v>
+      </c>
+      <c r="I183" s="6" t="s">
+        <v>395</v>
+      </c>
+      <c r="J183" s="4"/>
+      <c r="K183" s="8"/>
+      <c r="L183" s="4"/>
+      <c r="M183" s="4"/>
+      <c r="N183" s="6"/>
+      <c r="O183" s="25"/>
+      <c r="P183" s="6"/>
+    </row>
+    <row r="184" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G184" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H184" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="I184" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J184" s="4"/>
+      <c r="K184" s="8"/>
+      <c r="L184" s="4"/>
+      <c r="M184" s="4"/>
+      <c r="N184" s="6"/>
+      <c r="O184" s="25"/>
+      <c r="P184" s="6"/>
+    </row>
+    <row r="185" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G185" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H185" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I185" s="6" t="s">
+        <v>380</v>
+      </c>
+      <c r="J185" s="4"/>
+      <c r="K185" s="8"/>
+      <c r="L185" s="4"/>
+      <c r="M185" s="4"/>
+      <c r="N185" s="6"/>
+      <c r="O185" s="25"/>
+      <c r="P185" s="6"/>
+    </row>
+    <row r="186" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G186" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H186" s="4" t="s">
+        <v>560</v>
+      </c>
+      <c r="I186" s="6" t="s">
+        <v>504</v>
+      </c>
+      <c r="J186" s="4"/>
+      <c r="K186" s="8"/>
+      <c r="L186" s="4"/>
+      <c r="M186" s="4"/>
+      <c r="N186" s="6"/>
+      <c r="O186" s="25"/>
+      <c r="P186" s="6"/>
+    </row>
+    <row r="187" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G187" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H187" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I187" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J187" s="4"/>
+      <c r="K187" s="8"/>
+      <c r="L187" s="4"/>
+      <c r="M187" s="4"/>
+      <c r="N187" s="6"/>
+      <c r="O187" s="25"/>
+      <c r="P187" s="6"/>
+    </row>
+    <row r="188" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G188" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H188" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I188" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="J188" s="4"/>
+      <c r="K188" s="8"/>
+      <c r="L188" s="4"/>
+      <c r="M188" s="4"/>
+      <c r="N188" s="6"/>
+      <c r="O188" s="25"/>
+      <c r="P188" s="6"/>
+    </row>
+    <row r="189" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G189" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H189" s="4"/>
+      <c r="I189" s="6"/>
+      <c r="J189" s="4"/>
+      <c r="K189" s="8"/>
+      <c r="L189" s="4"/>
+      <c r="M189" s="4"/>
+      <c r="N189" s="6"/>
+      <c r="O189" s="25"/>
+      <c r="P189" s="6"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -26743,15 +27156,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O171" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O180" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
-      <customFilters>
-        <customFilter operator="notEqual" val=" "/>
-      </customFilters>
-    </filterColumn>
-    <filterColumn colId="2">
       <filters>
-        <filter val="RYCHARD"/>
+        <dateGroupItem year="2026" month="2" day="4" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-05 11:53
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2126" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69C8073F-0053-44F2-A7D3-4A6B3B567D1C}"/>
+  <xr:revisionPtr revIDLastSave="2128" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC3C3107-5C85-47A2-9213-FB4D1A523C08}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$180</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$189</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -26427,7 +26427,7 @@
       <c r="O155" s="25"/>
       <c r="P155" s="6"/>
     </row>
-    <row r="156" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>46055</v>
       </c>
@@ -26523,7 +26523,7 @@
       <c r="O159" s="25"/>
       <c r="P159" s="6"/>
     </row>
-    <row r="160" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>46056</v>
       </c>
@@ -26763,7 +26763,7 @@
       <c r="O172" s="25"/>
       <c r="P172" s="6"/>
     </row>
-    <row r="173" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="173" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G173" s="3">
         <v>46057</v>
       </c>
@@ -26787,7 +26787,7 @@
       <c r="O173" s="25"/>
       <c r="P173" s="6"/>
     </row>
-    <row r="174" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="174" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G174" s="3">
         <v>46057</v>
       </c>
@@ -26811,7 +26811,7 @@
       <c r="O174" s="25"/>
       <c r="P174" s="6"/>
     </row>
-    <row r="175" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="175" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G175" s="3">
         <v>46057</v>
       </c>
@@ -26835,7 +26835,7 @@
       <c r="O175" s="25"/>
       <c r="P175" s="6"/>
     </row>
-    <row r="176" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="176" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G176" s="3">
         <v>46057</v>
       </c>
@@ -26859,7 +26859,7 @@
       <c r="O176" s="25"/>
       <c r="P176" s="6"/>
     </row>
-    <row r="177" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="177" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
         <v>46057</v>
       </c>
@@ -26883,7 +26883,7 @@
       <c r="O177" s="25"/>
       <c r="P177" s="6"/>
     </row>
-    <row r="178" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="178" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
         <v>46057</v>
       </c>
@@ -26907,7 +26907,7 @@
       <c r="O178" s="25"/>
       <c r="P178" s="6"/>
     </row>
-    <row r="179" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="179" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
         <v>46057</v>
       </c>
@@ -26931,7 +26931,7 @@
       <c r="O179" s="25"/>
       <c r="P179" s="6"/>
     </row>
-    <row r="180" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="180" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
         <v>46057</v>
       </c>
@@ -26955,7 +26955,7 @@
       <c r="O180" s="25"/>
       <c r="P180" s="6"/>
     </row>
-    <row r="181" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>46058</v>
       </c>
@@ -26979,7 +26979,7 @@
       <c r="O181" s="25"/>
       <c r="P181" s="6"/>
     </row>
-    <row r="182" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>46058</v>
       </c>
@@ -27003,7 +27003,7 @@
       <c r="O182" s="25"/>
       <c r="P182" s="6"/>
     </row>
-    <row r="183" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>46058</v>
       </c>
@@ -27021,7 +27021,7 @@
       <c r="O183" s="25"/>
       <c r="P183" s="6"/>
     </row>
-    <row r="184" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>46058</v>
       </c>
@@ -27039,7 +27039,7 @@
       <c r="O184" s="25"/>
       <c r="P184" s="6"/>
     </row>
-    <row r="185" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="185" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G185" s="3">
         <v>46058</v>
       </c>
@@ -27057,7 +27057,7 @@
       <c r="O185" s="25"/>
       <c r="P185" s="6"/>
     </row>
-    <row r="186" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="186" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G186" s="3">
         <v>46058</v>
       </c>
@@ -27075,7 +27075,7 @@
       <c r="O186" s="25"/>
       <c r="P186" s="6"/>
     </row>
-    <row r="187" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="187" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G187" s="3">
         <v>46058</v>
       </c>
@@ -27093,7 +27093,7 @@
       <c r="O187" s="25"/>
       <c r="P187" s="6"/>
     </row>
-    <row r="188" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="188" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G188" s="3">
         <v>46058</v>
       </c>
@@ -27111,7 +27111,7 @@
       <c r="O188" s="25"/>
       <c r="P188" s="6"/>
     </row>
-    <row r="189" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="189" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G189" s="3">
         <v>46058</v>
       </c>
@@ -27156,10 +27156,15 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O180" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O189" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="2" day="4" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="2" dateTimeGrouping="month"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="2">
+      <filters>
+        <filter val="GUILHERME"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-05 16:41
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2128" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC3C3107-5C85-47A2-9213-FB4D1A523C08}"/>
+  <xr:revisionPtr revIDLastSave="2211" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29E879A-5BBA-417F-BF5E-E6B176358ABD}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$189</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$195</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4852" uniqueCount="561">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4898" uniqueCount="564">
   <si>
     <t>DATA</t>
   </si>
@@ -1724,6 +1724,15 @@
   </si>
   <si>
     <t>JOSE ARILD</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>jose antonio</t>
+  </si>
+  <si>
+    <t>HOTEL CASARAO</t>
   </si>
 </sst>
 </file>
@@ -1870,7 +1879,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2010,6 +2019,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -26427,7 +26437,7 @@
       <c r="O155" s="25"/>
       <c r="P155" s="6"/>
     </row>
-    <row r="156" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="156" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
         <v>46055</v>
       </c>
@@ -26523,7 +26533,7 @@
       <c r="O159" s="25"/>
       <c r="P159" s="6"/>
     </row>
-    <row r="160" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="160" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G160" s="3">
         <v>46056</v>
       </c>
@@ -26739,7 +26749,7 @@
       <c r="O171" s="37"/>
       <c r="P171" s="29"/>
     </row>
-    <row r="172" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="172" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G172" s="3">
         <v>46057</v>
       </c>
@@ -26859,7 +26869,7 @@
       <c r="O176" s="25"/>
       <c r="P176" s="6"/>
     </row>
-    <row r="177" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
         <v>46057</v>
       </c>
@@ -26883,7 +26893,7 @@
       <c r="O177" s="25"/>
       <c r="P177" s="6"/>
     </row>
-    <row r="178" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
         <v>46057</v>
       </c>
@@ -26907,7 +26917,7 @@
       <c r="O178" s="25"/>
       <c r="P178" s="6"/>
     </row>
-    <row r="179" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
         <v>46057</v>
       </c>
@@ -26931,7 +26941,7 @@
       <c r="O179" s="25"/>
       <c r="P179" s="6"/>
     </row>
-    <row r="180" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
         <v>46057</v>
       </c>
@@ -26955,7 +26965,7 @@
       <c r="O180" s="25"/>
       <c r="P180" s="6"/>
     </row>
-    <row r="181" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="181" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>46058</v>
       </c>
@@ -26979,7 +26989,7 @@
       <c r="O181" s="25"/>
       <c r="P181" s="6"/>
     </row>
-    <row r="182" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="182" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>46058</v>
       </c>
@@ -27003,7 +27013,7 @@
       <c r="O182" s="25"/>
       <c r="P182" s="6"/>
     </row>
-    <row r="183" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="183" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>46058</v>
       </c>
@@ -27013,15 +27023,21 @@
       <c r="I183" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="J183" s="4"/>
-      <c r="K183" s="8"/>
-      <c r="L183" s="4"/>
+      <c r="J183" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="K183" s="8">
+        <v>209</v>
+      </c>
+      <c r="L183" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="M183" s="4"/>
       <c r="N183" s="6"/>
       <c r="O183" s="25"/>
       <c r="P183" s="6"/>
     </row>
-    <row r="184" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="184" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>46058</v>
       </c>
@@ -27031,15 +27047,21 @@
       <c r="I184" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="J184" s="4"/>
-      <c r="K184" s="8"/>
-      <c r="L184" s="4"/>
+      <c r="J184" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K184" s="8">
+        <v>240</v>
+      </c>
+      <c r="L184" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M184" s="4"/>
       <c r="N184" s="6"/>
       <c r="O184" s="25"/>
       <c r="P184" s="6"/>
     </row>
-    <row r="185" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="185" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G185" s="3">
         <v>46058</v>
       </c>
@@ -27049,15 +27071,21 @@
       <c r="I185" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="J185" s="4"/>
-      <c r="K185" s="8"/>
-      <c r="L185" s="4"/>
+      <c r="J185" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="K185" s="8">
+        <v>200</v>
+      </c>
+      <c r="L185" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="M185" s="4"/>
       <c r="N185" s="6"/>
       <c r="O185" s="25"/>
       <c r="P185" s="6"/>
     </row>
-    <row r="186" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="186" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G186" s="3">
         <v>46058</v>
       </c>
@@ -27067,15 +27095,21 @@
       <c r="I186" s="6" t="s">
         <v>504</v>
       </c>
-      <c r="J186" s="4"/>
-      <c r="K186" s="8"/>
-      <c r="L186" s="4"/>
+      <c r="J186" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K186" s="8">
+        <v>200</v>
+      </c>
+      <c r="L186" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="M186" s="4"/>
       <c r="N186" s="6"/>
       <c r="O186" s="25"/>
       <c r="P186" s="6"/>
     </row>
-    <row r="187" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="187" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G187" s="3">
         <v>46058</v>
       </c>
@@ -27085,15 +27119,24 @@
       <c r="I187" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="J187" s="4"/>
-      <c r="K187" s="8"/>
-      <c r="L187" s="4"/>
+      <c r="J187" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="K187" s="8">
+        <v>220</v>
+      </c>
+      <c r="L187" s="4" t="s">
+        <v>81</v>
+      </c>
       <c r="M187" s="4"/>
       <c r="N187" s="6"/>
       <c r="O187" s="25"/>
       <c r="P187" s="6"/>
     </row>
-    <row r="188" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="188" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F188" t="s">
+        <v>561</v>
+      </c>
       <c r="G188" s="3">
         <v>46058</v>
       </c>
@@ -27103,28 +27146,215 @@
       <c r="I188" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="J188" s="4"/>
-      <c r="K188" s="8"/>
-      <c r="L188" s="4"/>
+      <c r="J188" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K188" s="8">
+        <v>190</v>
+      </c>
+      <c r="L188" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="M188" s="4"/>
       <c r="N188" s="6"/>
       <c r="O188" s="25"/>
       <c r="P188" s="6"/>
     </row>
-    <row r="189" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="189" spans="6:16" x14ac:dyDescent="0.25">
       <c r="G189" s="3">
         <v>46058</v>
       </c>
-      <c r="H189" s="4"/>
-      <c r="I189" s="6"/>
-      <c r="J189" s="4"/>
-      <c r="K189" s="8"/>
-      <c r="L189" s="4"/>
+      <c r="H189" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I189" s="6" t="s">
+        <v>534</v>
+      </c>
+      <c r="J189" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K189" s="8">
+        <v>190</v>
+      </c>
+      <c r="L189" s="4" t="s">
+        <v>469</v>
+      </c>
       <c r="M189" s="4"/>
       <c r="N189" s="6"/>
       <c r="O189" s="25"/>
       <c r="P189" s="6"/>
     </row>
+    <row r="190" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G190" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H190" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="I190" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="J190" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="K190" s="8">
+        <v>279</v>
+      </c>
+      <c r="L190" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="M190" s="4"/>
+      <c r="N190" s="6"/>
+      <c r="O190" s="25"/>
+      <c r="P190" s="6"/>
+    </row>
+    <row r="191" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G191" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H191" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="I191" s="6" t="s">
+        <v>555</v>
+      </c>
+      <c r="J191" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K191" s="8">
+        <v>220</v>
+      </c>
+      <c r="L191" s="4" t="s">
+        <v>526</v>
+      </c>
+      <c r="M191" s="4"/>
+      <c r="N191" s="6"/>
+      <c r="O191" s="25"/>
+      <c r="P191" s="6"/>
+    </row>
+    <row r="192" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F192" t="s">
+        <v>561</v>
+      </c>
+      <c r="G192" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H192" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I192" s="6" t="s">
+        <v>556</v>
+      </c>
+      <c r="J192" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="K192" s="8">
+        <v>220</v>
+      </c>
+      <c r="L192" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="M192" s="4"/>
+      <c r="N192" s="6"/>
+      <c r="O192" s="25"/>
+      <c r="P192" s="6"/>
+    </row>
+    <row r="193" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G193" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H193" s="4" t="s">
+        <v>468</v>
+      </c>
+      <c r="I193" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J193" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K193" s="8">
+        <v>180</v>
+      </c>
+      <c r="L193" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M193" s="4"/>
+      <c r="N193" s="6"/>
+      <c r="O193" s="25"/>
+      <c r="P193" s="6"/>
+    </row>
+    <row r="194" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G194" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H194" s="4" t="s">
+        <v>492</v>
+      </c>
+      <c r="I194" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J194" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="K194" s="8">
+        <v>200</v>
+      </c>
+      <c r="L194" s="4" t="s">
+        <v>563</v>
+      </c>
+      <c r="M194" s="4"/>
+      <c r="N194" s="6"/>
+      <c r="O194" s="25"/>
+      <c r="P194" s="6"/>
+    </row>
+    <row r="195" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G195" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H195" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="I195" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J195" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="K195" s="8">
+        <v>200</v>
+      </c>
+      <c r="L195" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="M195" s="4"/>
+      <c r="N195" s="6"/>
+      <c r="O195" s="25"/>
+      <c r="P195" s="6"/>
+    </row>
+    <row r="196" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G196" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H196" s="4" t="s">
+        <v>562</v>
+      </c>
+      <c r="I196" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="J196" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K196" s="8">
+        <v>234.9</v>
+      </c>
+      <c r="L196" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M196" s="4"/>
+      <c r="N196" s="6"/>
+      <c r="O196" s="25"/>
+      <c r="P196" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -27156,15 +27386,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O189" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O195" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="2" dateTimeGrouping="month"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="2">
-      <filters>
-        <filter val="GUILHERME"/>
+        <dateGroupItem year="2026" month="2" day="5" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-05 17:09
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPastaDeTrabalho" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jrferragens\OneDrive - JR Ferragens &amp; Madeiras\Arquivos de Gabriela Costa - Transportes\ARQUIVOS TRANSPORTE\DASHBOARD\DASHBOARD\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2211" documentId="13_ncr:1_{A234A3DC-4FDD-45DC-9635-2C3752DFE17E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C29E879A-5BBA-417F-BF5E-E6B176358ABD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BE2E8C-4293-4DFE-9680-384111709CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$195</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$196</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4898" uniqueCount="564">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4892" uniqueCount="563">
   <si>
     <t>DATA</t>
   </si>
@@ -1724,9 +1724,6 @@
   </si>
   <si>
     <t>JOSE ARILD</t>
-  </si>
-  <si>
-    <t>p</t>
   </si>
   <si>
     <t>jose antonio</t>
@@ -1879,7 +1876,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2019,7 +2016,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -25136,21 +25132,96 @@
       <c r="P96" s="6"/>
     </row>
     <row r="97" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="I97" s="50"/>
+      <c r="G97" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H97" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I97" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="J97" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K97" s="8">
+        <v>180</v>
+      </c>
+      <c r="L97" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M97" s="4"/>
+      <c r="N97" s="6"/>
+      <c r="O97" s="25"/>
+      <c r="P97" s="6"/>
     </row>
     <row r="98" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="I98" s="50"/>
+      <c r="G98" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H98" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I98" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J98" s="4" t="s">
+        <v>523</v>
+      </c>
+      <c r="K98" s="8">
+        <v>240</v>
+      </c>
+      <c r="L98" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="M98" s="4"/>
+      <c r="N98" s="6"/>
+      <c r="O98" s="25"/>
+      <c r="P98" s="6"/>
     </row>
     <row r="99" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="I99" s="50"/>
+      <c r="G99" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H99" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I99" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="J99" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K99" s="8">
+        <v>170</v>
+      </c>
+      <c r="L99" s="4" t="s">
+        <v>521</v>
+      </c>
+      <c r="M99" s="4"/>
+      <c r="N99" s="6"/>
+      <c r="O99" s="25"/>
+      <c r="P99" s="6"/>
     </row>
     <row r="100" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G100" s="3"/>
-      <c r="H100" s="4"/>
-      <c r="I100" s="6"/>
-      <c r="J100" s="4"/>
-      <c r="K100" s="8"/>
-      <c r="L100" s="4"/>
+      <c r="G100" s="3">
+        <v>46044</v>
+      </c>
+      <c r="H100" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I100" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J100" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K100" s="8">
+        <v>190</v>
+      </c>
+      <c r="L100" s="4" t="s">
+        <v>469</v>
+      </c>
       <c r="M100" s="4"/>
       <c r="N100" s="6"/>
       <c r="O100" s="25"/>
@@ -25161,19 +25232,19 @@
         <v>46044</v>
       </c>
       <c r="H101" s="4" t="s">
-        <v>142</v>
+        <v>490</v>
       </c>
       <c r="I101" s="6" t="s">
-        <v>325</v>
+        <v>213</v>
       </c>
       <c r="J101" s="4" t="s">
-        <v>25</v>
+        <v>190</v>
       </c>
       <c r="K101" s="8">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="L101" s="4" t="s">
-        <v>100</v>
+        <v>191</v>
       </c>
       <c r="M101" s="4"/>
       <c r="N101" s="6"/>
@@ -25185,19 +25256,19 @@
         <v>46044</v>
       </c>
       <c r="H102" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I102" s="6" t="s">
-        <v>133</v>
+        <v>215</v>
       </c>
       <c r="J102" s="4" t="s">
-        <v>523</v>
+        <v>194</v>
       </c>
       <c r="K102" s="8">
         <v>240</v>
       </c>
       <c r="L102" s="4" t="s">
-        <v>224</v>
+        <v>522</v>
       </c>
       <c r="M102" s="4"/>
       <c r="N102" s="6"/>
@@ -25206,22 +25277,22 @@
     </row>
     <row r="103" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G103" s="3">
-        <v>46044</v>
+        <v>46048</v>
       </c>
       <c r="H103" s="4" t="s">
-        <v>147</v>
+        <v>490</v>
       </c>
       <c r="I103" s="6" t="s">
-        <v>124</v>
+        <v>213</v>
       </c>
       <c r="J103" s="4" t="s">
-        <v>359</v>
+        <v>45</v>
       </c>
       <c r="K103" s="8">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="L103" s="4" t="s">
-        <v>521</v>
+        <v>454</v>
       </c>
       <c r="M103" s="4"/>
       <c r="N103" s="6"/>
@@ -25230,22 +25301,22 @@
     </row>
     <row r="104" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G104" s="3">
-        <v>46044</v>
+        <v>46048</v>
       </c>
       <c r="H104" s="4" t="s">
-        <v>491</v>
+        <v>379</v>
       </c>
       <c r="I104" s="6" t="s">
-        <v>195</v>
+        <v>124</v>
       </c>
       <c r="J104" s="4" t="s">
-        <v>44</v>
+        <v>502</v>
       </c>
       <c r="K104" s="8">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="L104" s="4" t="s">
-        <v>469</v>
+        <v>527</v>
       </c>
       <c r="M104" s="4"/>
       <c r="N104" s="6"/>
@@ -25254,22 +25325,22 @@
     </row>
     <row r="105" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G105" s="3">
-        <v>46044</v>
+        <v>46048</v>
       </c>
       <c r="H105" s="4" t="s">
-        <v>490</v>
+        <v>500</v>
       </c>
       <c r="I105" s="6" t="s">
-        <v>213</v>
+        <v>395</v>
       </c>
       <c r="J105" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K105" s="8">
         <v>190</v>
       </c>
-      <c r="K105" s="8">
-        <v>230</v>
-      </c>
       <c r="L105" s="4" t="s">
-        <v>191</v>
+        <v>250</v>
       </c>
       <c r="M105" s="4"/>
       <c r="N105" s="6"/>
@@ -25278,22 +25349,22 @@
     </row>
     <row r="106" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G106" s="3">
-        <v>46044</v>
+        <v>46048</v>
       </c>
       <c r="H106" s="4" t="s">
-        <v>144</v>
+        <v>205</v>
       </c>
       <c r="I106" s="6" t="s">
-        <v>215</v>
+        <v>129</v>
       </c>
       <c r="J106" s="4" t="s">
-        <v>194</v>
+        <v>61</v>
       </c>
       <c r="K106" s="8">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="L106" s="4" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="M106" s="4"/>
       <c r="N106" s="6"/>
@@ -25305,19 +25376,19 @@
         <v>46048</v>
       </c>
       <c r="H107" s="4" t="s">
-        <v>490</v>
+        <v>136</v>
       </c>
       <c r="I107" s="6" t="s">
-        <v>213</v>
+        <v>525</v>
       </c>
       <c r="J107" s="4" t="s">
-        <v>45</v>
+        <v>252</v>
       </c>
       <c r="K107" s="8">
-        <v>200</v>
+        <v>175</v>
       </c>
       <c r="L107" s="4" t="s">
-        <v>454</v>
+        <v>253</v>
       </c>
       <c r="M107" s="4"/>
       <c r="N107" s="6"/>
@@ -25329,19 +25400,19 @@
         <v>46048</v>
       </c>
       <c r="H108" s="4" t="s">
-        <v>379</v>
+        <v>325</v>
       </c>
       <c r="I108" s="6" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="J108" s="4" t="s">
-        <v>502</v>
+        <v>25</v>
       </c>
       <c r="K108" s="8">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="L108" s="4" t="s">
-        <v>527</v>
+        <v>100</v>
       </c>
       <c r="M108" s="4"/>
       <c r="N108" s="6"/>
@@ -25353,19 +25424,19 @@
         <v>46048</v>
       </c>
       <c r="H109" s="4" t="s">
-        <v>500</v>
+        <v>508</v>
       </c>
       <c r="I109" s="6" t="s">
-        <v>395</v>
+        <v>125</v>
       </c>
       <c r="J109" s="4" t="s">
-        <v>227</v>
+        <v>270</v>
       </c>
       <c r="K109" s="8">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="L109" s="4" t="s">
-        <v>250</v>
+        <v>175</v>
       </c>
       <c r="M109" s="4"/>
       <c r="N109" s="6"/>
@@ -25374,22 +25445,22 @@
     </row>
     <row r="110" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G110" s="3">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="H110" s="4" t="s">
-        <v>205</v>
+        <v>325</v>
       </c>
       <c r="I110" s="6" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="J110" s="4" t="s">
-        <v>61</v>
+        <v>11</v>
       </c>
       <c r="K110" s="8">
-        <v>220</v>
+        <v>160</v>
       </c>
       <c r="L110" s="4" t="s">
-        <v>526</v>
+        <v>457</v>
       </c>
       <c r="M110" s="4"/>
       <c r="N110" s="6"/>
@@ -25398,22 +25469,22 @@
     </row>
     <row r="111" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G111" s="3">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="H111" s="4" t="s">
-        <v>136</v>
+        <v>157</v>
       </c>
       <c r="I111" s="6" t="s">
-        <v>525</v>
+        <v>354</v>
       </c>
       <c r="J111" s="4" t="s">
-        <v>252</v>
+        <v>41</v>
       </c>
       <c r="K111" s="8">
-        <v>175</v>
+        <v>240</v>
       </c>
       <c r="L111" s="4" t="s">
-        <v>253</v>
+        <v>480</v>
       </c>
       <c r="M111" s="4"/>
       <c r="N111" s="6"/>
@@ -25422,22 +25493,22 @@
     </row>
     <row r="112" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G112" s="3">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="H112" s="4" t="s">
-        <v>325</v>
+        <v>145</v>
       </c>
       <c r="I112" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J112" s="4" t="s">
-        <v>25</v>
+        <v>243</v>
       </c>
       <c r="K112" s="8">
-        <v>180</v>
+        <v>296</v>
       </c>
       <c r="L112" s="4" t="s">
-        <v>100</v>
+        <v>529</v>
       </c>
       <c r="M112" s="4"/>
       <c r="N112" s="6"/>
@@ -25446,22 +25517,22 @@
     </row>
     <row r="113" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G113" s="3">
-        <v>46048</v>
+        <v>46049</v>
       </c>
       <c r="H113" s="4" t="s">
-        <v>508</v>
+        <v>382</v>
       </c>
       <c r="I113" s="6" t="s">
-        <v>125</v>
+        <v>528</v>
       </c>
       <c r="J113" s="4" t="s">
-        <v>270</v>
+        <v>226</v>
       </c>
       <c r="K113" s="8">
         <v>220</v>
       </c>
       <c r="L113" s="4" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="M113" s="4"/>
       <c r="N113" s="6"/>
@@ -25473,19 +25544,19 @@
         <v>46049</v>
       </c>
       <c r="H114" s="4" t="s">
-        <v>325</v>
+        <v>144</v>
       </c>
       <c r="I114" s="6" t="s">
-        <v>135</v>
+        <v>215</v>
       </c>
       <c r="J114" s="4" t="s">
-        <v>11</v>
+        <v>335</v>
       </c>
       <c r="K114" s="8">
-        <v>160</v>
+        <v>200</v>
       </c>
       <c r="L114" s="4" t="s">
-        <v>457</v>
+        <v>161</v>
       </c>
       <c r="M114" s="4"/>
       <c r="N114" s="6"/>
@@ -25497,19 +25568,19 @@
         <v>46049</v>
       </c>
       <c r="H115" s="4" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="I115" s="6" t="s">
-        <v>354</v>
+        <v>325</v>
       </c>
       <c r="J115" s="4" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="K115" s="8">
-        <v>240</v>
+        <v>160</v>
       </c>
       <c r="L115" s="4" t="s">
-        <v>480</v>
+        <v>459</v>
       </c>
       <c r="M115" s="4"/>
       <c r="N115" s="6"/>
@@ -25521,19 +25592,19 @@
         <v>46049</v>
       </c>
       <c r="H116" s="4" t="s">
-        <v>145</v>
+        <v>508</v>
       </c>
       <c r="I116" s="6" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="J116" s="4" t="s">
-        <v>243</v>
+        <v>328</v>
       </c>
       <c r="K116" s="8">
-        <v>296</v>
+        <v>240</v>
       </c>
       <c r="L116" s="4" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="M116" s="4"/>
       <c r="N116" s="6"/>
@@ -25545,19 +25616,19 @@
         <v>46049</v>
       </c>
       <c r="H117" s="4" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="I117" s="6" t="s">
-        <v>528</v>
+        <v>124</v>
       </c>
       <c r="J117" s="4" t="s">
-        <v>226</v>
+        <v>185</v>
       </c>
       <c r="K117" s="8">
-        <v>220</v>
+        <v>175</v>
       </c>
       <c r="L117" s="4" t="s">
-        <v>92</v>
+        <v>363</v>
       </c>
       <c r="M117" s="4"/>
       <c r="N117" s="6"/>
@@ -25569,19 +25640,19 @@
         <v>46049</v>
       </c>
       <c r="H118" s="4" t="s">
-        <v>144</v>
+        <v>242</v>
       </c>
       <c r="I118" s="6" t="s">
-        <v>215</v>
+        <v>504</v>
       </c>
       <c r="J118" s="4" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="K118" s="8">
-        <v>200</v>
+        <v>340</v>
       </c>
       <c r="L118" s="4" t="s">
-        <v>161</v>
+        <v>256</v>
       </c>
       <c r="M118" s="4"/>
       <c r="N118" s="6"/>
@@ -25590,22 +25661,22 @@
     </row>
     <row r="119" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G119" s="3">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="H119" s="4" t="s">
-        <v>142</v>
+        <v>205</v>
       </c>
       <c r="I119" s="6" t="s">
-        <v>325</v>
+        <v>531</v>
       </c>
       <c r="J119" s="4" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="K119" s="8">
-        <v>160</v>
+        <v>220</v>
       </c>
       <c r="L119" s="4" t="s">
-        <v>459</v>
+        <v>526</v>
       </c>
       <c r="M119" s="4"/>
       <c r="N119" s="6"/>
@@ -25613,12 +25684,24 @@
       <c r="P119" s="6"/>
     </row>
     <row r="120" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G120" s="3"/>
-      <c r="H120" s="4"/>
-      <c r="I120" s="6"/>
-      <c r="J120" s="4"/>
-      <c r="K120" s="8"/>
-      <c r="L120" s="4"/>
+      <c r="G120" s="3">
+        <v>46050</v>
+      </c>
+      <c r="H120" s="4" t="s">
+        <v>507</v>
+      </c>
+      <c r="I120" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J120" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K120" s="8">
+        <v>245</v>
+      </c>
+      <c r="L120" s="4" t="s">
+        <v>464</v>
+      </c>
       <c r="M120" s="4"/>
       <c r="N120" s="6"/>
       <c r="O120" s="25"/>
@@ -25626,22 +25709,22 @@
     </row>
     <row r="121" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G121" s="3">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="H121" s="4" t="s">
-        <v>508</v>
+        <v>490</v>
       </c>
       <c r="I121" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="J121" s="4" t="s">
-        <v>328</v>
+        <v>45</v>
       </c>
       <c r="K121" s="8">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="L121" s="4" t="s">
-        <v>530</v>
+        <v>454</v>
       </c>
       <c r="M121" s="4"/>
       <c r="N121" s="6"/>
@@ -25650,22 +25733,22 @@
     </row>
     <row r="122" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G122" s="3">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="H122" s="4" t="s">
-        <v>379</v>
+        <v>491</v>
       </c>
       <c r="I122" s="6" t="s">
-        <v>124</v>
+        <v>195</v>
       </c>
       <c r="J122" s="4" t="s">
-        <v>185</v>
+        <v>46</v>
       </c>
       <c r="K122" s="8">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="L122" s="4" t="s">
-        <v>363</v>
+        <v>413</v>
       </c>
       <c r="M122" s="4"/>
       <c r="N122" s="6"/>
@@ -25674,22 +25757,22 @@
     </row>
     <row r="123" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G123" s="3">
-        <v>46049</v>
+        <v>46050</v>
       </c>
       <c r="H123" s="4" t="s">
-        <v>242</v>
+        <v>136</v>
       </c>
       <c r="I123" s="6" t="s">
-        <v>504</v>
+        <v>391</v>
       </c>
       <c r="J123" s="4" t="s">
-        <v>337</v>
+        <v>364</v>
       </c>
       <c r="K123" s="8">
-        <v>340</v>
+        <v>220</v>
       </c>
       <c r="L123" s="4" t="s">
-        <v>256</v>
+        <v>30</v>
       </c>
       <c r="M123" s="4"/>
       <c r="N123" s="6"/>
@@ -25701,19 +25784,19 @@
         <v>46050</v>
       </c>
       <c r="H124" s="4" t="s">
-        <v>205</v>
+        <v>509</v>
       </c>
       <c r="I124" s="6" t="s">
-        <v>531</v>
+        <v>131</v>
       </c>
       <c r="J124" s="4" t="s">
-        <v>61</v>
+        <v>21</v>
       </c>
       <c r="K124" s="8">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="L124" s="4" t="s">
-        <v>526</v>
+        <v>22</v>
       </c>
       <c r="M124" s="4"/>
       <c r="N124" s="6"/>
@@ -25725,19 +25808,19 @@
         <v>46050</v>
       </c>
       <c r="H125" s="4" t="s">
-        <v>507</v>
+        <v>147</v>
       </c>
       <c r="I125" s="6" t="s">
-        <v>213</v>
+        <v>467</v>
       </c>
       <c r="J125" s="4" t="s">
-        <v>414</v>
+        <v>252</v>
       </c>
       <c r="K125" s="8">
-        <v>245</v>
+        <v>205</v>
       </c>
       <c r="L125" s="4" t="s">
-        <v>464</v>
+        <v>512</v>
       </c>
       <c r="M125" s="4"/>
       <c r="N125" s="6"/>
@@ -25749,19 +25832,19 @@
         <v>46050</v>
       </c>
       <c r="H126" s="4" t="s">
-        <v>490</v>
+        <v>145</v>
       </c>
       <c r="I126" s="6" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="J126" s="4" t="s">
-        <v>45</v>
+        <v>162</v>
       </c>
       <c r="K126" s="8">
-        <v>200</v>
+        <v>220</v>
       </c>
       <c r="L126" s="4" t="s">
-        <v>454</v>
+        <v>341</v>
       </c>
       <c r="M126" s="4"/>
       <c r="N126" s="6"/>
@@ -25773,19 +25856,19 @@
         <v>46050</v>
       </c>
       <c r="H127" s="4" t="s">
-        <v>491</v>
+        <v>382</v>
       </c>
       <c r="I127" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="J127" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="K127" s="8">
-        <v>170</v>
-      </c>
-      <c r="L127" s="4" t="s">
-        <v>413</v>
+        <v>528</v>
+      </c>
+      <c r="J127" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="K127" s="10">
+        <v>266</v>
+      </c>
+      <c r="L127" s="1" t="s">
+        <v>358</v>
       </c>
       <c r="M127" s="4"/>
       <c r="N127" s="6"/>
@@ -25797,19 +25880,19 @@
         <v>46050</v>
       </c>
       <c r="H128" s="4" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="I128" s="6" t="s">
-        <v>391</v>
+        <v>325</v>
       </c>
       <c r="J128" s="4" t="s">
-        <v>364</v>
+        <v>107</v>
       </c>
       <c r="K128" s="8">
-        <v>220</v>
+        <v>180</v>
       </c>
       <c r="L128" s="4" t="s">
-        <v>30</v>
+        <v>212</v>
       </c>
       <c r="M128" s="4"/>
       <c r="N128" s="6"/>
@@ -25821,19 +25904,19 @@
         <v>46050</v>
       </c>
       <c r="H129" s="4" t="s">
-        <v>509</v>
+        <v>362</v>
       </c>
       <c r="I129" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="J129" s="4" t="s">
-        <v>21</v>
+        <v>101</v>
       </c>
       <c r="K129" s="8">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="L129" s="4" t="s">
-        <v>22</v>
+        <v>425</v>
       </c>
       <c r="M129" s="4"/>
       <c r="N129" s="6"/>
@@ -25842,22 +25925,22 @@
     </row>
     <row r="130" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G130" s="3">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="H130" s="4" t="s">
-        <v>147</v>
+        <v>507</v>
       </c>
       <c r="I130" s="6" t="s">
-        <v>467</v>
+        <v>213</v>
       </c>
       <c r="J130" s="4" t="s">
-        <v>252</v>
+        <v>364</v>
       </c>
       <c r="K130" s="8">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="L130" s="4" t="s">
-        <v>512</v>
+        <v>30</v>
       </c>
       <c r="M130" s="4"/>
       <c r="N130" s="6"/>
@@ -25865,11 +25948,24 @@
       <c r="P130" s="6"/>
     </row>
     <row r="131" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G131" s="3"/>
-      <c r="I131" s="50"/>
-      <c r="J131" s="4"/>
-      <c r="K131" s="8"/>
-      <c r="L131" s="4"/>
+      <c r="G131" s="3">
+        <v>46051</v>
+      </c>
+      <c r="H131" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I131" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J131" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K131" s="8">
+        <v>230</v>
+      </c>
+      <c r="L131" s="4" t="s">
+        <v>191</v>
+      </c>
       <c r="M131" s="4"/>
       <c r="N131" s="6"/>
       <c r="O131" s="25"/>
@@ -25877,22 +25973,22 @@
     </row>
     <row r="132" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G132" s="3">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="H132" s="4" t="s">
-        <v>145</v>
+        <v>491</v>
       </c>
       <c r="I132" s="6" t="s">
-        <v>133</v>
+        <v>195</v>
       </c>
       <c r="J132" s="4" t="s">
-        <v>162</v>
+        <v>44</v>
       </c>
       <c r="K132" s="8">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="L132" s="4" t="s">
-        <v>341</v>
+        <v>86</v>
       </c>
       <c r="M132" s="4"/>
       <c r="N132" s="6"/>
@@ -25901,22 +25997,22 @@
     </row>
     <row r="133" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G133" s="3">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="H133" s="4" t="s">
-        <v>382</v>
+        <v>509</v>
       </c>
       <c r="I133" s="6" t="s">
-        <v>528</v>
-      </c>
-      <c r="J133" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="K133" s="10">
-        <v>266</v>
-      </c>
-      <c r="L133" s="1" t="s">
-        <v>358</v>
+        <v>131</v>
+      </c>
+      <c r="J133" s="4" t="s">
+        <v>273</v>
+      </c>
+      <c r="K133" s="8">
+        <v>260</v>
+      </c>
+      <c r="L133" s="4" t="s">
+        <v>271</v>
       </c>
       <c r="M133" s="4"/>
       <c r="N133" s="6"/>
@@ -25924,12 +26020,24 @@
       <c r="P133" s="6"/>
     </row>
     <row r="134" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G134" s="3"/>
-      <c r="H134" s="4"/>
-      <c r="I134" s="6"/>
-      <c r="J134" s="4"/>
-      <c r="K134" s="8"/>
-      <c r="L134" s="4"/>
+      <c r="G134" s="3">
+        <v>46051</v>
+      </c>
+      <c r="H134" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I134" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J134" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K134" s="8">
+        <v>240</v>
+      </c>
+      <c r="L134" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M134" s="4"/>
       <c r="N134" s="6"/>
       <c r="O134" s="25"/>
@@ -25937,22 +26045,22 @@
     </row>
     <row r="135" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G135" s="3">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="H135" s="4" t="s">
-        <v>142</v>
+        <v>495</v>
       </c>
       <c r="I135" s="6" t="s">
-        <v>325</v>
+        <v>534</v>
       </c>
       <c r="J135" s="4" t="s">
-        <v>107</v>
+        <v>539</v>
       </c>
       <c r="K135" s="8">
-        <v>180</v>
+        <v>160</v>
       </c>
       <c r="L135" s="4" t="s">
-        <v>212</v>
+        <v>538</v>
       </c>
       <c r="M135" s="4"/>
       <c r="N135" s="6"/>
@@ -25961,22 +26069,22 @@
     </row>
     <row r="136" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G136" s="3">
-        <v>46050</v>
+        <v>46051</v>
       </c>
       <c r="H136" s="4" t="s">
-        <v>362</v>
+        <v>532</v>
       </c>
       <c r="I136" s="6" t="s">
-        <v>135</v>
+        <v>380</v>
       </c>
       <c r="J136" s="4" t="s">
-        <v>101</v>
+        <v>486</v>
       </c>
       <c r="K136" s="8">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="L136" s="4" t="s">
-        <v>425</v>
+        <v>412</v>
       </c>
       <c r="M136" s="4"/>
       <c r="N136" s="6"/>
@@ -25988,19 +26096,19 @@
         <v>46051</v>
       </c>
       <c r="H137" s="4" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="I137" s="6" t="s">
-        <v>213</v>
+        <v>504</v>
       </c>
       <c r="J137" s="4" t="s">
-        <v>364</v>
+        <v>10</v>
       </c>
       <c r="K137" s="8">
         <v>220</v>
       </c>
       <c r="L137" s="4" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="M137" s="4"/>
       <c r="N137" s="6"/>
@@ -26012,19 +26120,19 @@
         <v>46051</v>
       </c>
       <c r="H138" s="4" t="s">
-        <v>490</v>
+        <v>468</v>
       </c>
       <c r="I138" s="6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="J138" s="4" t="s">
-        <v>190</v>
-      </c>
-      <c r="K138" s="8">
-        <v>230</v>
+        <v>536</v>
+      </c>
+      <c r="K138" s="10">
+        <v>200</v>
       </c>
       <c r="L138" s="4" t="s">
-        <v>191</v>
+        <v>535</v>
       </c>
       <c r="M138" s="4"/>
       <c r="N138" s="6"/>
@@ -26036,19 +26144,19 @@
         <v>46051</v>
       </c>
       <c r="H139" s="4" t="s">
-        <v>491</v>
+        <v>533</v>
       </c>
       <c r="I139" s="6" t="s">
-        <v>195</v>
+        <v>125</v>
       </c>
       <c r="J139" s="4" t="s">
-        <v>44</v>
+        <v>270</v>
       </c>
       <c r="K139" s="8">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="L139" s="4" t="s">
-        <v>86</v>
+        <v>175</v>
       </c>
       <c r="M139" s="4"/>
       <c r="N139" s="6"/>
@@ -26060,19 +26168,19 @@
         <v>46051</v>
       </c>
       <c r="H140" s="4" t="s">
-        <v>509</v>
+        <v>136</v>
       </c>
       <c r="I140" s="6" t="s">
-        <v>131</v>
+        <v>391</v>
       </c>
       <c r="J140" s="4" t="s">
-        <v>273</v>
+        <v>364</v>
       </c>
       <c r="K140" s="8">
-        <v>260</v>
+        <v>220</v>
       </c>
       <c r="L140" s="4" t="s">
-        <v>271</v>
+        <v>30</v>
       </c>
       <c r="M140" s="4"/>
       <c r="N140" s="6"/>
@@ -26084,19 +26192,19 @@
         <v>46051</v>
       </c>
       <c r="H141" s="4" t="s">
-        <v>157</v>
+        <v>233</v>
       </c>
       <c r="I141" s="6" t="s">
-        <v>354</v>
+        <v>325</v>
       </c>
       <c r="J141" s="4" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="K141" s="8">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="L141" s="4" t="s">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="M141" s="4"/>
       <c r="N141" s="6"/>
@@ -26108,19 +26216,19 @@
         <v>46051</v>
       </c>
       <c r="H142" s="4" t="s">
-        <v>495</v>
+        <v>483</v>
       </c>
       <c r="I142" s="6" t="s">
-        <v>534</v>
+        <v>395</v>
       </c>
       <c r="J142" s="4" t="s">
-        <v>539</v>
+        <v>498</v>
       </c>
       <c r="K142" s="8">
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="L142" s="4" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="M142" s="4"/>
       <c r="N142" s="6"/>
@@ -26129,22 +26237,22 @@
     </row>
     <row r="143" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G143" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H143" s="4" t="s">
-        <v>532</v>
+        <v>147</v>
       </c>
       <c r="I143" s="6" t="s">
-        <v>380</v>
+        <v>174</v>
       </c>
       <c r="J143" s="4" t="s">
-        <v>486</v>
+        <v>226</v>
       </c>
       <c r="K143" s="8">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="L143" s="4" t="s">
-        <v>412</v>
+        <v>92</v>
       </c>
       <c r="M143" s="4"/>
       <c r="N143" s="6"/>
@@ -26153,22 +26261,22 @@
     </row>
     <row r="144" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G144" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H144" s="4" t="s">
-        <v>503</v>
+        <v>490</v>
       </c>
       <c r="I144" s="6" t="s">
-        <v>504</v>
+        <v>129</v>
       </c>
       <c r="J144" s="4" t="s">
-        <v>10</v>
+        <v>540</v>
       </c>
       <c r="K144" s="8">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="L144" s="4" t="s">
-        <v>9</v>
+        <v>454</v>
       </c>
       <c r="M144" s="4"/>
       <c r="N144" s="6"/>
@@ -26177,22 +26285,22 @@
     </row>
     <row r="145" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G145" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H145" s="4" t="s">
-        <v>468</v>
+        <v>541</v>
       </c>
       <c r="I145" s="6" t="s">
         <v>124</v>
       </c>
       <c r="J145" s="4" t="s">
-        <v>536</v>
-      </c>
-      <c r="K145" s="10">
+        <v>95</v>
+      </c>
+      <c r="K145" s="8">
         <v>200</v>
       </c>
       <c r="L145" s="4" t="s">
-        <v>535</v>
+        <v>161</v>
       </c>
       <c r="M145" s="4"/>
       <c r="N145" s="6"/>
@@ -26201,22 +26309,22 @@
     </row>
     <row r="146" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G146" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H146" s="4" t="s">
-        <v>533</v>
+        <v>483</v>
       </c>
       <c r="I146" s="6" t="s">
-        <v>125</v>
+        <v>395</v>
       </c>
       <c r="J146" s="4" t="s">
-        <v>270</v>
+        <v>227</v>
       </c>
       <c r="K146" s="8">
-        <v>220</v>
+        <v>190</v>
       </c>
       <c r="L146" s="4" t="s">
-        <v>175</v>
+        <v>250</v>
       </c>
       <c r="M146" s="4"/>
       <c r="N146" s="6"/>
@@ -26225,22 +26333,22 @@
     </row>
     <row r="147" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G147" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H147" s="4" t="s">
-        <v>136</v>
+        <v>542</v>
       </c>
       <c r="I147" s="6" t="s">
-        <v>391</v>
+        <v>534</v>
       </c>
       <c r="J147" s="4" t="s">
-        <v>364</v>
+        <v>226</v>
       </c>
       <c r="K147" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L147" s="4" t="s">
-        <v>30</v>
+        <v>92</v>
       </c>
       <c r="M147" s="4"/>
       <c r="N147" s="6"/>
@@ -26249,19 +26357,17 @@
     </row>
     <row r="148" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G148" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H148" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="I148" s="6" t="s">
-        <v>325</v>
-      </c>
+        <v>543</v>
+      </c>
+      <c r="I148" s="6"/>
       <c r="J148" s="4" t="s">
         <v>25</v>
       </c>
       <c r="K148" s="8">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="L148" s="4" t="s">
         <v>100</v>
@@ -26273,22 +26379,22 @@
     </row>
     <row r="149" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G149" s="3">
-        <v>46051</v>
+        <v>46055</v>
       </c>
       <c r="H149" s="4" t="s">
-        <v>483</v>
+        <v>362</v>
       </c>
       <c r="I149" s="6" t="s">
-        <v>395</v>
+        <v>195</v>
       </c>
       <c r="J149" s="4" t="s">
-        <v>498</v>
+        <v>25</v>
       </c>
       <c r="K149" s="8">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="L149" s="4" t="s">
-        <v>537</v>
+        <v>100</v>
       </c>
       <c r="M149" s="4"/>
       <c r="N149" s="6"/>
@@ -26300,19 +26406,19 @@
         <v>46055</v>
       </c>
       <c r="H150" s="4" t="s">
-        <v>147</v>
+        <v>533</v>
       </c>
       <c r="I150" s="6" t="s">
-        <v>174</v>
+        <v>125</v>
       </c>
       <c r="J150" s="4" t="s">
-        <v>226</v>
+        <v>270</v>
       </c>
       <c r="K150" s="8">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="L150" s="4" t="s">
-        <v>92</v>
+        <v>175</v>
       </c>
       <c r="M150" s="4"/>
       <c r="N150" s="6"/>
@@ -26321,22 +26427,22 @@
     </row>
     <row r="151" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G151" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H151" s="4" t="s">
-        <v>490</v>
+        <v>147</v>
       </c>
       <c r="I151" s="6" t="s">
-        <v>129</v>
+        <v>174</v>
       </c>
       <c r="J151" s="4" t="s">
-        <v>540</v>
+        <v>226</v>
       </c>
       <c r="K151" s="8">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="L151" s="4" t="s">
-        <v>454</v>
+        <v>92</v>
       </c>
       <c r="M151" s="4"/>
       <c r="N151" s="6"/>
@@ -26345,22 +26451,22 @@
     </row>
     <row r="152" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G152" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H152" s="4" t="s">
-        <v>541</v>
+        <v>490</v>
       </c>
       <c r="I152" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="J152" s="4" t="s">
-        <v>95</v>
+        <v>190</v>
       </c>
       <c r="K152" s="8">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="L152" s="4" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="M152" s="4"/>
       <c r="N152" s="6"/>
@@ -26369,22 +26475,22 @@
     </row>
     <row r="153" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G153" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H153" s="4" t="s">
-        <v>483</v>
+        <v>362</v>
       </c>
       <c r="I153" s="6" t="s">
-        <v>395</v>
+        <v>195</v>
       </c>
       <c r="J153" s="4" t="s">
-        <v>227</v>
+        <v>11</v>
       </c>
       <c r="K153" s="8">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="L153" s="4" t="s">
-        <v>250</v>
+        <v>550</v>
       </c>
       <c r="M153" s="4"/>
       <c r="N153" s="6"/>
@@ -26393,22 +26499,22 @@
     </row>
     <row r="154" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G154" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H154" s="4" t="s">
-        <v>542</v>
+        <v>533</v>
       </c>
       <c r="I154" s="6" t="s">
-        <v>534</v>
+        <v>125</v>
       </c>
       <c r="J154" s="4" t="s">
-        <v>226</v>
+        <v>328</v>
       </c>
       <c r="K154" s="8">
-        <v>240</v>
+        <v>190</v>
       </c>
       <c r="L154" s="4" t="s">
-        <v>92</v>
+        <v>55</v>
       </c>
       <c r="M154" s="4"/>
       <c r="N154" s="6"/>
@@ -26417,20 +26523,22 @@
     </row>
     <row r="155" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G155" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H155" s="4" t="s">
-        <v>543</v>
-      </c>
-      <c r="I155" s="6"/>
+        <v>157</v>
+      </c>
+      <c r="I155" s="6" t="s">
+        <v>354</v>
+      </c>
       <c r="J155" s="4" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="K155" s="8">
-        <v>100</v>
+        <v>240</v>
       </c>
       <c r="L155" s="4" t="s">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="M155" s="4"/>
       <c r="N155" s="6"/>
@@ -26439,22 +26547,22 @@
     </row>
     <row r="156" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G156" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H156" s="4" t="s">
-        <v>362</v>
+        <v>544</v>
       </c>
       <c r="I156" s="6" t="s">
-        <v>195</v>
+        <v>545</v>
       </c>
       <c r="J156" s="4" t="s">
-        <v>25</v>
+        <v>243</v>
       </c>
       <c r="K156" s="8">
-        <v>200</v>
+        <v>296</v>
       </c>
       <c r="L156" s="4" t="s">
-        <v>100</v>
+        <v>410</v>
       </c>
       <c r="M156" s="4"/>
       <c r="N156" s="6"/>
@@ -26463,22 +26571,22 @@
     </row>
     <row r="157" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G157" s="3">
-        <v>46055</v>
+        <v>46056</v>
       </c>
       <c r="H157" s="4" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="I157" s="6" t="s">
-        <v>125</v>
+        <v>547</v>
       </c>
       <c r="J157" s="4" t="s">
-        <v>270</v>
+        <v>226</v>
       </c>
       <c r="K157" s="8">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="L157" s="4" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="M157" s="4"/>
       <c r="N157" s="6"/>
@@ -26490,19 +26598,19 @@
         <v>46056</v>
       </c>
       <c r="H158" s="4" t="s">
-        <v>147</v>
+        <v>532</v>
       </c>
       <c r="I158" s="6" t="s">
-        <v>174</v>
+        <v>548</v>
       </c>
       <c r="J158" s="4" t="s">
-        <v>226</v>
+        <v>95</v>
       </c>
       <c r="K158" s="8">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="L158" s="4" t="s">
-        <v>92</v>
+        <v>161</v>
       </c>
       <c r="M158" s="4"/>
       <c r="N158" s="6"/>
@@ -26514,19 +26622,19 @@
         <v>46056</v>
       </c>
       <c r="H159" s="4" t="s">
-        <v>490</v>
+        <v>549</v>
       </c>
       <c r="I159" s="6" t="s">
-        <v>129</v>
+        <v>504</v>
       </c>
       <c r="J159" s="4" t="s">
-        <v>190</v>
+        <v>513</v>
       </c>
       <c r="K159" s="8">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="L159" s="4" t="s">
-        <v>191</v>
+        <v>551</v>
       </c>
       <c r="M159" s="4"/>
       <c r="N159" s="6"/>
@@ -26538,19 +26646,19 @@
         <v>46056</v>
       </c>
       <c r="H160" s="4" t="s">
-        <v>362</v>
+        <v>333</v>
       </c>
       <c r="I160" s="6" t="s">
-        <v>195</v>
+        <v>325</v>
       </c>
       <c r="J160" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K160" s="8">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="L160" s="4" t="s">
-        <v>550</v>
+        <v>459</v>
       </c>
       <c r="M160" s="4"/>
       <c r="N160" s="6"/>
@@ -26559,22 +26667,22 @@
     </row>
     <row r="161" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G161" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H161" s="4" t="s">
-        <v>533</v>
+        <v>362</v>
       </c>
       <c r="I161" s="6" t="s">
-        <v>125</v>
+        <v>195</v>
       </c>
       <c r="J161" s="4" t="s">
-        <v>328</v>
+        <v>101</v>
       </c>
       <c r="K161" s="8">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="L161" s="4" t="s">
-        <v>55</v>
+        <v>511</v>
       </c>
       <c r="M161" s="4"/>
       <c r="N161" s="6"/>
@@ -26583,22 +26691,22 @@
     </row>
     <row r="162" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G162" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H162" s="4" t="s">
-        <v>157</v>
+        <v>552</v>
       </c>
       <c r="I162" s="6" t="s">
-        <v>354</v>
+        <v>534</v>
       </c>
       <c r="J162" s="4" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="K162" s="8">
-        <v>240</v>
+        <v>265</v>
       </c>
       <c r="L162" s="4" t="s">
-        <v>115</v>
+        <v>413</v>
       </c>
       <c r="M162" s="4"/>
       <c r="N162" s="6"/>
@@ -26607,22 +26715,22 @@
     </row>
     <row r="163" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G163" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H163" s="4" t="s">
-        <v>544</v>
+        <v>333</v>
       </c>
       <c r="I163" s="6" t="s">
-        <v>545</v>
+        <v>325</v>
       </c>
       <c r="J163" s="4" t="s">
-        <v>243</v>
+        <v>107</v>
       </c>
       <c r="K163" s="8">
-        <v>296</v>
+        <v>180</v>
       </c>
       <c r="L163" s="4" t="s">
-        <v>410</v>
+        <v>212</v>
       </c>
       <c r="M163" s="4"/>
       <c r="N163" s="6"/>
@@ -26631,19 +26739,19 @@
     </row>
     <row r="164" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G164" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H164" s="4" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="I164" s="6" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="J164" s="4" t="s">
         <v>226</v>
       </c>
       <c r="K164" s="8">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="L164" s="4" t="s">
         <v>92</v>
@@ -26655,22 +26763,22 @@
     </row>
     <row r="165" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G165" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H165" s="4" t="s">
-        <v>532</v>
+        <v>236</v>
       </c>
       <c r="I165" s="6" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="J165" s="4" t="s">
-        <v>95</v>
+        <v>519</v>
       </c>
       <c r="K165" s="8">
-        <v>200</v>
+        <v>280</v>
       </c>
       <c r="L165" s="4" t="s">
-        <v>161</v>
+        <v>520</v>
       </c>
       <c r="M165" s="4"/>
       <c r="N165" s="6"/>
@@ -26679,22 +26787,22 @@
     </row>
     <row r="166" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G166" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H166" s="4" t="s">
-        <v>549</v>
+        <v>152</v>
       </c>
       <c r="I166" s="6" t="s">
-        <v>504</v>
+        <v>556</v>
       </c>
       <c r="J166" s="4" t="s">
-        <v>513</v>
+        <v>414</v>
       </c>
       <c r="K166" s="8">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="L166" s="4" t="s">
-        <v>551</v>
+        <v>464</v>
       </c>
       <c r="M166" s="4"/>
       <c r="N166" s="6"/>
@@ -26703,22 +26811,22 @@
     </row>
     <row r="167" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G167" s="3">
-        <v>46056</v>
+        <v>46057</v>
       </c>
       <c r="H167" s="4" t="s">
-        <v>333</v>
+        <v>468</v>
       </c>
       <c r="I167" s="6" t="s">
-        <v>325</v>
+        <v>124</v>
       </c>
       <c r="J167" s="4" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="K167" s="8">
-        <v>160</v>
+        <v>250</v>
       </c>
       <c r="L167" s="4" t="s">
-        <v>459</v>
+        <v>408</v>
       </c>
       <c r="M167" s="4"/>
       <c r="N167" s="6"/>
@@ -26726,635 +26834,425 @@
       <c r="P167" s="6"/>
     </row>
     <row r="168" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G168" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H168" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="I168" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J168" s="4" t="s">
+        <v>557</v>
+      </c>
+      <c r="K168" s="8">
+        <v>179</v>
+      </c>
+      <c r="L168" s="4" t="s">
+        <v>558</v>
+      </c>
       <c r="M168" s="4"/>
       <c r="N168" s="6"/>
       <c r="O168" s="25"/>
       <c r="P168" s="6"/>
     </row>
     <row r="169" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G169" s="3">
+        <v>46057</v>
+      </c>
+      <c r="H169" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="I169" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J169" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K169" s="8">
+        <v>234.9</v>
+      </c>
+      <c r="L169" s="4" t="s">
+        <v>210</v>
+      </c>
       <c r="M169" s="4"/>
       <c r="N169" s="6"/>
       <c r="O169" s="25"/>
       <c r="P169" s="6"/>
     </row>
-    <row r="170" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="170" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G170" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H170" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I170" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J170" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K170" s="8">
+        <v>240</v>
+      </c>
+      <c r="L170" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="M170" s="4"/>
       <c r="N170" s="6"/>
       <c r="O170" s="25"/>
       <c r="P170" s="6"/>
     </row>
-    <row r="171" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="M171" s="31"/>
-      <c r="N171" s="29"/>
-      <c r="O171" s="37"/>
-      <c r="P171" s="29"/>
-    </row>
-    <row r="172" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="171" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G171" s="3">
+        <v>46058</v>
+      </c>
+      <c r="H171" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I171" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J171" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K171" s="8">
+        <v>240</v>
+      </c>
+      <c r="L171" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M171" s="4"/>
+      <c r="N171" s="6"/>
+      <c r="O171" s="25"/>
+      <c r="P171" s="6"/>
+    </row>
+    <row r="172" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G172" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H172" s="4" t="s">
-        <v>362</v>
+        <v>500</v>
       </c>
       <c r="I172" s="6" t="s">
-        <v>195</v>
+        <v>395</v>
       </c>
       <c r="J172" s="4" t="s">
-        <v>101</v>
+        <v>349</v>
       </c>
       <c r="K172" s="8">
-        <v>200</v>
+        <v>209</v>
       </c>
       <c r="L172" s="4" t="s">
-        <v>511</v>
+        <v>88</v>
       </c>
       <c r="M172" s="4"/>
       <c r="N172" s="6"/>
       <c r="O172" s="25"/>
       <c r="P172" s="6"/>
     </row>
-    <row r="173" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="173" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G173" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H173" s="4" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="I173" s="6" t="s">
-        <v>534</v>
+        <v>354</v>
       </c>
       <c r="J173" s="4" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="K173" s="8">
-        <v>265</v>
+        <v>240</v>
       </c>
       <c r="L173" s="4" t="s">
-        <v>413</v>
+        <v>115</v>
       </c>
       <c r="M173" s="4"/>
       <c r="N173" s="6"/>
       <c r="O173" s="25"/>
       <c r="P173" s="6"/>
     </row>
-    <row r="174" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="174" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G174" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H174" s="4" t="s">
-        <v>333</v>
+        <v>144</v>
       </c>
       <c r="I174" s="6" t="s">
-        <v>325</v>
+        <v>380</v>
       </c>
       <c r="J174" s="4" t="s">
-        <v>107</v>
+        <v>95</v>
       </c>
       <c r="K174" s="8">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="L174" s="4" t="s">
-        <v>212</v>
+        <v>161</v>
       </c>
       <c r="M174" s="4"/>
       <c r="N174" s="6"/>
       <c r="O174" s="25"/>
       <c r="P174" s="6"/>
     </row>
-    <row r="175" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="175" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G175" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H175" s="4" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="I175" s="6" t="s">
-        <v>554</v>
+        <v>504</v>
       </c>
       <c r="J175" s="4" t="s">
-        <v>226</v>
+        <v>10</v>
       </c>
       <c r="K175" s="8">
-        <v>220</v>
+        <v>200</v>
       </c>
       <c r="L175" s="4" t="s">
-        <v>92</v>
+        <v>9</v>
       </c>
       <c r="M175" s="4"/>
       <c r="N175" s="6"/>
       <c r="O175" s="25"/>
       <c r="P175" s="6"/>
     </row>
-    <row r="176" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="176" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G176" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H176" s="4" t="s">
-        <v>236</v>
+        <v>157</v>
       </c>
       <c r="I176" s="6" t="s">
-        <v>555</v>
+        <v>125</v>
       </c>
       <c r="J176" s="4" t="s">
-        <v>519</v>
+        <v>82</v>
       </c>
       <c r="K176" s="8">
-        <v>280</v>
+        <v>220</v>
       </c>
       <c r="L176" s="4" t="s">
-        <v>520</v>
+        <v>81</v>
       </c>
       <c r="M176" s="4"/>
       <c r="N176" s="6"/>
       <c r="O176" s="25"/>
       <c r="P176" s="6"/>
     </row>
-    <row r="177" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="177" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G177" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H177" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="I177" s="6" t="s">
-        <v>556</v>
+        <v>172</v>
       </c>
       <c r="J177" s="4" t="s">
-        <v>414</v>
+        <v>328</v>
       </c>
       <c r="K177" s="8">
-        <v>245</v>
+        <v>190</v>
       </c>
       <c r="L177" s="4" t="s">
-        <v>464</v>
+        <v>55</v>
       </c>
       <c r="M177" s="4"/>
       <c r="N177" s="6"/>
       <c r="O177" s="25"/>
       <c r="P177" s="6"/>
     </row>
-    <row r="178" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="178" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G178" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H178" s="4" t="s">
-        <v>468</v>
+        <v>491</v>
       </c>
       <c r="I178" s="6" t="s">
-        <v>124</v>
+        <v>534</v>
       </c>
       <c r="J178" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K178" s="8">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="L178" s="4" t="s">
-        <v>408</v>
+        <v>469</v>
       </c>
       <c r="M178" s="4"/>
       <c r="N178" s="6"/>
       <c r="O178" s="25"/>
       <c r="P178" s="6"/>
     </row>
-    <row r="179" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="179" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G179" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H179" s="4" t="s">
-        <v>509</v>
+        <v>553</v>
       </c>
       <c r="I179" s="6" t="s">
-        <v>131</v>
+        <v>554</v>
       </c>
       <c r="J179" s="4" t="s">
-        <v>557</v>
+        <v>255</v>
       </c>
       <c r="K179" s="8">
-        <v>179</v>
+        <v>279</v>
       </c>
       <c r="L179" s="4" t="s">
-        <v>558</v>
+        <v>358</v>
       </c>
       <c r="M179" s="4"/>
       <c r="N179" s="6"/>
       <c r="O179" s="25"/>
       <c r="P179" s="6"/>
     </row>
-    <row r="180" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="180" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G180" s="3">
-        <v>46057</v>
+        <v>46058</v>
       </c>
       <c r="H180" s="4" t="s">
-        <v>495</v>
+        <v>152</v>
       </c>
       <c r="I180" s="6" t="s">
-        <v>133</v>
+        <v>556</v>
       </c>
       <c r="J180" s="4" t="s">
-        <v>162</v>
+        <v>364</v>
       </c>
       <c r="K180" s="8">
-        <v>234.9</v>
+        <v>220</v>
       </c>
       <c r="L180" s="4" t="s">
-        <v>210</v>
+        <v>30</v>
       </c>
       <c r="M180" s="4"/>
       <c r="N180" s="6"/>
       <c r="O180" s="25"/>
       <c r="P180" s="6"/>
     </row>
-    <row r="181" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="181" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G181" s="3">
         <v>46058</v>
       </c>
       <c r="H181" s="4" t="s">
-        <v>147</v>
+        <v>468</v>
       </c>
       <c r="I181" s="6" t="s">
-        <v>174</v>
+        <v>124</v>
       </c>
       <c r="J181" s="4" t="s">
-        <v>226</v>
+        <v>31</v>
       </c>
       <c r="K181" s="8">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="L181" s="4" t="s">
-        <v>92</v>
+        <v>32</v>
       </c>
       <c r="M181" s="4"/>
       <c r="N181" s="6"/>
       <c r="O181" s="25"/>
       <c r="P181" s="6"/>
     </row>
-    <row r="182" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="182" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G182" s="3">
         <v>46058</v>
       </c>
       <c r="H182" s="4" t="s">
-        <v>130</v>
+        <v>492</v>
       </c>
       <c r="I182" s="6" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="J182" s="4" t="s">
-        <v>226</v>
+        <v>83</v>
       </c>
       <c r="K182" s="8">
-        <v>240</v>
+        <v>200</v>
       </c>
       <c r="L182" s="4" t="s">
-        <v>92</v>
+        <v>562</v>
       </c>
       <c r="M182" s="4"/>
       <c r="N182" s="6"/>
       <c r="O182" s="25"/>
       <c r="P182" s="6"/>
     </row>
-    <row r="183" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="183" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G183" s="3">
         <v>46058</v>
       </c>
       <c r="H183" s="4" t="s">
-        <v>500</v>
+        <v>333</v>
       </c>
       <c r="I183" s="6" t="s">
-        <v>395</v>
+        <v>325</v>
       </c>
       <c r="J183" s="4" t="s">
-        <v>349</v>
+        <v>432</v>
       </c>
       <c r="K183" s="8">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="L183" s="4" t="s">
-        <v>88</v>
+        <v>433</v>
       </c>
       <c r="M183" s="4"/>
       <c r="N183" s="6"/>
       <c r="O183" s="25"/>
       <c r="P183" s="6"/>
     </row>
-    <row r="184" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="184" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G184" s="3">
         <v>46058</v>
       </c>
       <c r="H184" s="4" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="I184" s="6" t="s">
-        <v>354</v>
+        <v>133</v>
       </c>
       <c r="J184" s="4" t="s">
-        <v>41</v>
+        <v>162</v>
       </c>
       <c r="K184" s="8">
-        <v>240</v>
+        <v>234.9</v>
       </c>
       <c r="L184" s="4" t="s">
-        <v>115</v>
+        <v>210</v>
       </c>
       <c r="M184" s="4"/>
       <c r="N184" s="6"/>
       <c r="O184" s="25"/>
       <c r="P184" s="6"/>
     </row>
-    <row r="185" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G185" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H185" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="I185" s="6" t="s">
-        <v>380</v>
-      </c>
-      <c r="J185" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="K185" s="8">
-        <v>200</v>
-      </c>
-      <c r="L185" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="M185" s="4"/>
-      <c r="N185" s="6"/>
-      <c r="O185" s="25"/>
-      <c r="P185" s="6"/>
-    </row>
-    <row r="186" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G186" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H186" s="4" t="s">
-        <v>560</v>
-      </c>
-      <c r="I186" s="6" t="s">
-        <v>504</v>
-      </c>
-      <c r="J186" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="K186" s="8">
-        <v>200</v>
-      </c>
-      <c r="L186" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="M186" s="4"/>
-      <c r="N186" s="6"/>
-      <c r="O186" s="25"/>
-      <c r="P186" s="6"/>
-    </row>
-    <row r="187" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G187" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H187" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="I187" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="J187" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="K187" s="8">
-        <v>220</v>
-      </c>
-      <c r="L187" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="M187" s="4"/>
-      <c r="N187" s="6"/>
-      <c r="O187" s="25"/>
-      <c r="P187" s="6"/>
-    </row>
-    <row r="188" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="F188" t="s">
-        <v>561</v>
-      </c>
-      <c r="G188" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H188" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="I188" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="J188" s="4" t="s">
-        <v>328</v>
-      </c>
-      <c r="K188" s="8">
-        <v>190</v>
-      </c>
-      <c r="L188" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M188" s="4"/>
-      <c r="N188" s="6"/>
-      <c r="O188" s="25"/>
-      <c r="P188" s="6"/>
-    </row>
-    <row r="189" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G189" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H189" s="4" t="s">
-        <v>491</v>
-      </c>
-      <c r="I189" s="6" t="s">
-        <v>534</v>
-      </c>
-      <c r="J189" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="K189" s="8">
-        <v>190</v>
-      </c>
-      <c r="L189" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="M189" s="4"/>
-      <c r="N189" s="6"/>
-      <c r="O189" s="25"/>
-      <c r="P189" s="6"/>
-    </row>
-    <row r="190" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G190" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H190" s="4" t="s">
-        <v>553</v>
-      </c>
-      <c r="I190" s="6" t="s">
-        <v>554</v>
-      </c>
-      <c r="J190" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="K190" s="8">
-        <v>279</v>
-      </c>
-      <c r="L190" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="M190" s="4"/>
-      <c r="N190" s="6"/>
-      <c r="O190" s="25"/>
-      <c r="P190" s="6"/>
-    </row>
-    <row r="191" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G191" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H191" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I191" s="6" t="s">
-        <v>555</v>
-      </c>
-      <c r="J191" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="K191" s="8">
-        <v>220</v>
-      </c>
-      <c r="L191" s="4" t="s">
-        <v>526</v>
-      </c>
-      <c r="M191" s="4"/>
-      <c r="N191" s="6"/>
-      <c r="O191" s="25"/>
-      <c r="P191" s="6"/>
-    </row>
-    <row r="192" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="F192" t="s">
-        <v>561</v>
-      </c>
-      <c r="G192" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H192" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="I192" s="6" t="s">
-        <v>556</v>
-      </c>
-      <c r="J192" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="K192" s="8">
-        <v>220</v>
-      </c>
-      <c r="L192" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="M192" s="4"/>
-      <c r="N192" s="6"/>
-      <c r="O192" s="25"/>
-      <c r="P192" s="6"/>
-    </row>
-    <row r="193" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G193" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H193" s="4" t="s">
-        <v>468</v>
-      </c>
-      <c r="I193" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="J193" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="K193" s="8">
-        <v>180</v>
-      </c>
-      <c r="L193" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="M193" s="4"/>
-      <c r="N193" s="6"/>
-      <c r="O193" s="25"/>
-      <c r="P193" s="6"/>
-    </row>
-    <row r="194" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G194" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H194" s="4" t="s">
-        <v>492</v>
-      </c>
-      <c r="I194" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="J194" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="K194" s="8">
-        <v>200</v>
-      </c>
-      <c r="L194" s="4" t="s">
-        <v>563</v>
-      </c>
-      <c r="M194" s="4"/>
-      <c r="N194" s="6"/>
-      <c r="O194" s="25"/>
-      <c r="P194" s="6"/>
-    </row>
-    <row r="195" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G195" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H195" s="4" t="s">
-        <v>333</v>
-      </c>
-      <c r="I195" s="6" t="s">
-        <v>325</v>
-      </c>
-      <c r="J195" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="K195" s="8">
-        <v>200</v>
-      </c>
-      <c r="L195" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="M195" s="4"/>
-      <c r="N195" s="6"/>
-      <c r="O195" s="25"/>
-      <c r="P195" s="6"/>
-    </row>
-    <row r="196" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G196" s="3">
-        <v>46058</v>
-      </c>
-      <c r="H196" s="4" t="s">
-        <v>562</v>
-      </c>
-      <c r="I196" s="59" t="s">
-        <v>133</v>
-      </c>
-      <c r="J196" s="4" t="s">
-        <v>162</v>
-      </c>
-      <c r="K196" s="8">
-        <v>234.9</v>
-      </c>
-      <c r="L196" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="M196" s="4"/>
-      <c r="N196" s="6"/>
-      <c r="O196" s="25"/>
-      <c r="P196" s="6"/>
-    </row>
+    <row r="185" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="186" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="187" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="188" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="189" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="190" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="191" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="192" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="193" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="194" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="195" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="196" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -27386,7 +27284,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O195" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O196" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
         <dateGroupItem year="2026" month="2" day="5" dateTimeGrouping="day"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-09 10:45
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{82BE2E8C-4293-4DFE-9680-384111709CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD79298F-B6CE-4BD6-8910-3498A751B848}"/>
+  <xr:revisionPtr revIDLastSave="55" documentId="13_ncr:1_{82BE2E8C-4293-4DFE-9680-384111709CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EC09218-F801-41F5-9511-8F961C1695DC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4910" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4912" uniqueCount="556">
   <si>
     <t>DATA</t>
   </si>
@@ -27352,9 +27352,15 @@
       <c r="I202" s="6" t="s">
         <v>549</v>
       </c>
-      <c r="J202" s="4"/>
-      <c r="K202" s="8"/>
-      <c r="L202" s="4"/>
+      <c r="J202" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K202" s="8">
+        <v>190</v>
+      </c>
+      <c r="L202" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="M202" s="4"/>
       <c r="N202" s="6"/>
       <c r="O202" s="25"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-19 16:18
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CFDD7E5-D22E-4219-9163-E5CAD56F2AB0}"/>
+  <xr:revisionPtr revIDLastSave="106" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF726D96-AEC4-4AB4-9678-22942C9A3485}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,9 +19,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$243</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$262</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5069" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5131" uniqueCount="574">
   <si>
     <t>DATA</t>
   </si>
@@ -1748,6 +1749,21 @@
   </si>
   <si>
     <t>FERNANDO GOMES</t>
+  </si>
+  <si>
+    <t>rychard</t>
+  </si>
+  <si>
+    <t>MATEUS SEV</t>
+  </si>
+  <si>
+    <t>LUCAS GA</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>POUSADA AMERICA</t>
   </si>
 </sst>
 </file>
@@ -28221,7 +28237,7 @@
       <c r="O238" s="25"/>
       <c r="P238" s="6"/>
     </row>
-    <row r="239" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="239" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G239" s="3">
         <v>46071</v>
       </c>
@@ -28247,7 +28263,7 @@
       <c r="O239" s="25"/>
       <c r="P239" s="6"/>
     </row>
-    <row r="240" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="240" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G240" s="3">
         <v>46071</v>
       </c>
@@ -28258,13 +28274,13 @@
         <v>548</v>
       </c>
       <c r="J240" s="4" t="s">
-        <v>243</v>
+        <v>162</v>
       </c>
       <c r="K240" s="8">
-        <v>296</v>
+        <v>234.9</v>
       </c>
       <c r="L240" s="4" t="s">
-        <v>410</v>
+        <v>210</v>
       </c>
       <c r="M240" s="4"/>
       <c r="N240" s="6">
@@ -28273,7 +28289,7 @@
       <c r="O240" s="25"/>
       <c r="P240" s="6"/>
     </row>
-    <row r="241" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="241" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G241" s="3">
         <v>46071</v>
       </c>
@@ -28299,7 +28315,7 @@
       <c r="O241" s="25"/>
       <c r="P241" s="6"/>
     </row>
-    <row r="242" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="242" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G242" s="3">
         <v>46071</v>
       </c>
@@ -28325,7 +28341,7 @@
       <c r="O242" s="25"/>
       <c r="P242" s="6"/>
     </row>
-    <row r="243" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="243" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G243" s="3">
         <v>46071</v>
       </c>
@@ -28351,7 +28367,7 @@
       <c r="O243" s="25"/>
       <c r="P243" s="6"/>
     </row>
-    <row r="244" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="244" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G244" s="3">
         <v>46071</v>
       </c>
@@ -28377,7 +28393,7 @@
       <c r="O244" s="25"/>
       <c r="P244" s="6"/>
     </row>
-    <row r="245" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="245" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G245" s="3">
         <v>46071</v>
       </c>
@@ -28403,7 +28419,7 @@
       <c r="O245" s="25"/>
       <c r="P245" s="6"/>
     </row>
-    <row r="246" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="246" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G246" s="3">
         <v>46071</v>
       </c>
@@ -28414,13 +28430,13 @@
         <v>467</v>
       </c>
       <c r="J246" s="4" t="s">
-        <v>252</v>
+        <v>226</v>
       </c>
       <c r="K246" s="8">
-        <v>205</v>
+        <v>280</v>
       </c>
       <c r="L246" s="4" t="s">
-        <v>253</v>
+        <v>92</v>
       </c>
       <c r="M246" s="4"/>
       <c r="N246" s="6">
@@ -28429,7 +28445,7 @@
       <c r="O246" s="25"/>
       <c r="P246" s="6"/>
     </row>
-    <row r="247" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="247" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G247" s="3">
         <v>46071</v>
       </c>
@@ -28455,6 +28471,428 @@
       <c r="O247" s="25"/>
       <c r="P247" s="6"/>
     </row>
+    <row r="248" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G248" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H248" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I248" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="J248" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="K248" s="8">
+        <v>234.9</v>
+      </c>
+      <c r="L248" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M248" s="4"/>
+      <c r="N248" s="6">
+        <v>2</v>
+      </c>
+      <c r="O248" s="25"/>
+      <c r="P248" s="6"/>
+    </row>
+    <row r="249" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G249" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H249" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="I249" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="J249" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K249" s="8">
+        <v>190</v>
+      </c>
+      <c r="L249" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="M249" s="4"/>
+      <c r="N249" s="6">
+        <v>2</v>
+      </c>
+      <c r="O249" s="25"/>
+      <c r="P249" s="6"/>
+    </row>
+    <row r="250" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G250" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H250" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I250" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J250" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K250" s="8">
+        <v>230</v>
+      </c>
+      <c r="L250" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="M250" s="4"/>
+      <c r="N250" s="6">
+        <v>2</v>
+      </c>
+      <c r="O250" s="25"/>
+      <c r="P250" s="6"/>
+    </row>
+    <row r="251" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F251" t="s">
+        <v>572</v>
+      </c>
+      <c r="G251" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H251" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I251" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="J251" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="K251" s="8">
+        <v>200</v>
+      </c>
+      <c r="L251" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="M251" s="4"/>
+      <c r="N251" s="6">
+        <v>2</v>
+      </c>
+      <c r="O251" s="25"/>
+      <c r="P251" s="6"/>
+    </row>
+    <row r="252" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G252" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H252" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I252" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J252" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K252" s="8">
+        <v>190</v>
+      </c>
+      <c r="L252" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="M252" s="4"/>
+      <c r="N252" s="6">
+        <v>2</v>
+      </c>
+      <c r="O252" s="25"/>
+      <c r="P252" s="6"/>
+    </row>
+    <row r="253" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G253" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H253" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I253" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J253" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="K253" s="8">
+        <v>210</v>
+      </c>
+      <c r="L253" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="M253" s="4"/>
+      <c r="N253" s="6">
+        <v>2</v>
+      </c>
+      <c r="O253" s="25"/>
+      <c r="P253" s="6"/>
+    </row>
+    <row r="254" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G254" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H254" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I254" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J254" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="K254" s="8">
+        <v>200</v>
+      </c>
+      <c r="L254" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="M254" s="4"/>
+      <c r="N254" s="6">
+        <v>2</v>
+      </c>
+      <c r="O254" s="25"/>
+      <c r="P254" s="6"/>
+    </row>
+    <row r="255" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G255" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H255" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I255" s="6" t="s">
+        <v>569</v>
+      </c>
+      <c r="J255" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K255" s="8">
+        <v>190</v>
+      </c>
+      <c r="L255" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="M255" s="4"/>
+      <c r="N255" s="6">
+        <v>2</v>
+      </c>
+      <c r="O255" s="25"/>
+      <c r="P255" s="6"/>
+    </row>
+    <row r="256" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G256" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H256" s="4" t="s">
+        <v>554</v>
+      </c>
+      <c r="I256" s="6" t="s">
+        <v>462</v>
+      </c>
+      <c r="J256" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="K256" s="8">
+        <v>209</v>
+      </c>
+      <c r="L256" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="M256" s="4"/>
+      <c r="N256" s="6">
+        <v>2</v>
+      </c>
+      <c r="O256" s="25"/>
+      <c r="P256" s="6"/>
+    </row>
+    <row r="257" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G257" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H257" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="I257" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J257" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K257" s="8">
+        <v>240</v>
+      </c>
+      <c r="L257" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="M257" s="4"/>
+      <c r="N257" s="6">
+        <v>2</v>
+      </c>
+      <c r="O257" s="25"/>
+      <c r="P257" s="6"/>
+    </row>
+    <row r="258" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G258" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H258" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="I258" s="6" t="s">
+        <v>571</v>
+      </c>
+      <c r="J258" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="K258" s="8">
+        <v>220</v>
+      </c>
+      <c r="L258" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="M258" s="4"/>
+      <c r="N258" s="6"/>
+      <c r="O258" s="25"/>
+      <c r="P258" s="6"/>
+    </row>
+    <row r="259" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G259" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H259" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="I259" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="J259" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="K259" s="8">
+        <v>300</v>
+      </c>
+      <c r="L259" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="M259" s="4"/>
+      <c r="N259" s="6"/>
+      <c r="O259" s="25"/>
+      <c r="P259" s="6"/>
+    </row>
+    <row r="260" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G260" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H260" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I260" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J260" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K260" s="8">
+        <v>200</v>
+      </c>
+      <c r="L260" s="4" t="s">
+        <v>518</v>
+      </c>
+      <c r="M260" s="4"/>
+      <c r="N260" s="6"/>
+      <c r="O260" s="25"/>
+      <c r="P260" s="6"/>
+    </row>
+    <row r="261" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="F261" t="s">
+        <v>572</v>
+      </c>
+      <c r="G261" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H261" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="I261" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="J261" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K261" s="8">
+        <v>300</v>
+      </c>
+      <c r="L261" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M261" s="4"/>
+      <c r="N261" s="6"/>
+      <c r="O261" s="25"/>
+      <c r="P261" s="6"/>
+    </row>
+    <row r="262" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G262" s="3">
+        <v>46072</v>
+      </c>
+      <c r="H262" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I262" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J262" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="K262" s="8">
+        <v>220</v>
+      </c>
+      <c r="L262" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="M262" s="4"/>
+      <c r="N262" s="6"/>
+      <c r="O262" s="25"/>
+      <c r="P262" s="6"/>
+    </row>
+    <row r="263" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G263" s="4"/>
+      <c r="H263" s="4"/>
+      <c r="I263" s="6"/>
+      <c r="J263" s="4"/>
+      <c r="K263" s="8"/>
+      <c r="L263" s="4"/>
+      <c r="M263" s="4"/>
+      <c r="N263" s="6"/>
+      <c r="O263" s="25"/>
+      <c r="P263" s="6"/>
+    </row>
+    <row r="264" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G264" s="4"/>
+      <c r="H264" s="4"/>
+      <c r="I264" s="6"/>
+      <c r="J264" s="4"/>
+      <c r="K264" s="8"/>
+      <c r="L264" s="4"/>
+      <c r="M264" s="4"/>
+      <c r="N264" s="6"/>
+      <c r="O264" s="25"/>
+      <c r="P264" s="6"/>
+    </row>
+    <row r="265" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G265" s="4"/>
+      <c r="H265" s="4"/>
+      <c r="I265" s="6"/>
+      <c r="J265" s="4"/>
+      <c r="K265" s="8"/>
+      <c r="L265" s="4"/>
+      <c r="M265" s="4"/>
+      <c r="N265" s="6"/>
+      <c r="O265" s="25"/>
+      <c r="P265" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -28486,10 +28924,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O243" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O262" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="2" day="18" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="2" day="19" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-23 08:26
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="106" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF726D96-AEC4-4AB4-9678-22942C9A3485}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44CA8086-8220-46C6-A724-4BF84BD9724A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,10 +19,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$262</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$270</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5131" uniqueCount="574">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5149" uniqueCount="574">
   <si>
     <t>DATA</t>
   </si>
@@ -28471,7 +28470,7 @@
       <c r="O247" s="25"/>
       <c r="P247" s="6"/>
     </row>
-    <row r="248" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="248" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G248" s="3">
         <v>46072</v>
       </c>
@@ -28497,7 +28496,7 @@
       <c r="O248" s="25"/>
       <c r="P248" s="6"/>
     </row>
-    <row r="249" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="249" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G249" s="3">
         <v>46072</v>
       </c>
@@ -28523,7 +28522,7 @@
       <c r="O249" s="25"/>
       <c r="P249" s="6"/>
     </row>
-    <row r="250" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="250" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G250" s="3">
         <v>46072</v>
       </c>
@@ -28549,7 +28548,7 @@
       <c r="O250" s="25"/>
       <c r="P250" s="6"/>
     </row>
-    <row r="251" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="251" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="F251" t="s">
         <v>572</v>
       </c>
@@ -28578,7 +28577,7 @@
       <c r="O251" s="25"/>
       <c r="P251" s="6"/>
     </row>
-    <row r="252" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="252" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G252" s="3">
         <v>46072</v>
       </c>
@@ -28604,7 +28603,7 @@
       <c r="O252" s="25"/>
       <c r="P252" s="6"/>
     </row>
-    <row r="253" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="253" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G253" s="3">
         <v>46072</v>
       </c>
@@ -28630,7 +28629,7 @@
       <c r="O253" s="25"/>
       <c r="P253" s="6"/>
     </row>
-    <row r="254" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="254" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G254" s="3">
         <v>46072</v>
       </c>
@@ -28656,7 +28655,7 @@
       <c r="O254" s="25"/>
       <c r="P254" s="6"/>
     </row>
-    <row r="255" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="255" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G255" s="3">
         <v>46072</v>
       </c>
@@ -28682,7 +28681,7 @@
       <c r="O255" s="25"/>
       <c r="P255" s="6"/>
     </row>
-    <row r="256" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="256" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G256" s="3">
         <v>46072</v>
       </c>
@@ -28708,7 +28707,7 @@
       <c r="O256" s="25"/>
       <c r="P256" s="6"/>
     </row>
-    <row r="257" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="257" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G257" s="3">
         <v>46072</v>
       </c>
@@ -28734,7 +28733,7 @@
       <c r="O257" s="25"/>
       <c r="P257" s="6"/>
     </row>
-    <row r="258" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="258" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G258" s="3">
         <v>46072</v>
       </c>
@@ -28758,7 +28757,7 @@
       <c r="O258" s="25"/>
       <c r="P258" s="6"/>
     </row>
-    <row r="259" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="259" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G259" s="3">
         <v>46072</v>
       </c>
@@ -28782,7 +28781,7 @@
       <c r="O259" s="25"/>
       <c r="P259" s="6"/>
     </row>
-    <row r="260" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="260" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G260" s="3">
         <v>46072</v>
       </c>
@@ -28806,7 +28805,7 @@
       <c r="O260" s="25"/>
       <c r="P260" s="6"/>
     </row>
-    <row r="261" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="261" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="F261" t="s">
         <v>572</v>
       </c>
@@ -28833,7 +28832,7 @@
       <c r="O261" s="25"/>
       <c r="P261" s="6"/>
     </row>
-    <row r="262" spans="6:16" x14ac:dyDescent="0.25">
+    <row r="262" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G262" s="3">
         <v>46072</v>
       </c>
@@ -28858,40 +28857,170 @@
       <c r="P262" s="6"/>
     </row>
     <row r="263" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G263" s="4"/>
-      <c r="H263" s="4"/>
-      <c r="I263" s="6"/>
-      <c r="J263" s="4"/>
-      <c r="K263" s="8"/>
-      <c r="L263" s="4"/>
+      <c r="G263" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H263" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I263" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J263" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K263" s="8">
+        <v>240</v>
+      </c>
+      <c r="L263" s="4" t="s">
+        <v>92</v>
+      </c>
       <c r="M263" s="4"/>
-      <c r="N263" s="6"/>
+      <c r="N263" s="6">
+        <v>2</v>
+      </c>
       <c r="O263" s="25"/>
       <c r="P263" s="6"/>
     </row>
     <row r="264" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G264" s="4"/>
-      <c r="H264" s="4"/>
-      <c r="I264" s="6"/>
+      <c r="G264" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H264" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I264" s="6" t="s">
+        <v>569</v>
+      </c>
       <c r="J264" s="4"/>
       <c r="K264" s="8"/>
       <c r="L264" s="4"/>
       <c r="M264" s="4"/>
-      <c r="N264" s="6"/>
+      <c r="N264" s="6">
+        <v>2</v>
+      </c>
       <c r="O264" s="25"/>
       <c r="P264" s="6"/>
     </row>
     <row r="265" spans="6:16" x14ac:dyDescent="0.25">
-      <c r="G265" s="4"/>
-      <c r="H265" s="4"/>
-      <c r="I265" s="6"/>
+      <c r="G265" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H265" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I265" s="6" t="s">
+        <v>174</v>
+      </c>
       <c r="J265" s="4"/>
       <c r="K265" s="8"/>
       <c r="L265" s="4"/>
       <c r="M265" s="4"/>
-      <c r="N265" s="6"/>
+      <c r="N265" s="6">
+        <v>2</v>
+      </c>
       <c r="O265" s="25"/>
       <c r="P265" s="6"/>
+    </row>
+    <row r="266" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G266" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H266" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="I266" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="J266" s="4"/>
+      <c r="K266" s="8"/>
+      <c r="L266" s="4"/>
+      <c r="M266" s="4"/>
+      <c r="N266" s="6">
+        <v>2</v>
+      </c>
+      <c r="O266" s="25"/>
+      <c r="P266" s="6"/>
+    </row>
+    <row r="267" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G267" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H267" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I267" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J267" s="4"/>
+      <c r="K267" s="8"/>
+      <c r="L267" s="4"/>
+      <c r="M267" s="4"/>
+      <c r="N267" s="6">
+        <v>2</v>
+      </c>
+      <c r="O267" s="25"/>
+      <c r="P267" s="6"/>
+    </row>
+    <row r="268" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G268" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H268" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I268" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J268" s="4"/>
+      <c r="K268" s="8"/>
+      <c r="L268" s="4"/>
+      <c r="M268" s="4"/>
+      <c r="N268" s="6">
+        <v>2</v>
+      </c>
+      <c r="O268" s="25"/>
+      <c r="P268" s="6"/>
+    </row>
+    <row r="269" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G269" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H269" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="I269" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J269" s="4"/>
+      <c r="K269" s="8"/>
+      <c r="L269" s="4"/>
+      <c r="M269" s="4"/>
+      <c r="N269" s="6">
+        <v>2</v>
+      </c>
+      <c r="O269" s="25"/>
+      <c r="P269" s="6"/>
+    </row>
+    <row r="270" spans="6:16" x14ac:dyDescent="0.25">
+      <c r="G270" s="3">
+        <v>46076</v>
+      </c>
+      <c r="H270" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I270" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J270" s="4"/>
+      <c r="K270" s="8"/>
+      <c r="L270" s="4"/>
+      <c r="M270" s="4"/>
+      <c r="N270" s="6">
+        <v>3</v>
+      </c>
+      <c r="O270" s="25"/>
+      <c r="P270" s="6"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -28924,10 +29053,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O262" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O270" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="2" day="19" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="2" day="23" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-26 16:46
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="392" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0EC667A-4454-46A3-B903-34F2B52692E1}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEED7075-44B6-4FBD-B6AB-10F0217A0840}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5275" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5279" uniqueCount="588">
   <si>
     <t>DATA</t>
   </si>
@@ -1951,7 +1951,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2091,6 +2091,7 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -29805,7 +29806,7 @@
         <v>414</v>
       </c>
       <c r="K299" s="8">
-        <v>190</v>
+        <v>290</v>
       </c>
       <c r="L299" s="4" t="s">
         <v>464</v>
@@ -29842,6 +29843,26 @@
       <c r="P300" s="6"/>
     </row>
     <row r="301" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G301" s="3">
+        <v>46079</v>
+      </c>
+      <c r="H301" s="4" t="s">
+        <v>497</v>
+      </c>
+      <c r="I301" s="59" t="s">
+        <v>129</v>
+      </c>
+      <c r="J301" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="K301" s="8">
+        <v>230</v>
+      </c>
+      <c r="L301" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="M301" s="4"/>
+      <c r="N301" s="6"/>
       <c r="O301" s="25"/>
       <c r="P301" s="6"/>
     </row>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-27 08:40
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEED7075-44B6-4FBD-B6AB-10F0217A0840}"/>
+  <xr:revisionPtr revIDLastSave="408" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F32BF347-85EC-4299-A20A-87C45AF61CCA}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$302</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5279" uniqueCount="588">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5283" uniqueCount="588">
   <si>
     <t>DATA</t>
   </si>
@@ -1951,7 +1951,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2091,7 +2091,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -29324,7 +29323,7 @@
       <c r="O280" s="25"/>
       <c r="P280" s="6"/>
     </row>
-    <row r="281" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="281" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G281" s="3">
         <v>46078</v>
       </c>
@@ -29350,7 +29349,7 @@
       <c r="O281" s="25"/>
       <c r="P281" s="6"/>
     </row>
-    <row r="282" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="282" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G282" s="3">
         <v>46078</v>
       </c>
@@ -29376,7 +29375,7 @@
       <c r="O282" s="25"/>
       <c r="P282" s="6"/>
     </row>
-    <row r="283" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="283" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G283" s="3">
         <v>46078</v>
       </c>
@@ -29402,7 +29401,7 @@
       <c r="O283" s="25"/>
       <c r="P283" s="6"/>
     </row>
-    <row r="284" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="284" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G284" s="3">
         <v>46078</v>
       </c>
@@ -29428,7 +29427,7 @@
       <c r="O284" s="25"/>
       <c r="P284" s="6"/>
     </row>
-    <row r="285" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="285" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G285" s="3">
         <v>46078</v>
       </c>
@@ -29454,7 +29453,7 @@
       <c r="O285" s="25"/>
       <c r="P285" s="6"/>
     </row>
-    <row r="286" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="286" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G286" s="3">
         <v>46078</v>
       </c>
@@ -29480,7 +29479,7 @@
       <c r="O286" s="25"/>
       <c r="P286" s="6"/>
     </row>
-    <row r="287" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="287" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G287" s="3">
         <v>46078</v>
       </c>
@@ -29506,7 +29505,7 @@
       <c r="O287" s="25"/>
       <c r="P287" s="6"/>
     </row>
-    <row r="288" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="288" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G288" s="3">
         <v>46078</v>
       </c>
@@ -29532,7 +29531,7 @@
       <c r="O288" s="25"/>
       <c r="P288" s="6"/>
     </row>
-    <row r="289" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="289" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G289" s="3">
         <v>46078</v>
       </c>
@@ -29849,7 +29848,7 @@
       <c r="H301" s="4" t="s">
         <v>497</v>
       </c>
-      <c r="I301" s="59" t="s">
+      <c r="I301" s="6" t="s">
         <v>129</v>
       </c>
       <c r="J301" s="4" t="s">
@@ -29866,6 +29865,30 @@
       <c r="O301" s="25"/>
       <c r="P301" s="6"/>
     </row>
+    <row r="302" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G302" s="3">
+        <v>46079</v>
+      </c>
+      <c r="H302" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="I302" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="J302" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K302" s="8">
+        <v>200</v>
+      </c>
+      <c r="L302" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M302" s="4"/>
+      <c r="N302" s="6"/>
+      <c r="O302" s="25"/>
+      <c r="P302" s="6"/>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -29897,9 +29920,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O301" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O302" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
+        <dateGroupItem year="2026" month="2" day="25" dateTimeGrouping="day"/>
         <dateGroupItem year="2026" month="2" day="26" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-04 15:21
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="559" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{071D1C2C-3966-464C-A7C7-260868DD8D80}"/>
+  <xr:revisionPtr revIDLastSave="620" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4F7FB76-E793-48C6-88A9-5B6242962477}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$340</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5360" uniqueCount="596">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5389" uniqueCount="598">
   <si>
     <t>DATA</t>
   </si>
@@ -1829,6 +1829,12 @@
   </si>
   <si>
     <t>HOTEL ALVORADA DA SERRA</t>
+  </si>
+  <si>
+    <t>ELOI MENDER</t>
+  </si>
+  <si>
+    <t/>
   </si>
 </sst>
 </file>
@@ -1975,7 +1981,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2115,6 +2121,8 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -30145,7 +30153,7 @@
       <c r="O311" s="25"/>
       <c r="P311" s="6"/>
     </row>
-    <row r="312" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="312" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G312" s="3">
         <v>46084</v>
       </c>
@@ -30171,7 +30179,7 @@
       <c r="O312" s="25"/>
       <c r="P312" s="6"/>
     </row>
-    <row r="313" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="313" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G313" s="3">
         <v>46084</v>
       </c>
@@ -30197,7 +30205,7 @@
       <c r="O313" s="25"/>
       <c r="P313" s="6"/>
     </row>
-    <row r="314" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="314" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G314" s="3">
         <v>46084</v>
       </c>
@@ -30223,7 +30231,7 @@
       <c r="O314" s="25"/>
       <c r="P314" s="6"/>
     </row>
-    <row r="315" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="315" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G315" s="3">
         <v>46084</v>
       </c>
@@ -30249,7 +30257,7 @@
       <c r="O315" s="25"/>
       <c r="P315" s="6"/>
     </row>
-    <row r="316" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="316" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G316" s="3">
         <v>46084</v>
       </c>
@@ -30275,7 +30283,7 @@
       <c r="O316" s="25"/>
       <c r="P316" s="6"/>
     </row>
-    <row r="317" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="317" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G317" s="3">
         <v>46084</v>
       </c>
@@ -30301,7 +30309,7 @@
       <c r="O317" s="25"/>
       <c r="P317" s="6"/>
     </row>
-    <row r="318" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="318" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G318" s="3">
         <v>46084</v>
       </c>
@@ -30327,7 +30335,7 @@
       <c r="O318" s="25"/>
       <c r="P318" s="6"/>
     </row>
-    <row r="319" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="319" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G319" s="3">
         <v>46084</v>
       </c>
@@ -30353,7 +30361,7 @@
       <c r="O319" s="25"/>
       <c r="P319" s="6"/>
     </row>
-    <row r="320" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="320" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G320" s="3">
         <v>46084</v>
       </c>
@@ -30379,7 +30387,7 @@
       <c r="O320" s="25"/>
       <c r="P320" s="6"/>
     </row>
-    <row r="321" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="321" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G321" s="3">
         <v>46084</v>
       </c>
@@ -30416,6 +30424,213 @@
     <row r="328" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G328" s="3"/>
     </row>
+    <row r="329" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G329" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H329" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I329" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="J329" s="4" t="s">
+        <v>596</v>
+      </c>
+      <c r="K329" s="8">
+        <v>249.9</v>
+      </c>
+      <c r="L329" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M329" s="4"/>
+      <c r="N329" s="59">
+        <v>2</v>
+      </c>
+      <c r="O329" s="25"/>
+      <c r="P329" s="6"/>
+    </row>
+    <row r="330" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G330" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H330" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I330" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J330" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="K330" s="8">
+        <v>180</v>
+      </c>
+      <c r="L330" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="M330" s="4"/>
+      <c r="N330" s="59">
+        <v>2</v>
+      </c>
+      <c r="O330" s="25"/>
+      <c r="P330" s="6"/>
+    </row>
+    <row r="331" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G331" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H331" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="I331" s="59" t="s">
+        <v>515</v>
+      </c>
+      <c r="J331" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K331" s="8">
+        <v>250</v>
+      </c>
+      <c r="L331" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="M331" s="4"/>
+      <c r="N331" s="6">
+        <v>3</v>
+      </c>
+      <c r="O331" s="25"/>
+      <c r="P331" s="6"/>
+    </row>
+    <row r="332" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G332" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H332" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I332" s="59" t="s">
+        <v>133</v>
+      </c>
+      <c r="J332" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K332" s="8">
+        <v>280</v>
+      </c>
+      <c r="L332" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M332" s="4"/>
+      <c r="N332" s="6">
+        <v>2</v>
+      </c>
+      <c r="O332" s="25"/>
+      <c r="P332" s="6"/>
+    </row>
+    <row r="333" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G333" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H333" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I333" s="59" t="s">
+        <v>129</v>
+      </c>
+      <c r="J333" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K333" s="8">
+        <v>200</v>
+      </c>
+      <c r="L333" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M333" s="4"/>
+      <c r="N333" s="6">
+        <v>3</v>
+      </c>
+      <c r="O333" s="25"/>
+      <c r="P333" s="6"/>
+    </row>
+    <row r="334" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G334" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H334" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I334" s="59" t="s">
+        <v>125</v>
+      </c>
+      <c r="J334" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K334" s="8">
+        <v>265</v>
+      </c>
+      <c r="L334" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M334" s="4"/>
+      <c r="N334" s="6">
+        <v>3</v>
+      </c>
+      <c r="O334" s="25"/>
+      <c r="P334" s="6"/>
+    </row>
+    <row r="335" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G335" s="3">
+        <v>46085</v>
+      </c>
+      <c r="H335" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I335" s="59" t="s">
+        <v>195</v>
+      </c>
+      <c r="J335" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K335" s="8">
+        <v>230</v>
+      </c>
+      <c r="L335" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M335" s="4"/>
+      <c r="N335" s="6">
+        <v>3</v>
+      </c>
+      <c r="O335" s="25"/>
+      <c r="P335" s="6"/>
+    </row>
+    <row r="336" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="O336" s="25"/>
+      <c r="P336" s="6"/>
+    </row>
+    <row r="337" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O337" s="25"/>
+      <c r="P337" s="6"/>
+    </row>
+    <row r="338" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O338" s="25"/>
+      <c r="P338" s="6"/>
+    </row>
+    <row r="339" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O339" s="25"/>
+      <c r="P339" s="6"/>
+    </row>
+    <row r="340" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O340" s="25"/>
+      <c r="P340" s="6"/>
+    </row>
+    <row r="353" spans="15:15" x14ac:dyDescent="0.25">
+      <c r="O353" s="60" t="s">
+        <v>597</v>
+      </c>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -30447,10 +30662,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O328" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O340" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="3" day="3" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="3" day="4" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-05 12:37
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="620" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B4F7FB76-E793-48C6-88A9-5B6242962477}"/>
+  <xr:revisionPtr revIDLastSave="645" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2277ED9D-3A8B-42CE-B1BF-3689D69F149D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$340</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$353</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5389" uniqueCount="598">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5417" uniqueCount="601">
   <si>
     <t>DATA</t>
   </si>
@@ -1835,6 +1835,15 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>VALTER</t>
+  </si>
+  <si>
+    <t>CAIQUE LACER</t>
+  </si>
+  <si>
+    <t>JOSE AR</t>
   </si>
 </sst>
 </file>
@@ -2122,7 +2131,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -30424,7 +30433,7 @@
     <row r="328" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G328" s="3"/>
     </row>
-    <row r="329" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="329" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G329" s="3">
         <v>46085</v>
       </c>
@@ -30444,13 +30453,13 @@
         <v>210</v>
       </c>
       <c r="M329" s="4"/>
-      <c r="N329" s="59">
+      <c r="N329" s="6">
         <v>2</v>
       </c>
       <c r="O329" s="25"/>
       <c r="P329" s="6"/>
     </row>
-    <row r="330" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="330" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G330" s="3">
         <v>46085</v>
       </c>
@@ -30470,20 +30479,20 @@
         <v>212</v>
       </c>
       <c r="M330" s="4"/>
-      <c r="N330" s="59">
+      <c r="N330" s="6">
         <v>2</v>
       </c>
       <c r="O330" s="25"/>
       <c r="P330" s="6"/>
     </row>
-    <row r="331" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="331" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G331" s="3">
         <v>46085</v>
       </c>
       <c r="H331" s="4" t="s">
         <v>537</v>
       </c>
-      <c r="I331" s="59" t="s">
+      <c r="I331" s="6" t="s">
         <v>515</v>
       </c>
       <c r="J331" s="4" t="s">
@@ -30502,14 +30511,14 @@
       <c r="O331" s="25"/>
       <c r="P331" s="6"/>
     </row>
-    <row r="332" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="332" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G332" s="3">
         <v>46085</v>
       </c>
       <c r="H332" s="4" t="s">
         <v>130</v>
       </c>
-      <c r="I332" s="59" t="s">
+      <c r="I332" s="6" t="s">
         <v>133</v>
       </c>
       <c r="J332" s="4" t="s">
@@ -30528,14 +30537,14 @@
       <c r="O332" s="25"/>
       <c r="P332" s="6"/>
     </row>
-    <row r="333" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="333" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G333" s="3">
         <v>46085</v>
       </c>
       <c r="H333" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="I333" s="59" t="s">
+      <c r="I333" s="6" t="s">
         <v>129</v>
       </c>
       <c r="J333" s="4" t="s">
@@ -30554,14 +30563,14 @@
       <c r="O333" s="25"/>
       <c r="P333" s="6"/>
     </row>
-    <row r="334" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="334" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G334" s="3">
         <v>46085</v>
       </c>
       <c r="H334" s="4" t="s">
         <v>491</v>
       </c>
-      <c r="I334" s="59" t="s">
+      <c r="I334" s="6" t="s">
         <v>125</v>
       </c>
       <c r="J334" s="4" t="s">
@@ -30580,14 +30589,14 @@
       <c r="O334" s="25"/>
       <c r="P334" s="6"/>
     </row>
-    <row r="335" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="335" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G335" s="3">
         <v>46085</v>
       </c>
       <c r="H335" s="4" t="s">
         <v>506</v>
       </c>
-      <c r="I335" s="59" t="s">
+      <c r="I335" s="6" t="s">
         <v>195</v>
       </c>
       <c r="J335" s="4" t="s">
@@ -30606,30 +30615,267 @@
       <c r="O335" s="25"/>
       <c r="P335" s="6"/>
     </row>
-    <row r="336" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="336" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O336" s="25"/>
       <c r="P336" s="6"/>
     </row>
-    <row r="337" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O337" s="25"/>
       <c r="P337" s="6"/>
     </row>
-    <row r="338" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O338" s="25"/>
       <c r="P338" s="6"/>
     </row>
-    <row r="339" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O339" s="25"/>
       <c r="P339" s="6"/>
     </row>
-    <row r="340" spans="15:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="O340" s="25"/>
-      <c r="P340" s="6"/>
-    </row>
-    <row r="353" spans="15:15" x14ac:dyDescent="0.25">
+    <row r="340" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O340" s="37"/>
+      <c r="P340" s="29"/>
+    </row>
+    <row r="341" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G341" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H341" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I341" s="6" t="s">
+        <v>593</v>
+      </c>
+      <c r="J341" s="4"/>
+      <c r="K341" s="8"/>
+      <c r="L341" s="4"/>
+      <c r="M341" s="4"/>
+      <c r="N341" s="6"/>
+      <c r="O341" s="25"/>
+      <c r="P341" s="6"/>
+    </row>
+    <row r="342" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G342" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H342" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I342" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J342" s="4"/>
+      <c r="K342" s="8"/>
+      <c r="L342" s="4"/>
+      <c r="M342" s="4"/>
+      <c r="N342" s="6"/>
+      <c r="O342" s="25"/>
+      <c r="P342" s="6"/>
+    </row>
+    <row r="343" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G343" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H343" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="I343" s="6" t="s">
+        <v>515</v>
+      </c>
+      <c r="J343" s="4"/>
+      <c r="K343" s="8"/>
+      <c r="L343" s="4"/>
+      <c r="M343" s="4"/>
+      <c r="N343" s="6"/>
+      <c r="O343" s="25"/>
+      <c r="P343" s="6"/>
+    </row>
+    <row r="344" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G344" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H344" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I344" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J344" s="4"/>
+      <c r="K344" s="8"/>
+      <c r="L344" s="4"/>
+      <c r="M344" s="4"/>
+      <c r="N344" s="6"/>
+      <c r="O344" s="25"/>
+      <c r="P344" s="6"/>
+    </row>
+    <row r="345" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G345" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H345" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I345" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J345" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="K345" s="8">
+        <v>239</v>
+      </c>
+      <c r="L345" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="M345" s="4"/>
+      <c r="N345" s="6"/>
+      <c r="O345" s="25"/>
+      <c r="P345" s="6"/>
+    </row>
+    <row r="346" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G346" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H346" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I346" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J346" s="4"/>
+      <c r="K346" s="8"/>
+      <c r="L346" s="4"/>
+      <c r="M346" s="4"/>
+      <c r="N346" s="6"/>
+      <c r="O346" s="25"/>
+      <c r="P346" s="6"/>
+    </row>
+    <row r="347" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G347" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H347" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I347" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J347" s="4"/>
+      <c r="K347" s="8"/>
+      <c r="L347" s="4"/>
+      <c r="M347" s="4"/>
+      <c r="N347" s="6"/>
+      <c r="O347" s="25"/>
+      <c r="P347" s="6"/>
+    </row>
+    <row r="348" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G348" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H348" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I348" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J348" s="4"/>
+      <c r="K348" s="8"/>
+      <c r="L348" s="4"/>
+      <c r="M348" s="4"/>
+      <c r="N348" s="6"/>
+      <c r="O348" s="25"/>
+      <c r="P348" s="6"/>
+    </row>
+    <row r="349" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G349" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H349" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I349" s="6" t="s">
+        <v>598</v>
+      </c>
+      <c r="J349" s="4"/>
+      <c r="K349" s="8"/>
+      <c r="L349" s="4"/>
+      <c r="M349" s="4"/>
+      <c r="N349" s="6"/>
+      <c r="O349" s="25"/>
+      <c r="P349" s="6"/>
+    </row>
+    <row r="350" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G350" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H350" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="I350" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="J350" s="4"/>
+      <c r="K350" s="8"/>
+      <c r="L350" s="4"/>
+      <c r="M350" s="4"/>
+      <c r="N350" s="6"/>
+      <c r="O350" s="25"/>
+      <c r="P350" s="6"/>
+    </row>
+    <row r="351" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G351" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H351" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="I351" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="J351" s="4"/>
+      <c r="K351" s="8"/>
+      <c r="L351" s="4"/>
+      <c r="M351" s="4"/>
+      <c r="N351" s="6"/>
+      <c r="O351" s="25"/>
+      <c r="P351" s="6"/>
+    </row>
+    <row r="352" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G352" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H352" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I352" s="59" t="s">
+        <v>213</v>
+      </c>
+      <c r="J352" s="4"/>
+      <c r="K352" s="8"/>
+      <c r="L352" s="4"/>
+      <c r="M352" s="4"/>
+      <c r="N352" s="6"/>
+      <c r="O352" s="25"/>
+      <c r="P352" s="6"/>
+    </row>
+    <row r="353" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G353" s="3">
+        <v>46086</v>
+      </c>
+      <c r="H353" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="I353" s="59" t="s">
+        <v>131</v>
+      </c>
+      <c r="J353" s="4"/>
+      <c r="K353" s="8"/>
+      <c r="L353" s="4"/>
+      <c r="M353" s="4"/>
+      <c r="N353" s="6"/>
       <c r="O353" s="60" t="s">
         <v>597</v>
       </c>
+      <c r="P353" s="6"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -30662,10 +30908,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O340" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O353" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="3" day="4" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="3" day="5" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-12 16:27
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="645" documentId="13_ncr:1_{2D0A47D7-273B-4CA0-B44B-89F09CAFB401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2277ED9D-3A8B-42CE-B1BF-3689D69F149D}"/>
+  <xr:revisionPtr revIDLastSave="288" documentId="13_ncr:1_{CF87F821-98AE-4A1A-B4F9-A70BAAFD478B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A6A9892-D45A-4B38-84A5-EF67E28B7C2E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,9 +19,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$353</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$389</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5417" uniqueCount="601">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5578" uniqueCount="615">
   <si>
     <t>DATA</t>
   </si>
@@ -1844,6 +1845,48 @@
   </si>
   <si>
     <t>JOSE AR</t>
+  </si>
+  <si>
+    <t>HOTEL MAIA</t>
+  </si>
+  <si>
+    <t>aldemir</t>
+  </si>
+  <si>
+    <t>fernando gomes</t>
+  </si>
+  <si>
+    <t>jose</t>
+  </si>
+  <si>
+    <t>iago</t>
+  </si>
+  <si>
+    <t>ELOI</t>
+  </si>
+  <si>
+    <t>HOTEL GONZAGA</t>
+  </si>
+  <si>
+    <t>CAPITOLIO</t>
+  </si>
+  <si>
+    <t>HOTEL NAIM</t>
+  </si>
+  <si>
+    <t>PERDOES</t>
+  </si>
+  <si>
+    <t>HOTEL VILHAMAR</t>
+  </si>
+  <si>
+    <t>HOTEL BH RIOS</t>
+  </si>
+  <si>
+    <t>NACIONAL INN</t>
+  </si>
+  <si>
+    <t>SP SOROCABA</t>
   </si>
 </sst>
 </file>
@@ -1990,7 +2033,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2130,7 +2173,6 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
@@ -30619,23 +30661,23 @@
       <c r="O336" s="25"/>
       <c r="P336" s="6"/>
     </row>
-    <row r="337" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="337" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O337" s="25"/>
       <c r="P337" s="6"/>
     </row>
-    <row r="338" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="338" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O338" s="25"/>
       <c r="P338" s="6"/>
     </row>
-    <row r="339" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="339" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O339" s="25"/>
       <c r="P339" s="6"/>
     </row>
-    <row r="340" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="340" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="O340" s="37"/>
       <c r="P340" s="29"/>
     </row>
-    <row r="341" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="341" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G341" s="3">
         <v>46086</v>
       </c>
@@ -30645,15 +30687,21 @@
       <c r="I341" s="6" t="s">
         <v>593</v>
       </c>
-      <c r="J341" s="4"/>
-      <c r="K341" s="8"/>
-      <c r="L341" s="4"/>
+      <c r="J341" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="K341" s="8">
+        <v>170</v>
+      </c>
+      <c r="L341" s="4" t="s">
+        <v>187</v>
+      </c>
       <c r="M341" s="4"/>
       <c r="N341" s="6"/>
       <c r="O341" s="25"/>
       <c r="P341" s="6"/>
     </row>
-    <row r="342" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="342" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G342" s="3">
         <v>46086</v>
       </c>
@@ -30663,15 +30711,21 @@
       <c r="I342" s="6" t="s">
         <v>529</v>
       </c>
-      <c r="J342" s="4"/>
-      <c r="K342" s="8"/>
-      <c r="L342" s="4"/>
+      <c r="J342" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="K342" s="8">
+        <v>200</v>
+      </c>
+      <c r="L342" s="4" t="s">
+        <v>433</v>
+      </c>
       <c r="M342" s="4"/>
       <c r="N342" s="6"/>
       <c r="O342" s="25"/>
       <c r="P342" s="6"/>
     </row>
-    <row r="343" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="343" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G343" s="3">
         <v>46086</v>
       </c>
@@ -30681,15 +30735,21 @@
       <c r="I343" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="J343" s="4"/>
-      <c r="K343" s="8"/>
-      <c r="L343" s="4"/>
+      <c r="J343" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="K343" s="8">
+        <v>220</v>
+      </c>
+      <c r="L343" s="4" t="s">
+        <v>30</v>
+      </c>
       <c r="M343" s="4"/>
       <c r="N343" s="6"/>
       <c r="O343" s="25"/>
       <c r="P343" s="6"/>
     </row>
-    <row r="344" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="344" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G344" s="3">
         <v>46086</v>
       </c>
@@ -30699,15 +30759,21 @@
       <c r="I344" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="J344" s="4"/>
-      <c r="K344" s="8"/>
-      <c r="L344" s="4"/>
+      <c r="J344" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K344" s="8">
+        <v>200</v>
+      </c>
+      <c r="L344" s="4" t="s">
+        <v>518</v>
+      </c>
       <c r="M344" s="4"/>
       <c r="N344" s="6"/>
       <c r="O344" s="25"/>
       <c r="P344" s="6"/>
     </row>
-    <row r="345" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="345" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G345" s="3">
         <v>46086</v>
       </c>
@@ -30731,7 +30797,7 @@
       <c r="O345" s="25"/>
       <c r="P345" s="6"/>
     </row>
-    <row r="346" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="346" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G346" s="3">
         <v>46086</v>
       </c>
@@ -30741,15 +30807,21 @@
       <c r="I346" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="J346" s="4"/>
-      <c r="K346" s="8"/>
-      <c r="L346" s="4"/>
+      <c r="J346" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K346" s="8">
+        <v>190</v>
+      </c>
+      <c r="L346" s="4" t="s">
+        <v>469</v>
+      </c>
       <c r="M346" s="4"/>
       <c r="N346" s="6"/>
       <c r="O346" s="25"/>
       <c r="P346" s="6"/>
     </row>
-    <row r="347" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="347" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G347" s="3">
         <v>46086</v>
       </c>
@@ -30759,15 +30831,21 @@
       <c r="I347" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="J347" s="4"/>
-      <c r="K347" s="8"/>
-      <c r="L347" s="4"/>
+      <c r="J347" s="4" t="s">
+        <v>449</v>
+      </c>
+      <c r="K347" s="8">
+        <v>260</v>
+      </c>
+      <c r="L347" s="4" t="s">
+        <v>271</v>
+      </c>
       <c r="M347" s="4"/>
       <c r="N347" s="6"/>
       <c r="O347" s="25"/>
       <c r="P347" s="6"/>
     </row>
-    <row r="348" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="348" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G348" s="3">
         <v>46086</v>
       </c>
@@ -30777,15 +30855,24 @@
       <c r="I348" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="J348" s="4"/>
-      <c r="K348" s="8"/>
-      <c r="L348" s="4"/>
+      <c r="J348" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K348" s="8">
+        <v>240</v>
+      </c>
+      <c r="L348" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="M348" s="4"/>
       <c r="N348" s="6"/>
       <c r="O348" s="25"/>
       <c r="P348" s="6"/>
     </row>
-    <row r="349" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="349" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F349" t="s">
+        <v>566</v>
+      </c>
       <c r="G349" s="3">
         <v>46086</v>
       </c>
@@ -30795,15 +30882,21 @@
       <c r="I349" s="6" t="s">
         <v>598</v>
       </c>
-      <c r="J349" s="4"/>
-      <c r="K349" s="8"/>
-      <c r="L349" s="4"/>
+      <c r="J349" s="4" t="s">
+        <v>402</v>
+      </c>
+      <c r="K349" s="8">
+        <v>209</v>
+      </c>
+      <c r="L349" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="M349" s="4"/>
       <c r="N349" s="6"/>
       <c r="O349" s="25"/>
       <c r="P349" s="6"/>
     </row>
-    <row r="350" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="350" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G350" s="3">
         <v>46086</v>
       </c>
@@ -30813,15 +30906,21 @@
       <c r="I350" s="6" t="s">
         <v>599</v>
       </c>
-      <c r="J350" s="4"/>
-      <c r="K350" s="8"/>
-      <c r="L350" s="4"/>
+      <c r="J350" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="K350" s="8">
+        <v>200</v>
+      </c>
+      <c r="L350" s="4" t="s">
+        <v>518</v>
+      </c>
       <c r="M350" s="4"/>
       <c r="N350" s="6"/>
       <c r="O350" s="25"/>
       <c r="P350" s="6"/>
     </row>
-    <row r="351" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="351" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G351" s="3">
         <v>46086</v>
       </c>
@@ -30831,51 +30930,963 @@
       <c r="I351" s="6" t="s">
         <v>502</v>
       </c>
-      <c r="J351" s="4"/>
-      <c r="K351" s="8"/>
-      <c r="L351" s="4"/>
+      <c r="J351" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K351" s="8">
+        <v>220</v>
+      </c>
+      <c r="L351" s="4" t="s">
+        <v>9</v>
+      </c>
       <c r="M351" s="4"/>
       <c r="N351" s="6"/>
       <c r="O351" s="25"/>
       <c r="P351" s="6"/>
     </row>
-    <row r="352" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="352" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G352" s="3">
         <v>46086</v>
       </c>
       <c r="H352" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="I352" s="59" t="s">
+      <c r="I352" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="J352" s="4"/>
-      <c r="K352" s="8"/>
-      <c r="L352" s="4"/>
+      <c r="J352" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K352" s="8">
+        <v>190</v>
+      </c>
+      <c r="L352" s="4" t="s">
+        <v>55</v>
+      </c>
       <c r="M352" s="4"/>
       <c r="N352" s="6"/>
       <c r="O352" s="25"/>
       <c r="P352" s="6"/>
     </row>
-    <row r="353" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="353" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G353" s="3">
         <v>46086</v>
       </c>
       <c r="H353" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="I353" s="59" t="s">
+      <c r="I353" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="J353" s="4"/>
-      <c r="K353" s="8"/>
-      <c r="L353" s="4"/>
+      <c r="J353" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="K353" s="8">
+        <v>220</v>
+      </c>
+      <c r="L353" s="4" t="s">
+        <v>412</v>
+      </c>
       <c r="M353" s="4"/>
       <c r="N353" s="6"/>
-      <c r="O353" s="60" t="s">
+      <c r="O353" s="59" t="s">
         <v>597</v>
       </c>
       <c r="P353" s="6"/>
+    </row>
+    <row r="354" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G354" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H354" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="I354" s="6" t="s">
+        <v>599</v>
+      </c>
+      <c r="J354" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K354" s="8">
+        <v>240</v>
+      </c>
+      <c r="L354" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="M354" s="4"/>
+      <c r="N354" s="6">
+        <v>2</v>
+      </c>
+      <c r="O354" s="25"/>
+      <c r="P354" s="6"/>
+    </row>
+    <row r="355" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G355" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H355" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I355" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="J355" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K355" s="8">
+        <v>190</v>
+      </c>
+      <c r="L355" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="M355" s="4"/>
+      <c r="N355" s="6">
+        <v>2</v>
+      </c>
+      <c r="O355" s="25"/>
+      <c r="P355" s="6"/>
+    </row>
+    <row r="356" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G356" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H356" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I356" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J356" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K356" s="8">
+        <v>240</v>
+      </c>
+      <c r="L356" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M356" s="4"/>
+      <c r="N356" s="6">
+        <v>2</v>
+      </c>
+      <c r="O356" s="25"/>
+      <c r="P356" s="6"/>
+    </row>
+    <row r="357" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G357" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H357" s="4" t="s">
+        <v>494</v>
+      </c>
+      <c r="I357" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J357" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K357" s="8">
+        <v>240</v>
+      </c>
+      <c r="L357" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M357" s="4"/>
+      <c r="N357" s="6">
+        <v>2</v>
+      </c>
+      <c r="O357" s="25"/>
+      <c r="P357" s="6"/>
+    </row>
+    <row r="358" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G358" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H358" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I358" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J358" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K358" s="8">
+        <v>200</v>
+      </c>
+      <c r="L358" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M358" s="4"/>
+      <c r="N358" s="6">
+        <v>2</v>
+      </c>
+      <c r="O358" s="25"/>
+      <c r="P358" s="6"/>
+    </row>
+    <row r="359" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G359" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H359" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I359" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J359" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K359" s="8">
+        <v>190</v>
+      </c>
+      <c r="L359" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M359" s="4"/>
+      <c r="N359" s="6">
+        <v>2</v>
+      </c>
+      <c r="O359" s="25"/>
+      <c r="P359" s="6"/>
+    </row>
+    <row r="360" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G360" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H360" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="I360" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="J360" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K360" s="8">
+        <v>170</v>
+      </c>
+      <c r="L360" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="M360" s="4"/>
+      <c r="N360" s="6">
+        <v>2</v>
+      </c>
+      <c r="O360" s="25"/>
+      <c r="P360" s="6"/>
+    </row>
+    <row r="361" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G361" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H361" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I361" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J361" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="K361" s="8">
+        <v>170</v>
+      </c>
+      <c r="L361" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="M361" s="4"/>
+      <c r="N361" s="6">
+        <v>3</v>
+      </c>
+      <c r="O361" s="25"/>
+      <c r="P361" s="6"/>
+    </row>
+    <row r="362" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G362" s="3">
+        <v>46090</v>
+      </c>
+      <c r="H362" s="4" t="s">
+        <v>505</v>
+      </c>
+      <c r="I362" s="6" t="s">
+        <v>548</v>
+      </c>
+      <c r="J362" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K362" s="8">
+        <v>200</v>
+      </c>
+      <c r="L362" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M362" s="4"/>
+      <c r="N362" s="6">
+        <v>2</v>
+      </c>
+      <c r="O362" s="25"/>
+      <c r="P362" s="6"/>
+    </row>
+    <row r="363" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G363" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H363" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I363" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J363" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="K363" s="8">
+        <v>200</v>
+      </c>
+      <c r="L363" s="4" t="s">
+        <v>573</v>
+      </c>
+      <c r="M363" s="4"/>
+      <c r="N363" s="6"/>
+      <c r="O363" s="25"/>
+      <c r="P363" s="6"/>
+    </row>
+    <row r="364" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G364" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H364" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="I364" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J364" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K364" s="8">
+        <v>240</v>
+      </c>
+      <c r="L364" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="M364" s="4"/>
+      <c r="N364" s="6">
+        <v>2</v>
+      </c>
+      <c r="O364" s="25"/>
+      <c r="P364" s="6"/>
+    </row>
+    <row r="365" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G365" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H365" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I365" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="J365" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="K365" s="8">
+        <v>249.9</v>
+      </c>
+      <c r="L365" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="M365" s="4"/>
+      <c r="N365" s="6">
+        <v>3</v>
+      </c>
+      <c r="O365" s="25"/>
+      <c r="P365" s="6"/>
+    </row>
+    <row r="366" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G366" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H366" s="4" t="s">
+        <v>604</v>
+      </c>
+      <c r="I366" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="J366" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="K366" s="8">
+        <v>300</v>
+      </c>
+      <c r="L366" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="M366" s="4"/>
+      <c r="N366" s="6">
+        <v>3</v>
+      </c>
+      <c r="O366" s="25"/>
+      <c r="P366" s="6"/>
+    </row>
+    <row r="367" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G367" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H367" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="I367" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J367" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="K367" s="8">
+        <v>160</v>
+      </c>
+      <c r="L367" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="M367" s="4"/>
+      <c r="N367" s="6">
+        <v>2</v>
+      </c>
+      <c r="O367" s="25"/>
+      <c r="P367" s="6"/>
+    </row>
+    <row r="368" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G368" s="3">
+        <v>46091</v>
+      </c>
+      <c r="H368" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="I368" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J368" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="K368" s="8">
+        <v>239</v>
+      </c>
+      <c r="L368" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="M368" s="4"/>
+      <c r="N368" s="6">
+        <v>2</v>
+      </c>
+      <c r="O368" s="25"/>
+      <c r="P368" s="6"/>
+    </row>
+    <row r="369" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G369" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H369" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="I369" s="6" t="s">
+        <v>603</v>
+      </c>
+      <c r="J369" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="K369" s="8">
+        <v>240</v>
+      </c>
+      <c r="L369" s="4" t="s">
+        <v>611</v>
+      </c>
+      <c r="M369" s="4"/>
+      <c r="N369" s="6"/>
+      <c r="O369" s="25"/>
+      <c r="P369" s="6"/>
+    </row>
+    <row r="370" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G370" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H370" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="I370" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J370" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="K370" s="8">
+        <v>200</v>
+      </c>
+      <c r="L370" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="M370" s="4"/>
+      <c r="N370" s="6"/>
+      <c r="O370" s="25"/>
+      <c r="P370" s="6"/>
+    </row>
+    <row r="371" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G371" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H371" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="I371" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="J371" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="K371" s="8">
+        <v>220</v>
+      </c>
+      <c r="L371" s="4" t="s">
+        <v>464</v>
+      </c>
+      <c r="M371" s="4"/>
+      <c r="N371" s="6"/>
+      <c r="O371" s="25"/>
+      <c r="P371" s="6"/>
+    </row>
+    <row r="372" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G372" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H372" s="4" t="s">
+        <v>377</v>
+      </c>
+      <c r="I372" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="J372" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K372" s="8">
+        <v>240</v>
+      </c>
+      <c r="L372" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M372" s="4"/>
+      <c r="N372" s="6">
+        <v>3</v>
+      </c>
+      <c r="O372" s="25"/>
+      <c r="P372" s="6"/>
+    </row>
+    <row r="373" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G373" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H373" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I373" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J373" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="K373" s="8">
+        <v>200</v>
+      </c>
+      <c r="L373" s="4" t="s">
+        <v>454</v>
+      </c>
+      <c r="M373" s="4"/>
+      <c r="N373" s="6">
+        <v>2</v>
+      </c>
+      <c r="O373" s="25"/>
+      <c r="P373" s="6"/>
+    </row>
+    <row r="374" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G374" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H374" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I374" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J374" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="K374" s="8">
+        <v>170</v>
+      </c>
+      <c r="L374" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="M374" s="4"/>
+      <c r="N374" s="6">
+        <v>3</v>
+      </c>
+      <c r="O374" s="25"/>
+      <c r="P374" s="6"/>
+    </row>
+    <row r="375" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G375" s="3">
+        <v>46092</v>
+      </c>
+      <c r="H375" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I375" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J375" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="K375" s="8">
+        <v>230</v>
+      </c>
+      <c r="L375" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M375" s="4"/>
+      <c r="N375" s="6">
+        <v>3</v>
+      </c>
+      <c r="O375" s="25"/>
+      <c r="P375" s="6"/>
+    </row>
+    <row r="376" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G376" s="30">
+        <v>46092</v>
+      </c>
+      <c r="H376" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="I376" s="50" t="s">
+        <v>599</v>
+      </c>
+      <c r="J376" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K376" s="10">
+        <v>240</v>
+      </c>
+      <c r="L376" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="M376" s="31"/>
+      <c r="N376" s="29">
+        <v>3</v>
+      </c>
+      <c r="O376" s="37"/>
+      <c r="P376" s="6"/>
+    </row>
+    <row r="377" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G377" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H377" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="I377" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="J377" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="K377" s="8">
+        <v>180</v>
+      </c>
+      <c r="L377" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="M377" s="4"/>
+      <c r="N377" s="6">
+        <v>2</v>
+      </c>
+      <c r="O377" s="25"/>
+      <c r="P377" s="6"/>
+    </row>
+    <row r="378" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G378" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H378" s="4" t="s">
+        <v>491</v>
+      </c>
+      <c r="I378" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="J378" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="K378" s="8">
+        <v>190</v>
+      </c>
+      <c r="L378" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="M378" s="4"/>
+      <c r="N378" s="6">
+        <v>2</v>
+      </c>
+      <c r="O378" s="25"/>
+      <c r="P378" s="6"/>
+    </row>
+    <row r="379" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G379" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H379" s="4" t="s">
+        <v>506</v>
+      </c>
+      <c r="I379" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="J379" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="K379" s="8">
+        <v>200</v>
+      </c>
+      <c r="L379" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="M379" s="4"/>
+      <c r="N379" s="6">
+        <v>2</v>
+      </c>
+      <c r="O379" s="25"/>
+      <c r="P379" s="6"/>
+    </row>
+    <row r="380" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G380" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H380" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I380" s="6" t="s">
+        <v>354</v>
+      </c>
+      <c r="J380" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="K380" s="8">
+        <v>240</v>
+      </c>
+      <c r="L380" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="M380" s="4"/>
+      <c r="N380" s="6">
+        <v>2</v>
+      </c>
+      <c r="O380" s="25"/>
+      <c r="P380" s="6"/>
+    </row>
+    <row r="381" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G381" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H381" s="4" t="s">
+        <v>498</v>
+      </c>
+      <c r="I381" s="6" t="s">
+        <v>586</v>
+      </c>
+      <c r="J381" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="K381" s="8">
+        <v>190</v>
+      </c>
+      <c r="L381" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="M381" s="4"/>
+      <c r="N381" s="6">
+        <v>2</v>
+      </c>
+      <c r="O381" s="25"/>
+      <c r="P381" s="6"/>
+    </row>
+    <row r="382" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G382" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H382" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="I382" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="J382" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="K382" s="8">
+        <v>240</v>
+      </c>
+      <c r="L382" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="M382" s="4"/>
+      <c r="N382" s="6">
+        <v>2</v>
+      </c>
+      <c r="O382" s="25"/>
+      <c r="P382" s="6"/>
+    </row>
+    <row r="383" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G383" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H383" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="I383" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="J383" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="K383" s="8">
+        <v>220</v>
+      </c>
+      <c r="L383" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="M383" s="4"/>
+      <c r="N383" s="6">
+        <v>2</v>
+      </c>
+      <c r="O383" s="25"/>
+      <c r="P383" s="6"/>
+    </row>
+    <row r="384" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G384" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H384" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="I384" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="J384" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="K384" s="8">
+        <v>190</v>
+      </c>
+      <c r="L384" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="M384" s="4"/>
+      <c r="N384" s="6">
+        <v>2</v>
+      </c>
+      <c r="O384" s="25"/>
+      <c r="P384" s="6"/>
+    </row>
+    <row r="385" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G385" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H385" s="4" t="s">
+        <v>527</v>
+      </c>
+      <c r="I385" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="J385" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="K385" s="8">
+        <v>220</v>
+      </c>
+      <c r="L385" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="M385" s="4"/>
+      <c r="N385" s="6">
+        <v>2</v>
+      </c>
+      <c r="O385" s="25"/>
+      <c r="P385" s="6"/>
+    </row>
+    <row r="386" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G386" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H386" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="I386" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="J386" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="K386" s="8">
+        <v>304</v>
+      </c>
+      <c r="L386" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="M386" s="4"/>
+      <c r="N386" s="6">
+        <v>2</v>
+      </c>
+      <c r="O386" s="25"/>
+      <c r="P386" s="6"/>
+    </row>
+    <row r="387" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O387" s="25"/>
+      <c r="P387" s="6"/>
+    </row>
+    <row r="388" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="O388" s="25"/>
+      <c r="P388" s="6"/>
+    </row>
+    <row r="389" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G389" s="3">
+        <v>46093</v>
+      </c>
+      <c r="H389" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="I389" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="J389" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K389" s="8">
+        <v>200</v>
+      </c>
+      <c r="L389" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M389" s="4"/>
+      <c r="N389" s="6"/>
+      <c r="O389" s="25"/>
+      <c r="P389" s="6"/>
+    </row>
+    <row r="390" spans="7:16" x14ac:dyDescent="0.25">
+      <c r="G390" s="3"/>
+      <c r="H390" s="4"/>
+      <c r="I390" s="6"/>
+      <c r="J390" s="4"/>
+      <c r="K390" s="8"/>
+      <c r="L390" s="4"/>
+      <c r="M390" s="4"/>
+      <c r="N390" s="6"/>
+      <c r="O390" s="25"/>
+      <c r="P390" s="6"/>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
@@ -30908,10 +31919,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O353" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O389" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="3" day="5" dateTimeGrouping="day"/>
+        <dateGroupItem year="2026" month="3" day="12" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-16 16:23
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="344" documentId="13_ncr:1_{CF87F821-98AE-4A1A-B4F9-A70BAAFD478B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B44A797-802B-4787-AB79-8446BE6FE8BC}"/>
+  <xr:revisionPtr revIDLastSave="351" documentId="13_ncr:1_{CF87F821-98AE-4A1A-B4F9-A70BAAFD478B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6178A346-399A-4396-9638-AC21282E8D2C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5603" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5607" uniqueCount="615">
   <si>
     <t>DATA</t>
   </si>
@@ -1883,9 +1883,6 @@
   </si>
   <si>
     <t>LUIS ED</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PIRAPORA </t>
   </si>
   <si>
     <t xml:space="preserve">BELLA POUSADA </t>
@@ -31890,9 +31887,15 @@
       <c r="I390" s="6" t="s">
         <v>611</v>
       </c>
-      <c r="J390" s="4"/>
-      <c r="K390" s="8"/>
-      <c r="L390" s="4"/>
+      <c r="J390" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="K390" s="8">
+        <v>240</v>
+      </c>
+      <c r="L390" s="4" t="s">
+        <v>598</v>
+      </c>
       <c r="M390" s="4"/>
       <c r="N390" s="6"/>
       <c r="O390" s="25"/>
@@ -31980,9 +31983,15 @@
       <c r="I394" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="J394" s="4"/>
-      <c r="K394" s="8"/>
-      <c r="L394" s="4"/>
+      <c r="J394" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="K394" s="8">
+        <v>170</v>
+      </c>
+      <c r="L394" s="4" t="s">
+        <v>363</v>
+      </c>
       <c r="M394" s="4"/>
       <c r="N394" s="6"/>
       <c r="O394" s="25"/>
@@ -31999,13 +32008,13 @@
         <v>135</v>
       </c>
       <c r="J395" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="K395" s="8">
+        <v>270</v>
+      </c>
+      <c r="L395" s="1" t="s">
         <v>614</v>
-      </c>
-      <c r="K395" s="8">
-        <v>170</v>
-      </c>
-      <c r="L395" s="4" t="s">
-        <v>229</v>
       </c>
       <c r="M395" s="4"/>
       <c r="N395" s="6">
@@ -32031,7 +32040,7 @@
         <v>270</v>
       </c>
       <c r="L396" s="1" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="M396" s="4"/>
       <c r="N396" s="6"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-04-02 12:07
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="572" documentId="13_ncr:1_{BFA144AC-8546-4E96-AEA1-F63AAF6602E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{288A5444-A530-4BAF-873F-619997D2E652}"/>
+  <xr:revisionPtr revIDLastSave="717" documentId="13_ncr:1_{BFA144AC-8546-4E96-AEA1-F63AAF6602E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{698A3BD4-68C6-4D21-BD60-234BAF10698E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
+    <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
   <sheets>
     <sheet name="HOTEIS2025" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$505</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NÚMERO DE HOTEIS'!$B$2:$D$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$506</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NÚMERO DE HOTEIS'!$B$2:$D$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6019" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6122" uniqueCount="681">
   <si>
     <t>DATA</t>
   </si>
@@ -1919,9 +1919,6 @@
     <t>VESPASIANO</t>
   </si>
   <si>
-    <t>PIUMI</t>
-  </si>
-  <si>
     <t>CORONEL FABRICIANO</t>
   </si>
   <si>
@@ -1994,9 +1991,6 @@
     <t>POUSADA CAETANO</t>
   </si>
   <si>
-    <t>PODE</t>
-  </si>
-  <si>
     <t>HOTEL CANIDEZ</t>
   </si>
   <si>
@@ -2004,6 +1998,93 @@
   </si>
   <si>
     <t>HOTEL FENIX</t>
+  </si>
+  <si>
+    <t>HOTEL POUSADA SOLAR</t>
+  </si>
+  <si>
+    <t>37 8827-0895</t>
+  </si>
+  <si>
+    <t>31 8325-0210</t>
+  </si>
+  <si>
+    <t>31 9573-2072</t>
+  </si>
+  <si>
+    <t>35 9930-1770</t>
+  </si>
+  <si>
+    <t>31 7100-8438</t>
+  </si>
+  <si>
+    <t> (31) 3532-1319</t>
+  </si>
+  <si>
+    <t>31 8246-4071</t>
+  </si>
+  <si>
+    <t>32 9165-7875</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 31 3184-1256</t>
+  </si>
+  <si>
+    <t>31 7144-8527</t>
+  </si>
+  <si>
+    <t> (35) 3235-3600</t>
+  </si>
+  <si>
+    <t> (35) 2146-5700</t>
+  </si>
+  <si>
+    <t>31 3841-9250</t>
+  </si>
+  <si>
+    <t>31 8201-6949</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 37 3524-1423</t>
+  </si>
+  <si>
+    <t>31 7212-7985</t>
+  </si>
+  <si>
+    <t>38 8807-5974</t>
+  </si>
+  <si>
+    <t>31 9254-3335</t>
+  </si>
+  <si>
+    <t>37 9992-9937</t>
+  </si>
+  <si>
+    <t>31 9832-2198</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 33 3416-2531</t>
+  </si>
+  <si>
+    <t>35 9935-1835</t>
+  </si>
+  <si>
+    <t>31 9940-9119</t>
+  </si>
+  <si>
+    <t>33 3421-7055</t>
+  </si>
+  <si>
+    <t>37 9870-4008</t>
+  </si>
+  <si>
+    <t>37 3551-1466</t>
+  </si>
+  <si>
+    <t>31 9238-1171</t>
+  </si>
+  <si>
+    <t>34 3851-2133</t>
   </si>
 </sst>
 </file>
@@ -2150,7 +2231,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2230,9 +2311,6 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2294,7 +2372,13 @@
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
@@ -2677,7 +2761,7 @@
       <c r="O5" s="24" t="s">
         <v>247</v>
       </c>
-      <c r="P5" s="40" t="s">
+      <c r="P5" s="39" t="s">
         <v>351</v>
       </c>
     </row>
@@ -4446,7 +4530,7 @@
       <c r="N64" s="19">
         <v>2</v>
       </c>
-      <c r="O64" s="38">
+      <c r="O64" s="37">
         <v>1</v>
       </c>
       <c r="P64" t="s">
@@ -5594,7 +5678,7 @@
       <c r="N102" s="19">
         <v>1</v>
       </c>
-      <c r="O102" s="38">
+      <c r="O102" s="37">
         <v>1</v>
       </c>
       <c r="P102" t="s">
@@ -7267,7 +7351,7 @@
       <c r="K158" s="20">
         <v>220</v>
       </c>
-      <c r="L158" s="35" t="s">
+      <c r="L158" s="34" t="s">
         <v>228</v>
       </c>
       <c r="M158" s="18" t="s">
@@ -12694,13 +12778,13 @@
       <c r="I339" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="J339" s="35" t="s">
+      <c r="J339" s="34" t="s">
         <v>245</v>
       </c>
-      <c r="K339" s="36">
+      <c r="K339" s="35">
         <v>150</v>
       </c>
-      <c r="L339" s="35" t="s">
+      <c r="L339" s="34" t="s">
         <v>246</v>
       </c>
       <c r="M339" s="18" t="s">
@@ -14371,7 +14455,7 @@
       <c r="N395" s="29">
         <v>2</v>
       </c>
-      <c r="O395" s="37"/>
+      <c r="O395" s="36"/>
       <c r="P395" t="s">
         <v>352</v>
       </c>
@@ -15215,10 +15299,10 @@
         <v>8</v>
       </c>
       <c r="N424" s="19"/>
-      <c r="O424" s="41" t="s">
+      <c r="O424" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P424" s="38" t="s">
+      <c r="P424" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -15455,10 +15539,10 @@
       <c r="N432" s="19">
         <v>2</v>
       </c>
-      <c r="O432" s="41" t="s">
+      <c r="O432" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P432" s="38" t="s">
+      <c r="P432" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -15491,7 +15575,7 @@
       </c>
     </row>
     <row r="434" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G434" s="51">
+      <c r="G434" s="50">
         <v>45966</v>
       </c>
       <c r="H434" s="18" t="s">
@@ -15513,15 +15597,15 @@
       <c r="N434" s="19">
         <v>2</v>
       </c>
-      <c r="O434" s="41" t="s">
+      <c r="O434" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P434" s="38" t="s">
+      <c r="P434" s="37" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="435" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G435" s="39">
+      <c r="G435" s="38">
         <v>45966</v>
       </c>
       <c r="H435" s="4" t="s">
@@ -15549,7 +15633,7 @@
       </c>
     </row>
     <row r="436" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G436" s="39">
+      <c r="G436" s="38">
         <v>45966</v>
       </c>
       <c r="H436" s="4" t="s">
@@ -15577,7 +15661,7 @@
       </c>
     </row>
     <row r="437" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G437" s="39">
+      <c r="G437" s="38">
         <v>45966</v>
       </c>
       <c r="H437" s="4" t="s">
@@ -15711,10 +15795,10 @@
       <c r="N441" s="19">
         <v>1</v>
       </c>
-      <c r="O441" s="41" t="s">
+      <c r="O441" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P441" s="38" t="s">
+      <c r="P441" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -15927,10 +16011,10 @@
       </c>
       <c r="M449" s="18"/>
       <c r="N449" s="19"/>
-      <c r="O449" s="41" t="s">
+      <c r="O449" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P449" s="38" t="s">
+      <c r="P449" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -15955,7 +16039,7 @@
       </c>
       <c r="M450" s="31"/>
       <c r="N450" s="29"/>
-      <c r="O450" s="37"/>
+      <c r="O450" s="36"/>
       <c r="P450" t="s">
         <v>352</v>
       </c>
@@ -15985,10 +16069,10 @@
       <c r="N451" s="19">
         <v>3</v>
       </c>
-      <c r="O451" s="41" t="s">
+      <c r="O451" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P451" s="38" t="s">
+      <c r="P451" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16225,38 +16309,38 @@
       <c r="N459" s="29">
         <v>3</v>
       </c>
-      <c r="O459" s="37"/>
+      <c r="O459" s="36"/>
       <c r="P459" t="s">
         <v>352</v>
       </c>
     </row>
     <row r="460" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G460" s="45">
+      <c r="G460" s="44">
         <v>45973</v>
       </c>
-      <c r="H460" s="46" t="s">
+      <c r="H460" s="45" t="s">
         <v>355</v>
       </c>
-      <c r="I460" s="47"/>
-      <c r="J460" s="46" t="s">
+      <c r="I460" s="46"/>
+      <c r="J460" s="45" t="s">
         <v>65</v>
       </c>
-      <c r="K460" s="48">
+      <c r="K460" s="47">
         <v>100</v>
       </c>
-      <c r="L460" s="46" t="s">
+      <c r="L460" s="45" t="s">
         <v>249</v>
       </c>
-      <c r="M460" s="46" t="s">
-        <v>8</v>
-      </c>
-      <c r="N460" s="47">
+      <c r="M460" s="45" t="s">
+        <v>8</v>
+      </c>
+      <c r="N460" s="46">
         <v>1</v>
       </c>
-      <c r="O460" s="49" t="s">
+      <c r="O460" s="48" t="s">
         <v>248</v>
       </c>
-      <c r="P460" s="38" t="s">
+      <c r="P460" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16372,10 +16456,10 @@
         <v>8</v>
       </c>
       <c r="N469" s="19"/>
-      <c r="O469" s="41" t="s">
+      <c r="O469" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P469" s="38" t="s">
+      <c r="P469" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16484,10 +16568,10 @@
         <v>7</v>
       </c>
       <c r="N473" s="19"/>
-      <c r="O473" s="41" t="s">
+      <c r="O473" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P473" s="38" t="s">
+      <c r="P473" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16514,10 +16598,10 @@
         <v>8</v>
       </c>
       <c r="N474" s="19"/>
-      <c r="O474" s="41" t="s">
+      <c r="O474" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P474" s="38" t="s">
+      <c r="P474" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16630,10 +16714,10 @@
         <v>8</v>
       </c>
       <c r="N478" s="19"/>
-      <c r="O478" s="41" t="s">
+      <c r="O478" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="P478" s="38" t="s">
+      <c r="P478" s="37" t="s">
         <v>352</v>
       </c>
     </row>
@@ -16723,7 +16807,7 @@
     </row>
     <row r="482" spans="7:16" hidden="1" x14ac:dyDescent="0.25"/>
     <row r="483" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G483" s="45">
+      <c r="G483" s="44">
         <v>45974</v>
       </c>
       <c r="H483" s="18" t="s">
@@ -16745,7 +16829,7 @@
       <c r="N483" s="19">
         <v>2</v>
       </c>
-      <c r="O483" s="41" t="s">
+      <c r="O483" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P483" s="19" t="s">
@@ -16792,20 +16876,20 @@
       <c r="I485" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="J485" s="42" t="s">
+      <c r="J485" s="41" t="s">
         <v>46</v>
       </c>
-      <c r="K485" s="43">
+      <c r="K485" s="42">
         <v>170</v>
       </c>
-      <c r="L485" s="42" t="s">
+      <c r="L485" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="M485" s="42"/>
+      <c r="M485" s="41"/>
       <c r="N485" s="6">
         <v>2</v>
       </c>
-      <c r="O485" s="44"/>
+      <c r="O485" s="43"/>
       <c r="P485" s="6" t="s">
         <v>352</v>
       </c>
@@ -17035,7 +17119,7 @@
       </c>
     </row>
     <row r="494" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G494" s="45">
+      <c r="G494" s="44">
         <v>45974</v>
       </c>
       <c r="H494" s="18" t="s">
@@ -17057,7 +17141,7 @@
       <c r="N494" s="19">
         <v>2</v>
       </c>
-      <c r="O494" s="41" t="s">
+      <c r="O494" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P494" s="19" t="s">
@@ -17547,7 +17631,7 @@
       <c r="N511" s="19">
         <v>1</v>
       </c>
-      <c r="O511" s="41" t="s">
+      <c r="O511" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P511" s="19" t="s">
@@ -17631,7 +17715,7 @@
       </c>
       <c r="M514" s="18"/>
       <c r="N514" s="19"/>
-      <c r="O514" s="41" t="s">
+      <c r="O514" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P514" s="19" t="s">
@@ -17661,7 +17745,7 @@
       <c r="N515" s="19">
         <v>2</v>
       </c>
-      <c r="O515" s="41" t="s">
+      <c r="O515" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P515" s="19" t="s">
@@ -18078,7 +18162,7 @@
       <c r="N531" s="19">
         <v>2</v>
       </c>
-      <c r="O531" s="41" t="s">
+      <c r="O531" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P531" s="19" t="s">
@@ -18106,7 +18190,7 @@
       </c>
       <c r="M532" s="18"/>
       <c r="N532" s="19"/>
-      <c r="O532" s="41" t="s">
+      <c r="O532" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P532" s="19" t="s">
@@ -18186,7 +18270,7 @@
       </c>
       <c r="M535" s="18"/>
       <c r="N535" s="19"/>
-      <c r="O535" s="41" t="s">
+      <c r="O535" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P535" s="19" t="s">
@@ -18287,7 +18371,7 @@
       <c r="I539" s="19" t="s">
         <v>174</v>
       </c>
-      <c r="J539" s="35" t="s">
+      <c r="J539" s="34" t="s">
         <v>226</v>
       </c>
       <c r="K539" s="20">
@@ -18300,7 +18384,7 @@
       <c r="N539" s="19">
         <v>2</v>
       </c>
-      <c r="O539" s="41" t="s">
+      <c r="O539" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P539" s="19" t="s">
@@ -18345,20 +18429,20 @@
       <c r="I541" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="J541" s="35" t="s">
+      <c r="J541" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="K541" s="52">
+      <c r="K541" s="51">
         <v>180</v>
       </c>
-      <c r="L541" s="35" t="s">
+      <c r="L541" s="34" t="s">
         <v>100</v>
       </c>
       <c r="M541" s="18"/>
       <c r="N541" s="19">
         <v>2</v>
       </c>
-      <c r="O541" s="41" t="s">
+      <c r="O541" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P541" s="19" t="s">
@@ -18584,7 +18668,7 @@
       <c r="N549" s="19">
         <v>2</v>
       </c>
-      <c r="O549" s="41" t="s">
+      <c r="O549" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P549" s="19" t="s">
@@ -18650,7 +18734,7 @@
       <c r="N553" s="19">
         <v>1</v>
       </c>
-      <c r="O553" s="41" t="s">
+      <c r="O553" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P553" s="19" t="s">
@@ -18736,7 +18820,7 @@
       <c r="N556" s="19">
         <v>2</v>
       </c>
-      <c r="O556" s="41" t="s">
+      <c r="O556" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P556" s="19" t="s">
@@ -18878,7 +18962,7 @@
       <c r="N561" s="19">
         <v>2</v>
       </c>
-      <c r="O561" s="41" t="s">
+      <c r="O561" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P561" s="19" t="s">
@@ -18908,7 +18992,7 @@
       <c r="N562" s="19">
         <v>1</v>
       </c>
-      <c r="O562" s="41" t="s">
+      <c r="O562" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P562" s="19" t="s">
@@ -19050,7 +19134,7 @@
       <c r="N567" s="19">
         <v>1</v>
       </c>
-      <c r="O567" s="41" t="s">
+      <c r="O567" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P567" s="19" t="s">
@@ -19274,7 +19358,7 @@
       <c r="N575" s="19">
         <v>1</v>
       </c>
-      <c r="O575" s="41" t="s">
+      <c r="O575" s="40" t="s">
         <v>248</v>
       </c>
       <c r="P575" s="19" t="s">
@@ -19738,7 +19822,7 @@
       <c r="H596" s="1" t="s">
         <v>377</v>
       </c>
-      <c r="I596" s="50" t="s">
+      <c r="I596" s="49" t="s">
         <v>129</v>
       </c>
       <c r="J596" s="1" t="s">
@@ -22529,7 +22613,7 @@
       <c r="L700" s="31"/>
       <c r="M700" s="31"/>
       <c r="N700" s="29"/>
-      <c r="O700" s="37"/>
+      <c r="O700" s="36"/>
       <c r="P700" s="29" t="s">
         <v>352</v>
       </c>
@@ -22986,34 +23070,34 @@
   </cols>
   <sheetData>
     <row r="5" spans="7:16" x14ac:dyDescent="0.25">
-      <c r="G5" s="53" t="s">
+      <c r="G5" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="H5" s="53" t="s">
+      <c r="H5" s="52" t="s">
         <v>138</v>
       </c>
-      <c r="I5" s="54" t="s">
+      <c r="I5" s="53" t="s">
         <v>118</v>
       </c>
-      <c r="J5" s="53" t="s">
+      <c r="J5" s="52" t="s">
         <v>1</v>
       </c>
-      <c r="K5" s="55" t="s">
-        <v>2</v>
-      </c>
-      <c r="L5" s="53" t="s">
+      <c r="K5" s="54" t="s">
+        <v>2</v>
+      </c>
+      <c r="L5" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="53" t="s">
+      <c r="M5" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="N5" s="53" t="s">
+      <c r="N5" s="52" t="s">
         <v>20</v>
       </c>
-      <c r="O5" s="56" t="s">
+      <c r="O5" s="55" t="s">
         <v>247</v>
       </c>
-      <c r="P5" s="40" t="s">
+      <c r="P5" s="39" t="s">
         <v>351</v>
       </c>
     </row>
@@ -23938,27 +24022,27 @@
       </c>
     </row>
     <row r="40" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="G40" s="58">
+      <c r="G40" s="57">
         <v>46035</v>
       </c>
-      <c r="H40" s="42" t="s">
+      <c r="H40" s="41" t="s">
         <v>490</v>
       </c>
       <c r="I40" s="28" t="s">
         <v>127</v>
       </c>
-      <c r="J40" s="42" t="s">
+      <c r="J40" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="K40" s="43">
+      <c r="K40" s="42">
         <v>170</v>
       </c>
-      <c r="L40" s="42" t="s">
+      <c r="L40" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="M40" s="42"/>
+      <c r="M40" s="41"/>
       <c r="N40" s="28"/>
-      <c r="O40" s="44"/>
+      <c r="O40" s="43"/>
       <c r="P40" s="28" t="s">
         <v>352</v>
       </c>
@@ -24336,7 +24420,7 @@
       </c>
       <c r="M54" s="31"/>
       <c r="N54" s="29"/>
-      <c r="O54" s="37"/>
+      <c r="O54" s="36"/>
       <c r="P54" s="6" t="s">
         <v>352</v>
       </c>
@@ -24371,10 +24455,10 @@
       <c r="G56" s="3">
         <v>46037</v>
       </c>
-      <c r="H56" s="57" t="s">
+      <c r="H56" s="56" t="s">
         <v>145</v>
       </c>
-      <c r="I56" s="50" t="s">
+      <c r="I56" s="49" t="s">
         <v>133</v>
       </c>
       <c r="P56" s="6" t="s">
@@ -25263,7 +25347,7 @@
       </c>
       <c r="M90" s="31"/>
       <c r="N90" s="29"/>
-      <c r="O90" s="37"/>
+      <c r="O90" s="36"/>
       <c r="P90" s="29"/>
     </row>
     <row r="91" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
@@ -30117,7 +30201,7 @@
       <c r="O303" s="25"/>
       <c r="P303" s="6"/>
     </row>
-    <row r="304" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+    <row r="304" spans="7:16" x14ac:dyDescent="0.25">
       <c r="G304" s="3">
         <v>46080</v>
       </c>
@@ -30795,7 +30879,7 @@
       <c r="P339" s="6"/>
     </row>
     <row r="340" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="O340" s="37"/>
+      <c r="O340" s="36"/>
       <c r="P340" s="29"/>
     </row>
     <row r="341" spans="6:16" hidden="1" x14ac:dyDescent="0.25">
@@ -31110,7 +31194,7 @@
       </c>
       <c r="M353" s="4"/>
       <c r="N353" s="6"/>
-      <c r="O353" s="59" t="s">
+      <c r="O353" s="58" t="s">
         <v>594</v>
       </c>
       <c r="P353" s="6"/>
@@ -31686,7 +31770,7 @@
       <c r="H376" s="1" t="s">
         <v>494</v>
       </c>
-      <c r="I376" s="50" t="s">
+      <c r="I376" s="49" t="s">
         <v>596</v>
       </c>
       <c r="J376" s="1" t="s">
@@ -31702,7 +31786,7 @@
       <c r="N376" s="29">
         <v>3</v>
       </c>
-      <c r="O376" s="37"/>
+      <c r="O376" s="36"/>
       <c r="P376" s="6"/>
     </row>
     <row r="377" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
@@ -32612,7 +32696,7 @@
       <c r="N414" s="29">
         <v>2</v>
       </c>
-      <c r="O414" s="37"/>
+      <c r="O414" s="36"/>
       <c r="P414" s="29"/>
     </row>
     <row r="415" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
@@ -33240,7 +33324,7 @@
         <v>131</v>
       </c>
       <c r="J440" s="4" t="s">
-        <v>625</v>
+        <v>486</v>
       </c>
       <c r="K440" s="8">
         <v>220</v>
@@ -33362,13 +33446,13 @@
         <v>501</v>
       </c>
       <c r="J445" s="4" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="K445" s="8">
         <v>159</v>
       </c>
       <c r="L445" s="4" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="M445" s="4"/>
       <c r="N445" s="6"/>
@@ -33556,16 +33640,16 @@
       <c r="P452" s="6"/>
     </row>
     <row r="453" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="K453" s="60"/>
+      <c r="K453" s="59"/>
     </row>
     <row r="454" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="K454" s="60"/>
+      <c r="K454" s="59"/>
     </row>
     <row r="455" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="K455" s="60"/>
+      <c r="K455" s="59"/>
     </row>
     <row r="456" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
-      <c r="K456" s="60"/>
+      <c r="K456" s="59"/>
     </row>
     <row r="457" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G457" s="3">
@@ -33695,7 +33779,7 @@
         <v>497</v>
       </c>
       <c r="I462" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="J462" s="4" t="s">
         <v>402</v>
@@ -33794,7 +33878,7 @@
         <v>144</v>
       </c>
       <c r="I466" s="6" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="J466" s="4" t="s">
         <v>95</v>
@@ -33818,7 +33902,7 @@
         <v>130</v>
       </c>
       <c r="I467" s="6" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J467" s="4" t="s">
         <v>515</v>
@@ -33827,7 +33911,7 @@
         <v>300</v>
       </c>
       <c r="L467" s="4" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="P467" s="6"/>
     </row>
@@ -33869,13 +33953,13 @@
         <v>131</v>
       </c>
       <c r="J470" s="4" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="K470" s="8">
         <v>315</v>
       </c>
       <c r="L470" s="4" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="M470" s="4"/>
       <c r="N470" s="6"/>
@@ -33901,7 +33985,7 @@
         <v>270</v>
       </c>
       <c r="L471" s="4" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="M471" s="4"/>
       <c r="N471" s="6"/>
@@ -33916,10 +34000,10 @@
         <v>497</v>
       </c>
       <c r="I472" s="6" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="J472" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="K472" s="8">
         <v>158</v>
@@ -34107,19 +34191,19 @@
         <v>46107</v>
       </c>
       <c r="H480" s="4" t="s">
+        <v>634</v>
+      </c>
+      <c r="I480" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="I480" s="6" t="s">
-        <v>636</v>
-      </c>
       <c r="J480" s="4" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="K480" s="8">
         <v>200</v>
       </c>
       <c r="L480" s="4" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="M480" s="4"/>
       <c r="N480" s="6"/>
@@ -34167,7 +34251,7 @@
         <v>220</v>
       </c>
       <c r="L482" s="4" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="M482" s="4"/>
       <c r="N482" s="6">
@@ -34239,13 +34323,13 @@
         <v>133</v>
       </c>
       <c r="J485" s="4" t="s">
-        <v>648</v>
+        <v>647</v>
       </c>
       <c r="K485" s="8">
         <v>160</v>
       </c>
       <c r="L485" s="4" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="M485" s="4"/>
       <c r="N485" s="6">
@@ -34259,10 +34343,10 @@
         <v>46112</v>
       </c>
       <c r="H486" s="4" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I486" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J486" s="4" t="s">
         <v>414</v>
@@ -34271,7 +34355,7 @@
         <v>190</v>
       </c>
       <c r="L486" s="4" t="s">
-        <v>650</v>
+        <v>464</v>
       </c>
       <c r="M486" s="4"/>
       <c r="N486" s="6">
@@ -34340,7 +34424,7 @@
         <v>382</v>
       </c>
       <c r="I489" s="6" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="J489" s="4" t="s">
         <v>262</v>
@@ -34369,7 +34453,7 @@
         <v>584</v>
       </c>
       <c r="J490" s="4" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
       <c r="K490" s="8">
         <v>259</v>
@@ -34382,7 +34466,7 @@
       <c r="O490" s="25"/>
       <c r="P490" s="6"/>
     </row>
-    <row r="491" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="491" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G491" s="3">
         <v>46113</v>
       </c>
@@ -34406,7 +34490,7 @@
       <c r="O491" s="25"/>
       <c r="P491" s="6"/>
     </row>
-    <row r="492" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="492" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G492" s="3">
         <v>46113</v>
       </c>
@@ -34430,31 +34514,31 @@
       <c r="O492" s="25"/>
       <c r="P492" s="6"/>
     </row>
-    <row r="493" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="493" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G493" s="3">
         <v>46113</v>
       </c>
       <c r="H493" s="4" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="I493" s="6" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J493" s="4" t="s">
-        <v>337</v>
+        <v>450</v>
       </c>
       <c r="K493" s="8">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="L493" s="4" t="s">
-        <v>256</v>
+        <v>652</v>
       </c>
       <c r="M493" s="4"/>
       <c r="N493" s="6"/>
       <c r="O493" s="25"/>
       <c r="P493" s="6"/>
     </row>
-    <row r="494" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="494" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G494" s="3">
         <v>46113</v>
       </c>
@@ -34478,7 +34562,7 @@
       <c r="O494" s="25"/>
       <c r="P494" s="6"/>
     </row>
-    <row r="495" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="495" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G495" s="3">
         <v>46113</v>
       </c>
@@ -34502,7 +34586,7 @@
       <c r="O495" s="25"/>
       <c r="P495" s="6"/>
     </row>
-    <row r="496" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="496" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G496" s="3">
         <v>46113</v>
       </c>
@@ -34528,7 +34612,7 @@
       <c r="O496" s="25"/>
       <c r="P496" s="6"/>
     </row>
-    <row r="497" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="497" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G497" s="3">
         <v>46113</v>
       </c>
@@ -34554,7 +34638,7 @@
       <c r="O497" s="25"/>
       <c r="P497" s="6"/>
     </row>
-    <row r="498" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="498" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G498" s="3">
         <v>46113</v>
       </c>
@@ -34571,7 +34655,7 @@
         <v>237</v>
       </c>
       <c r="L498" s="4" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="M498" s="4"/>
       <c r="N498" s="6">
@@ -34580,18 +34664,18 @@
       <c r="O498" s="25"/>
       <c r="P498" s="6"/>
     </row>
-    <row r="499" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="499" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G499" s="3">
         <v>46113</v>
       </c>
       <c r="H499" s="1" t="s">
         <v>491</v>
       </c>
-      <c r="I499" s="61" t="s">
+      <c r="I499" s="49" t="s">
         <v>547</v>
       </c>
       <c r="J499" s="1" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="K499" s="10">
         <v>190</v>
@@ -34602,14 +34686,14 @@
       <c r="O499" s="25"/>
       <c r="P499" s="6"/>
     </row>
-    <row r="500" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="500" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G500" s="3">
         <v>46113</v>
       </c>
       <c r="H500" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="I500" s="61" t="s">
+      <c r="I500" s="49" t="s">
         <v>135</v>
       </c>
       <c r="J500" s="1" t="s">
@@ -34668,6 +34752,26 @@
       <c r="O505" s="25"/>
       <c r="P505" s="6"/>
     </row>
+    <row r="506" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
+      <c r="G506" s="3">
+        <v>46113</v>
+      </c>
+      <c r="H506" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I506" s="49" t="s">
+        <v>631</v>
+      </c>
+      <c r="J506" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="K506" s="10">
+        <v>230</v>
+      </c>
+      <c r="L506" s="1" t="s">
+        <v>521</v>
+      </c>
+    </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
       <c r="F639">
         <v>1</v>
@@ -34699,10 +34803,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O505" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O506" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="4" dateTimeGrouping="month"/>
+        <dateGroupItem year="2026" month="2" day="27" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -34713,27 +34817,26 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FE6273D-5F38-4F53-8D59-CFF970DDA070}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="B2:E53"/>
+  <dimension ref="B2:E88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="27.5703125" style="34" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="29.5703125" style="34" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" style="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.5703125" style="33" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.5703125" style="33" customWidth="1"/>
+    <col min="4" max="4" width="13.7109375" style="33" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="7" t="s">
+        <v>638</v>
+      </c>
+      <c r="C2" s="7" t="s">
         <v>639</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="D2" s="7" t="s">
         <v>640</v>
       </c>
-      <c r="D2" s="7" t="s">
-        <v>641</v>
-      </c>
-    </row>
-    <row r="3" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="7" t="s">
         <v>107</v>
       </c>
@@ -34744,7 +34847,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="4" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="7" t="s">
         <v>25</v>
       </c>
@@ -34755,7 +34858,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="5" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="7" t="s">
         <v>31</v>
       </c>
@@ -34766,7 +34869,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="6" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="7" t="s">
         <v>243</v>
       </c>
@@ -34777,7 +34880,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="7" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="7" t="s">
         <v>60</v>
       </c>
@@ -34788,18 +34891,18 @@
         <v>279</v>
       </c>
     </row>
-    <row r="8" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>515</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>632</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="7" t="s">
         <v>46</v>
       </c>
@@ -34810,7 +34913,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="10" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="7" t="s">
         <v>93</v>
       </c>
@@ -34821,7 +34924,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="7" t="s">
         <v>227</v>
       </c>
@@ -34832,7 +34935,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="12" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="7" t="s">
         <v>252</v>
       </c>
@@ -34843,7 +34946,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="13" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="7" t="s">
         <v>10</v>
       </c>
@@ -34854,7 +34957,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="14" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B14" s="7" t="s">
         <v>237</v>
       </c>
@@ -34865,7 +34968,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="15" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="7" t="s">
         <v>83</v>
       </c>
@@ -34876,7 +34979,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="16" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="7" t="s">
         <v>41</v>
       </c>
@@ -34887,7 +34990,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="17" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="7" t="s">
         <v>85</v>
       </c>
@@ -34898,7 +35001,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="18" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="7" t="s">
         <v>107</v>
       </c>
@@ -34909,7 +35012,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="19" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="7" t="s">
         <v>13</v>
       </c>
@@ -34920,7 +35023,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="20" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="7" t="s">
         <v>75</v>
       </c>
@@ -34931,7 +35034,7 @@
         <v>293</v>
       </c>
     </row>
-    <row r="21" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="7" t="s">
         <v>101</v>
       </c>
@@ -34942,7 +35045,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="22" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="7" t="s">
         <v>190</v>
       </c>
@@ -34953,7 +35056,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="23" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="7" t="s">
         <v>262</v>
       </c>
@@ -34964,7 +35067,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="24" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="7" t="s">
         <v>181</v>
       </c>
@@ -34975,15 +35078,15 @@
         <v>297</v>
       </c>
     </row>
-    <row r="25" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="7" t="s">
-        <v>245</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>246</v>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>87</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>298</v>
+        <v>661</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
@@ -34997,7 +35100,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="27" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="7" t="s">
         <v>106</v>
       </c>
@@ -35008,7 +35111,7 @@
         <v>3532353600</v>
       </c>
     </row>
-    <row r="28" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="7" t="s">
         <v>106</v>
       </c>
@@ -35019,7 +35122,7 @@
         <v>3521465700</v>
       </c>
     </row>
-    <row r="29" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="7" t="s">
         <v>21</v>
       </c>
@@ -35030,7 +35133,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="30" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="7" t="s">
         <v>11</v>
       </c>
@@ -35041,7 +35144,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="31" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="7" t="s">
         <v>27</v>
       </c>
@@ -35052,7 +35155,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="32" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="7" t="s">
         <v>64</v>
       </c>
@@ -35063,7 +35166,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="33" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="7" t="s">
         <v>65</v>
       </c>
@@ -35074,7 +35177,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="34" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="7" t="s">
         <v>38</v>
       </c>
@@ -35085,7 +35188,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="35" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="7" t="s">
         <v>201</v>
       </c>
@@ -35096,7 +35199,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="36" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="7" t="s">
         <v>82</v>
       </c>
@@ -35107,7 +35210,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="37" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="7" t="s">
         <v>179</v>
       </c>
@@ -35118,7 +35221,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="38" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="7" t="s">
         <v>273</v>
       </c>
@@ -35129,7 +35232,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="39" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="7" t="s">
         <v>11</v>
       </c>
@@ -35140,7 +35243,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="40" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="7" t="s">
         <v>13</v>
       </c>
@@ -35151,7 +35254,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="41" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="21" t="s">
         <v>65</v>
       </c>
@@ -35162,7 +35265,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="42" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="7" t="s">
         <v>116</v>
       </c>
@@ -35173,7 +35276,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="43" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="7" t="s">
         <v>194</v>
       </c>
@@ -35184,7 +35287,7 @@
         <v>314</v>
       </c>
     </row>
-    <row r="44" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="7" t="s">
         <v>42</v>
       </c>
@@ -35195,7 +35298,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="45" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="7" t="s">
         <v>95</v>
       </c>
@@ -35206,7 +35309,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="46" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="7" t="s">
         <v>23</v>
       </c>
@@ -35217,7 +35320,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="47" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" s="7" t="s">
         <v>24</v>
       </c>
@@ -35228,7 +35331,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="48" spans="2:4" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B48" s="7" t="s">
         <v>103</v>
       </c>
@@ -35239,7 +35342,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="49" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B49" s="7" t="s">
         <v>34</v>
       </c>
@@ -35250,8 +35353,8 @@
         <v>320</v>
       </c>
     </row>
-    <row r="50" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B50" s="34" t="s">
+    <row r="50" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B50" s="33" t="s">
         <v>70</v>
       </c>
       <c r="C50" s="7" t="s">
@@ -35261,8 +35364,8 @@
         <v>318</v>
       </c>
     </row>
-    <row r="51" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="34" t="s">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B51" s="33" t="s">
         <v>364</v>
       </c>
       <c r="C51" s="7" t="s">
@@ -35272,41 +35375,413 @@
         <v>290</v>
       </c>
     </row>
-    <row r="52" spans="2:5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B52" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C52" s="34" t="s">
+      <c r="C52" s="33" t="s">
         <v>220</v>
       </c>
-      <c r="D52" s="34" t="s">
-        <v>642</v>
+      <c r="D52" s="33" t="s">
+        <v>641</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B53" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="C53" s="34" t="s">
+      <c r="C53" s="33" t="s">
         <v>341</v>
       </c>
-      <c r="D53" s="34" t="s">
+      <c r="D53" s="33" t="s">
+        <v>642</v>
+      </c>
+      <c r="E53" t="s">
         <v>643</v>
       </c>
-      <c r="E53" t="s">
+    </row>
+    <row r="54" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B54" s="4" t="s">
+        <v>486</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="D54" s="33" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="55" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B55" s="4" t="s">
+        <v>432</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>433</v>
+      </c>
+      <c r="D55" s="33" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="56" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B56" s="4" t="s">
+        <v>450</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="D56" s="33" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="57" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B57" s="33" t="s">
+        <v>5</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D57" s="7" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="58" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B58" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>651</v>
+      </c>
+      <c r="D58" s="33" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="59" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B59" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="D59" s="33" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="60" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B60" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>521</v>
+      </c>
+      <c r="D60" s="60" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="61" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B61" s="4" t="s">
+        <v>400</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D61" s="33" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="62" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B62" s="4" t="s">
+        <v>647</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>648</v>
+      </c>
+      <c r="D62" s="33" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="63" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B63" s="4" t="s">
         <v>644</v>
       </c>
+      <c r="C63" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D63" s="33" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="64" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B64" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="D64" s="62" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="65" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B65" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="D65" s="33" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="66" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B66" s="7" t="s">
+        <v>245</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="D66" s="61" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="67" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B67" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="D67" s="60" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="68" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B68" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D68" s="60" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="69" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B69" s="4" t="s">
+        <v>625</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>626</v>
+      </c>
+      <c r="D69" s="33" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="70" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B70" s="4"/>
+      <c r="C70" s="4"/>
+    </row>
+    <row r="71" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B71" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="D71" s="33" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="72" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B72" s="4" t="s">
+        <v>621</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="D72" s="33" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="73" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B73" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>623</v>
+      </c>
+      <c r="D73" s="33" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="74" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B74" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="D74" s="33" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="75" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B75" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="D75" s="33" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="76" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B76" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="D76" s="33" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="77" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B77" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D77" s="33" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="78" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B78" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="D78" s="33" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="79" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B79" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="D79" s="33" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="80" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B80" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="D80" s="33" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="81" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B81" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="D81" s="33" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="82" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B82" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D82" s="33" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="83" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B83" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D83" s="33" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="84" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B84" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="D84" s="33" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="85" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B85" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="C85" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D85" s="33" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="86" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B86" s="4" t="s">
+        <v>509</v>
+      </c>
+      <c r="C86" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="D86" s="33" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="87" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B87" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="C87" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="D87" s="33" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="88" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B88" s="4"/>
+      <c r="C88" s="4"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:D52" xr:uid="{4FE6273D-5F38-4F53-8D59-CFF970DDA070}">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="ELOI MENDES"/>
-      </filters>
-    </filterColumn>
+  <autoFilter ref="B2:D87" xr:uid="{4FE6273D-5F38-4F53-8D59-CFF970DDA070}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B8:D66">
+      <sortCondition ref="B2:B63"/>
+    </sortState>
   </autoFilter>
   <hyperlinks>
-    <hyperlink ref="D8" r:id="rId1" display="https://www.google.com/search?q=aguas+claras+hotelMARIANA&amp;sca_esv=2369d6cd51414d5b&amp;sxsrf=AE3TifN90vqarBjXmJsGMNTX1Qk1VEbDnQ%3A1761930672555&amp;ei=sO0EadLUIfi_5OUPpZjsmAI&amp;ved=0ahUKEwjS7Oye986QAxX4H7kGHSUMGyMQ4dUDCBQ&amp;uact=5&amp;oq=aguas+claras+hotelMARIANA&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiGWFndWFzIGNsYXJhcyBob3RlbE1BUklBTkEyBhAAGBYYHjIIEAAYCBgNGB4yCBAAGAgYDRgeMggQABiABBiiBDIIEAAYogQYiQUyCBAAGIAEGKIESJYWUPYNWLQUcAF4AZABAJgBpgGgAdsHqgEDMC43uAEDyAEA-AEBmAIIoAKFCMICChAAGLADGNYEGEfCAg0QABiABBiwAxhDGIoFwgIHECMYsAIYJ8ICBxAAGIAEGA3CAhMQLhiABBjHARiYBRiZBRgNGK8BwgIGEAAYDRgemAMAiAYBkAYKkgcDMS43oAfiP7IHAzAuN7gH-wfCBwcwLjQuMy4xyAch&amp;sclient=gws-wiz-serp" xr:uid="{87444837-14E2-4EF1-BE11-4D2D7B64B6B1}"/>
+    <hyperlink ref="D64" r:id="rId1" display="https://www.google.com/search?q=aguas+claras+hotelMARIANA&amp;sca_esv=2369d6cd51414d5b&amp;sxsrf=AE3TifN90vqarBjXmJsGMNTX1Qk1VEbDnQ%3A1761930672555&amp;ei=sO0EadLUIfi_5OUPpZjsmAI&amp;ved=0ahUKEwjS7Oye986QAxX4H7kGHSUMGyMQ4dUDCBQ&amp;uact=5&amp;oq=aguas+claras+hotelMARIANA&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiGWFndWFzIGNsYXJhcyBob3RlbE1BUklBTkEyBhAAGBYYHjIIEAAYCBgNGB4yCBAAGAgYDRgeMggQABiABBiiBDIIEAAYogQYiQUyCBAAGIAEGKIESJYWUPYNWLQUcAF4AZABAJgBpgGgAdsHqgEDMC43uAEDyAEA-AEBmAIIoAKFCMICChAAGLADGNYEGEfCAg0QABiABBiwAxhDGIoFwgIHECMYsAIYJ8ICBxAAGIAEGA3CAhMQLhiABBjHARiYBRiZBRgNGK8BwgIGEAAYDRgemAMAiAYBkAYKkgcDMS43oAfiP7IHAzAuN7gH-wfCBwcwLjQuMy4xyAch&amp;sclient=gws-wiz-serp" xr:uid="{87444837-14E2-4EF1-BE11-4D2D7B64B6B1}"/>
+    <hyperlink ref="D60" r:id="rId2" display="https://www.google.com/search?q=hotel+panoramic+betim+whatsapp&amp;oq=HOTEL+PANORAMIC&amp;gs_lcrp=EgZjaHJvbWUqBggBECMYJzIGCAAQRRg5MgYIARAjGCcyEwgCEC4YrwEYxwEYgAQYmAUYmQUyEwgDEC4YrwEYxwEYgAQYmAUYmQUyBwgEEAAYgAQyBwgFEAAYgAQyBwgGEAAYgAQyBwgHEAAYgAQyBwgIEAAYgAQyBwgJEAAYgATSAQk4NDI2ajBqMTWoAgiwAgHxBUkySMQuGzBx8QVJMkjELhswcQ&amp;sourceid=chrome&amp;ie=UTF-8" xr:uid="{A2188972-5010-4F50-9FF6-ACBA608EF578}"/>
+    <hyperlink ref="D67" r:id="rId3" display="https://www.google.com/search?q=hotel+medieval+1&amp;sca_esv=2d30375674e67280&amp;sxsrf=ANbL-n5zOvkJ73_nVtj6E1viK7q-0CzatA%3A1775138630262&amp;ei=RnfOabfaD9Ld5OUP5IWxmQE&amp;biw=1067&amp;bih=910&amp;oq=HOTEL+MEDI&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAaAhgCIgpIT1RFTCBNRURJKgIIAzIEECMYJzIKECMYgAQYJxiKBTIFEAAYgAQyBRAAGIAEMgUQABiABDIFEAAYgAQyBRAAGIAEMgUQABiABDIFEAAYgAQyBRAAGIAESJUnUMUJWJQYcAF4AJABAJgB_gGgAeILqgEFMC45LjG4AQPIAQD4AQGYAgugAugMqAIKwgIHECMYJxjqAsICDRAjGPAFGCcYyQIY6gLCAgoQIxgnGOoCGIsDwgIWEC4YgAQYQxjHARiYBRiZBRiKBRivAcICChAAGIAEGEMYigXCAgsQABiABBixAxiDAcICEBAuGIAEGMcBGCcYigUYrwHCAhAQLhiABBhDGMcBGIoFGK8BwgILEAAYgAQYkgMYigXCAhQQLhiABBjHARiYBRiZBRieBRivAcICCBAAGIAEGLEDwgIKEAAYgAQYFBiHApgDGvEFLJloD39LYEaSBwUxLjguMqAH9KMBsgcFMC44LjK4B80MwgcJMi05LjAuMS4xyAd1gAgA&amp;sclient=gws-wiz-serp" xr:uid="{E1FF049D-9A6E-4A15-979A-40CE6DF966F6}"/>
+    <hyperlink ref="D68" r:id="rId4" display="https://www.google.com/search?q=hotel+medieval+2&amp;sca_esv=2d30375674e67280&amp;biw=1067&amp;bih=910&amp;sxsrf=ANbL-n4eBzyt9PVcWHuJyNwzuoAl2A0Plg%3A1775139224874&amp;ei=mHnOaYCHNaz35OUPyv7ssAk&amp;ved=0ahUKEwiAs7P3rM-TAxWsO7kGHUo_G5YQ4dUDCBE&amp;uact=5&amp;oq=hotel+medieval+2&amp;gs_lp=Egxnd3Mtd2l6LXNlcnAiEGhvdGVsIG1lZGlldmFsIDIyBBAjGCcyChAjGIAEGCcYigUyBRAAGIAEMgUQABiABDIFEAAYgAQyBhAAGBYYHjIIEAAYgAQYogRI-wVQrQRY_ARwAXgBkAEAmAGFAaAB9AGqAQMwLjK4AQPIAQD4AQGYAgOgAoMCwgIKEAAYsAMY1gQYR8ICDRAAGIAEGLADGEMYigXCAgoQABiABBgUGIcCwgIKEAAYgAQYQxiKBZgDAIgGAZAGCpIHAzEuMqAH_BCyBwMwLjK4B_0BwgcFMC4xLjLIBwuACAA&amp;sclient=gws-wiz-serp" xr:uid="{4AB55217-289A-4D2E-A730-771095A9BB44}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-05-07 12:16
</commit_message>
<xml_diff>
--- a/data/reserva de hoteis.xlsx
+++ b/data/reserva de hoteis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="799" documentId="13_ncr:1_{BFA144AC-8546-4E96-AEA1-F63AAF6602E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5A51CB8-4AE9-4660-A891-9BAE6332B824}"/>
+  <xr:revisionPtr revIDLastSave="817" documentId="13_ncr:1_{BFA144AC-8546-4E96-AEA1-F63AAF6602E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2252B741-32F7-46B3-9CC7-CD2BE5B1111E}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{72B7B767-51BF-4851-A118-4A4FFA047337}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">HOTEIS2025!$G$5:$O$716</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$507</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">HOTEIS2026!$G$5:$O$526</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'NÚMERO DE HOTEIS'!$B$2:$D$87</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6162" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6184" uniqueCount="693">
   <si>
     <t>DATA</t>
   </si>
@@ -34806,7 +34806,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="507" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="507" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G507" s="3">
         <v>46148</v>
       </c>
@@ -34829,7 +34829,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="508" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="508" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G508" s="3">
         <v>46148</v>
       </c>
@@ -34852,7 +34852,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="509" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="509" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G509" s="3">
         <v>46148</v>
       </c>
@@ -34875,7 +34875,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="510" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="510" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G510" s="3">
         <v>46148</v>
       </c>
@@ -34898,7 +34898,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="511" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="511" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G511" s="3">
         <v>46148</v>
       </c>
@@ -34921,7 +34921,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="512" spans="7:16" x14ac:dyDescent="0.25">
+    <row r="512" spans="7:16" hidden="1" x14ac:dyDescent="0.25">
       <c r="G512" s="3">
         <v>46148</v>
       </c>
@@ -34944,7 +34944,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="513" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="513" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G513" s="3">
         <v>46148</v>
       </c>
@@ -34967,7 +34967,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="514" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="514" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G514" s="3">
         <v>46148</v>
       </c>
@@ -34987,7 +34987,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="515" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="515" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G515" s="3">
         <v>46148</v>
       </c>
@@ -35007,7 +35007,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="516" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="516" spans="7:14" hidden="1" x14ac:dyDescent="0.25">
       <c r="G516" s="3">
         <v>46148</v>
       </c>
@@ -35025,6 +35025,146 @@
       </c>
       <c r="L516" s="1" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="517" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G517" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H517" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="I517" t="s">
+        <v>562</v>
+      </c>
+      <c r="N517">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="518" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G518" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H518" s="1" t="s">
+        <v>681</v>
+      </c>
+      <c r="I518" t="s">
+        <v>682</v>
+      </c>
+      <c r="N518">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="519" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G519" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H519" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="I519" t="s">
+        <v>683</v>
+      </c>
+      <c r="N519">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="520" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G520" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H520" s="1" t="s">
+        <v>684</v>
+      </c>
+      <c r="I520" t="s">
+        <v>516</v>
+      </c>
+      <c r="N520">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="521" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G521" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H521" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="I521" t="s">
+        <v>686</v>
+      </c>
+      <c r="N521">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="522" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G522" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H522" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="I522" t="s">
+        <v>685</v>
+      </c>
+      <c r="J522" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K522" s="10">
+        <v>190</v>
+      </c>
+      <c r="L522" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="N522">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="523" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G523" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H523" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="I523" t="s">
+        <v>688</v>
+      </c>
+      <c r="N523">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="524" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G524" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H524" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I524" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="525" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G525" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H525" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I525" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="526" spans="7:14" x14ac:dyDescent="0.25">
+      <c r="G526" s="3">
+        <v>46149</v>
+      </c>
+      <c r="H526" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I526" t="s">
+        <v>690</v>
       </c>
     </row>
     <row r="639" spans="6:6" x14ac:dyDescent="0.25">
@@ -35058,10 +35198,10 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="G5:O507" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
+  <autoFilter ref="G5:O526" xr:uid="{0BF69182-D7BE-468C-B7FF-43AE3F66B93B}">
     <filterColumn colId="0">
       <filters>
-        <dateGroupItem year="2026" month="5" dateTimeGrouping="month"/>
+        <dateGroupItem year="2026" month="5" day="7" dateTimeGrouping="day"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>